<commit_message>
Add NP-SP-03: Route Profitability Analysis — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -1,13 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Master Catalog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="NP-SP-03" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +60,22 @@
       <name val="Calibri"/>
       <color rgb="007F4F00"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="9">
@@ -129,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +184,30 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -683,13 +725,21 @@
           <t>Route Profitability Analysis</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr"/>
-      <c r="G5" s="10" t="inlineStr"/>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>network-planning-scheduling/schedule-planning/np-sp-03</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -4997,4 +5047,2540 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Airlines Process Catalog — Master L4 Row Catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Extract O&amp;D Revenue &amp; Booking Data</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal booking history, MIDT data feeds, BSP/ARC settlement files</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix by route, cabin class, and booking window</t>
+        </is>
+      </c>
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>Data extract completeness ≥99%; query SLA &lt;4 hrs</t>
+        </is>
+      </c>
+      <c r="L3" s="16" t="inlineStr">
+        <is>
+          <t>MIDT data covers only ~65% of bookings; direct/NDC channel bookings require separate aggregation from Altéa DCS, causing analyst reconciliation overhead</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Pull Route Operating Cost Data</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>General ledger actuals, cost centre allocations, fuel price feeds</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Direct operating cost per departure by route and aircraft type</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Cost data refresh lag &lt;24 hrs; CASM variance vs budget &lt;2%</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Fleet commonality (737 family) limits aircraft-type cost granularity; fuel hedging gains/losses allocated at entity level not route level, distorting route CASM</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Retrieve Competitive Fare Intelligence</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Competitor SSIM files, OAG traffic data, ATPCO fare tariff feeds</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Competitive fare matrix and capacity share by route</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Competitor fare coverage ≥90% of routes under review</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>LCC and ULCC competitors file fares with minimal lead time; ATPCO refresh cycle (2x weekly) creates stale data windows that allow mispriced response strategies</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate Data Completeness &amp; Reconcile</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix, cost extract, competitive data, Altéa PNR data</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled route data package; data quality scorecard</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Reconciliation exceptions &lt;1% of route-months; sign-off completed within 1 business day</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Cross-system reconciliation between Altéa settlement data and SAP GL actuals regularly surfaces timing differences of 3–5 days for interline and codeshare revenue</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Analyse Load Factor &amp; Yield by Route</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Reconciled route data package, cabin inventory records</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Load factor and yield report by route, DOW, and season</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>System-wide load factor target ≥83%; yield degradation alert threshold &gt;5% YoY</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Altéa NRM optimises at O&amp;D level; thin point-to-point routes with no connecting traffic receive less sophisticated demand modelling, leading to premature sell-down</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Model O&amp;D Traffic Spill &amp; Recapture</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Load factor report, O&amp;D demand signals, competitor capacity data</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Spill/recapture estimates; demand elasticity coefficients by route</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Spill model accuracy ≥88% vs actual post-departure; recapture rate assumption validated quarterly</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Pure point-to-point network means spilled passengers rarely recaptured on connecting itineraries; recapture assumptions borrowed from hub-and-spoke models overstate true recapture by 10–15%</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Assess Route Against Break-Even Load Factor</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Yield data, direct operating costs per ASM, average fare</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Break-even load factor by route; routes flagged for detailed cost review</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Break-even LF calculation completed for 100% of routes under review</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Break-even LF sensitive to fuel price assumptions; a ±10% fuel swing shifts break-even by 3–4 pp, requiring frequent scenario refreshes that strain analyst bandwidth</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Attribute Direct Operating Costs to Route</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Cost centre actuals, block hours by route, fuel consumption by tail</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Direct CASM (crew, fuel, maintenance, airport fees) per route</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Direct cost attribution covers ≥95% of route operating cost; CASM per ASM variance &lt;1.5¢ vs prior period</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Maintenance event timing distorts monthly route CASM; an A-check occurring mid-month inflates CASM for that route by 8–12%, masking underlying profitability</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Allocate Overhead &amp; Indirect Costs to Route</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Corporate overhead pools (IT, HR, HQ), fleet lease costs, depreciation schedules</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Fully-loaded CASM per route including overhead allocation</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Overhead allocation methodology reviewed annually; allocation variance &lt;3% across fleet</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>No universally agreed overhead allocation driver; switching from ASM-based to departure-based allocation changes route rankings by up to 15 positions, creating internal disagreement on route verdicts</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Compare CASM Against Fleet-Type Benchmark</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Fully-loaded CASM, benchmark CASM by 737 variant (700/800/MAX 8)</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>CASM variance report; routes flagged for gauge optimisation review</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Routes with CASM &gt;110% of fleet benchmark escalated for review</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>737-700 has ~18% higher CASM per ASM vs MAX 8; routes locked to -700 gauge due to gate constraints or runway length restrictions cannot benefit from gauge upgrades</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Build Route Contribution Margin P&amp;L Model</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix, direct CASM, overhead allocation, ancillary revenue estimates</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Route P&amp;L model: RASM, CASM, contribution margin, EBIT per route</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>P&amp;L model completed for 100% of routes under review; contribution margin &gt;0 for ≥85% of network routes</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary revenue (EarlyBird, upgraded boarding, baggage) not disaggregated at route level in Altéa; lump-sum allocation from corporate finance understates ancillary contribution on leisure-heavy routes by up to 20%</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Run Frequency &amp; Gauge Sensitivity Scenarios</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Route P&amp;L model, fleet assignment options, schedule constraints from SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Scenario comparison matrix: +1 freq, -1 freq, gauge-up, gauge-down, suspend</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>At least 3 scenarios modelled per underperforming route; scenario run time &lt;2 hrs per route</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Fleet commonality reduces gauge flexibility to 737-700 vs 737-800/MAX 8; slot-constrained airports (DCA, LGA) limit frequency increase scenarios regardless of P&amp;L outcome</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Assess Network Contribution &amp; Connectivity Value</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Scenario matrix, network connectivity model, Rapid Rewards contribution data</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Revised profitability ranking incorporating network externality value</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Network contribution adjustment applied to ≥100% of reviewed routes; connectivity premium &gt;5% of direct P&amp;L flagged for executive review</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Point-to-point model lacks hub feed economics; connectivity value difficult to quantify without connecting passenger data — WN does not sell connecting itineraries through GDS, limiting third-party validation</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Prepare Route Profitability Scorecard</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Route P&amp;L models, scenario outputs, competitive benchmarks</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Executive route profitability dashboard: RAG status, trend, strategic recommendation</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Scorecard delivered within 5 business days of data extract; dashboard refresh SLA &lt;1 hr</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Tableau dashboards sourced from AWS Redshift data lake; ETL pipeline latency of 6–8 hrs means executives sometimes review overnight decisions against stale figures</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Review Findings with Commercial Leadership</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Route profitability scorecard, RM yield forecast, Sales channel input</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Reviewed recommendation with leadership commentary; routes approved/deferred/escalated</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Leadership review completed within 10 business days of analysis; ≥90% of recommendations resolved without escalation to CEO</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management and Network Planning use different optimisation horizons (RM: 90-day, NP: 12-18 month); misalignment on route verdicts for routes in near-term yield recovery frequently causes review rework</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Document Decision &amp; Update Route Status</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Approved recommendation, leadership sign-off record</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Route status updated in SkyWORKS (Grow/Maintain/Reduce/Suspend); decision audit trail</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Route status update completed within 2 business days of approval; 100% of decisions documented with rationale</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS decision log is free-text; no structured field for profitability verdict — audit trail relies on manual documentation discipline, creating compliance risk during DOT reviews</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-03 — Route Profitability Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Route Profitability Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract O&amp;D Revenue &amp; Booking Data</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal booking history, MIDT data feeds, BSP/ARC settlement files</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix by route, cabin class, and booking window</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Data extract completeness ≥99%; query SLA &lt;4 hrs</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>MIDT data covers only ~65% of bookings; direct/NDC channel bookings require separate aggregation from Altéa DCS, causing analyst reconciliation overhead</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Pull Route Operating Cost Data</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>General ledger actuals, cost centre allocations, fuel price feeds</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Direct operating cost per departure by route and aircraft type</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Cost data refresh lag &lt;24 hrs; CASM variance vs budget &lt;2%</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Fleet commonality (737 family) limits aircraft-type cost granularity; fuel hedging gains/losses allocated at entity level not route level, distorting route CASM</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Retrieve Competitive Fare Intelligence</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Competitor SSIM files, OAG traffic data, ATPCO fare tariff feeds</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Competitive fare matrix and capacity share by route</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Competitor fare coverage ≥90% of routes under review</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>LCC and ULCC competitors file fares with minimal lead time; ATPCO refresh cycle (2x weekly) creates stale data windows that allow mispriced response strategies</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Validate Data Completeness &amp; Reconcile</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix, cost extract, competitive data, Altéa PNR data</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Reconciled route data package; data quality scorecard</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Reconciliation exceptions &lt;1% of route-months; sign-off completed within 1 business day</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Cross-system reconciliation between Altéa settlement data and SAP GL actuals regularly surfaces timing differences of 3–5 days for interline and codeshare revenue</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Analyse Load Factor &amp; Yield by Route</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled route data package, cabin inventory records</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Load factor and yield report by route, DOW, and season</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>System-wide load factor target ≥83%; yield degradation alert threshold &gt;5% YoY</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Altéa NRM optimises at O&amp;D level; thin point-to-point routes with no connecting traffic receive less sophisticated demand modelling, leading to premature sell-down</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Model O&amp;D Traffic Spill &amp; Recapture</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Load factor report, O&amp;D demand signals, competitor capacity data</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Spill/recapture estimates; demand elasticity coefficients by route</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Spill model accuracy ≥88% vs actual post-departure; recapture rate assumption validated quarterly</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Pure point-to-point network means spilled passengers rarely recaptured on connecting itineraries; recapture assumptions borrowed from hub-and-spoke models overstate true recapture by 10–15%</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Assess Route Against Break-Even Load Factor</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Yield data, direct operating costs per ASM, average fare</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Break-even load factor by route; routes flagged for detailed cost review</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Break-even LF calculation completed for 100% of routes under review</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Break-even LF sensitive to fuel price assumptions; a ±10% fuel swing shifts break-even by 3–4 pp, requiring frequent scenario refreshes that strain analyst bandwidth</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Attribute Direct Operating Costs to Route</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Cost centre actuals, block hours by route, fuel consumption by tail</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Direct CASM (crew, fuel, maintenance, airport fees) per route</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Direct cost attribution covers ≥95% of route operating cost; CASM per ASM variance &lt;1.5¢ vs prior period</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Maintenance event timing distorts monthly route CASM; an A-check occurring mid-month inflates CASM for that route by 8–12%, masking underlying profitability</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Allocate Overhead &amp; Indirect Costs to Route</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Corporate overhead pools (IT, HR, HQ), fleet lease costs, depreciation schedules</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Fully-loaded CASM per route including overhead allocation</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Overhead allocation methodology reviewed annually; allocation variance &lt;3% across fleet</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>No universally agreed overhead allocation driver; switching from ASM-based to departure-based allocation changes route rankings by up to 15 positions, creating internal disagreement on route verdicts</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Compare CASM Against Fleet-Type Benchmark</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Fully-loaded CASM, benchmark CASM by 737 variant (700/800/MAX 8)</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>CASM variance report; routes flagged for gauge optimisation review</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Routes with CASM &gt;110% of fleet benchmark escalated for review</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>737-700 has ~18% higher CASM per ASM vs MAX 8; routes locked to -700 gauge due to gate constraints or runway length restrictions cannot benefit from gauge upgrades</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Build Route Contribution Margin P&amp;L Model</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix, direct CASM, overhead allocation, ancillary revenue estimates</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Route P&amp;L model: RASM, CASM, contribution margin, EBIT per route</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>P&amp;L model completed for 100% of routes under review; contribution margin &gt;0 for ≥85% of network routes</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue (EarlyBird, upgraded boarding, baggage) not disaggregated at route level in Altéa; lump-sum allocation from corporate finance understates ancillary contribution on leisure-heavy routes by up to 20%</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Run Frequency &amp; Gauge Sensitivity Scenarios</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Route P&amp;L model, fleet assignment options, schedule constraints from SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Scenario comparison matrix: +1 freq, -1 freq, gauge-up, gauge-down, suspend</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>At least 3 scenarios modelled per underperforming route; scenario run time &lt;2 hrs per route</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Fleet commonality reduces gauge flexibility to 737-700 vs 737-800/MAX 8; slot-constrained airports (DCA, LGA) limit frequency increase scenarios regardless of P&amp;L outcome</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Assess Network Contribution &amp; Connectivity Value</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Scenario matrix, network connectivity model, Rapid Rewards contribution data</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Revised profitability ranking incorporating network externality value</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Network contribution adjustment applied to ≥100% of reviewed routes; connectivity premium &gt;5% of direct P&amp;L flagged for executive review</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Point-to-point model lacks hub feed economics; connectivity value difficult to quantify without connecting passenger data — WN does not sell connecting itineraries through GDS, limiting third-party validation</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Prepare Route Profitability Scorecard</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Route P&amp;L models, scenario outputs, competitive benchmarks</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Executive route profitability dashboard: RAG status, trend, strategic recommendation</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Scorecard delivered within 5 business days of data extract; dashboard refresh SLA &lt;1 hr</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Tableau dashboards sourced from AWS Redshift data lake; ETL pipeline latency of 6–8 hrs means executives sometimes review overnight decisions against stale figures</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Review Findings with Commercial Leadership</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Route profitability scorecard, RM yield forecast, Sales channel input</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Reviewed recommendation with leadership commentary; routes approved/deferred/escalated</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Leadership review completed within 10 business days of analysis; ≥90% of recommendations resolved without escalation to CEO</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management and Network Planning use different optimisation horizons (RM: 90-day, NP: 12-18 month); misalignment on route verdicts for routes in near-term yield recovery frequently causes review rework</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-03</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Route Profitability Analysis</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Document Decision &amp; Update Route Status</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Network Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Approved recommendation, leadership sign-off record</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Route status updated in SkyWORKS (Grow/Maintain/Reduce/Suspend); decision audit trail</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Route status update completed within 2 business days of approval; 100% of decisions documented with rationale</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS decision log is free-text; no structured field for profitability verdict — audit trail relies on manual documentation discipline, creating compliance risk during DOT reviews</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-04: Slot Coordination & Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Master Catalog" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="NP-SP-03" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NP-SP-04" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -762,13 +763,21 @@
           <t>Slot Coordination &amp; Management</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr"/>
-      <c r="G6" s="8" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>network-planning-scheduling/schedule-planning/np-sp-04</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -5055,7 +5064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6302,6 +6311,1302 @@
       <c r="N18" s="17" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Analyse seasonal schedule demand vs slot inventory</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Approved seasonal schedule build, prior-season slot inventory</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Slot gap analysis report identifying constrained O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Slot gap identification rate ≥95% before coordinator submission deadline</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST demand forecasts do not auto-reconcile with live coordinator slot libraries — manual cross-check required, introducing errors in high-frequency bank builds</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Classify constrained airports by IATA Level 2 / Level 3</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Slot gap analysis report, OAG airport level classification data</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Constrained airport register with Level 2/3 designation and coordinator contact</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>100% of Level 3 airports correctly classified before coordinator submission window opens</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>IATA airport level classification updates lag real-world congestion changes by up to one season; misclassification causes incorrect submission routing and missed deadlines</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Generate prioritised slot request register</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Constrained airport register, route profitability data from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Prioritised slot request register ranked by revenue impact</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Slot requests submitted ≥8 weeks before IATA coordination deadline</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Late submission forfeits priority queue position at 47% of Level 3 coordinators; SkyWORKS has no built-in deadline tracking for each coordinator's unique submission calendar</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Extract historical slot series from IATA CRS portal</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Prior-season SSIM files, coordinator portal access credentials</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Historical slot series inventory per airport with series reference codes</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>100% of historical series extracted before coordinator portal submission window closes</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS portal availability falls below 99.5% during peak submission windows; fallback is manual email-based SSIM exchange with no automated validation</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>Validate 80/20 utilisation rule compliance per series</t>
+        </is>
+      </c>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>Slot Compliance Analyst</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Historical slot series inventory, actual operations data from prior season</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Series compliance report with used/available ratio per airport per series</t>
+        </is>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>Grandfather right retention rate ≥98% of eligible series per IATA WSG</t>
+        </is>
+      </c>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>Operational disruptions (weather, ATC) erode utilisation ratios; airlines must file force majeure exemptions within 5 days of each triggering event — SkyWORKS does not auto-flag breaches in real time</t>
+        </is>
+      </c>
+      <c r="M23" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N23" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>File force majeure exemptions for at-risk series</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Series compliance report, confirmed disruption log with ATC/weather evidence</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>Accepted exemption filing per affected slot series</t>
+        </is>
+      </c>
+      <c r="K24" s="18" t="inlineStr">
+        <is>
+          <t>Exemption filed within 5 calendar days of triggering disruption event</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr">
+        <is>
+          <t>Missed exemption window results in permanent series loss with no appeals mechanism at most Level 3 airports; coordinator acceptance rates vary by region (EU coordinators accept ~82%, US FAA exempt)</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Generate SSIM-formatted SCR slot request messages</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Prioritised slot request register, validated historical series inventory</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>SSIM SCR message set ready for coordinator submission</t>
+        </is>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>SSIM file validation error rate &lt; 1% on first submission</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export requires manual field mapping for airports not in the standard IATA airport list; common source of format errors that delay acceptance by coordinator systems</t>
+        </is>
+      </c>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N25" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>Submit slot requests to each airport coordinator</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>SSIM SCR message set, coordinator portal credentials per airport</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="inlineStr">
+        <is>
+          <t>Submitted SCR messages with coordinator receipt confirmations</t>
+        </is>
+      </c>
+      <c r="K26" s="18" t="inlineStr">
+        <is>
+          <t>100% of requests submitted before each coordinator's unique deadline</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
+          <t>Airport coordinators (ACNUSA, NATS, DFS, FAA, etc.) each operate different portal UIs with no single API standard; multi-airport submissions require manual portal navigation per coordinator</t>
+        </is>
+      </c>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Evaluate initial slot allocation vs requested schedule</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Coordinator SCT (slot confirmation) messages, original slot request register</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>Allocation gap report identifying unmatched or partially matched requests</t>
+        </is>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Allocation match rate ≥85% of requested slots in initial SCT response</t>
+        </is>
+      </c>
+      <c r="L27" s="16" t="inlineStr">
+        <is>
+          <t>Coordinators allocate on grandfather-then-new-entrant priority; late filers receive only residual slots, which are frequently at off-peak times incompatible with planned bank structures</t>
+        </is>
+      </c>
+      <c r="M27" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N27" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Prepare negotiation brief for IATA slot conference</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>Allocation gap report, network simulation scenarios from SkySYM</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="inlineStr">
+        <is>
+          <t>Negotiation brief with ranked alternative slot windows and revenue impact estimates</t>
+        </is>
+      </c>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>Brief finalised ≥2 weeks before IATA slot conference opening date</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM scenario export does not auto-generate slot swap proposals; analyst must manually map network simulation outputs to coordinator slot pool data, taking 3–5 days per conference cycle</t>
+        </is>
+      </c>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>Negotiate slot swaps and alternatives at conference</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>Negotiation brief, coordinator available slot pool published at conference</t>
+        </is>
+      </c>
+      <c r="J29" s="16" t="inlineStr">
+        <is>
+          <t>Agreed slot swaps or confirmed alternative allocations</t>
+        </is>
+      </c>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>≥70% of critical slot gaps (top 10 revenue routes) resolved at conference</t>
+        </is>
+      </c>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>Bilateral swap negotiations are blocked when the counterparty airline holds conflicting grandfather claims on the same series; coordinator cannot force swaps without both parties' consent under IATA WSG §9</t>
+        </is>
+      </c>
+      <c r="M29" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N29" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>File appeal for unresolved critical slot gaps</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>Unresolved slot gap list post-conference, coordinator appeal process documentation</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
+        <is>
+          <t>Formal appeal filing or coordinator mediation request</t>
+        </is>
+      </c>
+      <c r="K30" s="18" t="inlineStr">
+        <is>
+          <t>Appeal response received within 5 business days of filing</t>
+        </is>
+      </c>
+      <c r="L30" s="18" t="inlineStr">
+        <is>
+          <t>Appeal panels have no binding authority at most coordinators; outcomes are advisory only, leaving airlines with no recourse if coordinator declines to intervene in grandfather disputes</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Confirm final slot allocation and accept coordinator offer</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Final SCT messages from all coordinators including post-conference revisions</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>Accepted slot confirmation records per airport per series</t>
+        </is>
+      </c>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>100% of confirmed slots acknowledged within 24h of coordinator receipt</t>
+        </is>
+      </c>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>Coordinator systems deliver SCT messages in overnight batch files; missed or delayed messages require manual reconciliation with coordinator helpdesk, often taking 2–3 business days to resolve</t>
+        </is>
+      </c>
+      <c r="M31" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N31" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>Integrate confirmed slots into SkyWORKS schedule build</t>
+        </is>
+      </c>
+      <c r="G32" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>Accepted slot confirmation records, current SkyWORKS seasonal schedule</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr">
+        <is>
+          <t>Updated SkyWORKS schedule with slot-validated departure and arrival times per flight leg</t>
+        </is>
+      </c>
+      <c r="K32" s="18" t="inlineStr">
+        <is>
+          <t>Schedule-to-slot reconciliation accuracy ≥99.5% before SSIM publication</t>
+        </is>
+      </c>
+      <c r="L32" s="18" t="inlineStr">
+        <is>
+          <t>Slot times and SkyWORKS schedule times drift due to timezone and DST mapping errors during SSIM import; DST boundary airports (e.g. LORD, EIDW) are a recurring source of off-by-one-hour faults</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>Publish season SSIM file to GDS channels and PSS</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <t>Slot-validated SkyWORKS schedule</t>
+        </is>
+      </c>
+      <c r="J33" s="16" t="inlineStr">
+        <is>
+          <t>Published SSIM file distributed to Sabre GDS, Travelport GDS, Amadeus GDS, and Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>SSIM distributed to all GDS ≤72h after final coordinator confirmation</t>
+        </is>
+      </c>
+      <c r="L33" s="16" t="inlineStr">
+        <is>
+          <t>GDS distribution from SkyWORKS is fire-and-forget with no real-time ACK; distribution failures are silent and only detected when downstream booking discrepancies surface 24–48h later</t>
+        </is>
+      </c>
+      <c r="M33" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N33" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>Monitor weekly slot utilisation against 80% threshold</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="inlineStr">
+        <is>
+          <t>Slot Compliance Analyst</t>
+        </is>
+      </c>
+      <c r="H34" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>Weekly actual operations data, slot series inventory with coordinator reference codes</t>
+        </is>
+      </c>
+      <c r="J34" s="18" t="inlineStr">
+        <is>
+          <t>Weekly slot utilisation compliance report per series per airport</t>
+        </is>
+      </c>
+      <c r="K34" s="18" t="inlineStr">
+        <is>
+          <t>Slot series utilisation ≥80% per IATA WSG standard throughout season</t>
+        </is>
+      </c>
+      <c r="L34" s="18" t="inlineStr">
+        <is>
+          <t>Operational cancellations and schedule swaps erode utilisation without triggering automated alerts in SkyWORKS; compliance analysts must run manual SQL queries against ops data to compute rolling utilisation ratios</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>Return or swap underperforming slot series</t>
+        </is>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Utilisation compliance report identifying series below 80%, coordinator return deadlines</t>
+        </is>
+      </c>
+      <c r="J35" s="16" t="inlineStr">
+        <is>
+          <t>Slot return confirmations or approved swap records per series</t>
+        </is>
+      </c>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>Slot returns submitted ≥48h before departure per IATA WSG in-season return deadline</t>
+        </is>
+      </c>
+      <c r="L35" s="16" t="inlineStr">
+        <is>
+          <t>Late returns are forfeited to the slot pool with no recovery; repeated late-return flags accumulate as coordinator penalty records that reduce priority scoring in subsequent season bids</t>
+        </is>
+      </c>
+      <c r="M35" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N35" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>Execute ad-hoc slot swaps for operational recovery</t>
+        </is>
+      </c>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>Operations disruption report, coordinator available slot pool for swap</t>
+        </is>
+      </c>
+      <c r="J36" s="18" t="inlineStr">
+        <is>
+          <t>Ad-hoc swap confirmation and updated slot record in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="K36" s="18" t="inlineStr">
+        <is>
+          <t>Ad-hoc swap processed within 2h of disruption notification during coordinator office hours</t>
+        </is>
+      </c>
+      <c r="L36" s="18" t="inlineStr">
+        <is>
+          <t>Coordinator swap availability is limited to office hours (typically 07:00–19:00 local); out-of-hours disruptions at Level 3 airports have no swap mechanism, forcing cancellation or slot violation</t>
+        </is>
+      </c>
+      <c r="M36" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -7583,4 +8888,1420 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-04 — Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Analyse seasonal schedule demand vs slot inventory</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Approved seasonal schedule build, prior-season slot inventory</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Slot gap analysis report identifying constrained O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Slot gap identification rate ≥95% before coordinator submission deadline</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST demand forecasts do not auto-reconcile with live coordinator slot libraries — manual cross-check required, introducing errors in high-frequency bank builds</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Classify constrained airports by IATA Level 2 / Level 3</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Slot gap analysis report, OAG airport level classification data</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Constrained airport register with Level 2/3 designation and coordinator contact</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>100% of Level 3 airports correctly classified before coordinator submission window opens</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>IATA airport level classification updates lag real-world congestion changes by up to one season; misclassification causes incorrect submission routing and missed deadlines</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Generate prioritised slot request register</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Constrained airport register, route profitability data from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised slot request register ranked by revenue impact</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Slot requests submitted ≥8 weeks before IATA coordination deadline</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Late submission forfeits priority queue position at 47% of Level 3 coordinators; SkyWORKS has no built-in deadline tracking for each coordinator's unique submission calendar</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Extract historical slot series from IATA CRS portal</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Prior-season SSIM files, coordinator portal access credentials</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Historical slot series inventory per airport with series reference codes</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>100% of historical series extracted before coordinator portal submission window closes</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS portal availability falls below 99.5% during peak submission windows; fallback is manual email-based SSIM exchange with no automated validation</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Validate 80/20 utilisation rule compliance per series</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Slot Compliance Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Historical slot series inventory, actual operations data from prior season</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Series compliance report with used/available ratio per airport per series</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Grandfather right retention rate ≥98% of eligible series per IATA WSG</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Operational disruptions (weather, ATC) erode utilisation ratios; airlines must file force majeure exemptions within 5 days of each triggering event — SkyWORKS does not auto-flag breaches in real time</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>File force majeure exemptions for at-risk series</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Series compliance report, confirmed disruption log with ATC/weather evidence</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Accepted exemption filing per affected slot series</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Exemption filed within 5 calendar days of triggering disruption event</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Missed exemption window results in permanent series loss with no appeals mechanism at most Level 3 airports; coordinator acceptance rates vary by region (EU coordinators accept ~82%, US FAA exempt)</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Generate SSIM-formatted SCR slot request messages</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised slot request register, validated historical series inventory</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>SSIM SCR message set ready for coordinator submission</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>SSIM file validation error rate &lt; 1% on first submission</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export requires manual field mapping for airports not in the standard IATA airport list; common source of format errors that delay acceptance by coordinator systems</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Submit slot requests to each airport coordinator</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>SSIM SCR message set, coordinator portal credentials per airport</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Submitted SCR messages with coordinator receipt confirmations</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>100% of requests submitted before each coordinator's unique deadline</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Airport coordinators (ACNUSA, NATS, DFS, FAA, etc.) each operate different portal UIs with no single API standard; multi-airport submissions require manual portal navigation per coordinator</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate initial slot allocation vs requested schedule</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Coordinator SCT (slot confirmation) messages, original slot request register</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Allocation gap report identifying unmatched or partially matched requests</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Allocation match rate ≥85% of requested slots in initial SCT response</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Coordinators allocate on grandfather-then-new-entrant priority; late filers receive only residual slots, which are frequently at off-peak times incompatible with planned bank structures</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Prepare negotiation brief for IATA slot conference</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Allocation gap report, network simulation scenarios from SkySYM</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Negotiation brief with ranked alternative slot windows and revenue impact estimates</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Brief finalised ≥2 weeks before IATA slot conference opening date</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario export does not auto-generate slot swap proposals; analyst must manually map network simulation outputs to coordinator slot pool data, taking 3–5 days per conference cycle</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Negotiate slot swaps and alternatives at conference</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Negotiation brief, coordinator available slot pool published at conference</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Agreed slot swaps or confirmed alternative allocations</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>≥70% of critical slot gaps (top 10 revenue routes) resolved at conference</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Bilateral swap negotiations are blocked when the counterparty airline holds conflicting grandfather claims on the same series; coordinator cannot force swaps without both parties' consent under IATA WSG §9</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>File appeal for unresolved critical slot gaps</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Unresolved slot gap list post-conference, coordinator appeal process documentation</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Formal appeal filing or coordinator mediation request</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Appeal response received within 5 business days of filing</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Appeal panels have no binding authority at most coordinators; outcomes are advisory only, leaving airlines with no recourse if coordinator declines to intervene in grandfather disputes</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Confirm final slot allocation and accept coordinator offer</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Final SCT messages from all coordinators including post-conference revisions</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Accepted slot confirmation records per airport per series</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>100% of confirmed slots acknowledged within 24h of coordinator receipt</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Coordinator systems deliver SCT messages in overnight batch files; missed or delayed messages require manual reconciliation with coordinator helpdesk, often taking 2–3 business days to resolve</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Integrate confirmed slots into SkyWORKS schedule build</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Accepted slot confirmation records, current SkyWORKS seasonal schedule</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Updated SkyWORKS schedule with slot-validated departure and arrival times per flight leg</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule-to-slot reconciliation accuracy ≥99.5% before SSIM publication</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Slot times and SkyWORKS schedule times drift due to timezone and DST mapping errors during SSIM import; DST boundary airports (e.g. LORD, EIDW) are a recurring source of off-by-one-hour faults</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Publish season SSIM file to GDS channels and PSS</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Slot-validated SkyWORKS schedule</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Published SSIM file distributed to Sabre GDS, Travelport GDS, Amadeus GDS, and Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>SSIM distributed to all GDS ≤72h after final coordinator confirmation</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>GDS distribution from SkyWORKS is fire-and-forget with no real-time ACK; distribution failures are silent and only detected when downstream booking discrepancies surface 24–48h later</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Monitor weekly slot utilisation against 80% threshold</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Slot Compliance Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Weekly actual operations data, slot series inventory with coordinator reference codes</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Weekly slot utilisation compliance report per series per airport</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Slot series utilisation ≥80% per IATA WSG standard throughout season</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Operational cancellations and schedule swaps erode utilisation without triggering automated alerts in SkyWORKS; compliance analysts must run manual SQL queries against ops data to compute rolling utilisation ratios</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Return or swap underperforming slot series</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Utilisation compliance report identifying series below 80%, coordinator return deadlines</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Slot return confirmations or approved swap records per series</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Slot returns submitted ≥48h before departure per IATA WSG in-season return deadline</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Late returns are forfeited to the slot pool with no recovery; repeated late-return flags accumulate as coordinator penalty records that reduce priority scoring in subsequent season bids</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-04</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination &amp; Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Execute ad-hoc slot swaps for operational recovery</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Operations disruption report, coordinator available slot pool for swap</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Ad-hoc swap confirmation and updated slot record in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Ad-hoc swap processed within 2h of disruption notification during coordinator office hours</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Coordinator swap availability is limited to office hours (typically 07:00–19:00 local); out-of-hours disruptions at Level 3 airports have no swap mechanism, forcing cancellation or slot violation</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-05: Codeshare & Interline Schedule Planning — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Master Catalog" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="NP-SP-03" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="NP-SP-04" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="NP-SP-05" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -800,13 +801,21 @@
           <t>Codeshare &amp; Interline Schedule Planning</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-05</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -5064,7 +5073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11421,6 +11430,1158 @@
         </is>
       </c>
       <c r="N89" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D90" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E90" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>Identify codeshare &amp; interline partner candidates</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Manager</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I90" s="18" t="inlineStr">
+        <is>
+          <t>Network gap analysis, O&amp;D demand data, commercial strategy brief</t>
+        </is>
+      </c>
+      <c r="J90" s="18" t="inlineStr">
+        <is>
+          <t>Ranked partner shortlist with O&amp;D overlap scores</t>
+        </is>
+      </c>
+      <c r="K90" s="18" t="inlineStr">
+        <is>
+          <t>Min 5 candidate partners assessed per planning cycle</t>
+        </is>
+      </c>
+      <c r="L90" s="18" t="inlineStr">
+        <is>
+          <t>OAG data latency (updated weekly) may miss recent partner schedule changes; analysts must cross-check with SSIM direct feeds</t>
+        </is>
+      </c>
+      <c r="M90" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N90" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E91" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F91" s="16" t="inlineStr">
+        <is>
+          <t>Analyse partner O&amp;D network overlap and revenue potential</t>
+        </is>
+      </c>
+      <c r="G91" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H91" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I91" s="16" t="inlineStr">
+        <is>
+          <t>Partner SSIM schedule, OAG market share data, own O&amp;D traffic database</t>
+        </is>
+      </c>
+      <c r="J91" s="16" t="inlineStr">
+        <is>
+          <t>Revenue opportunity model: incremental pax and yield per route</t>
+        </is>
+      </c>
+      <c r="K91" s="16" t="inlineStr">
+        <is>
+          <t>Projected incremental load factor contribution ≥3 ppts on thin O&amp;D routes</t>
+        </is>
+      </c>
+      <c r="L91" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D demand models assume point-to-point flows; interline connecting itineraries require manual traffic splitting adjustments</t>
+        </is>
+      </c>
+      <c r="M91" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N91" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E92" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>Verify IIA and SPA agreement status with legal</t>
+        </is>
+      </c>
+      <c r="G92" s="18" t="inlineStr">
+        <is>
+          <t>Interline Agreements Specialist</t>
+        </is>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I92" s="18" t="inlineStr">
+        <is>
+          <t>Partner carrier code, IATA IIA registry extract</t>
+        </is>
+      </c>
+      <c r="J92" s="18" t="inlineStr">
+        <is>
+          <t>Agreement status confirmation (IIA active / SPA in place / none)</t>
+        </is>
+      </c>
+      <c r="K92" s="18" t="inlineStr">
+        <is>
+          <t>Agreement status verified within 2 business days of partner selection</t>
+        </is>
+      </c>
+      <c r="L92" s="18" t="inlineStr">
+        <is>
+          <t>IATA IIA registry updates lag actual bilateral negotiations by up to 30 days; expired SPAs may not be flagged in the finance system</t>
+        </is>
+      </c>
+      <c r="M92" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N92" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>Request SSIM schedule data feed from partner airline</t>
+        </is>
+      </c>
+      <c r="G93" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H93" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I93" s="16" t="inlineStr">
+        <is>
+          <t>Partner carrier approval, IATA SSIM Chapter 7 format specification</t>
+        </is>
+      </c>
+      <c r="J93" s="16" t="inlineStr">
+        <is>
+          <t>Received partner SSIM file imported into SkyWORKS schedule database</t>
+        </is>
+      </c>
+      <c r="K93" s="16" t="inlineStr">
+        <is>
+          <t>SSIM file received and validated within 5 business days of partner agreement</t>
+        </is>
+      </c>
+      <c r="L93" s="16" t="inlineStr">
+        <is>
+          <t>Non-IATA partners (charter, regional) may supply non-standard SSIM variants requiring manual field mapping before SkyWORKS can import</t>
+        </is>
+      </c>
+      <c r="M93" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N93" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E94" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>Validate connection times against airport MCT tables</t>
+        </is>
+      </c>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I94" s="18" t="inlineStr">
+        <is>
+          <t>Partner SSIM flights, own schedule, IATA MCT database per airport</t>
+        </is>
+      </c>
+      <c r="J94" s="18" t="inlineStr">
+        <is>
+          <t>MCT compliance report: list of connections meeting/failing minimum connect time</t>
+        </is>
+      </c>
+      <c r="K94" s="18" t="inlineStr">
+        <is>
+          <t>100% of proposed connect itineraries MCT-compliant before GDS loading</t>
+        </is>
+      </c>
+      <c r="L94" s="18" t="inlineStr">
+        <is>
+          <t>MCT tables vary by terminal and domestic/international split; SkyWORKS uses airport-level MCTs and may not reflect terminal reassignments after gate changes</t>
+        </is>
+      </c>
+      <c r="M94" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N94" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F95" s="16" t="inlineStr">
+        <is>
+          <t>Resolve schedule conflicts via SSIM SCR negotiation</t>
+        </is>
+      </c>
+      <c r="G95" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H95" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I95" s="16" t="inlineStr">
+        <is>
+          <t>MCT non-compliance list, partner contact, SSIM SCR message format</t>
+        </is>
+      </c>
+      <c r="J95" s="16" t="inlineStr">
+        <is>
+          <t>Revised partner or own schedule achieving MCT compliance</t>
+        </is>
+      </c>
+      <c r="K95" s="16" t="inlineStr">
+        <is>
+          <t>Schedule conflicts resolved within 10 business days; &lt;5% of proposed connections requiring rescheduling</t>
+        </is>
+      </c>
+      <c r="L95" s="16" t="inlineStr">
+        <is>
+          <t>Partner airlines prioritise own network optimisation; schedule adjustment requests are often rejected or delayed beyond SSIM submission deadlines (D-180)</t>
+        </is>
+      </c>
+      <c r="M95" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N95" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="30" customHeight="1">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E96" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>Confirm aligned codeshare schedule and flight numbering</t>
+        </is>
+      </c>
+      <c r="G96" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I96" s="18" t="inlineStr">
+        <is>
+          <t>MCT-compliant schedule, codeshare designator allocation (IATA two-letter code)</t>
+        </is>
+      </c>
+      <c r="J96" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare flight number series filed in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="K96" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare flight numbers registered with IATA within 7 days of schedule confirmation</t>
+        </is>
+      </c>
+      <c r="L96" s="18" t="inlineStr">
+        <is>
+          <t>Duplicate flight number conflicts with own metal flights require manual deconfliction; SkyWORKS does not auto-detect cross-carrier designator clashes</t>
+        </is>
+      </c>
+      <c r="M96" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N96" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E97" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F97" s="16" t="inlineStr">
+        <is>
+          <t>Configure block-space or free-sale inventory allocation</t>
+        </is>
+      </c>
+      <c r="G97" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H97" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altea PSS</t>
+        </is>
+      </c>
+      <c r="I97" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare schedule, capacity agreement (block vs free-sale terms)</t>
+        </is>
+      </c>
+      <c r="J97" s="16" t="inlineStr">
+        <is>
+          <t>Inventory allocation rules loaded into Altéa PSS for codeshare flight numbers</t>
+        </is>
+      </c>
+      <c r="K97" s="16" t="inlineStr">
+        <is>
+          <t>Block-space utilisation target ≥70% within 30 days of schedule launch</t>
+        </is>
+      </c>
+      <c r="L97" s="16" t="inlineStr">
+        <is>
+          <t>Free-sale arrangements require real-time availability sharing via IATA Type B TELETYPE or PADIS; latency &gt;500ms causes ghost availability in partner booking systems</t>
+        </is>
+      </c>
+      <c r="M97" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N97" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C98" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E98" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>File interline prorate and SPA agreements via ATPCO</t>
+        </is>
+      </c>
+      <c r="G98" s="18" t="inlineStr">
+        <is>
+          <t>Interline Agreements Specialist</t>
+        </is>
+      </c>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I98" s="18" t="inlineStr">
+        <is>
+          <t>Bilateral prorate formula, revenue split percentage, SPA effective date</t>
+        </is>
+      </c>
+      <c r="J98" s="18" t="inlineStr">
+        <is>
+          <t>Published ATPCO prorate agreement record accessible by all GDS and PSS</t>
+        </is>
+      </c>
+      <c r="K98" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO filing effective within 24 hours of D-1 activation date; 0 unpriced itineraries at launch</t>
+        </is>
+      </c>
+      <c r="L98" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO prorate amendments require 3–5 business days for GDS propagation; last-minute schedule changes can create gaps where interline fares are unresolvable</t>
+        </is>
+      </c>
+      <c r="M98" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N98" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D99" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F99" s="16" t="inlineStr">
+        <is>
+          <t>Validate fare combinability and through-fare rules in PSS</t>
+        </is>
+      </c>
+      <c r="G99" s="16" t="inlineStr">
+        <is>
+          <t>Fares &amp; Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H99" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altea PSS</t>
+        </is>
+      </c>
+      <c r="I99" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO prorate records, own published fares, partner fare tariff</t>
+        </is>
+      </c>
+      <c r="J99" s="16" t="inlineStr">
+        <is>
+          <t>Validated combinability matrix: list of valid fare combinations per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K99" s="16" t="inlineStr">
+        <is>
+          <t>100% of marketed O&amp;D pairs have at least one priceable interline itinerary at launch</t>
+        </is>
+      </c>
+      <c r="L99" s="16" t="inlineStr">
+        <is>
+          <t>Global Indicator and Routing restrictions in ATPCO records frequently cause combinability failures for multi-sector interline itineraries that are not caught until passenger booking attempts</t>
+        </is>
+      </c>
+      <c r="M99" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N99" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C100" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E100" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="inlineStr">
+        <is>
+          <t>Load codeshare designators into GDS participant tables</t>
+        </is>
+      </c>
+      <c r="G100" s="18" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H100" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I100" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare flight numbers, operating carrier codes, effective/discontinue dates</t>
+        </is>
+      </c>
+      <c r="J100" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare flights live in Sabre, Travelport, and Amadeus GDS participant tables</t>
+        </is>
+      </c>
+      <c r="K100" s="18" t="inlineStr">
+        <is>
+          <t>GDS loading complete ≥14 days before first codeshare departure</t>
+        </is>
+      </c>
+      <c r="L100" s="18" t="inlineStr">
+        <is>
+          <t>Each GDS has separate participant-table submission portals with different lead-time requirements (Sabre: 14 days, Travelport: 10 days, Amadeus GDS: 7 days); misaligned loading creates uneven availability windows</t>
+        </is>
+      </c>
+      <c r="M100" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N100" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="30" customHeight="1">
+      <c r="A101" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F101" s="16" t="inlineStr">
+        <is>
+          <t>Validate end-to-end booking and ticketing path in GDS</t>
+        </is>
+      </c>
+      <c r="G101" s="16" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H101" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I101" s="16" t="inlineStr">
+        <is>
+          <t>Live GDS participant table entries, test PNR scenario set</t>
+        </is>
+      </c>
+      <c r="J101" s="16" t="inlineStr">
+        <is>
+          <t>UAT sign-off: booking, pricing, and ticketing confirmed for all O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K101" s="16" t="inlineStr">
+        <is>
+          <t>Zero pricing errors in UAT across 100% of marketed O&amp;D pairs before go-live</t>
+        </is>
+      </c>
+      <c r="L101" s="16" t="inlineStr">
+        <is>
+          <t>Travelport Galileo and Worldspan display codeshare availability differently from Sabre; availability masking rules may suppress partner availability in certain agencies without explicit GDS-specific configuration</t>
+        </is>
+      </c>
+      <c r="M101" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N101" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E102" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>Activate NDC API connection for partner direct-channel booking</t>
+        </is>
+      </c>
+      <c r="G102" s="18" t="inlineStr">
+        <is>
+          <t>Digital Distribution Manager</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I102" s="18" t="inlineStr">
+        <is>
+          <t>Partner NDC Level 3 certification status, API credential exchange</t>
+        </is>
+      </c>
+      <c r="J102" s="18" t="inlineStr">
+        <is>
+          <t>Live NDC offers including codeshare itineraries available via partner direct channel</t>
+        </is>
+      </c>
+      <c r="K102" s="18" t="inlineStr">
+        <is>
+          <t>NDC channel contributing ≥10% of codeshare bookings within 90 days of launch</t>
+        </is>
+      </c>
+      <c r="L102" s="18" t="inlineStr">
+        <is>
+          <t>Many regional and medium-haul interline partners are not NDC Level 3 certified; interline itineraries in NDC require bilateral offer/order linking that is not yet standardised across vendors</t>
+        </is>
+      </c>
+      <c r="M102" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N102" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>Brief operations and customer service on interline procedures</t>
+        </is>
+      </c>
+      <c r="G103" s="16" t="inlineStr">
+        <is>
+          <t>Ground Operations Manager</t>
+        </is>
+      </c>
+      <c r="H103" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I103" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare operating procedures manual, baggage interline agreement, reaccommodation policy</t>
+        </is>
+      </c>
+      <c r="J103" s="16" t="inlineStr">
+        <is>
+          <t>Briefed airport teams; interline baggage rules loaded into SITA AMS</t>
+        </is>
+      </c>
+      <c r="K103" s="16" t="inlineStr">
+        <is>
+          <t>100% of affected airport stations briefed ≥7 days before first codeshare departure</t>
+        </is>
+      </c>
+      <c r="L103" s="16" t="inlineStr">
+        <is>
+          <t>Interline baggage tag reconciliation between dissimilar PSS platforms (e.g. Altéa vs Sabre PSS) causes baggage misrouting; SITA AMS does not auto-validate cross-carrier bag tags at transfer points</t>
+        </is>
+      </c>
+      <c r="M103" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N103" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E104" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="inlineStr">
+        <is>
+          <t>Monitor codeshare booking ramp-up and yield metrics</t>
+        </is>
+      </c>
+      <c r="G104" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>Daily PNR booking data, codeshare flight segment reports from Altéa</t>
+        </is>
+      </c>
+      <c r="J104" s="18" t="inlineStr">
+        <is>
+          <t>Weekly performance dashboard: pax volume, yield, load factor by O&amp;D and partner</t>
+        </is>
+      </c>
+      <c r="K104" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare load factor ≥70% by week 4 post-launch; interline yield within 5% of target prorate</t>
+        </is>
+      </c>
+      <c r="L104" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM O&amp;D attribution for codeshare legs requires manual segment-level override; automated RM bid-price optimisation does not natively distinguish codeshare pax from own-metal pax in mixed itineraries</t>
+        </is>
+      </c>
+      <c r="M104" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N104" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E105" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>Conduct 90-day post-launch performance review</t>
+        </is>
+      </c>
+      <c r="G105" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H105" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I105" s="16" t="inlineStr">
+        <is>
+          <t>90-day pax and revenue actuals, prorate settlement statements, partner capacity data</t>
+        </is>
+      </c>
+      <c r="J105" s="16" t="inlineStr">
+        <is>
+          <t>Performance review report with recommendations: expand, renegotiate, or discontinue</t>
+        </is>
+      </c>
+      <c r="K105" s="16" t="inlineStr">
+        <is>
+          <t>Incremental revenue per ASK (RASK) contribution ≥2% above baseline on target O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="L105" s="16" t="inlineStr">
+        <is>
+          <t>Prorate settlement data from IATA BSP/ACH arrives 60–90 days in arrears, making 90-day review reliant on estimated yields; actual margin impact may not be known until Q2 following launch</t>
+        </is>
+      </c>
+      <c r="M105" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N105" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -14120,4 +15281,1276 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-05 — Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Identify codeshare &amp; interline partner candidates</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Manager</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Network gap analysis, O&amp;D demand data, commercial strategy brief</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Ranked partner shortlist with O&amp;D overlap scores</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Min 5 candidate partners assessed per planning cycle</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>OAG data latency (updated weekly) may miss recent partner schedule changes; analysts must cross-check with SSIM direct feeds</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Analyse partner O&amp;D network overlap and revenue potential</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Partner SSIM schedule, OAG market share data, own O&amp;D traffic database</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue opportunity model: incremental pax and yield per route</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Projected incremental load factor contribution ≥3 ppts on thin O&amp;D routes</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D demand models assume point-to-point flows; interline connecting itineraries require manual traffic splitting adjustments</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Verify IIA and SPA agreement status with legal</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Interline Agreements Specialist</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Partner carrier code, IATA IIA registry extract</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Agreement status confirmation (IIA active / SPA in place / none)</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Agreement status verified within 2 business days of partner selection</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>IATA IIA registry updates lag actual bilateral negotiations by up to 30 days; expired SPAs may not be flagged in the finance system</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Request SSIM schedule data feed from partner airline</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Partner carrier approval, IATA SSIM Chapter 7 format specification</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Received partner SSIM file imported into SkyWORKS schedule database</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>SSIM file received and validated within 5 business days of partner agreement</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Non-IATA partners (charter, regional) may supply non-standard SSIM variants requiring manual field mapping before SkyWORKS can import</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Validate connection times against airport MCT tables</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Partner SSIM flights, own schedule, IATA MCT database per airport</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>MCT compliance report: list of connections meeting/failing minimum connect time</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>100% of proposed connect itineraries MCT-compliant before GDS loading</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>MCT tables vary by terminal and domestic/international split; SkyWORKS uses airport-level MCTs and may not reflect terminal reassignments after gate changes</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Resolve schedule conflicts via SSIM SCR negotiation</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>MCT non-compliance list, partner contact, SSIM SCR message format</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Revised partner or own schedule achieving MCT compliance</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule conflicts resolved within 10 business days; &lt;5% of proposed connections requiring rescheduling</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Partner airlines prioritise own network optimisation; schedule adjustment requests are often rejected or delayed beyond SSIM submission deadlines (D-180)</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Confirm aligned codeshare schedule and flight numbering</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>MCT-compliant schedule, codeshare designator allocation (IATA two-letter code)</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare flight number series filed in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare flight numbers registered with IATA within 7 days of schedule confirmation</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Duplicate flight number conflicts with own metal flights require manual deconfliction; SkyWORKS does not auto-detect cross-carrier designator clashes</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Configure block-space or free-sale inventory allocation</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altea PSS</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare schedule, capacity agreement (block vs free-sale terms)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Inventory allocation rules loaded into Altéa PSS for codeshare flight numbers</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Block-space utilisation target ≥70% within 30 days of schedule launch</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Free-sale arrangements require real-time availability sharing via IATA Type B TELETYPE or PADIS; latency &gt;500ms causes ghost availability in partner booking systems</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>File interline prorate and SPA agreements via ATPCO</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Interline Agreements Specialist</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Bilateral prorate formula, revenue split percentage, SPA effective date</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Published ATPCO prorate agreement record accessible by all GDS and PSS</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO filing effective within 24 hours of D-1 activation date; 0 unpriced itineraries at launch</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO prorate amendments require 3–5 business days for GDS propagation; last-minute schedule changes can create gaps where interline fares are unresolvable</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Validate fare combinability and through-fare rules in PSS</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Fares &amp; Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altea PSS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO prorate records, own published fares, partner fare tariff</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Validated combinability matrix: list of valid fare combinations per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>100% of marketed O&amp;D pairs have at least one priceable interline itinerary at launch</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Global Indicator and Routing restrictions in ATPCO records frequently cause combinability failures for multi-sector interline itineraries that are not caught until passenger booking attempts</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Load codeshare designators into GDS participant tables</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed codeshare flight numbers, operating carrier codes, effective/discontinue dates</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare flights live in Sabre, Travelport, and Amadeus GDS participant tables</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>GDS loading complete ≥14 days before first codeshare departure</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Each GDS has separate participant-table submission portals with different lead-time requirements (Sabre: 14 days, Travelport: 10 days, Amadeus GDS: 7 days); misaligned loading creates uneven availability windows</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Validate end-to-end booking and ticketing path in GDS</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Live GDS participant table entries, test PNR scenario set</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>UAT sign-off: booking, pricing, and ticketing confirmed for all O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Zero pricing errors in UAT across 100% of marketed O&amp;D pairs before go-live</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Travelport Galileo and Worldspan display codeshare availability differently from Sabre; availability masking rules may suppress partner availability in certain agencies without explicit GDS-specific configuration</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Activate NDC API connection for partner direct-channel booking</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Digital Distribution Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Partner NDC Level 3 certification status, API credential exchange</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Live NDC offers including codeshare itineraries available via partner direct channel</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>NDC channel contributing ≥10% of codeshare bookings within 90 days of launch</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Many regional and medium-haul interline partners are not NDC Level 3 certified; interline itineraries in NDC require bilateral offer/order linking that is not yet standardised across vendors</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Brief operations and customer service on interline procedures</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Ground Operations Manager</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare operating procedures manual, baggage interline agreement, reaccommodation policy</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Briefed airport teams; interline baggage rules loaded into SITA AMS</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>100% of affected airport stations briefed ≥7 days before first codeshare departure</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Interline baggage tag reconciliation between dissimilar PSS platforms (e.g. Altéa vs Sabre PSS) causes baggage misrouting; SITA AMS does not auto-validate cross-carrier bag tags at transfer points</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Monitor codeshare booking ramp-up and yield metrics</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Daily PNR booking data, codeshare flight segment reports from Altéa</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Weekly performance dashboard: pax volume, yield, load factor by O&amp;D and partner</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare load factor ≥70% by week 4 post-launch; interline yield within 5% of target prorate</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM O&amp;D attribution for codeshare legs requires manual segment-level override; automated RM bid-price optimisation does not natively distinguish codeshare pax from own-metal pax in mixed itineraries</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-05</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare &amp; Interline Schedule Planning</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Conduct 90-day post-launch performance review</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>90-day pax and revenue actuals, prorate settlement statements, partner capacity data</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Performance review report with recommendations: expand, renegotiate, or discontinue</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Incremental revenue per ASK (RASK) contribution ≥2% above baseline on target O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Prorate settlement data from IATA BSP/ACH arrives 60–90 days in arrears, making 90-day review reliant on estimated yields; actual margin impact may not be known until Q2 following launch</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-06: Schedule Change Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -12,6 +12,7 @@
     <sheet name="NP-SP-03" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="NP-SP-04" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="NP-SP-05" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="NP-SP-06" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -838,13 +839,21 @@
           <t>Schedule Change Management</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-06</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -5073,7 +5082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12582,6 +12591,1374 @@
         </is>
       </c>
       <c r="N105" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E106" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="inlineStr">
+        <is>
+          <t>Capture schedule change request in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G106" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I106" s="18" t="inlineStr">
+        <is>
+          <t>Change trigger: demand signal, slot relinquishment, aircraft swap, regulatory requirement, or commercial request</t>
+        </is>
+      </c>
+      <c r="J106" s="18" t="inlineStr">
+        <is>
+          <t>Change request record with originating source, affected flights, and proposed effective date</t>
+        </is>
+      </c>
+      <c r="K106" s="18" t="inlineStr">
+        <is>
+          <t>Request logged within 2 hours of trigger receipt</t>
+        </is>
+      </c>
+      <c r="L106" s="18" t="inlineStr">
+        <is>
+          <t>Change requests arrive via email, Slack, and verbal channels with no single intake system — risk of duplicate or conflicting change records in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="M106" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N106" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C107" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D107" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E107" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>Classify change type, scope, and urgency</t>
+        </is>
+      </c>
+      <c r="G107" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H107" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I107" s="16" t="inlineStr">
+        <is>
+          <t>Change request record</t>
+        </is>
+      </c>
+      <c r="J107" s="16" t="inlineStr">
+        <is>
+          <t>Classification: seasonal adjustment, IRROP-driven, equipment swap, slot relinquishment, or capacity change; urgency tier (P1/P2/P3)</t>
+        </is>
+      </c>
+      <c r="K107" s="16" t="inlineStr">
+        <is>
+          <t>Classification completed within 4 hours of request capture</t>
+        </is>
+      </c>
+      <c r="L107" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal vs. irregular-operations changes require different downstream workflows; mis-classification delays IATA slot filing deadlines (SCR/ACR windows)</t>
+        </is>
+      </c>
+      <c r="M107" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N107" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="A108" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D108" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E108" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="inlineStr">
+        <is>
+          <t>Confirm route licence and fleet authority</t>
+        </is>
+      </c>
+      <c r="G108" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I108" s="18" t="inlineStr">
+        <is>
+          <t>Change classification, proposed route/frequency</t>
+        </is>
+      </c>
+      <c r="J108" s="18" t="inlineStr">
+        <is>
+          <t>Go/No-Go on initial feasibility: route DOT-licensed, aircraft type authorised for airport pair, bilateral traffic rights confirmed</t>
+        </is>
+      </c>
+      <c r="K108" s="18" t="inlineStr">
+        <is>
+          <t>Feasibility gate cleared within 1 business day; 100% of changes with regulatory exposure escalated before modelling</t>
+        </is>
+      </c>
+      <c r="L108" s="18" t="inlineStr">
+        <is>
+          <t>International route authority changes require DOT/foreign CAA coordination with 30–90 day lead times — late identification blocks schedule publication</t>
+        </is>
+      </c>
+      <c r="M108" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N108" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="30" customHeight="1">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D109" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F109" s="16" t="inlineStr">
+        <is>
+          <t>Simulate O&amp;D demand for proposed schedule</t>
+        </is>
+      </c>
+      <c r="G109" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H109" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I109" s="16" t="inlineStr">
+        <is>
+          <t>Proposed flight itinerary changes, historical booking curves, competitive schedule data from OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="J109" s="16" t="inlineStr">
+        <is>
+          <t>Projected O&amp;D demand, expected load factor, and unconstrained demand estimate for affected markets</t>
+        </is>
+      </c>
+      <c r="K109" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% on 90-day horizon; load factor projection ≥83% for change to proceed</t>
+        </is>
+      </c>
+      <c r="L109" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST demand models are calibrated on historical actuals — new or thin markets with &lt;12 months of data produce unreliable forecasts, requiring manual analyst override</t>
+        </is>
+      </c>
+      <c r="M109" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N109" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="30" customHeight="1">
+      <c r="A110" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E110" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>Model network-wide ripple effects in SkySYM</t>
+        </is>
+      </c>
+      <c r="G110" s="18" t="inlineStr">
+        <is>
+          <t>Network Simulation Analyst</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I110" s="18" t="inlineStr">
+        <is>
+          <t>Proposed schedule delta, current published schedule, connecting flow data</t>
+        </is>
+      </c>
+      <c r="J110" s="18" t="inlineStr">
+        <is>
+          <t>Connecting passenger impact report, minimum connect time (MCT) violations, spill/recapture estimates for disrupted flows</t>
+        </is>
+      </c>
+      <c r="K110" s="18" t="inlineStr">
+        <is>
+          <t>Zero MCT violations in output schedule; connecting flow spill ≤2% of total affected O&amp;D</t>
+        </is>
+      </c>
+      <c r="L110" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM scenario runs can take 45–90 minutes for full network simulation — time pressure during irregular operations compresses analysis window and increases error risk</t>
+        </is>
+      </c>
+      <c r="M110" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N110" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B111" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C111" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D111" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E111" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F111" s="16" t="inlineStr">
+        <is>
+          <t>Run fleet assignment optimisation to resolve conflicts</t>
+        </is>
+      </c>
+      <c r="G111" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H111" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I111" s="16" t="inlineStr">
+        <is>
+          <t>Network simulation output, available fleet positions, maintenance reservation blocks</t>
+        </is>
+      </c>
+      <c r="J111" s="16" t="inlineStr">
+        <is>
+          <t>Revised fleet assignment plan resolving aircraft-type conflicts; identified tail-swap or substitution options</t>
+        </is>
+      </c>
+      <c r="K111" s="16" t="inlineStr">
+        <is>
+          <t>Fleet conflict resolution rate ≥95% within 24 hours; gauge utilisation variance ≤5% vs. baseline plan</t>
+        </is>
+      </c>
+      <c r="L111" s="16" t="inlineStr">
+        <is>
+          <t>Fleet-constrained periods (peak summer, MAX grounding scenarios) leave SkyMAX with limited substitution options — manual intervention required and risks cascading reassignments</t>
+        </is>
+      </c>
+      <c r="M111" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N111" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B112" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C112" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D112" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E112" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="inlineStr">
+        <is>
+          <t>Gate: validate change against network thresholds</t>
+        </is>
+      </c>
+      <c r="G112" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H112" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I112" s="18" t="inlineStr">
+        <is>
+          <t>Demand simulation, ripple effect report, fleet assignment plan</t>
+        </is>
+      </c>
+      <c r="J112" s="18" t="inlineStr">
+        <is>
+          <t>Approval to proceed to slot/infrastructure assessment, or rejection with required redesign</t>
+        </is>
+      </c>
+      <c r="K112" s="18" t="inlineStr">
+        <is>
+          <t>Gate review completed within 1 business day; ≥90% of changes pass gate on first submission</t>
+        </is>
+      </c>
+      <c r="L112" s="18" t="inlineStr">
+        <is>
+          <t>Gate criteria (load factor, contribution margin, MCT compliance) are not formally codified — approval outcome varies by reviewer, creating schedule quality inconsistency</t>
+        </is>
+      </c>
+      <c r="M112" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N112" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="30" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B113" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C113" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D113" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F113" s="16" t="inlineStr">
+        <is>
+          <t>Check slot availability and filing deadlines</t>
+        </is>
+      </c>
+      <c r="G113" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Specialist</t>
+        </is>
+      </c>
+      <c r="H113" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I113" s="16" t="inlineStr">
+        <is>
+          <t>Proposed departure/arrival times, airport coordination level (L1/L2/L3), current season's slot holdings</t>
+        </is>
+      </c>
+      <c r="J113" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability confirmation or conflict flag; applicable SCR/ACR filing deadline</t>
+        </is>
+      </c>
+      <c r="K113" s="16" t="inlineStr">
+        <is>
+          <t>100% of slot change requests filed before IATA deadline; slot return compliance rate ≥98%</t>
+        </is>
+      </c>
+      <c r="L113" s="16" t="inlineStr">
+        <is>
+          <t>Level 3 coordinated airports (e.g., LHR, NRT) require slot exchanges negotiated bilaterally — lack of alliance membership limits swap leverage and can block desired time windows</t>
+        </is>
+      </c>
+      <c r="M113" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N113" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B114" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C114" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D114" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E114" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="inlineStr">
+        <is>
+          <t>Validate gate and terminal capacity at affected airports</t>
+        </is>
+      </c>
+      <c r="G114" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H114" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I114" s="18" t="inlineStr">
+        <is>
+          <t>Proposed schedule change, airport gate inventory, aircraft type (narrowbody vs. widebody)</t>
+        </is>
+      </c>
+      <c r="J114" s="18" t="inlineStr">
+        <is>
+          <t>Gate assignment confirmation or conflict flag; ground time adequacy assessment</t>
+        </is>
+      </c>
+      <c r="K114" s="18" t="inlineStr">
+        <is>
+          <t>Gate conflict resolution within 48 hours of identification; turnaround time ≥25 min protected for all affected rotations</t>
+        </is>
+      </c>
+      <c r="L114" s="18" t="inlineStr">
+        <is>
+          <t>Airport AMS data feeds are not always synchronised with SkyWORKS — gate conflicts discovered late in the process require emergency reassignments that increase ground delay risk</t>
+        </is>
+      </c>
+      <c r="M114" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N114" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B115" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C115" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D115" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E115" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F115" s="16" t="inlineStr">
+        <is>
+          <t>Gate: confirm slot and infrastructure availability</t>
+        </is>
+      </c>
+      <c r="G115" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H115" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I115" s="16" t="inlineStr">
+        <is>
+          <t>Slot confirmation or conflict report, gate capacity assessment</t>
+        </is>
+      </c>
+      <c r="J115" s="16" t="inlineStr">
+        <is>
+          <t>Infrastructure green-light or escalation to airport/slot coordinator for resolution</t>
+        </is>
+      </c>
+      <c r="K115" s="16" t="inlineStr">
+        <is>
+          <t>Slot and gate confirmation within 5 business days of change initiation; escalation resolved within 10 business days</t>
+        </is>
+      </c>
+      <c r="L115" s="16" t="inlineStr">
+        <is>
+          <t>Slot negotiation at congested airports (ORD, LAX, JFK) can extend beyond planning horizons — forces provisional schedule publication with risk of subsequent amendment</t>
+        </is>
+      </c>
+      <c r="M115" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N115" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B116" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C116" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D116" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E116" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="inlineStr">
+        <is>
+          <t>Model revenue and displacement impact in Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="G116" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I116" s="18" t="inlineStr">
+        <is>
+          <t>Approved schedule delta, current booking state for affected flights, O&amp;D demand forecasts</t>
+        </is>
+      </c>
+      <c r="J116" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact projection: incremental revenue, displacement cost, net contribution vs. status quo</t>
+        </is>
+      </c>
+      <c r="K116" s="18" t="inlineStr">
+        <is>
+          <t>Net revenue impact calculated within 2 business days; minimum threshold: net contribution change ≥ -$25K per changed rotation</t>
+        </is>
+      </c>
+      <c r="L116" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM O&amp;D optimisation recalibrates across all connected itineraries — a single frequency change can trigger widespread inventory reoptimisation that temporarily degrades load factors on unrelated flights</t>
+        </is>
+      </c>
+      <c r="M116" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N116" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C117" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D117" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E117" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F117" s="16" t="inlineStr">
+        <is>
+          <t>Assess fare structure and pricing impact via ATPCO</t>
+        </is>
+      </c>
+      <c r="G117" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H117" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I117" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact projection, current fare rules for affected markets, competitive pricing benchmarks</t>
+        </is>
+      </c>
+      <c r="J117" s="16" t="inlineStr">
+        <is>
+          <t>Fare rule amendment requirements; identification of fares requiring re-filing if schedule change breaches permitted connections or routing rules</t>
+        </is>
+      </c>
+      <c r="K117" s="16" t="inlineStr">
+        <is>
+          <t>100% of fares requiring re-filing identified before SSIM submission; fare amendment cycle ≤48 hours</t>
+        </is>
+      </c>
+      <c r="L117" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare rules contain explicit schedule-dependency conditions (permitted flights, connection times) — schedule changes that breach these rules automatically invalidate published fares and require emergency re-filing</t>
+        </is>
+      </c>
+      <c r="M117" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N117" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B118" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C118" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D118" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E118" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="inlineStr">
+        <is>
+          <t>Gate: commercial approval of net revenue impact</t>
+        </is>
+      </c>
+      <c r="G118" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H118" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I118" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact projection, fare amendment requirements, infrastructure cost estimates</t>
+        </is>
+      </c>
+      <c r="J118" s="18" t="inlineStr">
+        <is>
+          <t>Executive approval to proceed to filing, or directive to redesign change to improve commercial outcome</t>
+        </is>
+      </c>
+      <c r="K118" s="18" t="inlineStr">
+        <is>
+          <t>Commercial gate decision within 2 business days; ≤15% of changes recycled at this gate</t>
+        </is>
+      </c>
+      <c r="L118" s="18" t="inlineStr">
+        <is>
+          <t>Commercial gate approval is sequential with no parallel workstream — schedule change velocity is capped at VP availability, creating bottlenecks during peak planning periods (S/W season transitions)</t>
+        </is>
+      </c>
+      <c r="M118" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N118" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C119" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E119" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F119" s="16" t="inlineStr">
+        <is>
+          <t>Update master schedule and generate SSIM file</t>
+        </is>
+      </c>
+      <c r="G119" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H119" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I119" s="16" t="inlineStr">
+        <is>
+          <t>Approved schedule change, fleet assignment plan, effective date range</t>
+        </is>
+      </c>
+      <c r="J119" s="16" t="inlineStr">
+        <is>
+          <t>Updated published schedule in SkyWORKS; SSIM Chapter 7 message file for distribution</t>
+        </is>
+      </c>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>SSIM generated within 4 hours of commercial approval; zero data integrity errors in SSIM validation report</t>
+        </is>
+      </c>
+      <c r="L119" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export requires manual mapping of airline-internal equipment codes to IATA aircraft type designators — mapping errors cause GDS display discrepancies and passenger booking failures</t>
+        </is>
+      </c>
+      <c r="M119" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N119" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B120" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C120" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D120" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F120" s="18" t="inlineStr">
+        <is>
+          <t>Submit SSIM to GDS channels and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="G120" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H120" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I120" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file, NDC schedule change notification payload</t>
+        </is>
+      </c>
+      <c r="J120" s="18" t="inlineStr">
+        <is>
+          <t>Schedule update acknowledgement from Sabre GDS, Travelport GDS, Amadeus GDS, and NDC API Gateway; error report for failed segments</t>
+        </is>
+      </c>
+      <c r="K120" s="18" t="inlineStr">
+        <is>
+          <t>GDS schedule propagation within 24 hours of SSIM submission; NDC channel update within 4 hours; zero unacknowledged submissions</t>
+        </is>
+      </c>
+      <c r="L120" s="18" t="inlineStr">
+        <is>
+          <t>Each GDS has a different SSIM ingestion pipeline and error-reporting format — failures in one channel are not visible in another, requiring manual cross-channel reconciliation to confirm schedule accuracy</t>
+        </is>
+      </c>
+      <c r="M120" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N120" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="30" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C121" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D121" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E121" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F121" s="16" t="inlineStr">
+        <is>
+          <t>Gate: validate schedule accuracy across all channels</t>
+        </is>
+      </c>
+      <c r="G121" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H121" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I121" s="16" t="inlineStr">
+        <is>
+          <t>Live GDS schedule data, published SkyWORKS schedule, NDC content feed</t>
+        </is>
+      </c>
+      <c r="J121" s="16" t="inlineStr">
+        <is>
+          <t>Channel accuracy report; confirmed schedule match or list of discrepancies requiring re-submission</t>
+        </is>
+      </c>
+      <c r="K121" s="16" t="inlineStr">
+        <is>
+          <t>Schedule accuracy ≥99.5% across all channels within 48 hours of submission; zero flight-level discrepancies in departure time or equipment type</t>
+        </is>
+      </c>
+      <c r="L121" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser is updated on a 48-hour lag — real-time discrepancy detection requires direct GDS API queries that are not automated in the current toolchain</t>
+        </is>
+      </c>
+      <c r="M121" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N121" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B122" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C122" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D122" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E122" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F122" s="18" t="inlineStr">
+        <is>
+          <t>Trigger involuntary change notifications via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="G122" s="18" t="inlineStr">
+        <is>
+          <t>Customer Experience Operations Specialist</t>
+        </is>
+      </c>
+      <c r="H122" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I122" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed schedule change, affected PNR list, change type (significant vs. minor per DOT thresholds)</t>
+        </is>
+      </c>
+      <c r="J122" s="18" t="inlineStr">
+        <is>
+          <t>Passenger notification emails/SMS sent; re-accommodation offers generated for significantly affected itineraries (&gt;90 min departure change)</t>
+        </is>
+      </c>
+      <c r="K122" s="18" t="inlineStr">
+        <is>
+          <t>100% of affected passengers notified within 24 hours of schedule change publication; DOT significant change threshold compliance rate 100%</t>
+        </is>
+      </c>
+      <c r="L122" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS applies DOT notification rules based on schedule delta thresholds — but interline and codeshare bookings held in partner PSS systems are not automatically notified, creating DOT compliance risk</t>
+        </is>
+      </c>
+      <c r="M122" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N122" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C123" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D123" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E123" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F123" s="16" t="inlineStr">
+        <is>
+          <t>Process re-accommodation requests and fee waivers</t>
+        </is>
+      </c>
+      <c r="G123" s="16" t="inlineStr">
+        <is>
+          <t>Customer Experience Operations Specialist</t>
+        </is>
+      </c>
+      <c r="H123" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I123" s="16" t="inlineStr">
+        <is>
+          <t>Passenger rebooking requests, waiver policy (significant change = full flexibility), alternative flight inventory</t>
+        </is>
+      </c>
+      <c r="J123" s="16" t="inlineStr">
+        <is>
+          <t>Rebooked PNRs; refund transactions for passengers who opt out; waiver codes applied</t>
+        </is>
+      </c>
+      <c r="K123" s="16" t="inlineStr">
+        <is>
+          <t>Re-accommodation rate ≥92% on same-day alternatives; average re-booking handle time ≤8 minutes; refund processing within DOT 7-day credit card window</t>
+        </is>
+      </c>
+      <c r="L123" s="16" t="inlineStr">
+        <is>
+          <t>High-volume schedule changes (e.g., full season overhaul) generate re-accommodation queues that exceed contact centre capacity — automated re-accommodation via Altéa rebooking engine has a 78% acceptance rate, leaving 22% requiring agent intervention</t>
+        </is>
+      </c>
+      <c r="M123" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N123" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B124" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C124" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D124" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E124" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F124" s="18" t="inlineStr">
+        <is>
+          <t>Monitor post-implementation KPIs and close change record</t>
+        </is>
+      </c>
+      <c r="G124" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H124" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I124" s="18" t="inlineStr">
+        <is>
+          <t>Live booking data (Altéa), load factor actuals, OTP data, re-accommodation completion rate</t>
+        </is>
+      </c>
+      <c r="J124" s="18" t="inlineStr">
+        <is>
+          <t>Post-implementation review report; change record closed in SkyWORKS with outcome classification (successful / modified / reversed)</t>
+        </is>
+      </c>
+      <c r="K124" s="18" t="inlineStr">
+        <is>
+          <t>Load factor on changed flights ≥83% within 30 days; OTP ≥78% D0; re-accommodation completion rate ≥98% within 72 hours of notification</t>
+        </is>
+      </c>
+      <c r="L124" s="18" t="inlineStr">
+        <is>
+          <t>Post-implementation tracking is done manually in Tableau by pulling Altéa booking exports — there is no automated feedback loop from actuals into SkyCAST demand models, so forecast accuracy improvements from change outcomes are not systematically captured</t>
+        </is>
+      </c>
+      <c r="M124" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N124" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -16553,4 +17930,1492 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-06 — Schedule Change Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Schedule Change Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Capture schedule change request in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Change trigger: demand signal, slot relinquishment, aircraft swap, regulatory requirement, or commercial request</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Change request record with originating source, affected flights, and proposed effective date</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Request logged within 2 hours of trigger receipt</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Change requests arrive via email, Slack, and verbal channels with no single intake system — risk of duplicate or conflicting change records in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Classify change type, scope, and urgency</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Change request record</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Classification: seasonal adjustment, IRROP-driven, equipment swap, slot relinquishment, or capacity change; urgency tier (P1/P2/P3)</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Classification completed within 4 hours of request capture</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal vs. irregular-operations changes require different downstream workflows; mis-classification delays IATA slot filing deadlines (SCR/ACR windows)</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Confirm route licence and fleet authority</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Change classification, proposed route/frequency</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Go/No-Go on initial feasibility: route DOT-licensed, aircraft type authorised for airport pair, bilateral traffic rights confirmed</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Feasibility gate cleared within 1 business day; 100% of changes with regulatory exposure escalated before modelling</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>International route authority changes require DOT/foreign CAA coordination with 30–90 day lead times — late identification blocks schedule publication</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Simulate O&amp;D demand for proposed schedule</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Proposed flight itinerary changes, historical booking curves, competitive schedule data from OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Projected O&amp;D demand, expected load factor, and unconstrained demand estimate for affected markets</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% on 90-day horizon; load factor projection ≥83% for change to proceed</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST demand models are calibrated on historical actuals — new or thin markets with &lt;12 months of data produce unreliable forecasts, requiring manual analyst override</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Model network-wide ripple effects in SkySYM</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Network Simulation Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Proposed schedule delta, current published schedule, connecting flow data</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Connecting passenger impact report, minimum connect time (MCT) violations, spill/recapture estimates for disrupted flows</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Zero MCT violations in output schedule; connecting flow spill ≤2% of total affected O&amp;D</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM scenario runs can take 45–90 minutes for full network simulation — time pressure during irregular operations compresses analysis window and increases error risk</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Run fleet assignment optimisation to resolve conflicts</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Network simulation output, available fleet positions, maintenance reservation blocks</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Revised fleet assignment plan resolving aircraft-type conflicts; identified tail-swap or substitution options</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Fleet conflict resolution rate ≥95% within 24 hours; gauge utilisation variance ≤5% vs. baseline plan</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Fleet-constrained periods (peak summer, MAX grounding scenarios) leave SkyMAX with limited substitution options — manual intervention required and risks cascading reassignments</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Gate: validate change against network thresholds</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Demand simulation, ripple effect report, fleet assignment plan</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Approval to proceed to slot/infrastructure assessment, or rejection with required redesign</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Gate review completed within 1 business day; ≥90% of changes pass gate on first submission</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Gate criteria (load factor, contribution margin, MCT compliance) are not formally codified — approval outcome varies by reviewer, creating schedule quality inconsistency</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Check slot availability and filing deadlines</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Specialist</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Proposed departure/arrival times, airport coordination level (L1/L2/L3), current season's slot holdings</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability confirmation or conflict flag; applicable SCR/ACR filing deadline</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>100% of slot change requests filed before IATA deadline; slot return compliance rate ≥98%</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Level 3 coordinated airports (e.g., LHR, NRT) require slot exchanges negotiated bilaterally — lack of alliance membership limits swap leverage and can block desired time windows</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Validate gate and terminal capacity at affected airports</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Proposed schedule change, airport gate inventory, aircraft type (narrowbody vs. widebody)</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Gate assignment confirmation or conflict flag; ground time adequacy assessment</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Gate conflict resolution within 48 hours of identification; turnaround time ≥25 min protected for all affected rotations</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Airport AMS data feeds are not always synchronised with SkyWORKS — gate conflicts discovered late in the process require emergency reassignments that increase ground delay risk</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Gate: confirm slot and infrastructure availability</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Slot confirmation or conflict report, gate capacity assessment</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Infrastructure green-light or escalation to airport/slot coordinator for resolution</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Slot and gate confirmation within 5 business days of change initiation; escalation resolved within 10 business days</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Slot negotiation at congested airports (ORD, LAX, JFK) can extend beyond planning horizons — forces provisional schedule publication with risk of subsequent amendment</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Model revenue and displacement impact in Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Approved schedule delta, current booking state for affected flights, O&amp;D demand forecasts</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact projection: incremental revenue, displacement cost, net contribution vs. status quo</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Net revenue impact calculated within 2 business days; minimum threshold: net contribution change ≥ -$25K per changed rotation</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM O&amp;D optimisation recalibrates across all connected itineraries — a single frequency change can trigger widespread inventory reoptimisation that temporarily degrades load factors on unrelated flights</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Assess fare structure and pricing impact via ATPCO</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact projection, current fare rules for affected markets, competitive pricing benchmarks</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Fare rule amendment requirements; identification of fares requiring re-filing if schedule change breaches permitted connections or routing rules</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>100% of fares requiring re-filing identified before SSIM submission; fare amendment cycle ≤48 hours</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare rules contain explicit schedule-dependency conditions (permitted flights, connection times) — schedule changes that breach these rules automatically invalidate published fares and require emergency re-filing</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Gate: commercial approval of net revenue impact</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact projection, fare amendment requirements, infrastructure cost estimates</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Executive approval to proceed to filing, or directive to redesign change to improve commercial outcome</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Commercial gate decision within 2 business days; ≤15% of changes recycled at this gate</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Commercial gate approval is sequential with no parallel workstream — schedule change velocity is capped at VP availability, creating bottlenecks during peak planning periods (S/W season transitions)</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Update master schedule and generate SSIM file</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Approved schedule change, fleet assignment plan, effective date range</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Updated published schedule in SkyWORKS; SSIM Chapter 7 message file for distribution</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM generated within 4 hours of commercial approval; zero data integrity errors in SSIM validation report</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export requires manual mapping of airline-internal equipment codes to IATA aircraft type designators — mapping errors cause GDS display discrepancies and passenger booking failures</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Submit SSIM to GDS channels and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file, NDC schedule change notification payload</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule update acknowledgement from Sabre GDS, Travelport GDS, Amadeus GDS, and NDC API Gateway; error report for failed segments</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>GDS schedule propagation within 24 hours of SSIM submission; NDC channel update within 4 hours; zero unacknowledged submissions</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Each GDS has a different SSIM ingestion pipeline and error-reporting format — failures in one channel are not visible in another, requiring manual cross-channel reconciliation to confirm schedule accuracy</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Gate: validate schedule accuracy across all channels</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Live GDS schedule data, published SkyWORKS schedule, NDC content feed</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Channel accuracy report; confirmed schedule match or list of discrepancies requiring re-submission</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule accuracy ≥99.5% across all channels within 48 hours of submission; zero flight-level discrepancies in departure time or equipment type</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser is updated on a 48-hour lag — real-time discrepancy detection requires direct GDS API queries that are not automated in the current toolchain</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Trigger involuntary change notifications via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Customer Experience Operations Specialist</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed schedule change, affected PNR list, change type (significant vs. minor per DOT thresholds)</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Passenger notification emails/SMS sent; re-accommodation offers generated for significantly affected itineraries (&gt;90 min departure change)</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>100% of affected passengers notified within 24 hours of schedule change publication; DOT significant change threshold compliance rate 100%</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS applies DOT notification rules based on schedule delta thresholds — but interline and codeshare bookings held in partner PSS systems are not automatically notified, creating DOT compliance risk</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Process re-accommodation requests and fee waivers</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Customer Experience Operations Specialist</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Passenger rebooking requests, waiver policy (significant change = full flexibility), alternative flight inventory</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Rebooked PNRs; refund transactions for passengers who opt out; waiver codes applied</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Re-accommodation rate ≥92% on same-day alternatives; average re-booking handle time ≤8 minutes; refund processing within DOT 7-day credit card window</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>High-volume schedule changes (e.g., full season overhaul) generate re-accommodation queues that exceed contact centre capacity — automated re-accommodation via Altéa rebooking engine has a 78% acceptance rate, leaving 22% requiring agent intervention</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-06</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Change Management</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Monitor post-implementation KPIs and close change record</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Live booking data (Altéa), load factor actuals, OTP data, re-accommodation completion rate</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Post-implementation review report; change record closed in SkyWORKS with outcome classification (successful / modified / reversed)</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>Load factor on changed flights ≥83% within 30 days; OTP ≥78% D0; re-accommodation completion rate ≥98% within 72 hours of notification</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>Post-implementation tracking is done manually in Tableau by pulling Altéa booking exports — there is no automated feedback loop from actuals into SkyCAST demand models, so forecast accuracy improvements from change outcomes are not systematically captured</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-07: Capacity Planning & Utilization — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -13,6 +13,7 @@
     <sheet name="NP-SP-04" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="NP-SP-05" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="NP-SP-06" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NP-SP-07" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -876,13 +877,21 @@
           <t>Capacity Planning &amp; Utilization</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="10" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-07</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -5082,7 +5091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N124"/>
+  <dimension ref="A1:N142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13959,6 +13968,1302 @@
         </is>
       </c>
       <c r="N124" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B125" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C125" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F125" s="16" t="inlineStr">
+        <is>
+          <t>Extract historical O&amp;D traffic data</t>
+        </is>
+      </c>
+      <c r="G125" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H125" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I125" s="16" t="inlineStr">
+        <is>
+          <t>Planning cycle trigger; 24-month O&amp;D booking history</t>
+        </is>
+      </c>
+      <c r="J125" s="16" t="inlineStr">
+        <is>
+          <t>Baseline O&amp;D traffic dataset by market and quarter</t>
+        </is>
+      </c>
+      <c r="K125" s="16" t="inlineStr">
+        <is>
+          <t>Data completeness ≥98% of active markets</t>
+        </is>
+      </c>
+      <c r="L125" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST data feeds depend on Altéa PSS booking exports; delays in PSS batch jobs cause stale baseline traffic inputs, distorting forecasts for thin markets</t>
+        </is>
+      </c>
+      <c r="M125" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N125" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B126" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C126" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D126" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E126" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F126" s="18" t="inlineStr">
+        <is>
+          <t>Run demand forecast for planning horizon</t>
+        </is>
+      </c>
+      <c r="G126" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H126" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I126" s="18" t="inlineStr">
+        <is>
+          <t>Historical O&amp;D dataset; macro-economic indices; event calendar</t>
+        </is>
+      </c>
+      <c r="J126" s="18" t="inlineStr">
+        <is>
+          <t>12-month segment-level demand forecast by frequency band</t>
+        </is>
+      </c>
+      <c r="K126" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% at 90-day horizon</t>
+        </is>
+      </c>
+      <c r="L126" s="18" t="inlineStr">
+        <is>
+          <t>Thin LCC markets and new routes lack sufficient booking history; SkyCAST model defaults to industry averages, understating demand elasticity for fare-sensitive leisure segments</t>
+        </is>
+      </c>
+      <c r="M126" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N126" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B127" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C127" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D127" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E127" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F127" s="16" t="inlineStr">
+        <is>
+          <t>Validate forecast variance against prior cycle</t>
+        </is>
+      </c>
+      <c r="G127" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H127" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I127" s="16" t="inlineStr">
+        <is>
+          <t>Current forecast; prior planning cycle forecast</t>
+        </is>
+      </c>
+      <c r="J127" s="16" t="inlineStr">
+        <is>
+          <t>Variance report flagging markets with &gt;5% deviation</t>
+        </is>
+      </c>
+      <c r="K127" s="16" t="inlineStr">
+        <is>
+          <t>Forecast variance report produced within 2 business days of data extraction</t>
+        </is>
+      </c>
+      <c r="L127" s="16" t="inlineStr">
+        <is>
+          <t>Manual comparison between planning cycles is error-prone; no automated delta alerting in SkyCAST baseline module — analyst must export to Excel for comparison</t>
+        </is>
+      </c>
+      <c r="M127" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N127" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B128" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C128" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D128" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E128" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="inlineStr">
+        <is>
+          <t>Identify routes requiring capacity uplift</t>
+        </is>
+      </c>
+      <c r="G128" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H128" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I128" s="18" t="inlineStr">
+        <is>
+          <t>Validated demand forecast; current schedule frequencies</t>
+        </is>
+      </c>
+      <c r="J128" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised list of routes with capacity gap ≥10 seats/day average</t>
+        </is>
+      </c>
+      <c r="K128" s="18" t="inlineStr">
+        <is>
+          <t>Capacity gap identification covering 100% of markets with forecast load factor ≥85%</t>
+        </is>
+      </c>
+      <c r="L128" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM network simulation does not natively import SkyCAST output in real time; manual CSV handoff between tools introduces reconciliation lag of 1–2 days</t>
+        </is>
+      </c>
+      <c r="M128" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N128" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="A129" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C129" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E129" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F129" s="16" t="inlineStr">
+        <is>
+          <t>Run initial fleet assignment optimisation</t>
+        </is>
+      </c>
+      <c r="G129" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H129" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I129" s="16" t="inlineStr">
+        <is>
+          <t>Capacity gap list; available fleet inventory by subfleet</t>
+        </is>
+      </c>
+      <c r="J129" s="16" t="inlineStr">
+        <is>
+          <t>Draft fleet assignment plan with gauge per rotation</t>
+        </is>
+      </c>
+      <c r="K129" s="16" t="inlineStr">
+        <is>
+          <t>Fleet utilisation ≥13.5 block hours/aircraft/day across active rotations</t>
+        </is>
+      </c>
+      <c r="L129" s="16" t="inlineStr">
+        <is>
+          <t>SkyMAX optimiser is sensitive to input parameter sequencing; incorrect fleet availability seeding (e.g., aircraft in scheduled maintenance not flagged) generates infeasible rotations that require manual correction</t>
+        </is>
+      </c>
+      <c r="M129" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N129" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B130" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C130" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D130" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E130" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="inlineStr">
+        <is>
+          <t>Detect constraint violations in fleet plan</t>
+        </is>
+      </c>
+      <c r="G130" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H130" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I130" s="18" t="inlineStr">
+        <is>
+          <t>Draft fleet assignment plan</t>
+        </is>
+      </c>
+      <c r="J130" s="18" t="inlineStr">
+        <is>
+          <t>Constraint violation report (turn-time, gauge, balance)</t>
+        </is>
+      </c>
+      <c r="K130" s="18" t="inlineStr">
+        <is>
+          <t>Zero hard constraint violations (MTOW, turn-time) in approved plan</t>
+        </is>
+      </c>
+      <c r="L130" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX surface-level constraint checker does not model real-time gate availability at congested airports (e.g., LHR, JFK slots); gate conflicts surface only post-filing via airport coordination</t>
+        </is>
+      </c>
+      <c r="M130" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N130" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C131" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D131" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E131" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F131" s="16" t="inlineStr">
+        <is>
+          <t>Adjust gauge on constrained rotations</t>
+        </is>
+      </c>
+      <c r="G131" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H131" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I131" s="16" t="inlineStr">
+        <is>
+          <t>Constraint violation report; alternate fleet availability</t>
+        </is>
+      </c>
+      <c r="J131" s="16" t="inlineStr">
+        <is>
+          <t>Revised gauge assignments with documented trade-off notes</t>
+        </is>
+      </c>
+      <c r="K131" s="16" t="inlineStr">
+        <is>
+          <t>All gauge adjustments resolved and re-optimised within 3 business days</t>
+        </is>
+      </c>
+      <c r="L131" s="16" t="inlineStr">
+        <is>
+          <t>Downgrading gauge to resolve tail-count imbalance at outstations triggers yield loss on high-demand rotations; no automated revenue impact warning exists in SkyWORKS at point of gauge swap</t>
+        </is>
+      </c>
+      <c r="M131" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N131" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B132" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C132" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D132" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E132" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="inlineStr">
+        <is>
+          <t>Validate tail-count balance across network</t>
+        </is>
+      </c>
+      <c r="G132" s="18" t="inlineStr">
+        <is>
+          <t>Network Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H132" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I132" s="18" t="inlineStr">
+        <is>
+          <t>Revised fleet assignment plan; overnight parking constraints by station</t>
+        </is>
+      </c>
+      <c r="J132" s="18" t="inlineStr">
+        <is>
+          <t>Balanced fleet assignment confirming overnight positions by station</t>
+        </is>
+      </c>
+      <c r="K132" s="18" t="inlineStr">
+        <is>
+          <t>Overnight positioning plan with zero unresolved imbalances before SSIM submission</t>
+        </is>
+      </c>
+      <c r="L132" s="18" t="inlineStr">
+        <is>
+          <t>Overnight imbalances at spoke stations with no maintenance capability require costly ferry flights; SkyMAX does not auto-flag stations without MRO support when positioning aircraft</t>
+        </is>
+      </c>
+      <c r="M132" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N132" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B133" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C133" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D133" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E133" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F133" s="16" t="inlineStr">
+        <is>
+          <t>Assess slot and gate availability constraints</t>
+        </is>
+      </c>
+      <c r="G133" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H133" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I133" s="16" t="inlineStr">
+        <is>
+          <t>Validated fleet assignment plan; airport coordination level classifications</t>
+        </is>
+      </c>
+      <c r="J133" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability matrix for Level 2/3 airports</t>
+        </is>
+      </c>
+      <c r="K133" s="16" t="inlineStr">
+        <is>
+          <t>100% of Level 3 coordinated airports reviewed before SSIM submission</t>
+        </is>
+      </c>
+      <c r="L133" s="16" t="inlineStr">
+        <is>
+          <t>Slot exchanges with competing carriers at Level 3 airports require bilateral negotiation through IATA slot conferences; lead times of 6–12 months compress planning windows for seasonal capacity changes</t>
+        </is>
+      </c>
+      <c r="M133" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N133" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B134" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C134" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D134" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E134" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F134" s="18" t="inlineStr">
+        <is>
+          <t>Review maintenance capacity windows</t>
+        </is>
+      </c>
+      <c r="G134" s="18" t="inlineStr">
+        <is>
+          <t>Line Maintenance Planner</t>
+        </is>
+      </c>
+      <c r="H134" s="18" t="inlineStr">
+        <is>
+          <t>AMOS by Swiss AviationSoftware</t>
+        </is>
+      </c>
+      <c r="I134" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan; upcoming A/C-check and C-check schedules</t>
+        </is>
+      </c>
+      <c r="J134" s="18" t="inlineStr">
+        <is>
+          <t>Maintenance conflict report showing aircraft unavailability periods</t>
+        </is>
+      </c>
+      <c r="K134" s="18" t="inlineStr">
+        <is>
+          <t>Zero unplanned maintenance conflicts in 90-day rolling capacity plan</t>
+        </is>
+      </c>
+      <c r="L134" s="18" t="inlineStr">
+        <is>
+          <t>AMOS maintenance window data is not directly integrated with SkyMAX fleet assignment; planners rely on manual exports and cross-referencing in spreadsheets, creating reconciliation errors during peak planning periods</t>
+        </is>
+      </c>
+      <c r="M134" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N134" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B135" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C135" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D135" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E135" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F135" s="16" t="inlineStr">
+        <is>
+          <t>Validate crew availability against planned capacity</t>
+        </is>
+      </c>
+      <c r="G135" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H135" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I135" s="16" t="inlineStr">
+        <is>
+          <t>Validated fleet assignment plan; crew headcount and qualification data</t>
+        </is>
+      </c>
+      <c r="J135" s="16" t="inlineStr">
+        <is>
+          <t>Crew coverage report by base and crew position</t>
+        </is>
+      </c>
+      <c r="K135" s="16" t="inlineStr">
+        <is>
+          <t>Crew coverage ratio ≥105% (buffer above minimum legal complement)</t>
+        </is>
+      </c>
+      <c r="L135" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management pairing outputs are built on published schedule; capacity changes post-pairing require full rerun of crew pairings, increasing planning cycle time by 3–5 days and risking FAR Part 117 duty-time compliance gaps</t>
+        </is>
+      </c>
+      <c r="M135" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N135" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B136" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C136" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D136" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E136" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F136" s="18" t="inlineStr">
+        <is>
+          <t>Resolve crew or slot deficits via capacity swap</t>
+        </is>
+      </c>
+      <c r="G136" s="18" t="inlineStr">
+        <is>
+          <t>Network Planner</t>
+        </is>
+      </c>
+      <c r="H136" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I136" s="18" t="inlineStr">
+        <is>
+          <t>Crew coverage report; slot availability matrix; maintenance conflict report</t>
+        </is>
+      </c>
+      <c r="J136" s="18" t="inlineStr">
+        <is>
+          <t>Revised capacity plan with documented frequency or gauge reductions</t>
+        </is>
+      </c>
+      <c r="K136" s="18" t="inlineStr">
+        <is>
+          <t>All crew and slot deficits resolved before SSIM filing deadline</t>
+        </is>
+      </c>
+      <c r="L136" s="18" t="inlineStr">
+        <is>
+          <t>Reducing frequencies to resolve crew deficits at hub bases cascades into load factor pressure on remaining departures; decision lacks integrated revenue-impact modelling at point of resolution in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="M136" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N136" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B137" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C137" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E137" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F137" s="16" t="inlineStr">
+        <is>
+          <t>Generate SSIM schedule file for submission</t>
+        </is>
+      </c>
+      <c r="G137" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H137" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I137" s="16" t="inlineStr">
+        <is>
+          <t>Approved capacity plan; airline designator codes and flight number series</t>
+        </is>
+      </c>
+      <c r="J137" s="16" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 formatted schedule file</t>
+        </is>
+      </c>
+      <c r="K137" s="16" t="inlineStr">
+        <is>
+          <t>SSIM file generated within 1 business day of capacity plan sign-off</t>
+        </is>
+      </c>
+      <c r="L137" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export module requires manual mapping of codeshare flight suffixes for partner flights; errors in suffix formatting cause GDS rejection and require resubmission, delaying schedule availability by 24–48 hours</t>
+        </is>
+      </c>
+      <c r="M137" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N137" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B138" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C138" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D138" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E138" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F138" s="18" t="inlineStr">
+        <is>
+          <t>Validate SSIM file against IATA standards</t>
+        </is>
+      </c>
+      <c r="G138" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Coordinator</t>
+        </is>
+      </c>
+      <c r="H138" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I138" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J138" s="18" t="inlineStr">
+        <is>
+          <t>Validation report; corrected SSIM file if errors found</t>
+        </is>
+      </c>
+      <c r="K138" s="18" t="inlineStr">
+        <is>
+          <t>Zero critical SSIM errors at point of GDS submission</t>
+        </is>
+      </c>
+      <c r="L138" s="18" t="inlineStr">
+        <is>
+          <t>OAG validation catches structural SSIM errors but does not validate operational feasibility (e.g., turn-time violations at specific airports); operationally infeasible schedules pass SSIM validation and are caught only during operations</t>
+        </is>
+      </c>
+      <c r="M138" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N138" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B139" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C139" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E139" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F139" s="16" t="inlineStr">
+        <is>
+          <t>Submit validated schedule to GDS and NDC channels</t>
+        </is>
+      </c>
+      <c r="G139" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H139" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus GDS / Sabre GDS / NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I139" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J139" s="16" t="inlineStr">
+        <is>
+          <t>Schedule live in Amadeus, Sabre, Travelport, and NDC channel</t>
+        </is>
+      </c>
+      <c r="K139" s="16" t="inlineStr">
+        <is>
+          <t>Schedule available in all GDS channels within 4 hours of SSIM submission; NDC availability within 2 hours</t>
+        </is>
+      </c>
+      <c r="L139" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS schedule updates lag Amadeus and Sabre by up to 6 hours due to batch processing cadence; passengers booking via Travelport-connected TMCs may see stale capacity, resulting in overbooking conflicts at check-in</t>
+        </is>
+      </c>
+      <c r="M139" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N139" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B140" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C140" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D140" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E140" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="inlineStr">
+        <is>
+          <t>Monitor in-period seat utilization vs forecast</t>
+        </is>
+      </c>
+      <c r="G140" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H140" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I140" s="18" t="inlineStr">
+        <is>
+          <t>Live booking data; capacity plan baseline</t>
+        </is>
+      </c>
+      <c r="J140" s="18" t="inlineStr">
+        <is>
+          <t>Weekly utilization dashboard by market and departure date</t>
+        </is>
+      </c>
+      <c r="K140" s="18" t="inlineStr">
+        <is>
+          <t>System load factor ≥83% on average across active network; individual market load factor reviewed weekly</t>
+        </is>
+      </c>
+      <c r="L140" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM monitors inventory at O&amp;D level but does not natively surface segment-level spill and recapture estimates; capacity reoptimisation decisions rely on analyst judgment without automated spill quantification</t>
+        </is>
+      </c>
+      <c r="M140" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N140" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B141" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C141" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D141" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E141" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F141" s="16" t="inlineStr">
+        <is>
+          <t>Trigger capacity reoptimisation for underperforming routes</t>
+        </is>
+      </c>
+      <c r="G141" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H141" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I141" s="16" t="inlineStr">
+        <is>
+          <t>Utilization dashboard; routes with load factor &lt;78% within 60 days of departure</t>
+        </is>
+      </c>
+      <c r="J141" s="16" t="inlineStr">
+        <is>
+          <t>Reoptimisation recommendation: frequency reduction, gauge swap, or fare stimulus</t>
+        </is>
+      </c>
+      <c r="K141" s="16" t="inlineStr">
+        <is>
+          <t>Reoptimisation recommendation issued within 48 hours of load factor breach trigger</t>
+        </is>
+      </c>
+      <c r="L141" s="16" t="inlineStr">
+        <is>
+          <t>Within-60-day capacity changes require coordinated updates across Altéa PSS (inventory), SkyWORKS (schedule), and Jeppesen Crew (pairings); the lack of a unified change-management workflow causes synchronisation failures and involuntary passenger re-accommodation</t>
+        </is>
+      </c>
+      <c r="M141" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N141" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B142" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C142" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D142" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E142" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F142" s="18" t="inlineStr">
+        <is>
+          <t>Log final utilization KPIs and close planning cycle</t>
+        </is>
+      </c>
+      <c r="G142" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H142" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I142" s="18" t="inlineStr">
+        <is>
+          <t>Post-departure load factor actuals; forecast baseline</t>
+        </is>
+      </c>
+      <c r="J142" s="18" t="inlineStr">
+        <is>
+          <t>Post-cycle capacity utilization report with variance analysis</t>
+        </is>
+      </c>
+      <c r="K142" s="18" t="inlineStr">
+        <is>
+          <t>Post-cycle report published within 5 business days of season end; forecast vs actual load factor variance documented for model calibration</t>
+        </is>
+      </c>
+      <c r="L142" s="18" t="inlineStr">
+        <is>
+          <t>Redshift data pipeline aggregates actuals from Altéa PSS on a 24-hour delay; post-departure analysis for redeye and overnight flights often reflects next-day timestamps, distorting daily load factor KPIs in Tableau dashboards</t>
+        </is>
+      </c>
+      <c r="M142" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N142" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -19418,4 +20723,1420 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-07 — Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract historical O&amp;D traffic data</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Planning cycle trigger; 24-month O&amp;D booking history</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Baseline O&amp;D traffic dataset by market and quarter</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness ≥98% of active markets</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST data feeds depend on Altéa PSS booking exports; delays in PSS batch jobs cause stale baseline traffic inputs, distorting forecasts for thin markets</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Run demand forecast for planning horizon</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Historical O&amp;D dataset; macro-economic indices; event calendar</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>12-month segment-level demand forecast by frequency band</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% at 90-day horizon</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Thin LCC markets and new routes lack sufficient booking history; SkyCAST model defaults to industry averages, understating demand elasticity for fare-sensitive leisure segments</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate forecast variance against prior cycle</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Current forecast; prior planning cycle forecast</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Variance report flagging markets with &gt;5% deviation</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Forecast variance report produced within 2 business days of data extraction</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Manual comparison between planning cycles is error-prone; no automated delta alerting in SkyCAST baseline module — analyst must export to Excel for comparison</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Identify routes requiring capacity uplift</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated demand forecast; current schedule frequencies</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Prioritised list of routes with capacity gap ≥10 seats/day average</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Capacity gap identification covering 100% of markets with forecast load factor ≥85%</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM network simulation does not natively import SkyCAST output in real time; manual CSV handoff between tools introduces reconciliation lag of 1–2 days</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Run initial fleet assignment optimisation</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Capacity gap list; available fleet inventory by subfleet</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Draft fleet assignment plan with gauge per rotation</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Fleet utilisation ≥13.5 block hours/aircraft/day across active rotations</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX optimiser is sensitive to input parameter sequencing; incorrect fleet availability seeding (e.g., aircraft in scheduled maintenance not flagged) generates infeasible rotations that require manual correction</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Detect constraint violations in fleet plan</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Draft fleet assignment plan</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Constraint violation report (turn-time, gauge, balance)</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Zero hard constraint violations (MTOW, turn-time) in approved plan</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>SkyMAX surface-level constraint checker does not model real-time gate availability at congested airports (e.g., LHR, JFK slots); gate conflicts surface only post-filing via airport coordination</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Adjust gauge on constrained rotations</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Assignment Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Constraint violation report; alternate fleet availability</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Revised gauge assignments with documented trade-off notes</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>All gauge adjustments resolved and re-optimised within 3 business days</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Downgrading gauge to resolve tail-count imbalance at outstations triggers yield loss on high-demand rotations; no automated revenue impact warning exists in SkyWORKS at point of gauge swap</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Validate tail-count balance across network</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Network Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Revised fleet assignment plan; overnight parking constraints by station</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Balanced fleet assignment confirming overnight positions by station</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Overnight positioning plan with zero unresolved imbalances before SSIM submission</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Overnight imbalances at spoke stations with no maintenance capability require costly ferry flights; SkyMAX does not auto-flag stations without MRO support when positioning aircraft</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Assess slot and gate availability constraints</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Validated fleet assignment plan; airport coordination level classifications</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Slot availability matrix for Level 2/3 airports</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>100% of Level 3 coordinated airports reviewed before SSIM submission</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Slot exchanges with competing carriers at Level 3 airports require bilateral negotiation through IATA slot conferences; lead times of 6–12 months compress planning windows for seasonal capacity changes</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Review maintenance capacity windows</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Line Maintenance Planner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>AMOS by Swiss AviationSoftware</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan; upcoming A/C-check and C-check schedules</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Maintenance conflict report showing aircraft unavailability periods</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Zero unplanned maintenance conflicts in 90-day rolling capacity plan</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>AMOS maintenance window data is not directly integrated with SkyMAX fleet assignment; planners rely on manual exports and cross-referencing in spreadsheets, creating reconciliation errors during peak planning periods</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Validate crew availability against planned capacity</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Validated fleet assignment plan; crew headcount and qualification data</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Crew coverage report by base and crew position</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Crew coverage ratio ≥105% (buffer above minimum legal complement)</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management pairing outputs are built on published schedule; capacity changes post-pairing require full rerun of crew pairings, increasing planning cycle time by 3–5 days and risking FAR Part 117 duty-time compliance gaps</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Resolve crew or slot deficits via capacity swap</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planner</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Crew coverage report; slot availability matrix; maintenance conflict report</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Revised capacity plan with documented frequency or gauge reductions</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>All crew and slot deficits resolved before SSIM filing deadline</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Reducing frequencies to resolve crew deficits at hub bases cascades into load factor pressure on remaining departures; decision lacks integrated revenue-impact modelling at point of resolution in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Generate SSIM schedule file for submission</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Approved capacity plan; airline designator codes and flight number series</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 formatted schedule file</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>SSIM file generated within 1 business day of capacity plan sign-off</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM export module requires manual mapping of codeshare flight suffixes for partner flights; errors in suffix formatting cause GDS rejection and require resubmission, delaying schedule availability by 24–48 hours</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Validate SSIM file against IATA standards</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordinator</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Validation report; corrected SSIM file if errors found</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Zero critical SSIM errors at point of GDS submission</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>OAG validation catches structural SSIM errors but does not validate operational feasibility (e.g., turn-time violations at specific airports); operationally infeasible schedules pass SSIM validation and are caught only during operations</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Submit validated schedule to GDS and NDC channels</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS / Sabre GDS / NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule live in Amadeus, Sabre, Travelport, and NDC channel</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule available in all GDS channels within 4 hours of SSIM submission; NDC availability within 2 hours</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Travelport GDS schedule updates lag Amadeus and Sabre by up to 6 hours due to batch processing cadence; passengers booking via Travelport-connected TMCs may see stale capacity, resulting in overbooking conflicts at check-in</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Monitor in-period seat utilization vs forecast</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Live booking data; capacity plan baseline</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Weekly utilization dashboard by market and departure date</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>System load factor ≥83% on average across active network; individual market load factor reviewed weekly</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM monitors inventory at O&amp;D level but does not natively surface segment-level spill and recapture estimates; capacity reoptimisation decisions rely on analyst judgment without automated spill quantification</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Trigger capacity reoptimisation for underperforming routes</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Utilization dashboard; routes with load factor &lt;78% within 60 days of departure</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Reoptimisation recommendation: frequency reduction, gauge swap, or fare stimulus</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Reoptimisation recommendation issued within 48 hours of load factor breach trigger</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Within-60-day capacity changes require coordinated updates across Altéa PSS (inventory), SkyWORKS (schedule), and Jeppesen Crew (pairings); the lack of a unified change-management workflow causes synchronisation failures and involuntary passenger re-accommodation</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-07</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Capacity Planning &amp; Utilization</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Log final utilization KPIs and close planning cycle</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Post-departure load factor actuals; forecast baseline</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Post-cycle capacity utilization report with variance analysis</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Post-cycle report published within 5 business days of season end; forecast vs actual load factor variance documented for model calibration</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Redshift data pipeline aggregates actuals from Altéa PSS on a 24-hour delay; post-departure analysis for redeye and overnight flights often reflects next-day timestamps, distorting daily load factor KPIs in Tableau dashboards</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-08: New Market Entry Feasibility — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -14,6 +14,7 @@
     <sheet name="NP-SP-05" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="NP-SP-06" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="NP-SP-07" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NP-SP-08" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -914,13 +915,21 @@
           <t>New Market Entry Feasibility</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr"/>
-      <c r="G10" s="8" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-08</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -5091,7 +5100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N142"/>
+  <dimension ref="A1:N160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -15264,6 +15273,1302 @@
         </is>
       </c>
       <c r="N142" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B143" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C143" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D143" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E143" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F143" s="16" t="inlineStr">
+        <is>
+          <t>Scan unserved O&amp;D opportunities</t>
+        </is>
+      </c>
+      <c r="G143" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H143" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I143" s="16" t="inlineStr">
+        <is>
+          <t>Historical booking data, MIDT traffic feeds, interline itinerary reports</t>
+        </is>
+      </c>
+      <c r="J143" s="16" t="inlineStr">
+        <is>
+          <t>Long list of candidate unserved or underserved city pairs</t>
+        </is>
+      </c>
+      <c r="K143" s="16" t="inlineStr">
+        <is>
+          <t>Minimum 20 candidate markets identified per planning cycle</t>
+        </is>
+      </c>
+      <c r="L143" s="16" t="inlineStr">
+        <is>
+          <t>MIDT data excludes LCC-direct bookings, leading to demand underestimation in price-sensitive leisure markets</t>
+        </is>
+      </c>
+      <c r="M143" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N143" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B144" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C144" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D144" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E144" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F144" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark competitor schedules on candidates</t>
+        </is>
+      </c>
+      <c r="G144" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H144" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I144" s="18" t="inlineStr">
+        <is>
+          <t>Candidate city-pair list from step 1.1</t>
+        </is>
+      </c>
+      <c r="J144" s="18" t="inlineStr">
+        <is>
+          <t>Competitor capacity, frequency, and fare level summary per market</t>
+        </is>
+      </c>
+      <c r="K144" s="18" t="inlineStr">
+        <is>
+          <t>Competitive gap identified for ≥60% of shortlisted markets</t>
+        </is>
+      </c>
+      <c r="L144" s="18" t="inlineStr">
+        <is>
+          <t>OAG data lags real-time charter and codeshare capacity additions by up to 3 weeks</t>
+        </is>
+      </c>
+      <c r="M144" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N144" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B145" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C145" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D145" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E145" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F145" s="16" t="inlineStr">
+        <is>
+          <t>Screen markets against minimum demand threshold</t>
+        </is>
+      </c>
+      <c r="G145" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H145" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I145" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D traffic volumes and OAG competitor data</t>
+        </is>
+      </c>
+      <c r="J145" s="16" t="inlineStr">
+        <is>
+          <t>Shortlisted markets with ≥150 unserved or recapturable pax/day</t>
+        </is>
+      </c>
+      <c r="K145" s="16" t="inlineStr">
+        <is>
+          <t>Demand threshold screening accuracy ≥90% vs. post-launch actuals</t>
+        </is>
+      </c>
+      <c r="L145" s="16" t="inlineStr">
+        <is>
+          <t>Redshift demand cubes are refreshed weekly; intra-week traffic spikes from events or promotions not captured</t>
+        </is>
+      </c>
+      <c r="M145" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N145" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B146" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C146" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D146" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E146" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F146" s="18" t="inlineStr">
+        <is>
+          <t>Forecast 12-month O&amp;D demand per market</t>
+        </is>
+      </c>
+      <c r="G146" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H146" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I146" s="18" t="inlineStr">
+        <is>
+          <t>Shortlisted markets, seasonality curves, macro-economic indices</t>
+        </is>
+      </c>
+      <c r="J146" s="18" t="inlineStr">
+        <is>
+          <t>Monthly O&amp;D demand forecast with P10/P50/P90 confidence bands</t>
+        </is>
+      </c>
+      <c r="K146" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% at 90-day horizon</t>
+        </is>
+      </c>
+      <c r="L146" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST models calibrated on existing network may not reflect latent demand in markets with no prior service</t>
+        </is>
+      </c>
+      <c r="M146" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N146" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B147" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C147" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D147" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E147" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>Simulate network spill and recapture impact</t>
+        </is>
+      </c>
+      <c r="G147" s="16" t="inlineStr">
+        <is>
+          <t>Network Simulation Analyst</t>
+        </is>
+      </c>
+      <c r="H147" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I147" s="16" t="inlineStr">
+        <is>
+          <t>Demand forecast, existing schedule SSIM file</t>
+        </is>
+      </c>
+      <c r="J147" s="16" t="inlineStr">
+        <is>
+          <t>Incremental revenue estimate, spill/recapture matrix, connecting feed impact</t>
+        </is>
+      </c>
+      <c r="K147" s="16" t="inlineStr">
+        <is>
+          <t>Spill recapture rate ≥35% for new route</t>
+        </is>
+      </c>
+      <c r="L147" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM simulations assume fixed itinerary preference weights; actual passenger path choice in new markets is untested</t>
+        </is>
+      </c>
+      <c r="M147" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N147" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B148" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C148" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D148" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E148" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F148" s="18" t="inlineStr">
+        <is>
+          <t>Model yield and price elasticity</t>
+        </is>
+      </c>
+      <c r="G148" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H148" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I148" s="18" t="inlineStr">
+        <is>
+          <t>Demand forecast, competitor fare benchmarks from OAG</t>
+        </is>
+      </c>
+      <c r="J148" s="18" t="inlineStr">
+        <is>
+          <t>Projected RASM, average fare, and fare class mix by month</t>
+        </is>
+      </c>
+      <c r="K148" s="18" t="inlineStr">
+        <is>
+          <t>Projected RASM ≥ CASM + 15% margin at base-case load factor of 83%</t>
+        </is>
+      </c>
+      <c r="L148" s="18" t="inlineStr">
+        <is>
+          <t>NRM fare elasticity models trained on existing markets; new leisure markets may exhibit steeper price sensitivity than modelled</t>
+        </is>
+      </c>
+      <c r="M148" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N148" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B149" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C149" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D149" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E149" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>Produce consolidated revenue forecast report</t>
+        </is>
+      </c>
+      <c r="G149" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H149" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I149" s="16" t="inlineStr">
+        <is>
+          <t>RASM/CASM output from NRM and SkyCAST</t>
+        </is>
+      </c>
+      <c r="J149" s="16" t="inlineStr">
+        <is>
+          <t>Revenue forecast dashboard and market scorecard</t>
+        </is>
+      </c>
+      <c r="K149" s="16" t="inlineStr">
+        <is>
+          <t>Scorecard completed within 2 business days of demand model sign-off</t>
+        </is>
+      </c>
+      <c r="L149" s="16" t="inlineStr">
+        <is>
+          <t>Manual data collation from SkyCAST, SkySYM, and NRM increases error risk and delays review cycle</t>
+        </is>
+      </c>
+      <c r="M149" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N149" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B150" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C150" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D150" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E150" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F150" s="18" t="inlineStr">
+        <is>
+          <t>Optimise fleet assignment for candidate route</t>
+        </is>
+      </c>
+      <c r="G150" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H150" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I150" s="18" t="inlineStr">
+        <is>
+          <t>Proposed frequency and timing, existing fleet utilisation plan</t>
+        </is>
+      </c>
+      <c r="J150" s="18" t="inlineStr">
+        <is>
+          <t>Optimal aircraft gauge and rotation plan for new route</t>
+        </is>
+      </c>
+      <c r="K150" s="18" t="inlineStr">
+        <is>
+          <t>Fleet utilisation ≥12.5 block hours/aircraft/day post-addition</t>
+        </is>
+      </c>
+      <c r="L150" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX optimisation can downgrade candidate route gauge when existing network utilisation is near ceiling, creating circular infeasibility</t>
+        </is>
+      </c>
+      <c r="M150" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N150" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B151" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C151" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D151" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E151" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F151" s="16" t="inlineStr">
+        <is>
+          <t>Evaluate frequency and timing trade-offs</t>
+        </is>
+      </c>
+      <c r="G151" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H151" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I151" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment output, competitive departure timing benchmarks</t>
+        </is>
+      </c>
+      <c r="J151" s="16" t="inlineStr">
+        <is>
+          <t>Recommended departure times and frequency options (1x, 2x, 3x daily)</t>
+        </is>
+      </c>
+      <c r="K151" s="16" t="inlineStr">
+        <is>
+          <t>Scheduling conflict rate &lt;5% in SkyWORKS validation</t>
+        </is>
+      </c>
+      <c r="L151" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS turnaround time constraints at congested focus-city stations (e.g. LAS, MDW) restrict viable departure windows to &lt;3 options</t>
+        </is>
+      </c>
+      <c r="M151" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N151" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="30" customHeight="1">
+      <c r="A152" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C152" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D152" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E152" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F152" s="18" t="inlineStr">
+        <is>
+          <t>Confirm spare aircraft availability at launch date</t>
+        </is>
+      </c>
+      <c r="G152" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H152" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I152" s="18" t="inlineStr">
+        <is>
+          <t>Proposed launch date, fleet delivery schedule, maintenance forecast</t>
+        </is>
+      </c>
+      <c r="J152" s="18" t="inlineStr">
+        <is>
+          <t>Aircraft availability confirmation or gap identification</t>
+        </is>
+      </c>
+      <c r="K152" s="18" t="inlineStr">
+        <is>
+          <t>Spare cover ratio ≥5% of active fleet on launch date</t>
+        </is>
+      </c>
+      <c r="L152" s="18" t="inlineStr">
+        <is>
+          <t>Boeing 737 MAX delivery delays (post-FAA recertification cycle) have repeatedly compressed launch windows by 6–18 months</t>
+        </is>
+      </c>
+      <c r="M152" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N152" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="30" customHeight="1">
+      <c r="A153" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B153" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C153" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D153" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E153" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F153" s="16" t="inlineStr">
+        <is>
+          <t>Check slot availability at origin and destination</t>
+        </is>
+      </c>
+      <c r="G153" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H153" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I153" s="16" t="inlineStr">
+        <is>
+          <t>Proposed departure times, airport coordination level (L1/L2/L3)</t>
+        </is>
+      </c>
+      <c r="J153" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability status, coordination response, or waiver requirement</t>
+        </is>
+      </c>
+      <c r="K153" s="16" t="inlineStr">
+        <is>
+          <t>Preferred slot obtained within ±30 min of target for ≥80% of requests</t>
+        </is>
+      </c>
+      <c r="L153" s="16" t="inlineStr">
+        <is>
+          <t>Slot-coordinated airports (Level 3) at international gateways impose 6–12 month lead times; historical precedence rules favour incumbents over new entrants</t>
+        </is>
+      </c>
+      <c r="M153" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N153" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30" customHeight="1">
+      <c r="A154" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B154" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C154" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D154" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E154" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F154" s="18" t="inlineStr">
+        <is>
+          <t>Validate gate and ground handling feasibility</t>
+        </is>
+      </c>
+      <c r="G154" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Planner</t>
+        </is>
+      </c>
+      <c r="H154" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I154" s="18" t="inlineStr">
+        <is>
+          <t>Proposed departure and arrival times, station gate inventory</t>
+        </is>
+      </c>
+      <c r="J154" s="18" t="inlineStr">
+        <is>
+          <t>Gate assignment feasibility report and required turnaround buffer</t>
+        </is>
+      </c>
+      <c r="K154" s="18" t="inlineStr">
+        <is>
+          <t>Gate conflict rate &lt;2% for new route insertion</t>
+        </is>
+      </c>
+      <c r="L154" s="18" t="inlineStr">
+        <is>
+          <t>SITA AMS data quality at smaller domestic stations is often incomplete; manual verification with airport authority adds 1–2 weeks</t>
+        </is>
+      </c>
+      <c r="M154" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N154" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B155" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C155" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D155" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E155" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F155" s="16" t="inlineStr">
+        <is>
+          <t>Assess crew pairing efficiency for new route</t>
+        </is>
+      </c>
+      <c r="G155" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H155" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I155" s="16" t="inlineStr">
+        <is>
+          <t>Proposed schedule, crew base locations, FAR Part 117 duty limits</t>
+        </is>
+      </c>
+      <c r="J155" s="16" t="inlineStr">
+        <is>
+          <t>Crew pairing cost estimate and minimum crew headcount requirement</t>
+        </is>
+      </c>
+      <c r="K155" s="16" t="inlineStr">
+        <is>
+          <t>Crew cost per block hour for new route ≤ system average + 10%</t>
+        </is>
+      </c>
+      <c r="L155" s="16" t="inlineStr">
+        <is>
+          <t>Routes originating from non-crew-base stations require deadhead positioning, adding $800–$1,200/day per crew pair and inflating CASM</t>
+        </is>
+      </c>
+      <c r="M155" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N155" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="30" customHeight="1">
+      <c r="A156" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B156" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C156" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D156" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E156" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F156" s="18" t="inlineStr">
+        <is>
+          <t>Build full-route P&amp;L model</t>
+        </is>
+      </c>
+      <c r="G156" s="18" t="inlineStr">
+        <is>
+          <t>Network Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H156" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I156" s="18" t="inlineStr">
+        <is>
+          <t>RASM forecast, CASM drivers, crew cost estimate, airport fees</t>
+        </is>
+      </c>
+      <c r="J156" s="18" t="inlineStr">
+        <is>
+          <t>12-month route P&amp;L with EBIT, ROIC, and contribution margin</t>
+        </is>
+      </c>
+      <c r="K156" s="18" t="inlineStr">
+        <is>
+          <t>ROIC ≥12% in base-case scenario at month 12</t>
+        </is>
+      </c>
+      <c r="L156" s="18" t="inlineStr">
+        <is>
+          <t>Airport fee structures at new international destinations often require renegotiation; provisional estimates in SAP can overstate profitability by 8–15%</t>
+        </is>
+      </c>
+      <c r="M156" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N156" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="30" customHeight="1">
+      <c r="A157" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B157" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C157" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D157" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E157" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F157" s="16" t="inlineStr">
+        <is>
+          <t>Run sensitivity and break-even load factor analysis</t>
+        </is>
+      </c>
+      <c r="G157" s="16" t="inlineStr">
+        <is>
+          <t>Network Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H157" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I157" s="16" t="inlineStr">
+        <is>
+          <t>P&amp;L model, P10/P50/P90 demand scenarios from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J157" s="16" t="inlineStr">
+        <is>
+          <t>Break-even load factor, downside ROIC, and go/no-go recommendation</t>
+        </is>
+      </c>
+      <c r="K157" s="16" t="inlineStr">
+        <is>
+          <t>Break-even load factor ≤75%; downside P10 ROIC ≥6%</t>
+        </is>
+      </c>
+      <c r="L157" s="16" t="inlineStr">
+        <is>
+          <t>Sensitivity model inputs (fuel price, FX, competitor response) are manually refreshed quarterly; stale assumptions distort go/no-go threshold</t>
+        </is>
+      </c>
+      <c r="M157" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N157" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="30" customHeight="1">
+      <c r="A158" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B158" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C158" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D158" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E158" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F158" s="18" t="inlineStr">
+        <is>
+          <t>Compile and submit commercial committee pack</t>
+        </is>
+      </c>
+      <c r="G158" s="18" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H158" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I158" s="18" t="inlineStr">
+        <is>
+          <t>Business case deck, P&amp;L model, ops feasibility sign-off, demand forecast</t>
+        </is>
+      </c>
+      <c r="J158" s="18" t="inlineStr">
+        <is>
+          <t>Formal new market entry proposal submitted to Commercial Committee</t>
+        </is>
+      </c>
+      <c r="K158" s="18" t="inlineStr">
+        <is>
+          <t>Pack submission ≥10 business days before committee review date</t>
+        </is>
+      </c>
+      <c r="L158" s="18" t="inlineStr">
+        <is>
+          <t>Cross-functional sign-off (Revenue Mgmt, Ops, Finance) often delayed due to differing planning horizons; average pack completion takes 18 days vs. 10-day target</t>
+        </is>
+      </c>
+      <c r="M158" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N158" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B159" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C159" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D159" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E159" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F159" s="16" t="inlineStr">
+        <is>
+          <t>File approved schedule and slots in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G159" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I159" s="16" t="inlineStr">
+        <is>
+          <t>Commercial Committee approval, proposed SSIM schedule record</t>
+        </is>
+      </c>
+      <c r="J159" s="16" t="inlineStr">
+        <is>
+          <t>New market schedule inserted into official season file</t>
+        </is>
+      </c>
+      <c r="K159" s="16" t="inlineStr">
+        <is>
+          <t>Schedule filed ≥120 days before service start (IATA SSIM standard)</t>
+        </is>
+      </c>
+      <c r="L159" s="16" t="inlineStr">
+        <is>
+          <t>Late approvals compress the SSIM filing window, risking GDS distribution gaps and reducing advance booking lead time below optimal 90-day curve</t>
+        </is>
+      </c>
+      <c r="M159" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N159" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="30" customHeight="1">
+      <c r="A160" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B160" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C160" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D160" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E160" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F160" s="18" t="inlineStr">
+        <is>
+          <t>Publish new route to GDS and NDC channels</t>
+        </is>
+      </c>
+      <c r="G160" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H160" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I160" s="18" t="inlineStr">
+        <is>
+          <t>Approved SSIM schedule, fare filing from ATPCO</t>
+        </is>
+      </c>
+      <c r="J160" s="18" t="inlineStr">
+        <is>
+          <t>New route live in Sabre GDS, Travelport GDS, Amadeus GDS, and NDC channel</t>
+        </is>
+      </c>
+      <c r="K160" s="18" t="inlineStr">
+        <is>
+          <t>GDS content live ≥90 days before first departure; NDC content live within 24 hours of GDS</t>
+        </is>
+      </c>
+      <c r="L160" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO fare filing cycle runs twice daily; missed filing window delays public fare availability by up to 12 hours, impacting early adopter bookings on launch-day announcement</t>
+        </is>
+      </c>
+      <c r="M160" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N160" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -22139,4 +23444,1420 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-08 — New Market Entry Feasibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: New Market Entry Feasibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Scan unserved O&amp;D opportunities</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Historical booking data, MIDT traffic feeds, interline itinerary reports</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Long list of candidate unserved or underserved city pairs</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Minimum 20 candidate markets identified per planning cycle</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>MIDT data excludes LCC-direct bookings, leading to demand underestimation in price-sensitive leisure markets</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark competitor schedules on candidates</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Candidate city-pair list from step 1.1</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Competitor capacity, frequency, and fare level summary per market</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Competitive gap identified for ≥60% of shortlisted markets</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>OAG data lags real-time charter and codeshare capacity additions by up to 3 weeks</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Screen markets against minimum demand threshold</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D traffic volumes and OAG competitor data</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Shortlisted markets with ≥150 unserved or recapturable pax/day</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Demand threshold screening accuracy ≥90% vs. post-launch actuals</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Redshift demand cubes are refreshed weekly; intra-week traffic spikes from events or promotions not captured</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Forecast 12-month O&amp;D demand per market</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Shortlisted markets, seasonality curves, macro-economic indices</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Monthly O&amp;D demand forecast with P10/P50/P90 confidence bands</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤8% at 90-day horizon</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST models calibrated on existing network may not reflect latent demand in markets with no prior service</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Simulate network spill and recapture impact</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Network Simulation Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Demand forecast, existing schedule SSIM file</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Incremental revenue estimate, spill/recapture matrix, connecting feed impact</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Spill recapture rate ≥35% for new route</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM simulations assume fixed itinerary preference weights; actual passenger path choice in new markets is untested</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Model yield and price elasticity</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Demand forecast, competitor fare benchmarks from OAG</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Projected RASM, average fare, and fare class mix by month</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Projected RASM ≥ CASM + 15% margin at base-case load factor of 83%</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>NRM fare elasticity models trained on existing markets; new leisure markets may exhibit steeper price sensitivity than modelled</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Produce consolidated revenue forecast report</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>RASM/CASM output from NRM and SkyCAST</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue forecast dashboard and market scorecard</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Scorecard completed within 2 business days of demand model sign-off</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Manual data collation from SkyCAST, SkySYM, and NRM increases error risk and delays review cycle</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Optimise fleet assignment for candidate route</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Proposed frequency and timing, existing fleet utilisation plan</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Optimal aircraft gauge and rotation plan for new route</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Fleet utilisation ≥12.5 block hours/aircraft/day post-addition</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>SkyMAX optimisation can downgrade candidate route gauge when existing network utilisation is near ceiling, creating circular infeasibility</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate frequency and timing trade-offs</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment output, competitive departure timing benchmarks</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Recommended departure times and frequency options (1x, 2x, 3x daily)</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Scheduling conflict rate &lt;5% in SkyWORKS validation</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS turnaround time constraints at congested focus-city stations (e.g. LAS, MDW) restrict viable departure windows to &lt;3 options</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Confirm spare aircraft availability at launch date</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Proposed launch date, fleet delivery schedule, maintenance forecast</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Aircraft availability confirmation or gap identification</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Spare cover ratio ≥5% of active fleet on launch date</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Boeing 737 MAX delivery delays (post-FAA recertification cycle) have repeatedly compressed launch windows by 6–18 months</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Check slot availability at origin and destination</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Proposed departure times, airport coordination level (L1/L2/L3)</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Slot availability status, coordination response, or waiver requirement</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Preferred slot obtained within ±30 min of target for ≥80% of requests</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Slot-coordinated airports (Level 3) at international gateways impose 6–12 month lead times; historical precedence rules favour incumbents over new entrants</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Validate gate and ground handling feasibility</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Airport Operations Planner</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Proposed departure and arrival times, station gate inventory</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Gate assignment feasibility report and required turnaround buffer</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Gate conflict rate &lt;2% for new route insertion</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>SITA AMS data quality at smaller domestic stations is often incomplete; manual verification with airport authority adds 1–2 weeks</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Assess crew pairing efficiency for new route</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Proposed schedule, crew base locations, FAR Part 117 duty limits</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Crew pairing cost estimate and minimum crew headcount requirement</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Crew cost per block hour for new route ≤ system average + 10%</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Routes originating from non-crew-base stations require deadhead positioning, adding $800–$1,200/day per crew pair and inflating CASM</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Build full-route P&amp;L model</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Network Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>RASM forecast, CASM drivers, crew cost estimate, airport fees</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>12-month route P&amp;L with EBIT, ROIC, and contribution margin</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>ROIC ≥12% in base-case scenario at month 12</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Airport fee structures at new international destinations often require renegotiation; provisional estimates in SAP can overstate profitability by 8–15%</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Run sensitivity and break-even load factor analysis</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Network Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>P&amp;L model, P10/P50/P90 demand scenarios from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Break-even load factor, downside ROIC, and go/no-go recommendation</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Break-even load factor ≤75%; downside P10 ROIC ≥6%</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Sensitivity model inputs (fuel price, FX, competitor response) are manually refreshed quarterly; stale assumptions distort go/no-go threshold</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Compile and submit commercial committee pack</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Business case deck, P&amp;L model, ops feasibility sign-off, demand forecast</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Formal new market entry proposal submitted to Commercial Committee</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Pack submission ≥10 business days before committee review date</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Cross-functional sign-off (Revenue Mgmt, Ops, Finance) often delayed due to differing planning horizons; average pack completion takes 18 days vs. 10-day target</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>File approved schedule and slots in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Commercial Committee approval, proposed SSIM schedule record</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>New market schedule inserted into official season file</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule filed ≥120 days before service start (IATA SSIM standard)</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Late approvals compress the SSIM filing window, risking GDS distribution gaps and reducing advance booking lead time below optimal 90-day curve</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-08</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>New Market Entry Feasibility</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Publish new route to GDS and NDC channels</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Approved SSIM schedule, fare filing from ATPCO</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>New route live in Sabre GDS, Travelport GDS, Amadeus GDS, and NDC channel</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>GDS content live ≥90 days before first departure; NDC content live within 24 hours of GDS</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare filing cycle runs twice daily; missed filing window delays public fare availability by up to 12 hours, impacting early adopter bookings on launch-day announcement</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-09: Alliance & Partnership Network Strategy — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -15,6 +15,7 @@
     <sheet name="NP-SP-06" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="NP-SP-07" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="NP-SP-08" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="NP-SP-09" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -952,13 +953,21 @@
           <t>Alliance &amp; Partnership Network Strategy</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="10" t="inlineStr"/>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-09</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -5100,7 +5109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N160"/>
+  <dimension ref="A1:N179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16569,6 +16578,1374 @@
         </is>
       </c>
       <c r="N160" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B161" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C161" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D161" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E161" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F161" s="16" t="inlineStr">
+        <is>
+          <t>Scan competitive landscape for partnership gaps</t>
+        </is>
+      </c>
+      <c r="G161" s="16" t="inlineStr">
+        <is>
+          <t>Network Strategy Analyst</t>
+        </is>
+      </c>
+      <c r="H161" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I161" s="16" t="inlineStr">
+        <is>
+          <t>Annual network strategy review, O&amp;D demand data, competitor alliance footprint</t>
+        </is>
+      </c>
+      <c r="J161" s="16" t="inlineStr">
+        <is>
+          <t>Partnership opportunity heat-map with prioritised O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K161" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D market coverage gap ≥5% of total addressable revenue identified</t>
+        </is>
+      </c>
+      <c r="L161" s="16" t="inlineStr">
+        <is>
+          <t>OAG data lags IATA SSIM submissions by 4–6 weeks, causing stale competitive benchmarks during fast-moving alliance negotiations</t>
+        </is>
+      </c>
+      <c r="M161" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N161" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="30" customHeight="1">
+      <c r="A162" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C162" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D162" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E162" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F162" s="18" t="inlineStr">
+        <is>
+          <t>Assess network complementarity of candidate partners</t>
+        </is>
+      </c>
+      <c r="G162" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Analyst</t>
+        </is>
+      </c>
+      <c r="H162" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I162" s="18" t="inlineStr">
+        <is>
+          <t>Candidate airline schedules (OAG), own network SSIM, O&amp;D demand forecast</t>
+        </is>
+      </c>
+      <c r="J162" s="18" t="inlineStr">
+        <is>
+          <t>Network complementarity score and connecting-flow traffic simulation per candidate</t>
+        </is>
+      </c>
+      <c r="K162" s="18" t="inlineStr">
+        <is>
+          <t>Incremental connecting pax potential ≥50,000 pax/year per candidate to proceed</t>
+        </is>
+      </c>
+      <c r="L162" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM simulation accuracy degrades for thin O&amp;D markets (&lt;10 bookings/day) where demand signal is insufficient for reliable modelling</t>
+        </is>
+      </c>
+      <c r="M162" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N162" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="30" customHeight="1">
+      <c r="A163" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C163" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D163" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E163" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F163" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Approve candidate shortlist for business case</t>
+        </is>
+      </c>
+      <c r="G163" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H163" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I163" s="16" t="inlineStr">
+        <is>
+          <t>Network complementarity scores, SkyCAST demand forecast by O&amp;D</t>
+        </is>
+      </c>
+      <c r="J163" s="16" t="inlineStr">
+        <is>
+          <t>Approved shortlist of ≤3 partner candidates for full financial modelling</t>
+        </is>
+      </c>
+      <c r="K163" s="16" t="inlineStr">
+        <is>
+          <t>Shortlist decision cycle ≤10 business days from scan initiation</t>
+        </is>
+      </c>
+      <c r="L163" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST demand forecasts for new O&amp;D markets (no historical booking data) carry ±25% confidence intervals, creating executive pushback on go/no-go decisions</t>
+        </is>
+      </c>
+      <c r="M163" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N163" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="A164" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B164" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C164" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D164" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E164" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F164" s="18" t="inlineStr">
+        <is>
+          <t>Model incremental codeshare revenue per O&amp;D</t>
+        </is>
+      </c>
+      <c r="G164" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H164" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I164" s="18" t="inlineStr">
+        <is>
+          <t>Approved partner shortlist, O&amp;D demand forecast, own fare inventory data</t>
+        </is>
+      </c>
+      <c r="J164" s="18" t="inlineStr">
+        <is>
+          <t>Revenue uplift model: incremental yield, load factor impact, and fare dilution estimate per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K164" s="18" t="inlineStr">
+        <is>
+          <t>Projected revenue uplift ≥3% on affected O&amp;D markets within 12 months of go-live</t>
+        </is>
+      </c>
+      <c r="L164" s="18" t="inlineStr">
+        <is>
+          <t>NRM O&amp;D revenue attribution for connecting itineraries is split by leg, obscuring true contribution of partner-fed traffic; manual adjustment required</t>
+        </is>
+      </c>
+      <c r="M164" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N164" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="30" customHeight="1">
+      <c r="A165" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B165" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C165" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D165" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E165" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F165" s="16" t="inlineStr">
+        <is>
+          <t>Model interline prorate and revenue-share economics</t>
+        </is>
+      </c>
+      <c r="G165" s="16" t="inlineStr">
+        <is>
+          <t>Commercial Finance Analyst</t>
+        </is>
+      </c>
+      <c r="H165" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I165" s="16" t="inlineStr">
+        <is>
+          <t>Revenue uplift model, proposed prorate split (IATA pro-rata or bilateral rates), partner financial statements</t>
+        </is>
+      </c>
+      <c r="J165" s="16" t="inlineStr">
+        <is>
+          <t>NPV analysis and 5-year P&amp;L impact; minimum acceptable prorate floor rate</t>
+        </is>
+      </c>
+      <c r="K165" s="16" t="inlineStr">
+        <is>
+          <t>Partnership NPV ≥ $5M over 5-year horizon to proceed to regulatory review</t>
+        </is>
+      </c>
+      <c r="L165" s="16" t="inlineStr">
+        <is>
+          <t>IATA standard prorate methodology (IATA Resolution 850) frequently under-compensates short-haul feeder partners, leading to prolonged bilateral negotiation cycles averaging 6–9 months</t>
+        </is>
+      </c>
+      <c r="M165" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N165" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="30" customHeight="1">
+      <c r="A166" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B166" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C166" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D166" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E166" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F166" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Approve business case for regulatory submission</t>
+        </is>
+      </c>
+      <c r="G166" s="18" t="inlineStr">
+        <is>
+          <t>Chief Commercial Officer</t>
+        </is>
+      </c>
+      <c r="H166" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I166" s="18" t="inlineStr">
+        <is>
+          <t>NPV model, revenue uplift forecast, prorate economics, risk register</t>
+        </is>
+      </c>
+      <c r="J166" s="18" t="inlineStr">
+        <is>
+          <t>Signed business case approval; mandate for regulatory and legal teams to proceed</t>
+        </is>
+      </c>
+      <c r="K166" s="18" t="inlineStr">
+        <is>
+          <t>Business case approval decision ≤15 business days from financial model submission</t>
+        </is>
+      </c>
+      <c r="L166" s="18" t="inlineStr">
+        <is>
+          <t>Executive approval stalls when NPV is marginal (e.g. $5–8M) and downside scenarios show revenue dilution on own metal — no standardised sensitivity threshold exists</t>
+        </is>
+      </c>
+      <c r="M166" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N166" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="30" customHeight="1">
+      <c r="A167" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B167" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C167" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D167" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E167" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F167" s="16" t="inlineStr">
+        <is>
+          <t>File for antitrust immunity or bilateral ASA review</t>
+        </is>
+      </c>
+      <c r="G167" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Director</t>
+        </is>
+      </c>
+      <c r="H167" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I167" s="16" t="inlineStr">
+        <is>
+          <t>Signed business case, proposed route list, partner agreement term sheet</t>
+        </is>
+      </c>
+      <c r="J167" s="16" t="inlineStr">
+        <is>
+          <t>DOT antitrust immunity application (US routes) or bilateral ASA amendment filing; IATA CRS slot filing if applicable</t>
+        </is>
+      </c>
+      <c r="K167" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory filing submitted within 20 business days of business case approval</t>
+        </is>
+      </c>
+      <c r="L167" s="16" t="inlineStr">
+        <is>
+          <t>US DOT antitrust immunity reviews average 12–18 months; EU bilateral amendments require ECAA or bilateral renegotiation via member-state government, adding 6–24 months of uncertainty</t>
+        </is>
+      </c>
+      <c r="M167" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N167" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="30" customHeight="1">
+      <c r="A168" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B168" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C168" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D168" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E168" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F168" s="18" t="inlineStr">
+        <is>
+          <t>Assess slot availability at partner hub airports</t>
+        </is>
+      </c>
+      <c r="G168" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination Manager</t>
+        </is>
+      </c>
+      <c r="H168" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I168" s="18" t="inlineStr">
+        <is>
+          <t>Proposed connecting schedule, partner hub slot pool data, IATA WSG constraints</t>
+        </is>
+      </c>
+      <c r="J168" s="18" t="inlineStr">
+        <is>
+          <t>Slot feasibility report; list of required slot swaps or grandfather-right acquisitions</t>
+        </is>
+      </c>
+      <c r="K168" s="18" t="inlineStr">
+        <is>
+          <t>Required slots secured for ≥90% of planned codeshare frequency within IATA schedule season</t>
+        </is>
+      </c>
+      <c r="L168" s="18" t="inlineStr">
+        <is>
+          <t>Level 3 coordinated airports (e.g. LHR, JFK, CDG) have near-zero slot availability; grandfather rights are held by incumbents, making new entry dependent on costly secondary market transactions or seasonal swap negotiations</t>
+        </is>
+      </c>
+      <c r="M168" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N168" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="30" customHeight="1">
+      <c r="A169" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B169" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C169" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D169" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E169" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F169" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Confirm regulatory and slot approvals are obtainable</t>
+        </is>
+      </c>
+      <c r="G169" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H169" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I169" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory filing status, slot feasibility report, legal counsel opinion</t>
+        </is>
+      </c>
+      <c r="J169" s="16" t="inlineStr">
+        <is>
+          <t>Go/no-go decision on regulatory path; if no-go, revised route scope or exit recommendation</t>
+        </is>
+      </c>
+      <c r="K169" s="16" t="inlineStr">
+        <is>
+          <t>Clear regulatory pathway confirmed within 30 business days of filing; slot coverage ≥90%</t>
+        </is>
+      </c>
+      <c r="L169" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory timelines are non-deterministic; slot constraints at Level 3 airports can invalidate the entire business case after 3–6 months of investment, with no partial recovery mechanism</t>
+        </is>
+      </c>
+      <c r="M169" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N169" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B170" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C170" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D170" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E170" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F170" s="18" t="inlineStr">
+        <is>
+          <t>Negotiate Interline Traffic Agreement and prorate rates</t>
+        </is>
+      </c>
+      <c r="G170" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="H170" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I170" s="18" t="inlineStr">
+        <is>
+          <t>Approved business case, regulatory clearance, IATA prorate methodology benchmark</t>
+        </is>
+      </c>
+      <c r="J170" s="18" t="inlineStr">
+        <is>
+          <t>Signed Interline Traffic Agreement (ITA) with bilateral prorate rates; Altéa interline carrier setup request</t>
+        </is>
+      </c>
+      <c r="K170" s="18" t="inlineStr">
+        <is>
+          <t>ITA negotiation closed within 60 days of regulatory clearance; prorate floor ≥65% of published fare for feeder leg</t>
+        </is>
+      </c>
+      <c r="L170" s="18" t="inlineStr">
+        <is>
+          <t>Altéa interline carrier onboarding requires manual BSP/clearing house configuration (ARC/IATA) taking 4–8 weeks after ITA signing — creates gap between commercial agreement and operational readiness</t>
+        </is>
+      </c>
+      <c r="M170" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N170" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="A171" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B171" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C171" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D171" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E171" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F171" s="16" t="inlineStr">
+        <is>
+          <t>Negotiate codeshare block-space or free-sale agreement</t>
+        </is>
+      </c>
+      <c r="G171" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="H171" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I171" s="16" t="inlineStr">
+        <is>
+          <t>Signed ITA, revenue model (minimum guaranteed block vs free-sale risk), partner capacity plan</t>
+        </is>
+      </c>
+      <c r="J171" s="16" t="inlineStr">
+        <is>
+          <t>Signed codeshare agreement specifying seat-block size, free-sale cap, and operating/marketing carrier designations</t>
+        </is>
+      </c>
+      <c r="K171" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare seat utilisation ≥70% on protected block within 6 months of launch</t>
+        </is>
+      </c>
+      <c r="L171" s="16" t="inlineStr">
+        <is>
+          <t>Free-sale agreements create inventory cannibalisation risk when partner's own metal competes on overlapping O&amp;D segments; NRM O&amp;D controls do not natively arbitrate between own-metal and codeshare inventory in real time</t>
+        </is>
+      </c>
+      <c r="M171" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N171" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="30" customHeight="1">
+      <c r="A172" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B172" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C172" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D172" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E172" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F172" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Validate agreement terms against revenue policy</t>
+        </is>
+      </c>
+      <c r="G172" s="18" t="inlineStr">
+        <is>
+          <t>Chief Commercial Officer</t>
+        </is>
+      </c>
+      <c r="H172" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I172" s="18" t="inlineStr">
+        <is>
+          <t>Signed ITA, codeshare agreement, updated revenue model with final prorate and block-space terms</t>
+        </is>
+      </c>
+      <c r="J172" s="18" t="inlineStr">
+        <is>
+          <t>Final commercial approval; instruction to legal to execute agreements and initiate system configuration</t>
+        </is>
+      </c>
+      <c r="K172" s="18" t="inlineStr">
+        <is>
+          <t>Agreement terms deliver ≥90% of NPV projected in approved business case</t>
+        </is>
+      </c>
+      <c r="L172" s="18" t="inlineStr">
+        <is>
+          <t>Late-stage concessions (e.g. prorate adjustments, block-space size reductions) during final negotiation rounds can erode NPV below approval threshold without triggering a formal re-approval cycle</t>
+        </is>
+      </c>
+      <c r="M172" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N172" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="30" customHeight="1">
+      <c r="A173" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B173" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C173" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D173" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E173" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F173" s="16" t="inlineStr">
+        <is>
+          <t>File codeshare and interline fares via ATPCO</t>
+        </is>
+      </c>
+      <c r="G173" s="16" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Fares Analyst</t>
+        </is>
+      </c>
+      <c r="H173" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I173" s="16" t="inlineStr">
+        <is>
+          <t>Executed codeshare agreement, joint fare construction rules, partner published fares</t>
+        </is>
+      </c>
+      <c r="J173" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare filings: through-fares, combinability rules, and ticketing authority records (TAT/TAH)</t>
+        </is>
+      </c>
+      <c r="K173" s="16" t="inlineStr">
+        <is>
+          <t>100% of planned O&amp;D joint fares live in GDS within 14 days of agreement execution</t>
+        </is>
+      </c>
+      <c r="L173" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO filing errors in combinability rules (Cat 10) cause GDS repricing failures, leading to customer-facing booking errors and revenue leakage; testing requires manual GDS shop verification across Sabre, Travelport, and Amadeus</t>
+        </is>
+      </c>
+      <c r="M173" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N173" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="30" customHeight="1">
+      <c r="A174" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B174" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C174" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D174" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E174" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F174" s="18" t="inlineStr">
+        <is>
+          <t>Configure PSS codeshare inventory and host carrier setup</t>
+        </is>
+      </c>
+      <c r="G174" s="18" t="inlineStr">
+        <is>
+          <t>PSS Configuration Specialist</t>
+        </is>
+      </c>
+      <c r="H174" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I174" s="18" t="inlineStr">
+        <is>
+          <t>Signed codeshare agreement, ATPCO fare filings, partner IATA carrier code and BSP enrollment</t>
+        </is>
+      </c>
+      <c r="J174" s="18" t="inlineStr">
+        <is>
+          <t>Altéa codeshare host/operating carrier configuration; booking class mapping; through check-in profile</t>
+        </is>
+      </c>
+      <c r="K174" s="18" t="inlineStr">
+        <is>
+          <t>PSS configuration completed and unit-tested within 21 days of agreement execution</t>
+        </is>
+      </c>
+      <c r="L174" s="18" t="inlineStr">
+        <is>
+          <t>Altéa codeshare configuration requires coordination across PSS, DCS (Departure Control), and Loyalty modules; misaligned Rapid Rewards/FFP accrual rules on partner segments result in customer complaints and manual points corrections</t>
+        </is>
+      </c>
+      <c r="M174" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N174" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="30" customHeight="1">
+      <c r="A175" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B175" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D175" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E175" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F175" s="16" t="inlineStr">
+        <is>
+          <t>Configure GDS codeshare display and availability feed</t>
+        </is>
+      </c>
+      <c r="G175" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H175" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I175" s="16" t="inlineStr">
+        <is>
+          <t>Altéa codeshare configuration, partner SSIM schedule, ATPCO fare records</t>
+        </is>
+      </c>
+      <c r="J175" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare itineraries visible and bookable in Sabre, Travelport, and Amadeus GDS; NDC API feed updated</t>
+        </is>
+      </c>
+      <c r="K175" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare itinerary display accuracy ≥99% across all three GDS within 7 days of Altéa config completion</t>
+        </is>
+      </c>
+      <c r="L175" s="16" t="inlineStr">
+        <is>
+          <t>GDS display logic for codeshare itineraries varies by channel (Sabre vs Travelport vs Amadeus); duplicate or ghost inventory appears when schedule changes are not propagated simultaneously across all three, requiring manual suppression</t>
+        </is>
+      </c>
+      <c r="M175" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N175" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="30" customHeight="1">
+      <c r="A176" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B176" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C176" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D176" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E176" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F176" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Pass end-to-end interoperability test suite</t>
+        </is>
+      </c>
+      <c r="G176" s="18" t="inlineStr">
+        <is>
+          <t>Partnerships Implementation Lead</t>
+        </is>
+      </c>
+      <c r="H176" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I176" s="18" t="inlineStr">
+        <is>
+          <t>PSS and GDS configuration, ATPCO fare records, test booking scripts (≥50 scenarios)</t>
+        </is>
+      </c>
+      <c r="J176" s="18" t="inlineStr">
+        <is>
+          <t>Interoperability test report; pass/fail verdict; defect log for remediation</t>
+        </is>
+      </c>
+      <c r="K176" s="18" t="inlineStr">
+        <is>
+          <t>≥95% of test scenarios pass (booking, ticketing, check-in, FFP accrual, irregular ops rebooking)</t>
+        </is>
+      </c>
+      <c r="L176" s="18" t="inlineStr">
+        <is>
+          <t>Irregular operations (IROPS) rebooking on codeshare itineraries across PSS boundaries is the most common test failure; Altéa does not natively rebook passengers onto partner-operated flights without manual agent intervention</t>
+        </is>
+      </c>
+      <c r="M176" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N176" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="30" customHeight="1">
+      <c r="A177" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B177" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C177" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D177" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E177" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F177" s="16" t="inlineStr">
+        <is>
+          <t>Launch codeshare service and activate commercial marketing</t>
+        </is>
+      </c>
+      <c r="G177" s="16" t="inlineStr">
+        <is>
+          <t>Partnerships Implementation Lead</t>
+        </is>
+      </c>
+      <c r="H177" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I177" s="16" t="inlineStr">
+        <is>
+          <t>Passed interoperability test, regulatory approvals confirmed, GDS live</t>
+        </is>
+      </c>
+      <c r="J177" s="16" t="inlineStr">
+        <is>
+          <t>Codeshare service live; press release issued; joint marketing campaign activated</t>
+        </is>
+      </c>
+      <c r="K177" s="16" t="inlineStr">
+        <is>
+          <t>First-week codeshare booking volume ≥50% of 90-day ramp forecast</t>
+        </is>
+      </c>
+      <c r="L177" s="16" t="inlineStr">
+        <is>
+          <t>Launch delays caused by late regulatory clearance compress the marketing window before the IATA schedule season, reducing awareness and first-season load factors vs forecast by an average of 8–12 percentage points</t>
+        </is>
+      </c>
+      <c r="M177" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N177" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="30" customHeight="1">
+      <c r="A178" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B178" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C178" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D178" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E178" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F178" s="18" t="inlineStr">
+        <is>
+          <t>Monitor connecting yield, load factor, and prorate settlement</t>
+        </is>
+      </c>
+      <c r="G178" s="18" t="inlineStr">
+        <is>
+          <t>Alliance Performance Analyst</t>
+        </is>
+      </c>
+      <c r="H178" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I178" s="18" t="inlineStr">
+        <is>
+          <t>Daily booking and revenue data from Altéa, GDS booking reports, IATA BSP settlement files</t>
+        </is>
+      </c>
+      <c r="J178" s="18" t="inlineStr">
+        <is>
+          <t>Monthly partnership performance dashboard: connecting pax yield, load factor, prorate actuals vs model, ancillary attach rate</t>
+        </is>
+      </c>
+      <c r="K178" s="18" t="inlineStr">
+        <is>
+          <t>Connecting pax yield ≥80% of model projection; prorate settlement discrepancy ≤2% of billed revenue</t>
+        </is>
+      </c>
+      <c r="L178" s="18" t="inlineStr">
+        <is>
+          <t>IATA BSP prorate settlement cycles are monthly with 45-day lag, making real-time revenue performance tracking dependent on booking-level proxies in Redshift rather than actual settled amounts</t>
+        </is>
+      </c>
+      <c r="M178" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N178" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="30" customHeight="1">
+      <c r="A179" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B179" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C179" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D179" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E179" s="15" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F179" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Annual review — expand, renegotiate, or exit partnership</t>
+        </is>
+      </c>
+      <c r="G179" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H179" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I179" s="16" t="inlineStr">
+        <is>
+          <t>12-month performance dashboard, updated NPV reforecast, partner relationship assessment, regulatory renewal status</t>
+        </is>
+      </c>
+      <c r="J179" s="16" t="inlineStr">
+        <is>
+          <t>Strategic decision: expand routes, renegotiate prorate/block terms, or serve notice of termination per agreement exit clause</t>
+        </is>
+      </c>
+      <c r="K179" s="16" t="inlineStr">
+        <is>
+          <t>Annual review completed and decision issued ≤90 days before agreement renewal deadline; partnership retained if NPV reforecast ≥80% of original approval threshold</t>
+        </is>
+      </c>
+      <c r="L179" s="16" t="inlineStr">
+        <is>
+          <t>Exit clauses in codeshare agreements typically require 6–12 months notice; airlines that miss the review cycle are locked into underperforming partnerships for an additional year, absorbing continued prorate losses</t>
+        </is>
+      </c>
+      <c r="M179" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N179" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -24860,4 +26237,1492 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-09 — Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Scan competitive landscape for partnership gaps</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Annual network strategy review, O&amp;D demand data, competitor alliance footprint</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Partnership opportunity heat-map with prioritised O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D market coverage gap ≥5% of total addressable revenue identified</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>OAG data lags IATA SSIM submissions by 4–6 weeks, causing stale competitive benchmarks during fast-moving alliance negotiations</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Assess network complementarity of candidate partners</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Strategy Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Candidate airline schedules (OAG), own network SSIM, O&amp;D demand forecast</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Network complementarity score and connecting-flow traffic simulation per candidate</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Incremental connecting pax potential ≥50,000 pax/year per candidate to proceed</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM simulation accuracy degrades for thin O&amp;D markets (&lt;10 bookings/day) where demand signal is insufficient for reliable modelling</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Approve candidate shortlist for business case</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Network complementarity scores, SkyCAST demand forecast by O&amp;D</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Approved shortlist of ≤3 partner candidates for full financial modelling</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Shortlist decision cycle ≤10 business days from scan initiation</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST demand forecasts for new O&amp;D markets (no historical booking data) carry ±25% confidence intervals, creating executive pushback on go/no-go decisions</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Model incremental codeshare revenue per O&amp;D</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Approved partner shortlist, O&amp;D demand forecast, own fare inventory data</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue uplift model: incremental yield, load factor impact, and fare dilution estimate per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Projected revenue uplift ≥3% on affected O&amp;D markets within 12 months of go-live</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>NRM O&amp;D revenue attribution for connecting itineraries is split by leg, obscuring true contribution of partner-fed traffic; manual adjustment required</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Model interline prorate and revenue-share economics</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Commercial Finance Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue uplift model, proposed prorate split (IATA pro-rata or bilateral rates), partner financial statements</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>NPV analysis and 5-year P&amp;L impact; minimum acceptable prorate floor rate</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Partnership NPV ≥ $5M over 5-year horizon to proceed to regulatory review</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>IATA standard prorate methodology (IATA Resolution 850) frequently under-compensates short-haul feeder partners, leading to prolonged bilateral negotiation cycles averaging 6–9 months</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Approve business case for regulatory submission</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Chief Commercial Officer</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>NPV model, revenue uplift forecast, prorate economics, risk register</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Signed business case approval; mandate for regulatory and legal teams to proceed</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Business case approval decision ≤15 business days from financial model submission</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Executive approval stalls when NPV is marginal (e.g. $5–8M) and downside scenarios show revenue dilution on own metal — no standardised sensitivity threshold exists</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>File for antitrust immunity or bilateral ASA review</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Director</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Signed business case, proposed route list, partner agreement term sheet</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>DOT antitrust immunity application (US routes) or bilateral ASA amendment filing; IATA CRS slot filing if applicable</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory filing submitted within 20 business days of business case approval</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>US DOT antitrust immunity reviews average 12–18 months; EU bilateral amendments require ECAA or bilateral renegotiation via member-state government, adding 6–24 months of uncertainty</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Assess slot availability at partner hub airports</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Manager</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Proposed connecting schedule, partner hub slot pool data, IATA WSG constraints</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Slot feasibility report; list of required slot swaps or grandfather-right acquisitions</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Required slots secured for ≥90% of planned codeshare frequency within IATA schedule season</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Level 3 coordinated airports (e.g. LHR, JFK, CDG) have near-zero slot availability; grandfather rights are held by incumbents, making new entry dependent on costly secondary market transactions or seasonal swap negotiations</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Confirm regulatory and slot approvals are obtainable</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory filing status, slot feasibility report, legal counsel opinion</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Go/no-go decision on regulatory path; if no-go, revised route scope or exit recommendation</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Clear regulatory pathway confirmed within 30 business days of filing; slot coverage ≥90%</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory timelines are non-deterministic; slot constraints at Level 3 airports can invalidate the entire business case after 3–6 months of investment, with no partial recovery mechanism</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Negotiate Interline Traffic Agreement and prorate rates</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Approved business case, regulatory clearance, IATA prorate methodology benchmark</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Signed Interline Traffic Agreement (ITA) with bilateral prorate rates; Altéa interline carrier setup request</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>ITA negotiation closed within 60 days of regulatory clearance; prorate floor ≥65% of published fare for feeder leg</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Altéa interline carrier onboarding requires manual BSP/clearing house configuration (ARC/IATA) taking 4–8 weeks after ITA signing — creates gap between commercial agreement and operational readiness</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Negotiate codeshare block-space or free-sale agreement</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Signed ITA, revenue model (minimum guaranteed block vs free-sale risk), partner capacity plan</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Signed codeshare agreement specifying seat-block size, free-sale cap, and operating/marketing carrier designations</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare seat utilisation ≥70% on protected block within 6 months of launch</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Free-sale agreements create inventory cannibalisation risk when partner's own metal competes on overlapping O&amp;D segments; NRM O&amp;D controls do not natively arbitrate between own-metal and codeshare inventory in real time</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Validate agreement terms against revenue policy</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Chief Commercial Officer</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Signed ITA, codeshare agreement, updated revenue model with final prorate and block-space terms</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Final commercial approval; instruction to legal to execute agreements and initiate system configuration</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Agreement terms deliver ≥90% of NPV projected in approved business case</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Late-stage concessions (e.g. prorate adjustments, block-space size reductions) during final negotiation rounds can erode NPV below approval threshold without triggering a formal re-approval cycle</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>File codeshare and interline fares via ATPCO</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Fares Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Executed codeshare agreement, joint fare construction rules, partner published fares</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO fare filings: through-fares, combinability rules, and ticketing authority records (TAT/TAH)</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>100% of planned O&amp;D joint fares live in GDS within 14 days of agreement execution</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO filing errors in combinability rules (Cat 10) cause GDS repricing failures, leading to customer-facing booking errors and revenue leakage; testing requires manual GDS shop verification across Sabre, Travelport, and Amadeus</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Configure PSS codeshare inventory and host carrier setup</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>PSS Configuration Specialist</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Signed codeshare agreement, ATPCO fare filings, partner IATA carrier code and BSP enrollment</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Altéa codeshare host/operating carrier configuration; booking class mapping; through check-in profile</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>PSS configuration completed and unit-tested within 21 days of agreement execution</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Altéa codeshare configuration requires coordination across PSS, DCS (Departure Control), and Loyalty modules; misaligned Rapid Rewards/FFP accrual rules on partner segments result in customer complaints and manual points corrections</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Configure GDS codeshare display and availability feed</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Altéa codeshare configuration, partner SSIM schedule, ATPCO fare records</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare itineraries visible and bookable in Sabre, Travelport, and Amadeus GDS; NDC API feed updated</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare itinerary display accuracy ≥99% across all three GDS within 7 days of Altéa config completion</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>GDS display logic for codeshare itineraries varies by channel (Sabre vs Travelport vs Amadeus); duplicate or ghost inventory appears when schedule changes are not propagated simultaneously across all three, requiring manual suppression</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Gate: Pass end-to-end interoperability test suite</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Partnerships Implementation Lead</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>PSS and GDS configuration, ATPCO fare records, test booking scripts (≥50 scenarios)</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Interoperability test report; pass/fail verdict; defect log for remediation</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>≥95% of test scenarios pass (booking, ticketing, check-in, FFP accrual, irregular ops rebooking)</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Irregular operations (IROPS) rebooking on codeshare itineraries across PSS boundaries is the most common test failure; Altéa does not natively rebook passengers onto partner-operated flights without manual agent intervention</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Launch codeshare service and activate commercial marketing</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Partnerships Implementation Lead</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Passed interoperability test, regulatory approvals confirmed, GDS live</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Codeshare service live; press release issued; joint marketing campaign activated</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>First-week codeshare booking volume ≥50% of 90-day ramp forecast</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Launch delays caused by late regulatory clearance compress the marketing window before the IATA schedule season, reducing awareness and first-season load factors vs forecast by an average of 8–12 percentage points</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Monitor connecting yield, load factor, and prorate settlement</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Alliance Performance Analyst</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Daily booking and revenue data from Altéa, GDS booking reports, IATA BSP settlement files</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Monthly partnership performance dashboard: connecting pax yield, load factor, prorate actuals vs model, ancillary attach rate</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Connecting pax yield ≥80% of model projection; prorate settlement discrepancy ≤2% of billed revenue</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>IATA BSP prorate settlement cycles are monthly with 45-day lag, making real-time revenue performance tracking dependent on booking-level proxies in Redshift rather than actual settled amounts</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-09</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Alliance &amp; Partnership Network Strategy</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Gate: Annual review — expand, renegotiate, or exit partnership</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>12-month performance dashboard, updated NPV reforecast, partner relationship assessment, regulatory renewal status</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Strategic decision: expand routes, renegotiate prorate/block terms, or serve notice of termination per agreement exit clause</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>Annual review completed and decision issued ≤90 days before agreement renewal deadline; partnership retained if NPV reforecast ≥80% of original approval threshold</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>Exit clauses in codeshare agreements typically require 6–12 months notice; airlines that miss the review cycle are locked into underperforming partnerships for an additional year, absorbing continued prorate losses</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NP-SP-10: SSIM File Management & Distribution — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -16,6 +16,7 @@
     <sheet name="NP-SP-07" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="NP-SP-08" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="NP-SP-09" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="NP-SP-10" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -990,13 +991,21 @@
           <t>SSIM File Management &amp; Distribution</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-10</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -5098,6 +5107,1350 @@
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A154:D154"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-10 — SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Confirm seasonal schedule freeze milestone</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal schedule deadline calendar; IATA scheduling conference date</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Freeze confirmation memo; SkyWORKS workspace locked for SSIM export</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule frozen ≥8 weeks before IATA seasonal deadline</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS freeze locks the shared planning workspace; late changes require an emergency amendment process that triggers full GDS re-distribution</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Extract full flight schedule from SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed schedule freeze; all routes with equipment assignments and frequency patterns</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Raw schedule export file (flights, equipment ICAO codes, times, frequencies, cabin configs)</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Extract completeness ≥99.5% of scheduled flight legs</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS export occasionally omits wet-lease and codeshare-operated segments, requiring manual reconciliation before SSIM generation</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate schedule data completeness and codes</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Raw schedule export file</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Validated schedule dataset with exception log of missing or invalid fields</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Data quality score ≥99% (missing or invalid fields &lt;1% of records)</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Missing IATA airport codes or unrecognised aircraft ICAO type codes cause SSIM Chapter 7 format rejection at downstream GDS ingestion</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Generate SSIM Chapter 7 format file</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated schedule dataset</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 formatted file with header, record types 1–4, and trailer</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>File generated within 4 business hours of schedule freeze confirmation</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM output does not include non-IATA member charter operations; manual record append required, increasing error risk</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Run IATA SSIM syntax and schema validation</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Validation report: pass/fail status with line-level error list</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Zero critical format errors before external submission</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS embedded IATA SSIM validator version lags IATA annual publication cycle by up to 6 months, causing false positives on new record type extensions requiring manual sign-off</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Correct SSIM format errors and re-validate</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Validation error report with line references</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Corrected and revalidated SSIM file cleared for distribution</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Error resolution cycle completed within 2 business days</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Iterative correction loops frequently triggered by aircraft sub-fleet code changes (e.g. 73H vs 73W); no automated mapping maintained between SkyWORKS fleet types and SSIM equipment codes</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Identify slot-controlled airports in schedule</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM file; IATA Level 2 and Level 3 coordinated airport register</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Slot request list by airport, season, and designated coordinator body</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Slot request list submitted ≥4 weeks before IATA scheduling conference</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>IATA Level 2/3 coordination status changes seasonally with no automated alert; reclassification of an airport discovered post-SSIM generation forces last-minute slot programme additions</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Submit slot requests to airport coordinators</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Slot request list; SSIM extract for the relevant airports</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>SLOT/S2 and SAL messages submitted to ACL (UK), COHOR (France), FAA ATCSCC (US), and regional bodies</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Submission acknowledgement received from all coordinators within 5 business days</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Some regional coordinators (e.g. ACNUSA for Paris CDG, NACC for Caribbean) require national-format messages rather than standard IATA WSG SSIM; manual reformatting needed per coordinator</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Reconcile slot confirmations against requests</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Coordinator confirmation messages; original slot request register</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Reconciliation report: confirmed vs. requested vs. denied slots with variance analysis</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Slot hit rate ≥90% of requested times within ±30 minutes</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Slot denials at Level 3 constrained airports (LHR, JFK, FRA) require re-planning iterations with the Network team; no automated feedback loop into SkyWORKS to propagate confirmed times back to the live schedule</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Transmit SSIM to Sabre Schedule Distribution</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Sabre Schedule Distribution System (SDS)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Validated and slot-reconciled SSIM file</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Sabre SDS ingest confirmation receipt with processing timestamp</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Sabre display accuracy ≥99% within 48 hours of transmission</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Sabre SDS equipment type mapping for new aircraft variants (e.g. A321XLR, 737 MAX 10) lags IATA SSIM type code releases by up to one schedule season, causing booking class display errors</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Transmit SSIM to Amadeus and Travelport GDS</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS / Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>GDS ingest confirmation receipts from Amadeus and Travelport</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Display accuracy ≥99% within 48 hours on both GDS platforms</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus and Travelport have different SSIM ingestion cutoff times and batch processing windows; staggered submissions required to avoid inconsistent schedule displays across booking channels during the transition window</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Distribute schedule data to OAG and Cirium</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>OAG and Cirium data feed ingest acknowledgements</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule data live on OAG and Cirium within 72 hours of SSIM receipt</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>OAG charges amendment fees for mid-cycle corrections; unplanned network changes require budget pre-approval before re-submission, introducing a 2–5 day delay in schedule visibility for travel agencies and competitors</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Verify GDS schedule display accuracy post-load</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS / Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Submitted SSIM file; post-load GDS availability and schedule displays</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Display verification report: error rate by flight, equipment, and booking class</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>GDS display error rate &lt;0.5% across sampled flights</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>GDS automated post-load checks do not cover all booking class inheritance mappings for new routes; manual spot-check required for every new city-pair added to the schedule</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Distribute SSIM to codeshare and interline partners</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Alliance Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>SITA STB (Schedule Transfer Bridge)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM file; interline and codeshare partner agreement register</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM sub-files transmitted to each codeshare and interline partner via SITA STB</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Partner receipt confirmation received within 48 hours for ≥95% of partners</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>SITA STB acknowledgement messages do not distinguish between received and processed status; partners occasionally load superseded SSIM versions when multiple amendments are in flight simultaneously</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Notify airports of schedule via IATA AHM 090</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>SITA AMS (Airport Management System)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmed schedule with slot allocations</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>AHM 090 schedule notification messages transmitted to all served airports</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Airport acknowledgement received from ≥95% of notified airports within 5 business days</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>AHM 090 message format compliance varies by airport handler; some outstations require a direct email supplement alongside SITA MATIP messages, adding manual workload with no audit trail in AMS</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Archive versioned SSIM with change log</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Final SSIM file; amendment history register</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Versioned SSIM archive in AWS S3 with structured change log (season, date, amendment number, changed flights)</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>100% version retention; any historical SSIM retrievable within 1 business hour</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>No automated versioning in SkyWORKS SSIM module; manual naming conventions lead to version confusion when multiple mid-season amendments are active, creating audit and regulatory traceability risk</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Manage mid-season SSIM amendment cycle</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Network change requests; schedule irregularity reports; commercial re-routing decisions</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Amendment SSIM file; updated GDS displays; re-notified partners and airports</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Full amendment cycle (generate → validate → distribute → verify) completed within 5 business days</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Mid-season amendments trigger full re-distribution to all GDS, aggregators, and partners; SkyWORKS SSIM module has no selective-update capability, so even single-flight changes require a complete file re-transmission</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5109,7 +6462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N179"/>
+  <dimension ref="A1:N196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17948,6 +19301,1230 @@
       <c r="N179" s="15" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B180" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C180" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D180" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E180" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F180" s="18" t="inlineStr">
+        <is>
+          <t>Confirm seasonal schedule freeze milestone</t>
+        </is>
+      </c>
+      <c r="G180" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H180" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I180" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal schedule deadline calendar; IATA scheduling conference date</t>
+        </is>
+      </c>
+      <c r="J180" s="18" t="inlineStr">
+        <is>
+          <t>Freeze confirmation memo; SkyWORKS workspace locked for SSIM export</t>
+        </is>
+      </c>
+      <c r="K180" s="18" t="inlineStr">
+        <is>
+          <t>Schedule frozen ≥8 weeks before IATA seasonal deadline</t>
+        </is>
+      </c>
+      <c r="L180" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS freeze locks the shared planning workspace; late changes require an emergency amendment process that triggers full GDS re-distribution</t>
+        </is>
+      </c>
+      <c r="M180" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N180" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B181" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C181" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D181" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E181" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F181" s="16" t="inlineStr">
+        <is>
+          <t>Extract full flight schedule from SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G181" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H181" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I181" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed schedule freeze; all routes with equipment assignments and frequency patterns</t>
+        </is>
+      </c>
+      <c r="J181" s="16" t="inlineStr">
+        <is>
+          <t>Raw schedule export file (flights, equipment ICAO codes, times, frequencies, cabin configs)</t>
+        </is>
+      </c>
+      <c r="K181" s="16" t="inlineStr">
+        <is>
+          <t>Extract completeness ≥99.5% of scheduled flight legs</t>
+        </is>
+      </c>
+      <c r="L181" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS export occasionally omits wet-lease and codeshare-operated segments, requiring manual reconciliation before SSIM generation</t>
+        </is>
+      </c>
+      <c r="M181" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N181" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B182" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C182" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D182" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E182" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F182" s="18" t="inlineStr">
+        <is>
+          <t>Validate schedule data completeness and codes</t>
+        </is>
+      </c>
+      <c r="G182" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H182" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I182" s="18" t="inlineStr">
+        <is>
+          <t>Raw schedule export file</t>
+        </is>
+      </c>
+      <c r="J182" s="18" t="inlineStr">
+        <is>
+          <t>Validated schedule dataset with exception log of missing or invalid fields</t>
+        </is>
+      </c>
+      <c r="K182" s="18" t="inlineStr">
+        <is>
+          <t>Data quality score ≥99% (missing or invalid fields &lt;1% of records)</t>
+        </is>
+      </c>
+      <c r="L182" s="18" t="inlineStr">
+        <is>
+          <t>Missing IATA airport codes or unrecognised aircraft ICAO type codes cause SSIM Chapter 7 format rejection at downstream GDS ingestion</t>
+        </is>
+      </c>
+      <c r="M182" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N182" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B183" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C183" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D183" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E183" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F183" s="16" t="inlineStr">
+        <is>
+          <t>Generate SSIM Chapter 7 format file</t>
+        </is>
+      </c>
+      <c r="G183" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H183" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I183" s="16" t="inlineStr">
+        <is>
+          <t>Validated schedule dataset</t>
+        </is>
+      </c>
+      <c r="J183" s="16" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 formatted file with header, record types 1–4, and trailer</t>
+        </is>
+      </c>
+      <c r="K183" s="16" t="inlineStr">
+        <is>
+          <t>File generated within 4 business hours of schedule freeze confirmation</t>
+        </is>
+      </c>
+      <c r="L183" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS SSIM output does not include non-IATA member charter operations; manual record append required, increasing error risk</t>
+        </is>
+      </c>
+      <c r="M183" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N183" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B184" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C184" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D184" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E184" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F184" s="18" t="inlineStr">
+        <is>
+          <t>Run IATA SSIM syntax and schema validation</t>
+        </is>
+      </c>
+      <c r="G184" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H184" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I184" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J184" s="18" t="inlineStr">
+        <is>
+          <t>Validation report: pass/fail status with line-level error list</t>
+        </is>
+      </c>
+      <c r="K184" s="18" t="inlineStr">
+        <is>
+          <t>Zero critical format errors before external submission</t>
+        </is>
+      </c>
+      <c r="L184" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS embedded IATA SSIM validator version lags IATA annual publication cycle by up to 6 months, causing false positives on new record type extensions requiring manual sign-off</t>
+        </is>
+      </c>
+      <c r="M184" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N184" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B185" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C185" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D185" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E185" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F185" s="16" t="inlineStr">
+        <is>
+          <t>Correct SSIM format errors and re-validate</t>
+        </is>
+      </c>
+      <c r="G185" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H185" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I185" s="16" t="inlineStr">
+        <is>
+          <t>Validation error report with line references</t>
+        </is>
+      </c>
+      <c r="J185" s="16" t="inlineStr">
+        <is>
+          <t>Corrected and revalidated SSIM file cleared for distribution</t>
+        </is>
+      </c>
+      <c r="K185" s="16" t="inlineStr">
+        <is>
+          <t>Error resolution cycle completed within 2 business days</t>
+        </is>
+      </c>
+      <c r="L185" s="16" t="inlineStr">
+        <is>
+          <t>Iterative correction loops frequently triggered by aircraft sub-fleet code changes (e.g. 73H vs 73W); no automated mapping maintained between SkyWORKS fleet types and SSIM equipment codes</t>
+        </is>
+      </c>
+      <c r="M185" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N185" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B186" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C186" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D186" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E186" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F186" s="18" t="inlineStr">
+        <is>
+          <t>Identify slot-controlled airports in schedule</t>
+        </is>
+      </c>
+      <c r="G186" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H186" s="18" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I186" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM file; IATA Level 2 and Level 3 coordinated airport register</t>
+        </is>
+      </c>
+      <c r="J186" s="18" t="inlineStr">
+        <is>
+          <t>Slot request list by airport, season, and designated coordinator body</t>
+        </is>
+      </c>
+      <c r="K186" s="18" t="inlineStr">
+        <is>
+          <t>Slot request list submitted ≥4 weeks before IATA scheduling conference</t>
+        </is>
+      </c>
+      <c r="L186" s="18" t="inlineStr">
+        <is>
+          <t>IATA Level 2/3 coordination status changes seasonally with no automated alert; reclassification of an airport discovered post-SSIM generation forces last-minute slot programme additions</t>
+        </is>
+      </c>
+      <c r="M186" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N186" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B187" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C187" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D187" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E187" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F187" s="16" t="inlineStr">
+        <is>
+          <t>Submit slot requests to airport coordinators</t>
+        </is>
+      </c>
+      <c r="G187" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H187" s="16" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I187" s="16" t="inlineStr">
+        <is>
+          <t>Slot request list; SSIM extract for the relevant airports</t>
+        </is>
+      </c>
+      <c r="J187" s="16" t="inlineStr">
+        <is>
+          <t>SLOT/S2 and SAL messages submitted to ACL (UK), COHOR (France), FAA ATCSCC (US), and regional bodies</t>
+        </is>
+      </c>
+      <c r="K187" s="16" t="inlineStr">
+        <is>
+          <t>Submission acknowledgement received from all coordinators within 5 business days</t>
+        </is>
+      </c>
+      <c r="L187" s="16" t="inlineStr">
+        <is>
+          <t>Some regional coordinators (e.g. ACNUSA for Paris CDG, NACC for Caribbean) require national-format messages rather than standard IATA WSG SSIM; manual reformatting needed per coordinator</t>
+        </is>
+      </c>
+      <c r="M187" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N187" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="30" customHeight="1">
+      <c r="A188" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B188" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C188" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D188" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E188" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F188" s="18" t="inlineStr">
+        <is>
+          <t>Reconcile slot confirmations against requests</t>
+        </is>
+      </c>
+      <c r="G188" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H188" s="18" t="inlineStr">
+        <is>
+          <t>IATA WSG Slot Portal</t>
+        </is>
+      </c>
+      <c r="I188" s="18" t="inlineStr">
+        <is>
+          <t>Coordinator confirmation messages; original slot request register</t>
+        </is>
+      </c>
+      <c r="J188" s="18" t="inlineStr">
+        <is>
+          <t>Reconciliation report: confirmed vs. requested vs. denied slots with variance analysis</t>
+        </is>
+      </c>
+      <c r="K188" s="18" t="inlineStr">
+        <is>
+          <t>Slot hit rate ≥90% of requested times within ±30 minutes</t>
+        </is>
+      </c>
+      <c r="L188" s="18" t="inlineStr">
+        <is>
+          <t>Slot denials at Level 3 constrained airports (LHR, JFK, FRA) require re-planning iterations with the Network team; no automated feedback loop into SkyWORKS to propagate confirmed times back to the live schedule</t>
+        </is>
+      </c>
+      <c r="M188" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N188" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="30" customHeight="1">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B189" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C189" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D189" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E189" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F189" s="16" t="inlineStr">
+        <is>
+          <t>Transmit SSIM to Sabre Schedule Distribution</t>
+        </is>
+      </c>
+      <c r="G189" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H189" s="16" t="inlineStr">
+        <is>
+          <t>Sabre Schedule Distribution System (SDS)</t>
+        </is>
+      </c>
+      <c r="I189" s="16" t="inlineStr">
+        <is>
+          <t>Validated and slot-reconciled SSIM file</t>
+        </is>
+      </c>
+      <c r="J189" s="16" t="inlineStr">
+        <is>
+          <t>Sabre SDS ingest confirmation receipt with processing timestamp</t>
+        </is>
+      </c>
+      <c r="K189" s="16" t="inlineStr">
+        <is>
+          <t>Sabre display accuracy ≥99% within 48 hours of transmission</t>
+        </is>
+      </c>
+      <c r="L189" s="16" t="inlineStr">
+        <is>
+          <t>Sabre SDS equipment type mapping for new aircraft variants (e.g. A321XLR, 737 MAX 10) lags IATA SSIM type code releases by up to one schedule season, causing booking class display errors</t>
+        </is>
+      </c>
+      <c r="M189" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N189" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="30" customHeight="1">
+      <c r="A190" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B190" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C190" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D190" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E190" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F190" s="18" t="inlineStr">
+        <is>
+          <t>Transmit SSIM to Amadeus and Travelport GDS</t>
+        </is>
+      </c>
+      <c r="G190" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H190" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS / Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I190" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J190" s="18" t="inlineStr">
+        <is>
+          <t>GDS ingest confirmation receipts from Amadeus and Travelport</t>
+        </is>
+      </c>
+      <c r="K190" s="18" t="inlineStr">
+        <is>
+          <t>Display accuracy ≥99% within 48 hours on both GDS platforms</t>
+        </is>
+      </c>
+      <c r="L190" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus and Travelport have different SSIM ingestion cutoff times and batch processing windows; staggered submissions required to avoid inconsistent schedule displays across booking channels during the transition window</t>
+        </is>
+      </c>
+      <c r="M190" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N190" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B191" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C191" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D191" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E191" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F191" s="16" t="inlineStr">
+        <is>
+          <t>Distribute schedule data to OAG and Cirium</t>
+        </is>
+      </c>
+      <c r="G191" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H191" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I191" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM file</t>
+        </is>
+      </c>
+      <c r="J191" s="16" t="inlineStr">
+        <is>
+          <t>OAG and Cirium data feed ingest acknowledgements</t>
+        </is>
+      </c>
+      <c r="K191" s="16" t="inlineStr">
+        <is>
+          <t>Schedule data live on OAG and Cirium within 72 hours of SSIM receipt</t>
+        </is>
+      </c>
+      <c r="L191" s="16" t="inlineStr">
+        <is>
+          <t>OAG charges amendment fees for mid-cycle corrections; unplanned network changes require budget pre-approval before re-submission, introducing a 2–5 day delay in schedule visibility for travel agencies and competitors</t>
+        </is>
+      </c>
+      <c r="M191" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N191" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="30" customHeight="1">
+      <c r="A192" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B192" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C192" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D192" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E192" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F192" s="18" t="inlineStr">
+        <is>
+          <t>Verify GDS schedule display accuracy post-load</t>
+        </is>
+      </c>
+      <c r="G192" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H192" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS / Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I192" s="18" t="inlineStr">
+        <is>
+          <t>Submitted SSIM file; post-load GDS availability and schedule displays</t>
+        </is>
+      </c>
+      <c r="J192" s="18" t="inlineStr">
+        <is>
+          <t>Display verification report: error rate by flight, equipment, and booking class</t>
+        </is>
+      </c>
+      <c r="K192" s="18" t="inlineStr">
+        <is>
+          <t>GDS display error rate &lt;0.5% across sampled flights</t>
+        </is>
+      </c>
+      <c r="L192" s="18" t="inlineStr">
+        <is>
+          <t>GDS automated post-load checks do not cover all booking class inheritance mappings for new routes; manual spot-check required for every new city-pair added to the schedule</t>
+        </is>
+      </c>
+      <c r="M192" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N192" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="30" customHeight="1">
+      <c r="A193" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B193" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C193" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D193" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E193" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F193" s="16" t="inlineStr">
+        <is>
+          <t>Distribute SSIM to codeshare and interline partners</t>
+        </is>
+      </c>
+      <c r="G193" s="16" t="inlineStr">
+        <is>
+          <t>Alliance Operations Analyst</t>
+        </is>
+      </c>
+      <c r="H193" s="16" t="inlineStr">
+        <is>
+          <t>SITA STB (Schedule Transfer Bridge)</t>
+        </is>
+      </c>
+      <c r="I193" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM file; interline and codeshare partner agreement register</t>
+        </is>
+      </c>
+      <c r="J193" s="16" t="inlineStr">
+        <is>
+          <t>SSIM sub-files transmitted to each codeshare and interline partner via SITA STB</t>
+        </is>
+      </c>
+      <c r="K193" s="16" t="inlineStr">
+        <is>
+          <t>Partner receipt confirmation received within 48 hours for ≥95% of partners</t>
+        </is>
+      </c>
+      <c r="L193" s="16" t="inlineStr">
+        <is>
+          <t>SITA STB acknowledgement messages do not distinguish between received and processed status; partners occasionally load superseded SSIM versions when multiple amendments are in flight simultaneously</t>
+        </is>
+      </c>
+      <c r="M193" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N193" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="30" customHeight="1">
+      <c r="A194" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B194" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C194" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D194" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E194" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F194" s="18" t="inlineStr">
+        <is>
+          <t>Notify airports of schedule via IATA AHM 090</t>
+        </is>
+      </c>
+      <c r="G194" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H194" s="18" t="inlineStr">
+        <is>
+          <t>SITA AMS (Airport Management System)</t>
+        </is>
+      </c>
+      <c r="I194" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmed schedule with slot allocations</t>
+        </is>
+      </c>
+      <c r="J194" s="18" t="inlineStr">
+        <is>
+          <t>AHM 090 schedule notification messages transmitted to all served airports</t>
+        </is>
+      </c>
+      <c r="K194" s="18" t="inlineStr">
+        <is>
+          <t>Airport acknowledgement received from ≥95% of notified airports within 5 business days</t>
+        </is>
+      </c>
+      <c r="L194" s="18" t="inlineStr">
+        <is>
+          <t>AHM 090 message format compliance varies by airport handler; some outstations require a direct email supplement alongside SITA MATIP messages, adding manual workload with no audit trail in AMS</t>
+        </is>
+      </c>
+      <c r="M194" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N194" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="30" customHeight="1">
+      <c r="A195" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B195" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C195" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D195" s="16" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E195" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F195" s="16" t="inlineStr">
+        <is>
+          <t>Archive versioned SSIM with change log</t>
+        </is>
+      </c>
+      <c r="G195" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H195" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I195" s="16" t="inlineStr">
+        <is>
+          <t>Final SSIM file; amendment history register</t>
+        </is>
+      </c>
+      <c r="J195" s="16" t="inlineStr">
+        <is>
+          <t>Versioned SSIM archive in AWS S3 with structured change log (season, date, amendment number, changed flights)</t>
+        </is>
+      </c>
+      <c r="K195" s="16" t="inlineStr">
+        <is>
+          <t>100% version retention; any historical SSIM retrievable within 1 business hour</t>
+        </is>
+      </c>
+      <c r="L195" s="16" t="inlineStr">
+        <is>
+          <t>No automated versioning in SkyWORKS SSIM module; manual naming conventions lead to version confusion when multiple mid-season amendments are active, creating audit and regulatory traceability risk</t>
+        </is>
+      </c>
+      <c r="M195" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N195" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="A196" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-10</t>
+        </is>
+      </c>
+      <c r="B196" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C196" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D196" s="18" t="inlineStr">
+        <is>
+          <t>SSIM File Management &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="E196" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F196" s="18" t="inlineStr">
+        <is>
+          <t>Manage mid-season SSIM amendment cycle</t>
+        </is>
+      </c>
+      <c r="G196" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H196" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I196" s="18" t="inlineStr">
+        <is>
+          <t>Network change requests; schedule irregularity reports; commercial re-routing decisions</t>
+        </is>
+      </c>
+      <c r="J196" s="18" t="inlineStr">
+        <is>
+          <t>Amendment SSIM file; updated GDS displays; re-notified partners and airports</t>
+        </is>
+      </c>
+      <c r="K196" s="18" t="inlineStr">
+        <is>
+          <t>Full amendment cycle (generate → validate → distribute → verify) completed within 5 business days</t>
+        </is>
+      </c>
+      <c r="L196" s="18" t="inlineStr">
+        <is>
+          <t>Mid-season amendments trigger full re-distribution to all GDS, aggregators, and partners; SkyWORKS SSIM module has no selective-update capability, so even single-flight changes require a complete file re-transmission</t>
+        </is>
+      </c>
+      <c r="M196" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N196" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NP-SP-11: Schedule Publication & GDS Loading — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -17,6 +17,7 @@
     <sheet name="NP-SP-08" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="NP-SP-09" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="NP-SP-10" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="NP-SP-11" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1028,13 +1029,21 @@
           <t>Schedule Publication &amp; GDS Loading</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr"/>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-11</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -6456,13 +6465,1213 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-11 — Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Initiate seasonal schedule freeze in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Board-approved seasonal schedule (IATA season S26/W26)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Frozen schedule record with freeze timestamp and version lock</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule frozen ≥330 days before season start per IATA standard</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Late commercial decisions (new routes, frequency changes) force freeze date slippage, compressing the GDS loading window and risking incomplete availability at booking opening</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Validate schedule against airport slot constraints</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Frozen schedule from SkyWORKS, IATA slot declarations for coordinated airports</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Slot validation report with conflict flag per airport</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>100% slot compliance achieved before SSIM generation; zero unresolved conflicts at freeze</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Slot-constrained airports (LHR, JFK, CDG, NRT) require manual bilateral negotiation; automated IATA CRS checks surface conflicts but offer no resolution path, requiring scheduler intervention</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Resolve slot conflicts and revalidate schedule</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Slot validation report listing conflicting departure/arrival windows</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Revised schedule with adjusted slot times, resubmitted to IATA CRS</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Slot conflict resolution within 5 business days of detection</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Slot swaps require bilateral agreement with competing carriers; absence of a multilateral slot exchange platform means resolution depends on ad-hoc email negotiation with slot coordinators</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Generate SSIM Chapter 7 file from frozen schedule</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated, slot-compliant frozen schedule</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 flat file (.ssim) containing all flight records for the season</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>SSIM generated within 2 hours of freeze confirmation; file size validated within expected range</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Complex codeshare and interline agreements require precise segment-level carrier attribution in SSIM records; errors in marketing vs. operating carrier fields cause booking failures across all GDS channels</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Validate SSIM file against IATA format standards</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Generated SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>SSIM validation report detailing field-level errors, warnings, and record counts</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Zero format errors before transmission; validation run completed in &lt;30 minutes</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>IATA SSIM Chapter 7 format is field-position-exact; minor field-length violations or non-standard aircraft type codes cause full file rejection by GDS ingest pipelines, requiring a complete regeneration cycle</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Correct SSIM errors and regenerate file</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>SSIM validation error report with specific record and field references</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Corrected SSIM file ready for re-validation</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Correction and regeneration cycle completed in ≤4 hours per iteration</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Root cause of SSIM errors often lies in upstream schedule attributes (equipment codes, operating carrier flags); manual correction risks introducing new errors without an integrated diff-check tool</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Submit validated SSIM to OAG for GDS distribution</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM Chapter 7 file with zero format errors</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>OAG submission confirmation with distribution ticket ID and estimated processing completion time</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>SSIM submitted to OAG ≥12 months before season start for initial seasonal load; re-submissions within 4 hours of correction sign-off</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>OAG processing queue can introduce 24–48 hour delays during peak IATA schedule submission periods (March and October); cascading delay compresses the booking-open window for new routes</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Monitor Sabre GDS schedule ingestion and loading</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Sabre loading status feed</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Sabre loading confirmation report; discrepancy log if mismatches detected</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Sabre schedule parity ≥99.5% within 72 hours of SSIM submission</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Sabre's batch processing window is nightly; intraday schedule corrections are not reflected until the following day's run, requiring a manual Sabre support ticket for urgent changes such as flight cancellations or time shifts</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Monitor Travelport GDS schedule ingestion and loading</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Travelport Apollo/Galileo loading status</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Travelport loading confirmation report across Apollo and Galileo sub-platforms</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Travelport schedule parity ≥99.5% within 72 hours; Apollo/Galileo consistency 100%</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Travelport's Apollo and Galileo sub-platforms have different update cadences; inconsistency between the two creates agent booking confusion and potential duplicate or missing availability for the same flight</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Monitor Amadeus GDS schedule loading across all PCCs</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Amadeus PCC propagation status</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus parity report; consolidated GDS parity sign-off across Sabre, Travelport, and Amadeus</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus schedule parity ≥99.5% within 72 hours; full PCC propagation confirmed within 96 hours</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus GDS propagation to all Pseudo City Codes can lag by 24 hours; corporate TMC agents using affected PCCs see stale or missing schedules during the propagation window, generating avoidable calls to airline sales teams</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Publish schedule to NDC API Gateway for OTA partners</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Digital Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Validated SSIM, approved fare inventory from Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>NDC offer catalog updated; API endpoint live for OTA and metasearch partners</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>NDC schedule availability within 4 hours of SSIM freeze confirmation; API offer response latency &lt;200ms at P99</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>NDC schema versioning (IATA NDC 21.3) mismatches with OTA partner implementations cause silent failures where offer requests return empty results with no error surfaced to the traveller; debugging requires partner-by-partner API log analysis</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Update airline.com booking engine via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Digital Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Published SSIM, live fare inventory, NDC offer catalog</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Live schedule displayed in airline.com booking flow with correct availability and pricing</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Direct channel schedule accuracy 100%; booking engine page response time &lt;3 seconds; availability parity with GDS within 1 hour of schedule publication</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS schedule cache refresh requires a manual trigger for urgent changes; stale cache causes customers to see phantom flights or missing flights, generating misdirected bookings and call-centre volume spikes</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Execute cross-channel schedule parity audit</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Integrity Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Published schedules from Sabre GDS, Travelport GDS, Amadeus GDS, NDC API, and airline.com; master SSIM as reference</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Cross-channel parity audit report with discrepancy log (flight number, date, affected channel, nature of mismatch)</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Cross-channel schedule parity ≥99.8% within 5 business days of initial load; audit covering 100% of new and changed flights</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>No real-time automated parity monitoring tool spans all five distribution channels simultaneously; manual spot-checks via OAG miss low-frequency discrepancies such as wrong equipment type or missing return leg that only manifest at specific date ranges</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Issue SSIM delta file and re-submit for channel correction</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Parity audit discrepancy log with channel-specific mismatch details</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM delta file (update and cancel records) re-submitted to OAG; correction tracking ticket raised per affected channel</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Critical corrections (cancellations, departure time changes &gt;15 min) re-distributed within 4 hours; all corrections confirmed propagated within 48 hours</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>SSIM delta files require the same full validation cycle as the initial file; urgent corrections still take 24–48 hours to propagate across GDS batch pipelines, during which customers may purchase now-invalid itineraries requiring involuntary rerouting</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Notify Revenue Management and activate NRM inventory</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Final published schedule, parity audit sign-off document</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>NRM inventory controls activated for all new and changed flights; RM team notified with flight list and opening load factors</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>NRM inventory activation within 24 hours of schedule publication sign-off; 100% of new routes activated before booking opening date</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>NRM inventory loading following SSIM publication is not automated; the manual handoff between Schedule Planning and Revenue Management teams introduces activation delays of 1–3 days, causing new flights to go on sale without yield controls in place and exposing the airline to underpriced early bookings</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N196"/>
+  <dimension ref="A1:N211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -20525,6 +21734,1086 @@
       <c r="N196" s="17" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="30" customHeight="1">
+      <c r="A197" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B197" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C197" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D197" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E197" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F197" s="16" t="inlineStr">
+        <is>
+          <t>Initiate seasonal schedule freeze in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G197" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H197" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I197" s="16" t="inlineStr">
+        <is>
+          <t>Board-approved seasonal schedule (IATA season S26/W26)</t>
+        </is>
+      </c>
+      <c r="J197" s="16" t="inlineStr">
+        <is>
+          <t>Frozen schedule record with freeze timestamp and version lock</t>
+        </is>
+      </c>
+      <c r="K197" s="16" t="inlineStr">
+        <is>
+          <t>Schedule frozen ≥330 days before season start per IATA standard</t>
+        </is>
+      </c>
+      <c r="L197" s="16" t="inlineStr">
+        <is>
+          <t>Late commercial decisions (new routes, frequency changes) force freeze date slippage, compressing the GDS loading window and risking incomplete availability at booking opening</t>
+        </is>
+      </c>
+      <c r="M197" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N197" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="30" customHeight="1">
+      <c r="A198" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B198" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C198" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D198" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E198" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F198" s="18" t="inlineStr">
+        <is>
+          <t>Validate schedule against airport slot constraints</t>
+        </is>
+      </c>
+      <c r="G198" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H198" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I198" s="18" t="inlineStr">
+        <is>
+          <t>Frozen schedule from SkyWORKS, IATA slot declarations for coordinated airports</t>
+        </is>
+      </c>
+      <c r="J198" s="18" t="inlineStr">
+        <is>
+          <t>Slot validation report with conflict flag per airport</t>
+        </is>
+      </c>
+      <c r="K198" s="18" t="inlineStr">
+        <is>
+          <t>100% slot compliance achieved before SSIM generation; zero unresolved conflicts at freeze</t>
+        </is>
+      </c>
+      <c r="L198" s="18" t="inlineStr">
+        <is>
+          <t>Slot-constrained airports (LHR, JFK, CDG, NRT) require manual bilateral negotiation; automated IATA CRS checks surface conflicts but offer no resolution path, requiring scheduler intervention</t>
+        </is>
+      </c>
+      <c r="M198" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N198" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="30" customHeight="1">
+      <c r="A199" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B199" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C199" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D199" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E199" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F199" s="16" t="inlineStr">
+        <is>
+          <t>Resolve slot conflicts and revalidate schedule</t>
+        </is>
+      </c>
+      <c r="G199" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordination Analyst</t>
+        </is>
+      </c>
+      <c r="H199" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I199" s="16" t="inlineStr">
+        <is>
+          <t>Slot validation report listing conflicting departure/arrival windows</t>
+        </is>
+      </c>
+      <c r="J199" s="16" t="inlineStr">
+        <is>
+          <t>Revised schedule with adjusted slot times, resubmitted to IATA CRS</t>
+        </is>
+      </c>
+      <c r="K199" s="16" t="inlineStr">
+        <is>
+          <t>Slot conflict resolution within 5 business days of detection</t>
+        </is>
+      </c>
+      <c r="L199" s="16" t="inlineStr">
+        <is>
+          <t>Slot swaps require bilateral agreement with competing carriers; absence of a multilateral slot exchange platform means resolution depends on ad-hoc email negotiation with slot coordinators</t>
+        </is>
+      </c>
+      <c r="M199" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N199" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="30" customHeight="1">
+      <c r="A200" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B200" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C200" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D200" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E200" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F200" s="18" t="inlineStr">
+        <is>
+          <t>Generate SSIM Chapter 7 file from frozen schedule</t>
+        </is>
+      </c>
+      <c r="G200" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H200" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I200" s="18" t="inlineStr">
+        <is>
+          <t>Validated, slot-compliant frozen schedule</t>
+        </is>
+      </c>
+      <c r="J200" s="18" t="inlineStr">
+        <is>
+          <t>SSIM Chapter 7 flat file (.ssim) containing all flight records for the season</t>
+        </is>
+      </c>
+      <c r="K200" s="18" t="inlineStr">
+        <is>
+          <t>SSIM generated within 2 hours of freeze confirmation; file size validated within expected range</t>
+        </is>
+      </c>
+      <c r="L200" s="18" t="inlineStr">
+        <is>
+          <t>Complex codeshare and interline agreements require precise segment-level carrier attribution in SSIM records; errors in marketing vs. operating carrier fields cause booking failures across all GDS channels</t>
+        </is>
+      </c>
+      <c r="M200" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N200" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="30" customHeight="1">
+      <c r="A201" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B201" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C201" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D201" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E201" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F201" s="16" t="inlineStr">
+        <is>
+          <t>Validate SSIM file against IATA format standards</t>
+        </is>
+      </c>
+      <c r="G201" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H201" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I201" s="16" t="inlineStr">
+        <is>
+          <t>Generated SSIM Chapter 7 file</t>
+        </is>
+      </c>
+      <c r="J201" s="16" t="inlineStr">
+        <is>
+          <t>SSIM validation report detailing field-level errors, warnings, and record counts</t>
+        </is>
+      </c>
+      <c r="K201" s="16" t="inlineStr">
+        <is>
+          <t>Zero format errors before transmission; validation run completed in &lt;30 minutes</t>
+        </is>
+      </c>
+      <c r="L201" s="16" t="inlineStr">
+        <is>
+          <t>IATA SSIM Chapter 7 format is field-position-exact; minor field-length violations or non-standard aircraft type codes cause full file rejection by GDS ingest pipelines, requiring a complete regeneration cycle</t>
+        </is>
+      </c>
+      <c r="M201" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N201" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="30" customHeight="1">
+      <c r="A202" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B202" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C202" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D202" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E202" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F202" s="18" t="inlineStr">
+        <is>
+          <t>Correct SSIM errors and regenerate file</t>
+        </is>
+      </c>
+      <c r="G202" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H202" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I202" s="18" t="inlineStr">
+        <is>
+          <t>SSIM validation error report with specific record and field references</t>
+        </is>
+      </c>
+      <c r="J202" s="18" t="inlineStr">
+        <is>
+          <t>Corrected SSIM file ready for re-validation</t>
+        </is>
+      </c>
+      <c r="K202" s="18" t="inlineStr">
+        <is>
+          <t>Correction and regeneration cycle completed in ≤4 hours per iteration</t>
+        </is>
+      </c>
+      <c r="L202" s="18" t="inlineStr">
+        <is>
+          <t>Root cause of SSIM errors often lies in upstream schedule attributes (equipment codes, operating carrier flags); manual correction risks introducing new errors without an integrated diff-check tool</t>
+        </is>
+      </c>
+      <c r="M202" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N202" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="30" customHeight="1">
+      <c r="A203" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B203" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C203" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D203" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E203" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F203" s="16" t="inlineStr">
+        <is>
+          <t>Submit validated SSIM to OAG for GDS distribution</t>
+        </is>
+      </c>
+      <c r="G203" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H203" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I203" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM Chapter 7 file with zero format errors</t>
+        </is>
+      </c>
+      <c r="J203" s="16" t="inlineStr">
+        <is>
+          <t>OAG submission confirmation with distribution ticket ID and estimated processing completion time</t>
+        </is>
+      </c>
+      <c r="K203" s="16" t="inlineStr">
+        <is>
+          <t>SSIM submitted to OAG ≥12 months before season start for initial seasonal load; re-submissions within 4 hours of correction sign-off</t>
+        </is>
+      </c>
+      <c r="L203" s="16" t="inlineStr">
+        <is>
+          <t>OAG processing queue can introduce 24–48 hour delays during peak IATA schedule submission periods (March and October); cascading delay compresses the booking-open window for new routes</t>
+        </is>
+      </c>
+      <c r="M203" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N203" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="30" customHeight="1">
+      <c r="A204" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B204" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C204" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D204" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E204" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F204" s="18" t="inlineStr">
+        <is>
+          <t>Monitor Sabre GDS schedule ingestion and loading</t>
+        </is>
+      </c>
+      <c r="G204" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H204" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I204" s="18" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Sabre loading status feed</t>
+        </is>
+      </c>
+      <c r="J204" s="18" t="inlineStr">
+        <is>
+          <t>Sabre loading confirmation report; discrepancy log if mismatches detected</t>
+        </is>
+      </c>
+      <c r="K204" s="18" t="inlineStr">
+        <is>
+          <t>Sabre schedule parity ≥99.5% within 72 hours of SSIM submission</t>
+        </is>
+      </c>
+      <c r="L204" s="18" t="inlineStr">
+        <is>
+          <t>Sabre's batch processing window is nightly; intraday schedule corrections are not reflected until the following day's run, requiring a manual Sabre support ticket for urgent changes such as flight cancellations or time shifts</t>
+        </is>
+      </c>
+      <c r="M204" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N204" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="30" customHeight="1">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B205" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C205" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D205" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E205" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F205" s="16" t="inlineStr">
+        <is>
+          <t>Monitor Travelport GDS schedule ingestion and loading</t>
+        </is>
+      </c>
+      <c r="G205" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H205" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I205" s="16" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Travelport Apollo/Galileo loading status</t>
+        </is>
+      </c>
+      <c r="J205" s="16" t="inlineStr">
+        <is>
+          <t>Travelport loading confirmation report across Apollo and Galileo sub-platforms</t>
+        </is>
+      </c>
+      <c r="K205" s="16" t="inlineStr">
+        <is>
+          <t>Travelport schedule parity ≥99.5% within 72 hours; Apollo/Galileo consistency 100%</t>
+        </is>
+      </c>
+      <c r="L205" s="16" t="inlineStr">
+        <is>
+          <t>Travelport's Apollo and Galileo sub-platforms have different update cadences; inconsistency between the two creates agent booking confusion and potential duplicate or missing availability for the same flight</t>
+        </is>
+      </c>
+      <c r="M205" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N205" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="30" customHeight="1">
+      <c r="A206" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B206" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C206" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D206" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E206" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F206" s="18" t="inlineStr">
+        <is>
+          <t>Monitor Amadeus GDS schedule loading across all PCCs</t>
+        </is>
+      </c>
+      <c r="G206" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Coordinator</t>
+        </is>
+      </c>
+      <c r="H206" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I206" s="18" t="inlineStr">
+        <is>
+          <t>OAG distribution confirmation, Amadeus PCC propagation status</t>
+        </is>
+      </c>
+      <c r="J206" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus parity report; consolidated GDS parity sign-off across Sabre, Travelport, and Amadeus</t>
+        </is>
+      </c>
+      <c r="K206" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus schedule parity ≥99.5% within 72 hours; full PCC propagation confirmed within 96 hours</t>
+        </is>
+      </c>
+      <c r="L206" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS propagation to all Pseudo City Codes can lag by 24 hours; corporate TMC agents using affected PCCs see stale or missing schedules during the propagation window, generating avoidable calls to airline sales teams</t>
+        </is>
+      </c>
+      <c r="M206" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N206" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="30" customHeight="1">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B207" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C207" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D207" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E207" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F207" s="16" t="inlineStr">
+        <is>
+          <t>Publish schedule to NDC API Gateway for OTA partners</t>
+        </is>
+      </c>
+      <c r="G207" s="16" t="inlineStr">
+        <is>
+          <t>Digital Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H207" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I207" s="16" t="inlineStr">
+        <is>
+          <t>Validated SSIM, approved fare inventory from Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="J207" s="16" t="inlineStr">
+        <is>
+          <t>NDC offer catalog updated; API endpoint live for OTA and metasearch partners</t>
+        </is>
+      </c>
+      <c r="K207" s="16" t="inlineStr">
+        <is>
+          <t>NDC schedule availability within 4 hours of SSIM freeze confirmation; API offer response latency &lt;200ms at P99</t>
+        </is>
+      </c>
+      <c r="L207" s="16" t="inlineStr">
+        <is>
+          <t>NDC schema versioning (IATA NDC 21.3) mismatches with OTA partner implementations cause silent failures where offer requests return empty results with no error surfaced to the traveller; debugging requires partner-by-partner API log analysis</t>
+        </is>
+      </c>
+      <c r="M207" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N207" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="30" customHeight="1">
+      <c r="A208" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B208" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C208" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D208" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E208" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F208" s="18" t="inlineStr">
+        <is>
+          <t>Update airline.com booking engine via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="G208" s="18" t="inlineStr">
+        <is>
+          <t>Digital Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H208" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I208" s="18" t="inlineStr">
+        <is>
+          <t>Published SSIM, live fare inventory, NDC offer catalog</t>
+        </is>
+      </c>
+      <c r="J208" s="18" t="inlineStr">
+        <is>
+          <t>Live schedule displayed in airline.com booking flow with correct availability and pricing</t>
+        </is>
+      </c>
+      <c r="K208" s="18" t="inlineStr">
+        <is>
+          <t>Direct channel schedule accuracy 100%; booking engine page response time &lt;3 seconds; availability parity with GDS within 1 hour of schedule publication</t>
+        </is>
+      </c>
+      <c r="L208" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS schedule cache refresh requires a manual trigger for urgent changes; stale cache causes customers to see phantom flights or missing flights, generating misdirected bookings and call-centre volume spikes</t>
+        </is>
+      </c>
+      <c r="M208" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N208" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="30" customHeight="1">
+      <c r="A209" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B209" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C209" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D209" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E209" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F209" s="16" t="inlineStr">
+        <is>
+          <t>Execute cross-channel schedule parity audit</t>
+        </is>
+      </c>
+      <c r="G209" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Integrity Analyst</t>
+        </is>
+      </c>
+      <c r="H209" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I209" s="16" t="inlineStr">
+        <is>
+          <t>Published schedules from Sabre GDS, Travelport GDS, Amadeus GDS, NDC API, and airline.com; master SSIM as reference</t>
+        </is>
+      </c>
+      <c r="J209" s="16" t="inlineStr">
+        <is>
+          <t>Cross-channel parity audit report with discrepancy log (flight number, date, affected channel, nature of mismatch)</t>
+        </is>
+      </c>
+      <c r="K209" s="16" t="inlineStr">
+        <is>
+          <t>Cross-channel schedule parity ≥99.8% within 5 business days of initial load; audit covering 100% of new and changed flights</t>
+        </is>
+      </c>
+      <c r="L209" s="16" t="inlineStr">
+        <is>
+          <t>No real-time automated parity monitoring tool spans all five distribution channels simultaneously; manual spot-checks via OAG miss low-frequency discrepancies such as wrong equipment type or missing return leg that only manifest at specific date ranges</t>
+        </is>
+      </c>
+      <c r="M209" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N209" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="30" customHeight="1">
+      <c r="A210" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B210" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C210" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D210" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E210" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F210" s="18" t="inlineStr">
+        <is>
+          <t>Issue SSIM delta file and re-submit for channel correction</t>
+        </is>
+      </c>
+      <c r="G210" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Data Analyst</t>
+        </is>
+      </c>
+      <c r="H210" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I210" s="18" t="inlineStr">
+        <is>
+          <t>Parity audit discrepancy log with channel-specific mismatch details</t>
+        </is>
+      </c>
+      <c r="J210" s="18" t="inlineStr">
+        <is>
+          <t>SSIM delta file (update and cancel records) re-submitted to OAG; correction tracking ticket raised per affected channel</t>
+        </is>
+      </c>
+      <c r="K210" s="18" t="inlineStr">
+        <is>
+          <t>Critical corrections (cancellations, departure time changes &gt;15 min) re-distributed within 4 hours; all corrections confirmed propagated within 48 hours</t>
+        </is>
+      </c>
+      <c r="L210" s="18" t="inlineStr">
+        <is>
+          <t>SSIM delta files require the same full validation cycle as the initial file; urgent corrections still take 24–48 hours to propagate across GDS batch pipelines, during which customers may purchase now-invalid itineraries requiring involuntary rerouting</t>
+        </is>
+      </c>
+      <c r="M210" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N210" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="30" customHeight="1">
+      <c r="A211" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-11</t>
+        </is>
+      </c>
+      <c r="B211" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C211" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D211" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Publication &amp; GDS Loading</t>
+        </is>
+      </c>
+      <c r="E211" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F211" s="16" t="inlineStr">
+        <is>
+          <t>Notify Revenue Management and activate NRM inventory</t>
+        </is>
+      </c>
+      <c r="G211" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H211" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I211" s="16" t="inlineStr">
+        <is>
+          <t>Final published schedule, parity audit sign-off document</t>
+        </is>
+      </c>
+      <c r="J211" s="16" t="inlineStr">
+        <is>
+          <t>NRM inventory controls activated for all new and changed flights; RM team notified with flight list and opening load factors</t>
+        </is>
+      </c>
+      <c r="K211" s="16" t="inlineStr">
+        <is>
+          <t>NRM inventory activation within 24 hours of schedule publication sign-off; 100% of new routes activated before booking opening date</t>
+        </is>
+      </c>
+      <c r="L211" s="16" t="inlineStr">
+        <is>
+          <t>NRM inventory loading following SSIM publication is not automated; the manual handoff between Schedule Planning and Revenue Management teams introduces activation delays of 1–3 days, causing new flights to go on sale without yield controls in place and exposing the airline to underpriced early bookings</t>
+        </is>
+      </c>
+      <c r="M211" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N211" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NP-SP-12: Irregular Operations Recovery Planning — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -18,6 +18,7 @@
     <sheet name="NP-SP-09" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="NP-SP-10" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="NP-SP-11" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="NP-SP-12" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1066,13 +1067,21 @@
           <t>Irregular Operations Recovery Planning</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr"/>
-      <c r="G14" s="8" t="inlineStr"/>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-12</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -7665,13 +7674,1429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-12 — Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Ingest real-time disruption alerts from ops systems</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Operations Controller</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Weather service alerts, ATC NOTAMs, aircraft technical fault reports</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Unified disruption notification log with timestamp and source</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Alert-to-acknowledgement time ≤5 min</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Multiple alert streams (weather, ATC, maintenance) arrive in disparate systems with no unified ingestion layer, causing detection delays of 10–20 min during complex events</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Classify IROPS trigger type and severity tier</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Operations Controller</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Airport Management</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Disruption notification log, affected airport and flight list</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>IROPS classification (weather / ATC / technical / security / crew) and severity tier (1=local, 2=regional, 3=network-wide)</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Classification accuracy ≥95%; mis-classification rate &lt;5%</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>No AI-assisted triage in legacy NOC toolsets; mis-classification delays activation of the correct recovery playbook, costing 15–30 min of recovery time</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Activate IROPS command structure and war room</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Operations</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Telex / SITA ACARS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Severity tier, affected station list, initial disruption scope</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>IROPS war room activated; stakeholder notifications sent to crew, commercial, ground ops, and customer relations leads</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>War room activation time ≤15 min from trigger classification</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Escalation contact lists frequently stale; cross-functional mobilisation relies on manual phone trees rather than automated push notifications, adding 10–20 min delay</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Model affected flight propagation in network simulator</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>IROPS classification, affected airports, time window of disruption</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Affected flight list with downstream propagation map showing knock-on cancellation risk</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Network impact model run time ≤30 min; propagation accuracy ≥90%</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario setup is manual and not pre-loaded with IROPS templates; large weather events affecting 100+ flights can take 30–45 min to model, exceeding recovery window</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Identify aircraft and crew positioning conflicts</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Affected flight list, current crew duty records, aircraft position data</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Crew duty conflict report; aircraft position conflict map with stranded-asset flags</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Conflict identification complete ≤20 min; coverage of 100% of affected pairings</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>FAR Part 117 duty/rest legality checks are sequential in Jeppesen; large-scale events overwhelm manual review, and reserve pool visibility is not real-time</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Estimate disrupted passenger volume and missed connections</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Affected flight booking data from Altéa PSS, connection itinerary records</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Disrupted passenger count by segment, missed connection tally, estimated rebooking inventory gap</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Passenger impact estimate accuracy ≥85%; model run time ≤10 min</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>NRM is not designed for real-time IROPS queries; passenger impact models must be manually triggered outside normal RM workflow, creating data-currency risk</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Assess slot and regulatory constraints at affected airports</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Affected slot portfolio, airport coordination contacts, no-fly window data</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Waiveable slot list, regulatory no-fly windows, ATC Ground Delay Program parameters</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Slot waiver request accuracy ≥98%; assessment complete ≤15 min</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Slot waiver processes vary by country and airport authority; some regions require 24-hour advance notice incompatible with real-time IROPS response timelines</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Generate recovery schedule scenarios in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Impact assessment outputs, available aircraft count, crew availability, slot constraints</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>2–3 recovery schedule options with trade-off analysis (cost vs. OTP vs. coverage)</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Scenario generation time ≤45 min; minimum 2 viable options produced</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS is not optimised for real-time IROPS iteration; manual schedule editing under time pressure increases the risk of SSIM errors propagating to GDS</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate aircraft swap and ferry flight feasibility</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Aircraft availability roster, maintenance status from AMOS, ferry routing options, positioning cost estimates</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Approved ferry/swap plan or rejection rationale with cost-benefit summary</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Ferry cost vs. delay cost ratio assessed within 30 min; SkyMAX fleet assignment feasibility score ≥0.85</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>AMOS maintenance status sync delay (up to 15 min) risks assigning aircraft with open airworthiness items; no automated maintenance-status gate in SkyMAX IROPS workflows</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Validate crew legality for full recovery plan</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Proposed recovery schedule, current crew duty and rest records, reserve availability</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Crew-legal recovery schedule or exception list requiring reserve activation</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>100% FAR Part 117 compliance validated before plan publication; legality check ≤20 min</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Iterative crew legality re-checks slow plan finalisation; each SkyWORKS schedule change triggers a full Jeppesen re-validation cycle, compounding delay when multiple iterations are needed</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Publish revised recovery schedule to PSS and GDS</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS → Amadeus Altéa PSS → Sabre GDS / Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Approved, crew-legal recovery schedule</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Updated schedules live in Altéa PSS, Sabre GDS, Travelport GDS, and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>GDS schedule update latency ≤30 min from approval; distribution completeness 100% of active channels</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Multi-channel distribution (Altéa + Sabre + Travelport + NDC) requires sequential pushes with no atomic commit; partial-update windows create booking inconsistencies and duplicate inventory</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>File slot waivers and coordinate ATC ground delay program</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS + Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Waiveable slot list, ATC GDP parameters, airport authority contacts</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed slot waivers, revised approved departure windows per airport</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Slot waiver approval rate ≥90%; ATC GDP compliance 100%</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>ATC GDP parameters change frequently during active weather events; real-time coordination requires a dedicated FAA/EUROCONTROL liaison channel that is not always staffed at smaller carriers</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Confirm and dispatch aircraft ferry repositioning flights</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Flight Dispatcher</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>NAVBLUE + Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Approved swap/ferry plan, ATC clearances, confirmed slot windows</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Filed flight plans for ferry flights, repositioning confirmation messages to stations</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Ferry flight OTP ≥75%; repositioning within ±2 hrs of recovery plan target</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Ferry flight fuel burn is not pre-budgeted in standard IROPS cost models; post-event cost attribution to IROPS events is a manual, multi-week reconciliation process</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Initiate automated passenger rebooking</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Customer Operations Manager</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS + NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Disrupted passenger list, recovery flight inventory, passenger tier (FFP status)</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Rebooking confirmations sent to passengers; exception queue for manual handling</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Automated rebooking rate ≥70%; passenger notification delivered ≤30 min of flight cancellation</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Altéa automated rebooking rules are not always tuned for IROPS scenarios; high-volume events exhaust available recovery inventory before all passengers are rebooked, forcing costly offline handling</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Activate reserve crew and complete crew reassignments</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Crew Scheduling Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Recovery schedule, crew conflict report, reserve crew availability and location</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Final crew assignments for all recovery flights; reserve activation orders issued</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Reserve activation time ≤45 min; crew coverage rate ≥98% of recovery flights</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Reserve crew contact and activation is phone-based at many carriers; no push-notification system for mass activation means manual calling campaigns during high-stress IROPS events</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Issue passenger care and compensation entitlements</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Customer Relations Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Delay/cancellation duration, disruption cause classification, passenger loyalty tier</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Meal vouchers, hotel authorisations, transport allowances, and DOT/EU261 compensation notices</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>DOT / EU261 compensation filing accuracy ≥99%; voucher issuance within 60 min of entitlement trigger</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Compensation eligibility rules differ by jurisdiction (DOT, EU261, ANAC, DGAC); no unified entitlement engine forces manual legal review for international itineraries, creating under- or over-payment risk</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Conduct post-IROPS cost and performance analysis</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Finance Controller (Commercial)</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO) + AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Ferry fuel invoices, compensation payouts, rebooking costs, OTP and cancellation data</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>IROPS total cost report, OTP and cancellation deviation analysis vs. plan</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Report delivered ≤72 hrs post-event; cost capture accuracy ±2%</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Cost data is scattered across Altéa (compensation), SAP (vendor invoices), and Jeppesen (crew overtime); manual reconciliation typically takes 5–7 business days, delaying learning cycle</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Update IROPS recovery playbooks and SkySYM scenario library</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM + Confluence</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Post-event debrief findings, scenario performance data, cost report</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Updated recovery playbook version; new scenario added to SkySYM IROPS library for future use</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Playbook updated within 30 days of event; ≥1 new SkySYM scenario created per Tier 2+ IROPS</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Playbook updates are routinely deprioritised once normal operations resume; institutional recovery knowledge is frequently lost without a mandatory structured capture and review process</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N211"/>
+  <dimension ref="A1:N229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -22812,6 +24237,1302 @@
         </is>
       </c>
       <c r="N211" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="30" customHeight="1">
+      <c r="A212" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B212" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C212" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D212" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E212" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F212" s="18" t="inlineStr">
+        <is>
+          <t>Ingest real-time disruption alerts from ops systems</t>
+        </is>
+      </c>
+      <c r="G212" s="18" t="inlineStr">
+        <is>
+          <t>Network Operations Controller</t>
+        </is>
+      </c>
+      <c r="H212" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I212" s="18" t="inlineStr">
+        <is>
+          <t>Weather service alerts, ATC NOTAMs, aircraft technical fault reports</t>
+        </is>
+      </c>
+      <c r="J212" s="18" t="inlineStr">
+        <is>
+          <t>Unified disruption notification log with timestamp and source</t>
+        </is>
+      </c>
+      <c r="K212" s="18" t="inlineStr">
+        <is>
+          <t>Alert-to-acknowledgement time ≤5 min</t>
+        </is>
+      </c>
+      <c r="L212" s="18" t="inlineStr">
+        <is>
+          <t>Multiple alert streams (weather, ATC, maintenance) arrive in disparate systems with no unified ingestion layer, causing detection delays of 10–20 min during complex events</t>
+        </is>
+      </c>
+      <c r="M212" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N212" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="30" customHeight="1">
+      <c r="A213" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B213" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C213" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D213" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E213" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F213" s="16" t="inlineStr">
+        <is>
+          <t>Classify IROPS trigger type and severity tier</t>
+        </is>
+      </c>
+      <c r="G213" s="16" t="inlineStr">
+        <is>
+          <t>Network Operations Controller</t>
+        </is>
+      </c>
+      <c r="H213" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Airport Management</t>
+        </is>
+      </c>
+      <c r="I213" s="16" t="inlineStr">
+        <is>
+          <t>Disruption notification log, affected airport and flight list</t>
+        </is>
+      </c>
+      <c r="J213" s="16" t="inlineStr">
+        <is>
+          <t>IROPS classification (weather / ATC / technical / security / crew) and severity tier (1=local, 2=regional, 3=network-wide)</t>
+        </is>
+      </c>
+      <c r="K213" s="16" t="inlineStr">
+        <is>
+          <t>Classification accuracy ≥95%; mis-classification rate &lt;5%</t>
+        </is>
+      </c>
+      <c r="L213" s="16" t="inlineStr">
+        <is>
+          <t>No AI-assisted triage in legacy NOC toolsets; mis-classification delays activation of the correct recovery playbook, costing 15–30 min of recovery time</t>
+        </is>
+      </c>
+      <c r="M213" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N213" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="30" customHeight="1">
+      <c r="A214" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B214" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C214" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D214" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E214" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F214" s="18" t="inlineStr">
+        <is>
+          <t>Activate IROPS command structure and war room</t>
+        </is>
+      </c>
+      <c r="G214" s="18" t="inlineStr">
+        <is>
+          <t>VP Network Operations</t>
+        </is>
+      </c>
+      <c r="H214" s="18" t="inlineStr">
+        <is>
+          <t>Telex / SITA ACARS</t>
+        </is>
+      </c>
+      <c r="I214" s="18" t="inlineStr">
+        <is>
+          <t>Severity tier, affected station list, initial disruption scope</t>
+        </is>
+      </c>
+      <c r="J214" s="18" t="inlineStr">
+        <is>
+          <t>IROPS war room activated; stakeholder notifications sent to crew, commercial, ground ops, and customer relations leads</t>
+        </is>
+      </c>
+      <c r="K214" s="18" t="inlineStr">
+        <is>
+          <t>War room activation time ≤15 min from trigger classification</t>
+        </is>
+      </c>
+      <c r="L214" s="18" t="inlineStr">
+        <is>
+          <t>Escalation contact lists frequently stale; cross-functional mobilisation relies on manual phone trees rather than automated push notifications, adding 10–20 min delay</t>
+        </is>
+      </c>
+      <c r="M214" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N214" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="30" customHeight="1">
+      <c r="A215" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B215" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C215" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D215" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E215" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F215" s="16" t="inlineStr">
+        <is>
+          <t>Model affected flight propagation in network simulator</t>
+        </is>
+      </c>
+      <c r="G215" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H215" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I215" s="16" t="inlineStr">
+        <is>
+          <t>IROPS classification, affected airports, time window of disruption</t>
+        </is>
+      </c>
+      <c r="J215" s="16" t="inlineStr">
+        <is>
+          <t>Affected flight list with downstream propagation map showing knock-on cancellation risk</t>
+        </is>
+      </c>
+      <c r="K215" s="16" t="inlineStr">
+        <is>
+          <t>Network impact model run time ≤30 min; propagation accuracy ≥90%</t>
+        </is>
+      </c>
+      <c r="L215" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario setup is manual and not pre-loaded with IROPS templates; large weather events affecting 100+ flights can take 30–45 min to model, exceeding recovery window</t>
+        </is>
+      </c>
+      <c r="M215" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N215" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="30" customHeight="1">
+      <c r="A216" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B216" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C216" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D216" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E216" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F216" s="18" t="inlineStr">
+        <is>
+          <t>Identify aircraft and crew positioning conflicts</t>
+        </is>
+      </c>
+      <c r="G216" s="18" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H216" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I216" s="18" t="inlineStr">
+        <is>
+          <t>Affected flight list, current crew duty records, aircraft position data</t>
+        </is>
+      </c>
+      <c r="J216" s="18" t="inlineStr">
+        <is>
+          <t>Crew duty conflict report; aircraft position conflict map with stranded-asset flags</t>
+        </is>
+      </c>
+      <c r="K216" s="18" t="inlineStr">
+        <is>
+          <t>Conflict identification complete ≤20 min; coverage of 100% of affected pairings</t>
+        </is>
+      </c>
+      <c r="L216" s="18" t="inlineStr">
+        <is>
+          <t>FAR Part 117 duty/rest legality checks are sequential in Jeppesen; large-scale events overwhelm manual review, and reserve pool visibility is not real-time</t>
+        </is>
+      </c>
+      <c r="M216" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N216" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="30" customHeight="1">
+      <c r="A217" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B217" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C217" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D217" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E217" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F217" s="16" t="inlineStr">
+        <is>
+          <t>Estimate disrupted passenger volume and missed connections</t>
+        </is>
+      </c>
+      <c r="G217" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H217" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I217" s="16" t="inlineStr">
+        <is>
+          <t>Affected flight booking data from Altéa PSS, connection itinerary records</t>
+        </is>
+      </c>
+      <c r="J217" s="16" t="inlineStr">
+        <is>
+          <t>Disrupted passenger count by segment, missed connection tally, estimated rebooking inventory gap</t>
+        </is>
+      </c>
+      <c r="K217" s="16" t="inlineStr">
+        <is>
+          <t>Passenger impact estimate accuracy ≥85%; model run time ≤10 min</t>
+        </is>
+      </c>
+      <c r="L217" s="16" t="inlineStr">
+        <is>
+          <t>NRM is not designed for real-time IROPS queries; passenger impact models must be manually triggered outside normal RM workflow, creating data-currency risk</t>
+        </is>
+      </c>
+      <c r="M217" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N217" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="30" customHeight="1">
+      <c r="A218" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B218" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C218" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D218" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E218" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F218" s="18" t="inlineStr">
+        <is>
+          <t>Assess slot and regulatory constraints at affected airports</t>
+        </is>
+      </c>
+      <c r="G218" s="18" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H218" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I218" s="18" t="inlineStr">
+        <is>
+          <t>Affected slot portfolio, airport coordination contacts, no-fly window data</t>
+        </is>
+      </c>
+      <c r="J218" s="18" t="inlineStr">
+        <is>
+          <t>Waiveable slot list, regulatory no-fly windows, ATC Ground Delay Program parameters</t>
+        </is>
+      </c>
+      <c r="K218" s="18" t="inlineStr">
+        <is>
+          <t>Slot waiver request accuracy ≥98%; assessment complete ≤15 min</t>
+        </is>
+      </c>
+      <c r="L218" s="18" t="inlineStr">
+        <is>
+          <t>Slot waiver processes vary by country and airport authority; some regions require 24-hour advance notice incompatible with real-time IROPS response timelines</t>
+        </is>
+      </c>
+      <c r="M218" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N218" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="30" customHeight="1">
+      <c r="A219" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B219" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C219" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D219" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E219" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F219" s="16" t="inlineStr">
+        <is>
+          <t>Generate recovery schedule scenarios in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="G219" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H219" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I219" s="16" t="inlineStr">
+        <is>
+          <t>Impact assessment outputs, available aircraft count, crew availability, slot constraints</t>
+        </is>
+      </c>
+      <c r="J219" s="16" t="inlineStr">
+        <is>
+          <t>2–3 recovery schedule options with trade-off analysis (cost vs. OTP vs. coverage)</t>
+        </is>
+      </c>
+      <c r="K219" s="16" t="inlineStr">
+        <is>
+          <t>Scenario generation time ≤45 min; minimum 2 viable options produced</t>
+        </is>
+      </c>
+      <c r="L219" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS is not optimised for real-time IROPS iteration; manual schedule editing under time pressure increases the risk of SSIM errors propagating to GDS</t>
+        </is>
+      </c>
+      <c r="M219" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N219" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="30" customHeight="1">
+      <c r="A220" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B220" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C220" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D220" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E220" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F220" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate aircraft swap and ferry flight feasibility</t>
+        </is>
+      </c>
+      <c r="G220" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H220" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I220" s="18" t="inlineStr">
+        <is>
+          <t>Aircraft availability roster, maintenance status from AMOS, ferry routing options, positioning cost estimates</t>
+        </is>
+      </c>
+      <c r="J220" s="18" t="inlineStr">
+        <is>
+          <t>Approved ferry/swap plan or rejection rationale with cost-benefit summary</t>
+        </is>
+      </c>
+      <c r="K220" s="18" t="inlineStr">
+        <is>
+          <t>Ferry cost vs. delay cost ratio assessed within 30 min; SkyMAX fleet assignment feasibility score ≥0.85</t>
+        </is>
+      </c>
+      <c r="L220" s="18" t="inlineStr">
+        <is>
+          <t>AMOS maintenance status sync delay (up to 15 min) risks assigning aircraft with open airworthiness items; no automated maintenance-status gate in SkyMAX IROPS workflows</t>
+        </is>
+      </c>
+      <c r="M220" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N220" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="30" customHeight="1">
+      <c r="A221" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B221" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C221" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D221" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E221" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F221" s="16" t="inlineStr">
+        <is>
+          <t>Validate crew legality for full recovery plan</t>
+        </is>
+      </c>
+      <c r="G221" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H221" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I221" s="16" t="inlineStr">
+        <is>
+          <t>Proposed recovery schedule, current crew duty and rest records, reserve availability</t>
+        </is>
+      </c>
+      <c r="J221" s="16" t="inlineStr">
+        <is>
+          <t>Crew-legal recovery schedule or exception list requiring reserve activation</t>
+        </is>
+      </c>
+      <c r="K221" s="16" t="inlineStr">
+        <is>
+          <t>100% FAR Part 117 compliance validated before plan publication; legality check ≤20 min</t>
+        </is>
+      </c>
+      <c r="L221" s="16" t="inlineStr">
+        <is>
+          <t>Iterative crew legality re-checks slow plan finalisation; each SkyWORKS schedule change triggers a full Jeppesen re-validation cycle, compounding delay when multiple iterations are needed</t>
+        </is>
+      </c>
+      <c r="M221" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N221" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="30" customHeight="1">
+      <c r="A222" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B222" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C222" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D222" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E222" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F222" s="18" t="inlineStr">
+        <is>
+          <t>Publish revised recovery schedule to PSS and GDS</t>
+        </is>
+      </c>
+      <c r="G222" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H222" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS → Amadeus Altéa PSS → Sabre GDS / Travelport GDS</t>
+        </is>
+      </c>
+      <c r="I222" s="18" t="inlineStr">
+        <is>
+          <t>Approved, crew-legal recovery schedule</t>
+        </is>
+      </c>
+      <c r="J222" s="18" t="inlineStr">
+        <is>
+          <t>Updated schedules live in Altéa PSS, Sabre GDS, Travelport GDS, and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="K222" s="18" t="inlineStr">
+        <is>
+          <t>GDS schedule update latency ≤30 min from approval; distribution completeness 100% of active channels</t>
+        </is>
+      </c>
+      <c r="L222" s="18" t="inlineStr">
+        <is>
+          <t>Multi-channel distribution (Altéa + Sabre + Travelport + NDC) requires sequential pushes with no atomic commit; partial-update windows create booking inconsistencies and duplicate inventory</t>
+        </is>
+      </c>
+      <c r="M222" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N222" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="30" customHeight="1">
+      <c r="A223" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B223" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C223" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D223" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E223" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F223" s="16" t="inlineStr">
+        <is>
+          <t>File slot waivers and coordinate ATC ground delay program</t>
+        </is>
+      </c>
+      <c r="G223" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H223" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS + Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I223" s="16" t="inlineStr">
+        <is>
+          <t>Waiveable slot list, ATC GDP parameters, airport authority contacts</t>
+        </is>
+      </c>
+      <c r="J223" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed slot waivers, revised approved departure windows per airport</t>
+        </is>
+      </c>
+      <c r="K223" s="16" t="inlineStr">
+        <is>
+          <t>Slot waiver approval rate ≥90%; ATC GDP compliance 100%</t>
+        </is>
+      </c>
+      <c r="L223" s="16" t="inlineStr">
+        <is>
+          <t>ATC GDP parameters change frequently during active weather events; real-time coordination requires a dedicated FAA/EUROCONTROL liaison channel that is not always staffed at smaller carriers</t>
+        </is>
+      </c>
+      <c r="M223" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N223" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="30" customHeight="1">
+      <c r="A224" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B224" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C224" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D224" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E224" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F224" s="18" t="inlineStr">
+        <is>
+          <t>Confirm and dispatch aircraft ferry repositioning flights</t>
+        </is>
+      </c>
+      <c r="G224" s="18" t="inlineStr">
+        <is>
+          <t>Flight Dispatcher</t>
+        </is>
+      </c>
+      <c r="H224" s="18" t="inlineStr">
+        <is>
+          <t>NAVBLUE + Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I224" s="18" t="inlineStr">
+        <is>
+          <t>Approved swap/ferry plan, ATC clearances, confirmed slot windows</t>
+        </is>
+      </c>
+      <c r="J224" s="18" t="inlineStr">
+        <is>
+          <t>Filed flight plans for ferry flights, repositioning confirmation messages to stations</t>
+        </is>
+      </c>
+      <c r="K224" s="18" t="inlineStr">
+        <is>
+          <t>Ferry flight OTP ≥75%; repositioning within ±2 hrs of recovery plan target</t>
+        </is>
+      </c>
+      <c r="L224" s="18" t="inlineStr">
+        <is>
+          <t>Ferry flight fuel burn is not pre-budgeted in standard IROPS cost models; post-event cost attribution to IROPS events is a manual, multi-week reconciliation process</t>
+        </is>
+      </c>
+      <c r="M224" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N224" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="30" customHeight="1">
+      <c r="A225" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B225" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C225" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D225" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E225" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F225" s="16" t="inlineStr">
+        <is>
+          <t>Initiate automated passenger rebooking</t>
+        </is>
+      </c>
+      <c r="G225" s="16" t="inlineStr">
+        <is>
+          <t>Customer Operations Manager</t>
+        </is>
+      </c>
+      <c r="H225" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS + NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I225" s="16" t="inlineStr">
+        <is>
+          <t>Disrupted passenger list, recovery flight inventory, passenger tier (FFP status)</t>
+        </is>
+      </c>
+      <c r="J225" s="16" t="inlineStr">
+        <is>
+          <t>Rebooking confirmations sent to passengers; exception queue for manual handling</t>
+        </is>
+      </c>
+      <c r="K225" s="16" t="inlineStr">
+        <is>
+          <t>Automated rebooking rate ≥70%; passenger notification delivered ≤30 min of flight cancellation</t>
+        </is>
+      </c>
+      <c r="L225" s="16" t="inlineStr">
+        <is>
+          <t>Altéa automated rebooking rules are not always tuned for IROPS scenarios; high-volume events exhaust available recovery inventory before all passengers are rebooked, forcing costly offline handling</t>
+        </is>
+      </c>
+      <c r="M225" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N225" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="30" customHeight="1">
+      <c r="A226" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B226" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C226" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D226" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E226" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F226" s="18" t="inlineStr">
+        <is>
+          <t>Activate reserve crew and complete crew reassignments</t>
+        </is>
+      </c>
+      <c r="G226" s="18" t="inlineStr">
+        <is>
+          <t>Crew Scheduling Manager</t>
+        </is>
+      </c>
+      <c r="H226" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I226" s="18" t="inlineStr">
+        <is>
+          <t>Recovery schedule, crew conflict report, reserve crew availability and location</t>
+        </is>
+      </c>
+      <c r="J226" s="18" t="inlineStr">
+        <is>
+          <t>Final crew assignments for all recovery flights; reserve activation orders issued</t>
+        </is>
+      </c>
+      <c r="K226" s="18" t="inlineStr">
+        <is>
+          <t>Reserve activation time ≤45 min; crew coverage rate ≥98% of recovery flights</t>
+        </is>
+      </c>
+      <c r="L226" s="18" t="inlineStr">
+        <is>
+          <t>Reserve crew contact and activation is phone-based at many carriers; no push-notification system for mass activation means manual calling campaigns during high-stress IROPS events</t>
+        </is>
+      </c>
+      <c r="M226" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N226" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="30" customHeight="1">
+      <c r="A227" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B227" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C227" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D227" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E227" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F227" s="16" t="inlineStr">
+        <is>
+          <t>Issue passenger care and compensation entitlements</t>
+        </is>
+      </c>
+      <c r="G227" s="16" t="inlineStr">
+        <is>
+          <t>Customer Relations Manager</t>
+        </is>
+      </c>
+      <c r="H227" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I227" s="16" t="inlineStr">
+        <is>
+          <t>Delay/cancellation duration, disruption cause classification, passenger loyalty tier</t>
+        </is>
+      </c>
+      <c r="J227" s="16" t="inlineStr">
+        <is>
+          <t>Meal vouchers, hotel authorisations, transport allowances, and DOT/EU261 compensation notices</t>
+        </is>
+      </c>
+      <c r="K227" s="16" t="inlineStr">
+        <is>
+          <t>DOT / EU261 compensation filing accuracy ≥99%; voucher issuance within 60 min of entitlement trigger</t>
+        </is>
+      </c>
+      <c r="L227" s="16" t="inlineStr">
+        <is>
+          <t>Compensation eligibility rules differ by jurisdiction (DOT, EU261, ANAC, DGAC); no unified entitlement engine forces manual legal review for international itineraries, creating under- or over-payment risk</t>
+        </is>
+      </c>
+      <c r="M227" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N227" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="30" customHeight="1">
+      <c r="A228" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B228" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C228" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D228" s="18" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E228" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F228" s="18" t="inlineStr">
+        <is>
+          <t>Conduct post-IROPS cost and performance analysis</t>
+        </is>
+      </c>
+      <c r="G228" s="18" t="inlineStr">
+        <is>
+          <t>Finance Controller (Commercial)</t>
+        </is>
+      </c>
+      <c r="H228" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO) + AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I228" s="18" t="inlineStr">
+        <is>
+          <t>Ferry fuel invoices, compensation payouts, rebooking costs, OTP and cancellation data</t>
+        </is>
+      </c>
+      <c r="J228" s="18" t="inlineStr">
+        <is>
+          <t>IROPS total cost report, OTP and cancellation deviation analysis vs. plan</t>
+        </is>
+      </c>
+      <c r="K228" s="18" t="inlineStr">
+        <is>
+          <t>Report delivered ≤72 hrs post-event; cost capture accuracy ±2%</t>
+        </is>
+      </c>
+      <c r="L228" s="18" t="inlineStr">
+        <is>
+          <t>Cost data is scattered across Altéa (compensation), SAP (vendor invoices), and Jeppesen (crew overtime); manual reconciliation typically takes 5–7 business days, delaying learning cycle</t>
+        </is>
+      </c>
+      <c r="M228" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N228" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="30" customHeight="1">
+      <c r="A229" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-12</t>
+        </is>
+      </c>
+      <c r="B229" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C229" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D229" s="16" t="inlineStr">
+        <is>
+          <t>Irregular Operations Recovery Planning</t>
+        </is>
+      </c>
+      <c r="E229" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F229" s="16" t="inlineStr">
+        <is>
+          <t>Update IROPS recovery playbooks and SkySYM scenario library</t>
+        </is>
+      </c>
+      <c r="G229" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H229" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM + Confluence</t>
+        </is>
+      </c>
+      <c r="I229" s="16" t="inlineStr">
+        <is>
+          <t>Post-event debrief findings, scenario performance data, cost report</t>
+        </is>
+      </c>
+      <c r="J229" s="16" t="inlineStr">
+        <is>
+          <t>Updated recovery playbook version; new scenario added to SkySYM IROPS library for future use</t>
+        </is>
+      </c>
+      <c r="K229" s="16" t="inlineStr">
+        <is>
+          <t>Playbook updated within 30 days of event; ≥1 new SkySYM scenario created per Tier 2+ IROPS</t>
+        </is>
+      </c>
+      <c r="L229" s="16" t="inlineStr">
+        <is>
+          <t>Playbook updates are routinely deprioritised once normal operations resume; institutional recovery knowledge is frequently lost without a mandatory structured capture and review process</t>
+        </is>
+      </c>
+      <c r="M229" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N229" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-SP-13: Charter & Ad-Hoc Flight Planning — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -19,6 +19,7 @@
     <sheet name="NP-SP-10" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="NP-SP-11" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="NP-SP-12" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="NP-SP-13" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1104,13 +1105,21 @@
           <t>Charter &amp; Ad-Hoc Flight Planning</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr"/>
-      <c r="G15" s="10" t="inlineStr"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-13</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -9090,13 +9099,1357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-13 — Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Receive &amp; Log Charter Request</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Charter Sales Manager</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Client inquiry or broker RFQ (route, date, pax count, special requirements)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Logged charter request with unique reference number</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Request-to-quote turnaround ≤4 hours of receipt</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>No standardised intake form; requests arrive via email, phone, and broker portals with inconsistent data quality, causing re-work before feasibility can begin</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Validate Route &amp; Airport Feasibility</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Charter request log, airport infrastructure database, bilateral ASA register</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility report covering range, runway length, curfews, and handling agent availability</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility assessment completed ≤2 hours of request receipt</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Airport infrastructure constraints (runway PCN, curfews, Category III ILS availability) not always current in SkySYM, requiring manual NOTAM and AIP cross-check</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Assess Fleet Availability for Charter Date</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Current published schedule, maintenance release plan, feasibility report</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Available aircraft list with candidate tail numbers and estimated positioning cost</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Charter fleet utilisation rate ≥85% on confirmed charter days</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Charter demand routinely conflicts with peak scheduled operations; no dedicated charter fleet buffer exists, forcing displacement of scheduled rotations</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Verify Air Service Agreements &amp; Permit Scope</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Manager</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>IATA Timatic</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility report, destination country, charter type (commercial, private, government)</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>List of required permits, bilateral ASA status, advance-notice windows per country</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Permit scope identified ≤1 business day of feasibility sign-off</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>ASA gaps for new international charter destinations; some governments (Middle East, West Africa) require 72–120 hours advance notice, invalidating short-lead requests</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Apply for Overflight &amp; Landing Permits</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Manager</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>SITA Overflight Permit System</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Permit requirement list, aircraft registration, ICAO flight identifiers</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Filed permit applications, confirmation numbers, expected approval timeline</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Permit approval rate ≥95% within 48 hours of application</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Permit rejections or multi-day delays from foreign CAAs can invalidate charter date commitments already communicated to clients; no automated status polling in SITA system</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Coordinate Airport Slot &amp; Ground Handler</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Approved permits, flight schedule details, preferred handling agent contracts</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed slot allocation, ground handler assignment, and fuelling agreement</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Slot secured ≥5 days before departure; ground handler confirmed ≥72 hours before STD</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Ad-hoc charter requests often arrive within 48 hours of departure, leaving no slot buffer at Level 3 coordinated airports; late slots attract handling surcharges of 30–50% above standard rates</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Assign Aircraft Tail &amp; Confirm MX Release</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Operations Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>AMOS by Swiss AviationSoftware</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Available aircraft list, maintenance schedule, MEL status log</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed tail number with maintenance release, deferred defect check complete</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Aircraft assigned ≥72 hours before departure; MX release confirmed ≥24 hours before STD</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Last-minute MEL findings discovered during pre-departure inspection force tail swaps after crew pairing, catering, and ground handler briefings are complete, causing cascading delays</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Build Crew Pairing Within FAR Part 117 Limits</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed tail number, route, departure and arrival times, crew qualifications database</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Charter crew pairing with duty-time compliance check, rest period validated</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Crew assignment completed ≥48 hours before departure; 100% FAR Part 117 duty compliance</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Charter routes often exceed standard trip lengths or require international type ratings (ETOPS or specific country approvals); limited qualified crew pool for remote or new destinations</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Special Handling &amp; Catering Requirements</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Charter Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Client brief (VIP specifications, cargo manifest, special meal codes, security requirements)</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Special service order confirmed with caterer, ground handler, and security provider</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Special service confirmation delivered ≤24 hours after crew assignment</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>VIP and government charter clients frequently request bespoke catering and in-cabin configurations incompatible with standard galley setup; last-minute changes after catering uplift incur waste costs</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Calculate All-In Charter Price &amp; Margin</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Charter Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Route details, current fuel price (Platts jet fuel index), airport fees, crew cost, handling cost, positioning leg cost</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Itemised price quote with gross margin analysis and fuel surcharge buffer</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Gross margin on charter ≥15% above direct operating cost; quote issued ≤2 hours of feasibility confirmation</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Fuel price volatility between quote acceptance and flight date creates margin erosion; no automatic fuel surcharge adjustment mechanism is integrated into the charter pricing model</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Issue Charter Contract &amp; Collect Deposit</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Charter Sales Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Approved price quote, client details, payment terms</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Executed charter contract via DocuSign, 25% deposit posted to AR in SAP</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Contract executed ≤24 hours of quote acceptance; deposit received ≥5 days before departure</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Payment delays from charter brokers are common; deposit terms not enforced consistently; SAP AR integration gaps mean charter revenue recognition is sometimes deferred to the following month-end</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Load Charter Flight into PSS &amp; Block Inventory</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Signed contract, final pax manifest, special service order</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Active charter flight record in Altéa, inventory fully blocked, IATA SSR codes applied</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Flight created in PSS ≤4 hours of contract execution; zero open inventory seats on charter segment</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Charter flights must be created as special service segments in Altéa; misclassification as scheduled flights causes revenue leakage and double-counting in RM yield reporting</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>File ICAO Flight Plan &amp; Check NOTAMs</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Flight Dispatcher</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed route, tail number, fuel uplift plan, departure time</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Filed ICAO flight plan, NOTAM briefing pack, alternate aerodrome selected</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Flight plan filed ≥3 hours before STD; NOTAM briefing completed ≥90 min before STD</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Last-minute NOTAM closures (runway, restricted airspace, volcanic ash advisories) require re-routing; no automated re-route trigger exists for charter flights outside the scheduled network</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Conduct Pre-Departure Crew &amp; Cabin Briefing</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Captain / Charter Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Honeywell GoDirect</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Crew pairing, filed flight plan, weather package, special service order, security threat level</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Signed crew briefing record, cabin configuration confirmed, security clearances verified</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Briefing completed ≥90 min before STD; 100% crew attendance confirmed</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>VIP or government charter clients sometimes request last-minute route or timing changes post-briefing, requiring flight plan amendment and potential slot forfeiture at the destination</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Execute Charter Flight &amp; Capture Actuals</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Flight Crew / NOC Dispatcher</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Pre-departure checks complete, ATC clearance received, pax aboard</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Actual block time, fuel burn, pax count, and any ATC deviation logged in Altéa</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Block time variance ≤10 min vs. planned; fuel burn within ±3% of flight plan estimate</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>ATC delays on ad-hoc routes not automatically captured in Altéa; actual fuel and time data require manual post-flight reconciliation, creating a 24–48 hour reporting lag</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Reconcile Charter Revenue &amp; Costs in SAP</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Finance Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Actual flight data from Altéa, supplier invoices (fuel, catering, handling, permits)</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Charter P&amp;L report, variance analysis vs. quoted price, cost centre allocation</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue recognition completed ≤5 business days of flight; invoice matching rate ≥90% automated</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Charter cost allocation to cost centres is manual; catering and handling invoices frequently arrive 30+ days post-flight, requiring accruals that distort period-end reporting</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Update Charter Pricing Model &amp; Lessons Learned</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Charter P&amp;L report, operational incident log, client satisfaction feedback</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Updated charter pricing model parameters, lessons-learned record published in Tableau dashboard</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Pricing model refresh cycle: quarterly; margin forecast accuracy improvement ≥5% per cycle</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Lessons-learned data are not systematically fed back into the charter pricing model; repeat cost overruns on the same international routes indicate a structural feedback loop gap</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N229"/>
+  <dimension ref="A1:N246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -25533,6 +26886,1230 @@
         </is>
       </c>
       <c r="N229" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="30" customHeight="1">
+      <c r="A230" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B230" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C230" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D230" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E230" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F230" s="18" t="inlineStr">
+        <is>
+          <t>Receive &amp; Log Charter Request</t>
+        </is>
+      </c>
+      <c r="G230" s="18" t="inlineStr">
+        <is>
+          <t>Charter Sales Manager</t>
+        </is>
+      </c>
+      <c r="H230" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I230" s="18" t="inlineStr">
+        <is>
+          <t>Client inquiry or broker RFQ (route, date, pax count, special requirements)</t>
+        </is>
+      </c>
+      <c r="J230" s="18" t="inlineStr">
+        <is>
+          <t>Logged charter request with unique reference number</t>
+        </is>
+      </c>
+      <c r="K230" s="18" t="inlineStr">
+        <is>
+          <t>Request-to-quote turnaround ≤4 hours of receipt</t>
+        </is>
+      </c>
+      <c r="L230" s="18" t="inlineStr">
+        <is>
+          <t>No standardised intake form; requests arrive via email, phone, and broker portals with inconsistent data quality, causing re-work before feasibility can begin</t>
+        </is>
+      </c>
+      <c r="M230" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N230" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="30" customHeight="1">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B231" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C231" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D231" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E231" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F231" s="16" t="inlineStr">
+        <is>
+          <t>Validate Route &amp; Airport Feasibility</t>
+        </is>
+      </c>
+      <c r="G231" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H231" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I231" s="16" t="inlineStr">
+        <is>
+          <t>Charter request log, airport infrastructure database, bilateral ASA register</t>
+        </is>
+      </c>
+      <c r="J231" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility report covering range, runway length, curfews, and handling agent availability</t>
+        </is>
+      </c>
+      <c r="K231" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility assessment completed ≤2 hours of request receipt</t>
+        </is>
+      </c>
+      <c r="L231" s="16" t="inlineStr">
+        <is>
+          <t>Airport infrastructure constraints (runway PCN, curfews, Category III ILS availability) not always current in SkySYM, requiring manual NOTAM and AIP cross-check</t>
+        </is>
+      </c>
+      <c r="M231" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N231" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="30" customHeight="1">
+      <c r="A232" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B232" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C232" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D232" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E232" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F232" s="18" t="inlineStr">
+        <is>
+          <t>Assess Fleet Availability for Charter Date</t>
+        </is>
+      </c>
+      <c r="G232" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H232" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I232" s="18" t="inlineStr">
+        <is>
+          <t>Current published schedule, maintenance release plan, feasibility report</t>
+        </is>
+      </c>
+      <c r="J232" s="18" t="inlineStr">
+        <is>
+          <t>Available aircraft list with candidate tail numbers and estimated positioning cost</t>
+        </is>
+      </c>
+      <c r="K232" s="18" t="inlineStr">
+        <is>
+          <t>Charter fleet utilisation rate ≥85% on confirmed charter days</t>
+        </is>
+      </c>
+      <c r="L232" s="18" t="inlineStr">
+        <is>
+          <t>Charter demand routinely conflicts with peak scheduled operations; no dedicated charter fleet buffer exists, forcing displacement of scheduled rotations</t>
+        </is>
+      </c>
+      <c r="M232" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N232" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="30" customHeight="1">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B233" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C233" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D233" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F233" s="16" t="inlineStr">
+        <is>
+          <t>Verify Air Service Agreements &amp; Permit Scope</t>
+        </is>
+      </c>
+      <c r="G233" s="16" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Manager</t>
+        </is>
+      </c>
+      <c r="H233" s="16" t="inlineStr">
+        <is>
+          <t>IATA Timatic</t>
+        </is>
+      </c>
+      <c r="I233" s="16" t="inlineStr">
+        <is>
+          <t>Feasibility report, destination country, charter type (commercial, private, government)</t>
+        </is>
+      </c>
+      <c r="J233" s="16" t="inlineStr">
+        <is>
+          <t>List of required permits, bilateral ASA status, advance-notice windows per country</t>
+        </is>
+      </c>
+      <c r="K233" s="16" t="inlineStr">
+        <is>
+          <t>Permit scope identified ≤1 business day of feasibility sign-off</t>
+        </is>
+      </c>
+      <c r="L233" s="16" t="inlineStr">
+        <is>
+          <t>ASA gaps for new international charter destinations; some governments (Middle East, West Africa) require 72–120 hours advance notice, invalidating short-lead requests</t>
+        </is>
+      </c>
+      <c r="M233" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N233" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="30" customHeight="1">
+      <c r="A234" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B234" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C234" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D234" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E234" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F234" s="18" t="inlineStr">
+        <is>
+          <t>Apply for Overflight &amp; Landing Permits</t>
+        </is>
+      </c>
+      <c r="G234" s="18" t="inlineStr">
+        <is>
+          <t>Regulatory Affairs Manager</t>
+        </is>
+      </c>
+      <c r="H234" s="18" t="inlineStr">
+        <is>
+          <t>SITA Overflight Permit System</t>
+        </is>
+      </c>
+      <c r="I234" s="18" t="inlineStr">
+        <is>
+          <t>Permit requirement list, aircraft registration, ICAO flight identifiers</t>
+        </is>
+      </c>
+      <c r="J234" s="18" t="inlineStr">
+        <is>
+          <t>Filed permit applications, confirmation numbers, expected approval timeline</t>
+        </is>
+      </c>
+      <c r="K234" s="18" t="inlineStr">
+        <is>
+          <t>Permit approval rate ≥95% within 48 hours of application</t>
+        </is>
+      </c>
+      <c r="L234" s="18" t="inlineStr">
+        <is>
+          <t>Permit rejections or multi-day delays from foreign CAAs can invalidate charter date commitments already communicated to clients; no automated status polling in SITA system</t>
+        </is>
+      </c>
+      <c r="M234" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N234" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="30" customHeight="1">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B235" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C235" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D235" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E235" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F235" s="16" t="inlineStr">
+        <is>
+          <t>Coordinate Airport Slot &amp; Ground Handler</t>
+        </is>
+      </c>
+      <c r="G235" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H235" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I235" s="16" t="inlineStr">
+        <is>
+          <t>Approved permits, flight schedule details, preferred handling agent contracts</t>
+        </is>
+      </c>
+      <c r="J235" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed slot allocation, ground handler assignment, and fuelling agreement</t>
+        </is>
+      </c>
+      <c r="K235" s="16" t="inlineStr">
+        <is>
+          <t>Slot secured ≥5 days before departure; ground handler confirmed ≥72 hours before STD</t>
+        </is>
+      </c>
+      <c r="L235" s="16" t="inlineStr">
+        <is>
+          <t>Ad-hoc charter requests often arrive within 48 hours of departure, leaving no slot buffer at Level 3 coordinated airports; late slots attract handling surcharges of 30–50% above standard rates</t>
+        </is>
+      </c>
+      <c r="M235" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N235" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="30" customHeight="1">
+      <c r="A236" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B236" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C236" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D236" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E236" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F236" s="18" t="inlineStr">
+        <is>
+          <t>Assign Aircraft Tail &amp; Confirm MX Release</t>
+        </is>
+      </c>
+      <c r="G236" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Operations Manager</t>
+        </is>
+      </c>
+      <c r="H236" s="18" t="inlineStr">
+        <is>
+          <t>AMOS by Swiss AviationSoftware</t>
+        </is>
+      </c>
+      <c r="I236" s="18" t="inlineStr">
+        <is>
+          <t>Available aircraft list, maintenance schedule, MEL status log</t>
+        </is>
+      </c>
+      <c r="J236" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed tail number with maintenance release, deferred defect check complete</t>
+        </is>
+      </c>
+      <c r="K236" s="18" t="inlineStr">
+        <is>
+          <t>Aircraft assigned ≥72 hours before departure; MX release confirmed ≥24 hours before STD</t>
+        </is>
+      </c>
+      <c r="L236" s="18" t="inlineStr">
+        <is>
+          <t>Last-minute MEL findings discovered during pre-departure inspection force tail swaps after crew pairing, catering, and ground handler briefings are complete, causing cascading delays</t>
+        </is>
+      </c>
+      <c r="M236" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N236" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="30" customHeight="1">
+      <c r="A237" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B237" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C237" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D237" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F237" s="16" t="inlineStr">
+        <is>
+          <t>Build Crew Pairing Within FAR Part 117 Limits</t>
+        </is>
+      </c>
+      <c r="G237" s="16" t="inlineStr">
+        <is>
+          <t>Crew Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H237" s="16" t="inlineStr">
+        <is>
+          <t>Jeppesen Crew Management</t>
+        </is>
+      </c>
+      <c r="I237" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed tail number, route, departure and arrival times, crew qualifications database</t>
+        </is>
+      </c>
+      <c r="J237" s="16" t="inlineStr">
+        <is>
+          <t>Charter crew pairing with duty-time compliance check, rest period validated</t>
+        </is>
+      </c>
+      <c r="K237" s="16" t="inlineStr">
+        <is>
+          <t>Crew assignment completed ≥48 hours before departure; 100% FAR Part 117 duty compliance</t>
+        </is>
+      </c>
+      <c r="L237" s="16" t="inlineStr">
+        <is>
+          <t>Charter routes often exceed standard trip lengths or require international type ratings (ETOPS or specific country approvals); limited qualified crew pool for remote or new destinations</t>
+        </is>
+      </c>
+      <c r="M237" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N237" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="30" customHeight="1">
+      <c r="A238" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B238" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C238" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D238" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E238" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F238" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Special Handling &amp; Catering Requirements</t>
+        </is>
+      </c>
+      <c r="G238" s="18" t="inlineStr">
+        <is>
+          <t>Charter Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H238" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I238" s="18" t="inlineStr">
+        <is>
+          <t>Client brief (VIP specifications, cargo manifest, special meal codes, security requirements)</t>
+        </is>
+      </c>
+      <c r="J238" s="18" t="inlineStr">
+        <is>
+          <t>Special service order confirmed with caterer, ground handler, and security provider</t>
+        </is>
+      </c>
+      <c r="K238" s="18" t="inlineStr">
+        <is>
+          <t>Special service confirmation delivered ≤24 hours after crew assignment</t>
+        </is>
+      </c>
+      <c r="L238" s="18" t="inlineStr">
+        <is>
+          <t>VIP and government charter clients frequently request bespoke catering and in-cabin configurations incompatible with standard galley setup; last-minute changes after catering uplift incur waste costs</t>
+        </is>
+      </c>
+      <c r="M238" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N238" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="30" customHeight="1">
+      <c r="A239" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B239" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C239" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D239" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E239" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F239" s="16" t="inlineStr">
+        <is>
+          <t>Calculate All-In Charter Price &amp; Margin</t>
+        </is>
+      </c>
+      <c r="G239" s="16" t="inlineStr">
+        <is>
+          <t>Charter Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H239" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I239" s="16" t="inlineStr">
+        <is>
+          <t>Route details, current fuel price (Platts jet fuel index), airport fees, crew cost, handling cost, positioning leg cost</t>
+        </is>
+      </c>
+      <c r="J239" s="16" t="inlineStr">
+        <is>
+          <t>Itemised price quote with gross margin analysis and fuel surcharge buffer</t>
+        </is>
+      </c>
+      <c r="K239" s="16" t="inlineStr">
+        <is>
+          <t>Gross margin on charter ≥15% above direct operating cost; quote issued ≤2 hours of feasibility confirmation</t>
+        </is>
+      </c>
+      <c r="L239" s="16" t="inlineStr">
+        <is>
+          <t>Fuel price volatility between quote acceptance and flight date creates margin erosion; no automatic fuel surcharge adjustment mechanism is integrated into the charter pricing model</t>
+        </is>
+      </c>
+      <c r="M239" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N239" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="30" customHeight="1">
+      <c r="A240" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B240" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C240" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D240" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E240" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F240" s="18" t="inlineStr">
+        <is>
+          <t>Issue Charter Contract &amp; Collect Deposit</t>
+        </is>
+      </c>
+      <c r="G240" s="18" t="inlineStr">
+        <is>
+          <t>Charter Sales Manager</t>
+        </is>
+      </c>
+      <c r="H240" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I240" s="18" t="inlineStr">
+        <is>
+          <t>Approved price quote, client details, payment terms</t>
+        </is>
+      </c>
+      <c r="J240" s="18" t="inlineStr">
+        <is>
+          <t>Executed charter contract via DocuSign, 25% deposit posted to AR in SAP</t>
+        </is>
+      </c>
+      <c r="K240" s="18" t="inlineStr">
+        <is>
+          <t>Contract executed ≤24 hours of quote acceptance; deposit received ≥5 days before departure</t>
+        </is>
+      </c>
+      <c r="L240" s="18" t="inlineStr">
+        <is>
+          <t>Payment delays from charter brokers are common; deposit terms not enforced consistently; SAP AR integration gaps mean charter revenue recognition is sometimes deferred to the following month-end</t>
+        </is>
+      </c>
+      <c r="M240" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N240" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="30" customHeight="1">
+      <c r="A241" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B241" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C241" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D241" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E241" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F241" s="16" t="inlineStr">
+        <is>
+          <t>Load Charter Flight into PSS &amp; Block Inventory</t>
+        </is>
+      </c>
+      <c r="G241" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H241" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I241" s="16" t="inlineStr">
+        <is>
+          <t>Signed contract, final pax manifest, special service order</t>
+        </is>
+      </c>
+      <c r="J241" s="16" t="inlineStr">
+        <is>
+          <t>Active charter flight record in Altéa, inventory fully blocked, IATA SSR codes applied</t>
+        </is>
+      </c>
+      <c r="K241" s="16" t="inlineStr">
+        <is>
+          <t>Flight created in PSS ≤4 hours of contract execution; zero open inventory seats on charter segment</t>
+        </is>
+      </c>
+      <c r="L241" s="16" t="inlineStr">
+        <is>
+          <t>Charter flights must be created as special service segments in Altéa; misclassification as scheduled flights causes revenue leakage and double-counting in RM yield reporting</t>
+        </is>
+      </c>
+      <c r="M241" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N241" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="30" customHeight="1">
+      <c r="A242" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B242" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C242" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D242" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E242" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F242" s="18" t="inlineStr">
+        <is>
+          <t>File ICAO Flight Plan &amp; Check NOTAMs</t>
+        </is>
+      </c>
+      <c r="G242" s="18" t="inlineStr">
+        <is>
+          <t>Flight Dispatcher</t>
+        </is>
+      </c>
+      <c r="H242" s="18" t="inlineStr">
+        <is>
+          <t>Jeppesen FliteDeck</t>
+        </is>
+      </c>
+      <c r="I242" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed route, tail number, fuel uplift plan, departure time</t>
+        </is>
+      </c>
+      <c r="J242" s="18" t="inlineStr">
+        <is>
+          <t>Filed ICAO flight plan, NOTAM briefing pack, alternate aerodrome selected</t>
+        </is>
+      </c>
+      <c r="K242" s="18" t="inlineStr">
+        <is>
+          <t>Flight plan filed ≥3 hours before STD; NOTAM briefing completed ≥90 min before STD</t>
+        </is>
+      </c>
+      <c r="L242" s="18" t="inlineStr">
+        <is>
+          <t>Last-minute NOTAM closures (runway, restricted airspace, volcanic ash advisories) require re-routing; no automated re-route trigger exists for charter flights outside the scheduled network</t>
+        </is>
+      </c>
+      <c r="M242" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N242" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="30" customHeight="1">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B243" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C243" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D243" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F243" s="16" t="inlineStr">
+        <is>
+          <t>Conduct Pre-Departure Crew &amp; Cabin Briefing</t>
+        </is>
+      </c>
+      <c r="G243" s="16" t="inlineStr">
+        <is>
+          <t>Captain / Charter Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H243" s="16" t="inlineStr">
+        <is>
+          <t>Honeywell GoDirect</t>
+        </is>
+      </c>
+      <c r="I243" s="16" t="inlineStr">
+        <is>
+          <t>Crew pairing, filed flight plan, weather package, special service order, security threat level</t>
+        </is>
+      </c>
+      <c r="J243" s="16" t="inlineStr">
+        <is>
+          <t>Signed crew briefing record, cabin configuration confirmed, security clearances verified</t>
+        </is>
+      </c>
+      <c r="K243" s="16" t="inlineStr">
+        <is>
+          <t>Briefing completed ≥90 min before STD; 100% crew attendance confirmed</t>
+        </is>
+      </c>
+      <c r="L243" s="16" t="inlineStr">
+        <is>
+          <t>VIP or government charter clients sometimes request last-minute route or timing changes post-briefing, requiring flight plan amendment and potential slot forfeiture at the destination</t>
+        </is>
+      </c>
+      <c r="M243" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N243" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="30" customHeight="1">
+      <c r="A244" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B244" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C244" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D244" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E244" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F244" s="18" t="inlineStr">
+        <is>
+          <t>Execute Charter Flight &amp; Capture Actuals</t>
+        </is>
+      </c>
+      <c r="G244" s="18" t="inlineStr">
+        <is>
+          <t>Flight Crew / NOC Dispatcher</t>
+        </is>
+      </c>
+      <c r="H244" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I244" s="18" t="inlineStr">
+        <is>
+          <t>Pre-departure checks complete, ATC clearance received, pax aboard</t>
+        </is>
+      </c>
+      <c r="J244" s="18" t="inlineStr">
+        <is>
+          <t>Actual block time, fuel burn, pax count, and any ATC deviation logged in Altéa</t>
+        </is>
+      </c>
+      <c r="K244" s="18" t="inlineStr">
+        <is>
+          <t>Block time variance ≤10 min vs. planned; fuel burn within ±3% of flight plan estimate</t>
+        </is>
+      </c>
+      <c r="L244" s="18" t="inlineStr">
+        <is>
+          <t>ATC delays on ad-hoc routes not automatically captured in Altéa; actual fuel and time data require manual post-flight reconciliation, creating a 24–48 hour reporting lag</t>
+        </is>
+      </c>
+      <c r="M244" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N244" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="30" customHeight="1">
+      <c r="A245" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B245" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C245" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D245" s="16" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E245" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F245" s="16" t="inlineStr">
+        <is>
+          <t>Reconcile Charter Revenue &amp; Costs in SAP</t>
+        </is>
+      </c>
+      <c r="G245" s="16" t="inlineStr">
+        <is>
+          <t>Finance Analyst</t>
+        </is>
+      </c>
+      <c r="H245" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I245" s="16" t="inlineStr">
+        <is>
+          <t>Actual flight data from Altéa, supplier invoices (fuel, catering, handling, permits)</t>
+        </is>
+      </c>
+      <c r="J245" s="16" t="inlineStr">
+        <is>
+          <t>Charter P&amp;L report, variance analysis vs. quoted price, cost centre allocation</t>
+        </is>
+      </c>
+      <c r="K245" s="16" t="inlineStr">
+        <is>
+          <t>Revenue recognition completed ≤5 business days of flight; invoice matching rate ≥90% automated</t>
+        </is>
+      </c>
+      <c r="L245" s="16" t="inlineStr">
+        <is>
+          <t>Charter cost allocation to cost centres is manual; catering and handling invoices frequently arrive 30+ days post-flight, requiring accruals that distort period-end reporting</t>
+        </is>
+      </c>
+      <c r="M245" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N245" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="30" customHeight="1">
+      <c r="A246" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-13</t>
+        </is>
+      </c>
+      <c r="B246" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C246" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D246" s="18" t="inlineStr">
+        <is>
+          <t>Charter &amp; Ad-Hoc Flight Planning</t>
+        </is>
+      </c>
+      <c r="E246" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F246" s="18" t="inlineStr">
+        <is>
+          <t>Update Charter Pricing Model &amp; Lessons Learned</t>
+        </is>
+      </c>
+      <c r="G246" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H246" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I246" s="18" t="inlineStr">
+        <is>
+          <t>Charter P&amp;L report, operational incident log, client satisfaction feedback</t>
+        </is>
+      </c>
+      <c r="J246" s="18" t="inlineStr">
+        <is>
+          <t>Updated charter pricing model parameters, lessons-learned record published in Tableau dashboard</t>
+        </is>
+      </c>
+      <c r="K246" s="18" t="inlineStr">
+        <is>
+          <t>Pricing model refresh cycle: quarterly; margin forecast accuracy improvement ≥5% per cycle</t>
+        </is>
+      </c>
+      <c r="L246" s="18" t="inlineStr">
+        <is>
+          <t>Lessons-learned data are not systematically fed back into the charter pricing model; repeat cost overruns on the same international routes indicate a structural feedback loop gap</t>
+        </is>
+      </c>
+      <c r="M246" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N246" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-SP-14: Competition & Capacity Benchmarking — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -20,6 +20,7 @@
     <sheet name="NP-SP-11" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="NP-SP-12" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="NP-SP-13" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="NP-SP-14" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1142,13 +1143,21 @@
           <t>Competition &amp; Capacity Benchmarking</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr"/>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-14</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -10443,13 +10452,1357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-14 — Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract competitor schedule data from OAG feed</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Weekly OAG data subscription refresh (SSIM-format schedule file)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Structured competitor schedule dataset by route, frequency, and aircraft type</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Data currency: schedule feed ≤7 days old; coverage ≥95% of target markets</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>OAG schedule data lags actual GDS availability by 24–72 hrs; codeshare operating vs marketing carrier misclassification inflates competitor frequency counts</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Ingest DOT Form 41 traffic and capacity statistics</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>US DOT BTS Form 41 quarterly release (T-100 domestic segment data)</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Market-level ASM, RPM, and enplanement records loaded to Redshift</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Ingestion completeness ≥99% of published BTS records; pipeline SLA &lt;4 hrs post-BTS release</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>T-100 data is released with a 60-day lag; ultra-LCC capacity additions are visible in OAG weeks before T-100 confirms actual operation</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Pull GDS booking and availability data for share estimation</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Sabre MarketIntelligence booking data extract; Amadeus GDS availability snapshot</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Point-of-sale booking share estimates by O&amp;D market and carrier</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Market coverage: GDS data represents ≥70% of bookable seats on target routes</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>NDC channel bookings bypass GDS; LCC direct-channel share is structurally underrepresented, causing systematic underestimation of competitor capture rate</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Validate data completeness and trigger re-pull if gaps detected</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Automated data quality report from Redshift completeness checks</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Data validation sign-off or re-pull request to upstream pipeline</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Data quality gate pass rate ≥98% before advancing to analysis phase</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Partial OAG refreshes due to airline filing delays leave gaps for low-frequency international routes; manual gap-filling introduces analyst subjectivity</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Map competitor frequency and timing by route</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Validated competitor schedule dataset from Step 1.4</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Frequency matrix by competitor, route, and departure time bank</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Frequency gap identified on ≥80% of monitored routes within 5 business days of OAG refresh</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Ultra-LCC seasonal schedule volatility (Spirit, Frontier) makes frequency comparisons unstable; weekly snapshots miss intra-week capacity dumping tactics</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Assess competitor fleet gauge and seat capacity per route</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>SSIM aircraft type codes from OAG feed; Amadeus SkyWORKS fleet reference table</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Seat capacity report per competitor flight by route and equipment type</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Seat capacity variance vs prior period flagged within ±5% accuracy against T-100 actuals</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>SSIM equipment codes are often filed as generic family codes (e.g. 32A for any A320-family) making true gauge differentiation between A319/A320/A321neo unreliable</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Identify competitive schedule gaps and overlap windows</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Frequency matrix and seat capacity report from Steps 2.1–2.2</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Route priority list ranked by competitive exposure score; whitespace opportunity map</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>≥5 whitespace route opportunities or ≥3 overlap-reduction candidates identified per quarterly cycle</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM scenario modelling requires manual O&amp;D demand curves as input; stale demand assumptions from pre-COVID traffic models skew gap analysis in recovering thin markets</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Determine whether material competitive threat warrants escalation</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Competitive exposure score and whitespace map from Step 2.3</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Decision: escalate to capacity modelling (Y) or archive for quarterly review (N)</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Escalation decision issued within 5 business days of schedule gap analysis completion</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Threshold for 'material threat' is qualitatively defined; no standardised scoring rubric causes inconsistent escalation patterns across different analyst teams</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Compute ASM and RPM trends versus industry peers</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>T-100 records and OAG capacity data from Redshift; peer carrier selection list</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Rolling 12-month ASM/RPM trend report vs peer group (e.g. Delta, United, Southwest)</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>ASM CAGR benchmarked against top-5 network carriers; report produced within 3 days of T-100 release</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Peer group selection is subjective; including ULCCs in the peer set distorts unit cost benchmarks given fundamentally different cost structures and ancillary revenue models</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark CASK and RASK against published Form 41 data</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>DOT Form 41 P-12 financial schedules; internal cost allocation data from SAP S/4HANA Finance</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>CASK/RASK variance report with carrier ranking and gap-to-best-in-class analysis</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>RASK within ±3% of peer median; CASK gap-to-best flagged if &gt;10% adverse variance</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>SAP FI/CO cost data uses internal cost centre allocations that differ from DOT Form 41 reporting categories; reconciliation requires manual mapping table maintenance</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate whether own metrics fall below benchmark thresholds</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>CASK/RASK variance report and ASM/RPM trend analysis</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark status flag: within tolerance / below threshold / critical gap</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark review cycle completed quarterly; critical gaps escalated to VP Network within 48 hrs</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Power BI dashboards pull from Redshift snapshots with a 24-hr lag; real-time competitive capacity changes triggered by fare sales are invisible until next refresh cycle</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Run O&amp;D traffic share analysis by market</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>GDS booking share data; T-100 O&amp;D traffic estimates; SkyCAST demand model</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Market share report by O&amp;D pair: own share vs top-3 competitors, trend over 8 quarters</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Market share tracking coverage ≥90% of top-50 O&amp;D markets by revenue; report cycle ≤10 business days</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D demand models are calibrated on historical traffic; post-pandemic leisure demand shift to off-peak O&amp;D pairs is not yet fully reflected in SkyCAST baseline assumptions</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Model revenue impact of competitor capacity changes</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Market share report; competitor capacity delta from Phase 2; SkySYM demand elasticity curves</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact model: projected incremental revenue gain/loss under each competitive scenario</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact model completed within 5 business days; scenario accuracy validated against last 4 actuals within ±8%</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>SkySYM demand elasticity parameters require periodic recalibration; outdated elasticities overestimate diversion from legacy network carriers and underestimate LCC price sensitivity</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Assess whether schedule response is justified by revenue model</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact model from Step 4.2; available fleet and crew headroom data</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Go/no-go decision on capacity response; disposition for each flagged route</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Decision issued within 3 business days of revenue model delivery; routes with projected NPV &gt;$500K fast-tracked to schedule change workflow</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Fleet headroom data from the crew system and SkyMAX fleet assignment may reflect tentative aircraft swaps not yet confirmed; committing capacity response against uncommitted fleet creates downstream conflict</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Draft capacity response and schedule recommendations</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Approved route disposition list from Step 4.3; current season schedule in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Draft schedule change request: frequency additions, gauge upgrades, or withdrawals with effective dates</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Draft recommendations delivered within 5 business days of go-decision; SSIM-formatted change files ready for slot filing</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS schedule change workflow requires SSIM files to comply with IATA Season A/B slot deadlines; competitive response decisions made mid-season often miss the coordinated season window</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Cross-validate recommendations with Amadeus NRM inventory</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Draft schedule change request; NRM current fare class inventory and booking pace</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>NRM alignment sign-off or revised recommendation with RM-adjusted timing/frequency</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>NRM review completed within 3 business days; &lt;10% of recommendations require material revision due to inventory conflict</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>NRM inventory controls are set per flight departure; schedule changes that shift flights to new time slots reset booking pace baselines and require NRM recalibration, creating a 2–3 week blind spot in yield management</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Submit approved schedule changes to planning queue</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>NRM-approved schedule change request; IATA slot filing deadlines</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed schedule change submitted to SkyWORKS production queue; IATA CRS slot filing initiated where required</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>100% of approved changes submitted within IATA CRS filing window; zero capacity responses missed due to deadline breach</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>IATA CRS coordinated slot filings at Level 3 airports (e.g. LHR, JFK) require bilateral coordination that can delay competitive response by 3–6 months; uncoordinated airports still subject to airlines' own scheduling freeze windows</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N246"/>
+  <dimension ref="A1:N263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -28110,6 +29463,1230 @@
         </is>
       </c>
       <c r="N246" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="30" customHeight="1">
+      <c r="A247" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B247" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C247" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D247" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E247" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F247" s="16" t="inlineStr">
+        <is>
+          <t>Extract competitor schedule data from OAG feed</t>
+        </is>
+      </c>
+      <c r="G247" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H247" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I247" s="16" t="inlineStr">
+        <is>
+          <t>Weekly OAG data subscription refresh (SSIM-format schedule file)</t>
+        </is>
+      </c>
+      <c r="J247" s="16" t="inlineStr">
+        <is>
+          <t>Structured competitor schedule dataset by route, frequency, and aircraft type</t>
+        </is>
+      </c>
+      <c r="K247" s="16" t="inlineStr">
+        <is>
+          <t>Data currency: schedule feed ≤7 days old; coverage ≥95% of target markets</t>
+        </is>
+      </c>
+      <c r="L247" s="16" t="inlineStr">
+        <is>
+          <t>OAG schedule data lags actual GDS availability by 24–72 hrs; codeshare operating vs marketing carrier misclassification inflates competitor frequency counts</t>
+        </is>
+      </c>
+      <c r="M247" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N247" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="30" customHeight="1">
+      <c r="A248" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B248" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C248" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D248" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E248" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F248" s="18" t="inlineStr">
+        <is>
+          <t>Ingest DOT Form 41 traffic and capacity statistics</t>
+        </is>
+      </c>
+      <c r="G248" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H248" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I248" s="18" t="inlineStr">
+        <is>
+          <t>US DOT BTS Form 41 quarterly release (T-100 domestic segment data)</t>
+        </is>
+      </c>
+      <c r="J248" s="18" t="inlineStr">
+        <is>
+          <t>Market-level ASM, RPM, and enplanement records loaded to Redshift</t>
+        </is>
+      </c>
+      <c r="K248" s="18" t="inlineStr">
+        <is>
+          <t>Ingestion completeness ≥99% of published BTS records; pipeline SLA &lt;4 hrs post-BTS release</t>
+        </is>
+      </c>
+      <c r="L248" s="18" t="inlineStr">
+        <is>
+          <t>T-100 data is released with a 60-day lag; ultra-LCC capacity additions are visible in OAG weeks before T-100 confirms actual operation</t>
+        </is>
+      </c>
+      <c r="M248" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N248" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="30" customHeight="1">
+      <c r="A249" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B249" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C249" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D249" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E249" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F249" s="16" t="inlineStr">
+        <is>
+          <t>Pull GDS booking and availability data for share estimation</t>
+        </is>
+      </c>
+      <c r="G249" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H249" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I249" s="16" t="inlineStr">
+        <is>
+          <t>Sabre MarketIntelligence booking data extract; Amadeus GDS availability snapshot</t>
+        </is>
+      </c>
+      <c r="J249" s="16" t="inlineStr">
+        <is>
+          <t>Point-of-sale booking share estimates by O&amp;D market and carrier</t>
+        </is>
+      </c>
+      <c r="K249" s="16" t="inlineStr">
+        <is>
+          <t>Market coverage: GDS data represents ≥70% of bookable seats on target routes</t>
+        </is>
+      </c>
+      <c r="L249" s="16" t="inlineStr">
+        <is>
+          <t>NDC channel bookings bypass GDS; LCC direct-channel share is structurally underrepresented, causing systematic underestimation of competitor capture rate</t>
+        </is>
+      </c>
+      <c r="M249" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N249" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="30" customHeight="1">
+      <c r="A250" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B250" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C250" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D250" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E250" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F250" s="18" t="inlineStr">
+        <is>
+          <t>Validate data completeness and trigger re-pull if gaps detected</t>
+        </is>
+      </c>
+      <c r="G250" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H250" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I250" s="18" t="inlineStr">
+        <is>
+          <t>Automated data quality report from Redshift completeness checks</t>
+        </is>
+      </c>
+      <c r="J250" s="18" t="inlineStr">
+        <is>
+          <t>Data validation sign-off or re-pull request to upstream pipeline</t>
+        </is>
+      </c>
+      <c r="K250" s="18" t="inlineStr">
+        <is>
+          <t>Data quality gate pass rate ≥98% before advancing to analysis phase</t>
+        </is>
+      </c>
+      <c r="L250" s="18" t="inlineStr">
+        <is>
+          <t>Partial OAG refreshes due to airline filing delays leave gaps for low-frequency international routes; manual gap-filling introduces analyst subjectivity</t>
+        </is>
+      </c>
+      <c r="M250" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N250" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="30" customHeight="1">
+      <c r="A251" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B251" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C251" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D251" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E251" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F251" s="16" t="inlineStr">
+        <is>
+          <t>Map competitor frequency and timing by route</t>
+        </is>
+      </c>
+      <c r="G251" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H251" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I251" s="16" t="inlineStr">
+        <is>
+          <t>Validated competitor schedule dataset from Step 1.4</t>
+        </is>
+      </c>
+      <c r="J251" s="16" t="inlineStr">
+        <is>
+          <t>Frequency matrix by competitor, route, and departure time bank</t>
+        </is>
+      </c>
+      <c r="K251" s="16" t="inlineStr">
+        <is>
+          <t>Frequency gap identified on ≥80% of monitored routes within 5 business days of OAG refresh</t>
+        </is>
+      </c>
+      <c r="L251" s="16" t="inlineStr">
+        <is>
+          <t>Ultra-LCC seasonal schedule volatility (Spirit, Frontier) makes frequency comparisons unstable; weekly snapshots miss intra-week capacity dumping tactics</t>
+        </is>
+      </c>
+      <c r="M251" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N251" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="30" customHeight="1">
+      <c r="A252" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B252" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C252" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D252" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E252" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F252" s="18" t="inlineStr">
+        <is>
+          <t>Assess competitor fleet gauge and seat capacity per route</t>
+        </is>
+      </c>
+      <c r="G252" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H252" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I252" s="18" t="inlineStr">
+        <is>
+          <t>SSIM aircraft type codes from OAG feed; Amadeus SkyWORKS fleet reference table</t>
+        </is>
+      </c>
+      <c r="J252" s="18" t="inlineStr">
+        <is>
+          <t>Seat capacity report per competitor flight by route and equipment type</t>
+        </is>
+      </c>
+      <c r="K252" s="18" t="inlineStr">
+        <is>
+          <t>Seat capacity variance vs prior period flagged within ±5% accuracy against T-100 actuals</t>
+        </is>
+      </c>
+      <c r="L252" s="18" t="inlineStr">
+        <is>
+          <t>SSIM equipment codes are often filed as generic family codes (e.g. 32A for any A320-family) making true gauge differentiation between A319/A320/A321neo unreliable</t>
+        </is>
+      </c>
+      <c r="M252" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N252" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="30" customHeight="1">
+      <c r="A253" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B253" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C253" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D253" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E253" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F253" s="16" t="inlineStr">
+        <is>
+          <t>Identify competitive schedule gaps and overlap windows</t>
+        </is>
+      </c>
+      <c r="G253" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H253" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I253" s="16" t="inlineStr">
+        <is>
+          <t>Frequency matrix and seat capacity report from Steps 2.1–2.2</t>
+        </is>
+      </c>
+      <c r="J253" s="16" t="inlineStr">
+        <is>
+          <t>Route priority list ranked by competitive exposure score; whitespace opportunity map</t>
+        </is>
+      </c>
+      <c r="K253" s="16" t="inlineStr">
+        <is>
+          <t>≥5 whitespace route opportunities or ≥3 overlap-reduction candidates identified per quarterly cycle</t>
+        </is>
+      </c>
+      <c r="L253" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario modelling requires manual O&amp;D demand curves as input; stale demand assumptions from pre-COVID traffic models skew gap analysis in recovering thin markets</t>
+        </is>
+      </c>
+      <c r="M253" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N253" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="30" customHeight="1">
+      <c r="A254" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B254" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C254" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D254" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E254" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F254" s="18" t="inlineStr">
+        <is>
+          <t>Determine whether material competitive threat warrants escalation</t>
+        </is>
+      </c>
+      <c r="G254" s="18" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H254" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I254" s="18" t="inlineStr">
+        <is>
+          <t>Competitive exposure score and whitespace map from Step 2.3</t>
+        </is>
+      </c>
+      <c r="J254" s="18" t="inlineStr">
+        <is>
+          <t>Decision: escalate to capacity modelling (Y) or archive for quarterly review (N)</t>
+        </is>
+      </c>
+      <c r="K254" s="18" t="inlineStr">
+        <is>
+          <t>Escalation decision issued within 5 business days of schedule gap analysis completion</t>
+        </is>
+      </c>
+      <c r="L254" s="18" t="inlineStr">
+        <is>
+          <t>Threshold for 'material threat' is qualitatively defined; no standardised scoring rubric causes inconsistent escalation patterns across different analyst teams</t>
+        </is>
+      </c>
+      <c r="M254" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N254" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="30" customHeight="1">
+      <c r="A255" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B255" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C255" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D255" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E255" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F255" s="16" t="inlineStr">
+        <is>
+          <t>Compute ASM and RPM trends versus industry peers</t>
+        </is>
+      </c>
+      <c r="G255" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H255" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I255" s="16" t="inlineStr">
+        <is>
+          <t>T-100 records and OAG capacity data from Redshift; peer carrier selection list</t>
+        </is>
+      </c>
+      <c r="J255" s="16" t="inlineStr">
+        <is>
+          <t>Rolling 12-month ASM/RPM trend report vs peer group (e.g. Delta, United, Southwest)</t>
+        </is>
+      </c>
+      <c r="K255" s="16" t="inlineStr">
+        <is>
+          <t>ASM CAGR benchmarked against top-5 network carriers; report produced within 3 days of T-100 release</t>
+        </is>
+      </c>
+      <c r="L255" s="16" t="inlineStr">
+        <is>
+          <t>Peer group selection is subjective; including ULCCs in the peer set distorts unit cost benchmarks given fundamentally different cost structures and ancillary revenue models</t>
+        </is>
+      </c>
+      <c r="M255" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N255" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="30" customHeight="1">
+      <c r="A256" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B256" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C256" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D256" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E256" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F256" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark CASK and RASK against published Form 41 data</t>
+        </is>
+      </c>
+      <c r="G256" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H256" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I256" s="18" t="inlineStr">
+        <is>
+          <t>DOT Form 41 P-12 financial schedules; internal cost allocation data from SAP S/4HANA Finance</t>
+        </is>
+      </c>
+      <c r="J256" s="18" t="inlineStr">
+        <is>
+          <t>CASK/RASK variance report with carrier ranking and gap-to-best-in-class analysis</t>
+        </is>
+      </c>
+      <c r="K256" s="18" t="inlineStr">
+        <is>
+          <t>RASK within ±3% of peer median; CASK gap-to-best flagged if &gt;10% adverse variance</t>
+        </is>
+      </c>
+      <c r="L256" s="18" t="inlineStr">
+        <is>
+          <t>SAP FI/CO cost data uses internal cost centre allocations that differ from DOT Form 41 reporting categories; reconciliation requires manual mapping table maintenance</t>
+        </is>
+      </c>
+      <c r="M256" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N256" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="30" customHeight="1">
+      <c r="A257" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B257" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C257" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D257" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E257" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F257" s="16" t="inlineStr">
+        <is>
+          <t>Evaluate whether own metrics fall below benchmark thresholds</t>
+        </is>
+      </c>
+      <c r="G257" s="16" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H257" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I257" s="16" t="inlineStr">
+        <is>
+          <t>CASK/RASK variance report and ASM/RPM trend analysis</t>
+        </is>
+      </c>
+      <c r="J257" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark status flag: within tolerance / below threshold / critical gap</t>
+        </is>
+      </c>
+      <c r="K257" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark review cycle completed quarterly; critical gaps escalated to VP Network within 48 hrs</t>
+        </is>
+      </c>
+      <c r="L257" s="16" t="inlineStr">
+        <is>
+          <t>Power BI dashboards pull from Redshift snapshots with a 24-hr lag; real-time competitive capacity changes triggered by fare sales are invisible until next refresh cycle</t>
+        </is>
+      </c>
+      <c r="M257" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N257" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="30" customHeight="1">
+      <c r="A258" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B258" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C258" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D258" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E258" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F258" s="18" t="inlineStr">
+        <is>
+          <t>Run O&amp;D traffic share analysis by market</t>
+        </is>
+      </c>
+      <c r="G258" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H258" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I258" s="18" t="inlineStr">
+        <is>
+          <t>GDS booking share data; T-100 O&amp;D traffic estimates; SkyCAST demand model</t>
+        </is>
+      </c>
+      <c r="J258" s="18" t="inlineStr">
+        <is>
+          <t>Market share report by O&amp;D pair: own share vs top-3 competitors, trend over 8 quarters</t>
+        </is>
+      </c>
+      <c r="K258" s="18" t="inlineStr">
+        <is>
+          <t>Market share tracking coverage ≥90% of top-50 O&amp;D markets by revenue; report cycle ≤10 business days</t>
+        </is>
+      </c>
+      <c r="L258" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D demand models are calibrated on historical traffic; post-pandemic leisure demand shift to off-peak O&amp;D pairs is not yet fully reflected in SkyCAST baseline assumptions</t>
+        </is>
+      </c>
+      <c r="M258" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N258" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="30" customHeight="1">
+      <c r="A259" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B259" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C259" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D259" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E259" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F259" s="16" t="inlineStr">
+        <is>
+          <t>Model revenue impact of competitor capacity changes</t>
+        </is>
+      </c>
+      <c r="G259" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H259" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I259" s="16" t="inlineStr">
+        <is>
+          <t>Market share report; competitor capacity delta from Phase 2; SkySYM demand elasticity curves</t>
+        </is>
+      </c>
+      <c r="J259" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact model: projected incremental revenue gain/loss under each competitive scenario</t>
+        </is>
+      </c>
+      <c r="K259" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact model completed within 5 business days; scenario accuracy validated against last 4 actuals within ±8%</t>
+        </is>
+      </c>
+      <c r="L259" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM demand elasticity parameters require periodic recalibration; outdated elasticities overestimate diversion from legacy network carriers and underestimate LCC price sensitivity</t>
+        </is>
+      </c>
+      <c r="M259" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N259" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="30" customHeight="1">
+      <c r="A260" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B260" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C260" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D260" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E260" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F260" s="18" t="inlineStr">
+        <is>
+          <t>Assess whether schedule response is justified by revenue model</t>
+        </is>
+      </c>
+      <c r="G260" s="18" t="inlineStr">
+        <is>
+          <t>Director of Network Planning</t>
+        </is>
+      </c>
+      <c r="H260" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I260" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact model from Step 4.2; available fleet and crew headroom data</t>
+        </is>
+      </c>
+      <c r="J260" s="18" t="inlineStr">
+        <is>
+          <t>Go/no-go decision on capacity response; disposition for each flagged route</t>
+        </is>
+      </c>
+      <c r="K260" s="18" t="inlineStr">
+        <is>
+          <t>Decision issued within 3 business days of revenue model delivery; routes with projected NPV &gt;$500K fast-tracked to schedule change workflow</t>
+        </is>
+      </c>
+      <c r="L260" s="18" t="inlineStr">
+        <is>
+          <t>Fleet headroom data from the crew system and SkyMAX fleet assignment may reflect tentative aircraft swaps not yet confirmed; committing capacity response against uncommitted fleet creates downstream conflict</t>
+        </is>
+      </c>
+      <c r="M260" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N260" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="30" customHeight="1">
+      <c r="A261" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B261" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C261" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D261" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E261" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F261" s="16" t="inlineStr">
+        <is>
+          <t>Draft capacity response and schedule recommendations</t>
+        </is>
+      </c>
+      <c r="G261" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H261" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I261" s="16" t="inlineStr">
+        <is>
+          <t>Approved route disposition list from Step 4.3; current season schedule in SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J261" s="16" t="inlineStr">
+        <is>
+          <t>Draft schedule change request: frequency additions, gauge upgrades, or withdrawals with effective dates</t>
+        </is>
+      </c>
+      <c r="K261" s="16" t="inlineStr">
+        <is>
+          <t>Draft recommendations delivered within 5 business days of go-decision; SSIM-formatted change files ready for slot filing</t>
+        </is>
+      </c>
+      <c r="L261" s="16" t="inlineStr">
+        <is>
+          <t>SkyWORKS schedule change workflow requires SSIM files to comply with IATA Season A/B slot deadlines; competitive response decisions made mid-season often miss the coordinated season window</t>
+        </is>
+      </c>
+      <c r="M261" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N261" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="30" customHeight="1">
+      <c r="A262" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B262" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C262" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D262" s="18" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E262" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F262" s="18" t="inlineStr">
+        <is>
+          <t>Cross-validate recommendations with Amadeus NRM inventory</t>
+        </is>
+      </c>
+      <c r="G262" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H262" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I262" s="18" t="inlineStr">
+        <is>
+          <t>Draft schedule change request; NRM current fare class inventory and booking pace</t>
+        </is>
+      </c>
+      <c r="J262" s="18" t="inlineStr">
+        <is>
+          <t>NRM alignment sign-off or revised recommendation with RM-adjusted timing/frequency</t>
+        </is>
+      </c>
+      <c r="K262" s="18" t="inlineStr">
+        <is>
+          <t>NRM review completed within 3 business days; &lt;10% of recommendations require material revision due to inventory conflict</t>
+        </is>
+      </c>
+      <c r="L262" s="18" t="inlineStr">
+        <is>
+          <t>NRM inventory controls are set per flight departure; schedule changes that shift flights to new time slots reset booking pace baselines and require NRM recalibration, creating a 2–3 week blind spot in yield management</t>
+        </is>
+      </c>
+      <c r="M262" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N262" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="30" customHeight="1">
+      <c r="A263" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-14</t>
+        </is>
+      </c>
+      <c r="B263" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C263" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D263" s="16" t="inlineStr">
+        <is>
+          <t>Competition &amp; Capacity Benchmarking</t>
+        </is>
+      </c>
+      <c r="E263" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F263" s="16" t="inlineStr">
+        <is>
+          <t>Submit approved schedule changes to planning queue</t>
+        </is>
+      </c>
+      <c r="G263" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning Manager</t>
+        </is>
+      </c>
+      <c r="H263" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I263" s="16" t="inlineStr">
+        <is>
+          <t>NRM-approved schedule change request; IATA slot filing deadlines</t>
+        </is>
+      </c>
+      <c r="J263" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed schedule change submitted to SkyWORKS production queue; IATA CRS slot filing initiated where required</t>
+        </is>
+      </c>
+      <c r="K263" s="16" t="inlineStr">
+        <is>
+          <t>100% of approved changes submitted within IATA CRS filing window; zero capacity responses missed due to deadline breach</t>
+        </is>
+      </c>
+      <c r="L263" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS coordinated slot filings at Level 3 airports (e.g. LHR, JFK) require bilateral coordination that can delay competitive response by 3–6 months; uncoordinated airports still subject to airlines' own scheduling freeze windows</t>
+        </is>
+      </c>
+      <c r="M263" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N263" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-SP-15: Strategic Network Planning — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -21,6 +21,7 @@
     <sheet name="NP-SP-12" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="NP-SP-13" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="NP-SP-14" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="NP-SP-15" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1180,13 +1181,21 @@
           <t>Strategic Network Planning</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr"/>
-      <c r="G17" s="10" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/schedule-planning/np-sp-15</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -11796,13 +11805,1357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-SP-15 — Strategic Network Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Schedule Planning  |  L3: Strategic Network Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract competitive schedule &amp; capacity data</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Annual planning cycle trigger; prior-year SSIM schedules</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Competitor capacity matrix by O&amp;D market (seats, frequencies, ASMs)</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Market coverage: ≥95% of OAG universe validated within 5 business days</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>OAG data lags 48–72 hrs for LCC schedule changes; analyst must reconcile against GDS live availability</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Ingest historical O&amp;D traffic &amp; yield data</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>3-year rolling MIDT booking data, internal ticket coupon data</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand baseline with seasonality indices per market pair</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Demand model R² ≥0.90 vs actual bookings on back-test</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>MIDT coverage drops to ~60% for LCC-heavy markets where GDS penetration is low; distorts baseline</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate &amp; cleanse market intelligence dataset</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>OAG capacity matrix, SkyCAST O&amp;D baseline, macroeconomic indices</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Validated market intelligence dataset approved for modelling</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness ≥98% of target O&amp;D pairs before model run</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Macro data (GDP, tourism forecasts) sourced from multiple external vendors with inconsistent update cycles</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Generate long-haul &amp; medium-haul demand scenarios</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated market intelligence dataset; strategic growth targets from CEO brief</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>3 demand scenarios (base, upside, downside) per O&amp;D market for 3-year horizon</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Scenario variance within ±15% of base-case for primary markets</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario runtime scales poorly for networks &gt;500 O&amp;D pairs; overnight batch required for full network runs</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Score and rank route opportunities by strategic fit</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>3 demand scenarios, strategic priority filters (geography, alliance fit, connectivity)</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Ranked route opportunity scorecard (revenue potential, strategic score, competitive intensity)</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Top-20 route list updated within 2 weeks of scenario generation</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Scoring weights for 'strategic fit' are subjective; senior stakeholders override quantitative ranking without documented rationale</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Review route shortlist against network strategy guardrails</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Ranked route opportunity scorecard, board-approved network strategy KPIs</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Approved route shortlist (10–30 routes) for feasibility analysis</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Shortlist approved within 5 business days of scorecard publication</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>No system-enforced guardrail check; planner reliance on manual KPI dashboard review risks missing constraints</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Run fleet assignment optimisation for shortlisted routes</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Approved route shortlist, current fleet plan, aircraft availability calendar</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan with gauge recommendations per route</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Fleet utilisation uplift ≥2% vs current plan in optimised output</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX optimisation assumes unconstrained maintenance slots; MRO visit conflicts discovered post-optimisation require manual iteration</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Assess slot &amp; airport capacity constraints</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan, IATA WSG slot library for target airports</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Slot feasibility report (available, historic grandfather, needs application)</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Slot feasibility assessment completed ≥90 days before IATA scheduling conference</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability at Level 3 airports (LHR, AMS, CDG) is opaque until conference; strategic plans regularly revised post-conference</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate airport infrastructure &amp; ground handling readiness</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Airport Development Manager</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Slot feasibility report, proposed frequencies, aircraft gauge</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Airport readiness assessment (gates, ground handlers, customs, fuelling)</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Infrastructure gap identified ≥12 months before proposed launch date</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Ground handler capacity data at outstations not centrally held; planner must contact handlers individually, adding 3–6 weeks to cycle</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Confirm operational feasibility of candidate routes</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan, slot feasibility report, airport readiness assessment</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Operationally feasible route set confirmed in SkyWORKS schedule editor</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>≥80% of shortlisted routes confirmed feasible without major constraint</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Crew base restrictions and FAR Part 117 duty-time rules reduce feasible rotations, particularly for ultra-long-haul additions</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Build unit revenue &amp; yield forecast per candidate route</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed feasible route set, demand scenarios, competitive fare data from ATPCO</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>PRASM and RASM forecast per route across base/upside/downside scenarios</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>RASM forecast accuracy within ±8% of actuals on launched routes (tracked retrospectively)</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>NRM is calibrated on existing routes; forecast reliability for new O&amp;D markets with no booking history is low — often requires manual analyst override</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Model direct operating costs per route</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Finance Business Partner — Network</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan (aircraft type, block hours), fuel price assumptions, airport charges schedule</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>CASM breakdown per route (fuel, airport, crew, maintenance, overhead allocation)</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>CASM model completed within 10 business days of receiving fleet assignment input</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Airport charge schedules for new markets are not always available in SAP master data; finance team must source bilaterally from airport authorities</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Assess route contribution margin and breakeven load factor</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>RASM forecast, CASM breakdown, targeted load factor assumptions</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Route P&amp;L summary with breakeven load factor and payback period</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Target contribution margin ≥12% in Year 2; breakeven load factor ≤75%</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Sensitivity of breakeven load factor to fuel price is high; +10% fuel swing shifts breakeven by 4–6 ppts, making many routes marginal</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Aggregate network business case for plan period</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Individual route P&amp;L summaries, network-level synergy assumptions (feed, connectivity)</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>3-year network business case document (revenue, cost, EBIT impact)</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Network EBIT uplift ≥$150M over plan period vs do-nothing baseline</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Network synergy benefits (connecting traffic uplift) are difficult to isolate and often overstated in bottom-up aggregation</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Package strategic plan for governance review</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Network business case, route scorecard, risk register</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Executive briefing pack: network strategy summary, investment ask, risk matrix</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Briefing pack issued ≥5 business days before Network Strategy Committee meeting</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Version control of the briefing pack is manual; late assumption changes from Revenue Management or Finance require last-minute slides rebuild</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Present plan to Network Strategy Committee</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Executive briefing pack, committee member pre-read questions</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Committee decision: approved / approved with conditions / rejected with rationale</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Committee decision reached in ≤2 review cycles (no more than 1 deferral per plan)</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Committee quorum requires C-suite attendance; scheduling conflicts routinely delay decision by 2–4 weeks, compressing scheduling window</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Publish approved strategic network plan &amp; handoff to scheduling</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Approved committee decision, final route list with gauge and frequency targets</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Published strategic network plan loaded into SkyWORKS as planning baseline for Schedule Planning team</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Plan published in SkyWORKS ≤3 business days after committee approval</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS baseline lock-in creates downstream rigidity; late executive changes after publication require formal change request and delay tactical planning</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N263"/>
+  <dimension ref="A1:N280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -30689,6 +32042,1230 @@
       <c r="N263" s="15" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="30" customHeight="1">
+      <c r="A264" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B264" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C264" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D264" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E264" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F264" s="18" t="inlineStr">
+        <is>
+          <t>Extract competitive schedule &amp; capacity data</t>
+        </is>
+      </c>
+      <c r="G264" s="18" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H264" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I264" s="18" t="inlineStr">
+        <is>
+          <t>Annual planning cycle trigger; prior-year SSIM schedules</t>
+        </is>
+      </c>
+      <c r="J264" s="18" t="inlineStr">
+        <is>
+          <t>Competitor capacity matrix by O&amp;D market (seats, frequencies, ASMs)</t>
+        </is>
+      </c>
+      <c r="K264" s="18" t="inlineStr">
+        <is>
+          <t>Market coverage: ≥95% of OAG universe validated within 5 business days</t>
+        </is>
+      </c>
+      <c r="L264" s="18" t="inlineStr">
+        <is>
+          <t>OAG data lags 48–72 hrs for LCC schedule changes; analyst must reconcile against GDS live availability</t>
+        </is>
+      </c>
+      <c r="M264" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N264" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="30" customHeight="1">
+      <c r="A265" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B265" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C265" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D265" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E265" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F265" s="16" t="inlineStr">
+        <is>
+          <t>Ingest historical O&amp;D traffic &amp; yield data</t>
+        </is>
+      </c>
+      <c r="G265" s="16" t="inlineStr">
+        <is>
+          <t>Network Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H265" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I265" s="16" t="inlineStr">
+        <is>
+          <t>3-year rolling MIDT booking data, internal ticket coupon data</t>
+        </is>
+      </c>
+      <c r="J265" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand baseline with seasonality indices per market pair</t>
+        </is>
+      </c>
+      <c r="K265" s="16" t="inlineStr">
+        <is>
+          <t>Demand model R² ≥0.90 vs actual bookings on back-test</t>
+        </is>
+      </c>
+      <c r="L265" s="16" t="inlineStr">
+        <is>
+          <t>MIDT coverage drops to ~60% for LCC-heavy markets where GDS penetration is low; distorts baseline</t>
+        </is>
+      </c>
+      <c r="M265" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N265" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="30" customHeight="1">
+      <c r="A266" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B266" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C266" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D266" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E266" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F266" s="18" t="inlineStr">
+        <is>
+          <t>Validate &amp; cleanse market intelligence dataset</t>
+        </is>
+      </c>
+      <c r="G266" s="18" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H266" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I266" s="18" t="inlineStr">
+        <is>
+          <t>OAG capacity matrix, SkyCAST O&amp;D baseline, macroeconomic indices</t>
+        </is>
+      </c>
+      <c r="J266" s="18" t="inlineStr">
+        <is>
+          <t>Validated market intelligence dataset approved for modelling</t>
+        </is>
+      </c>
+      <c r="K266" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness ≥98% of target O&amp;D pairs before model run</t>
+        </is>
+      </c>
+      <c r="L266" s="18" t="inlineStr">
+        <is>
+          <t>Macro data (GDP, tourism forecasts) sourced from multiple external vendors with inconsistent update cycles</t>
+        </is>
+      </c>
+      <c r="M266" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N266" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="30" customHeight="1">
+      <c r="A267" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B267" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C267" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D267" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E267" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F267" s="16" t="inlineStr">
+        <is>
+          <t>Generate long-haul &amp; medium-haul demand scenarios</t>
+        </is>
+      </c>
+      <c r="G267" s="16" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H267" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkySYM</t>
+        </is>
+      </c>
+      <c r="I267" s="16" t="inlineStr">
+        <is>
+          <t>Validated market intelligence dataset; strategic growth targets from CEO brief</t>
+        </is>
+      </c>
+      <c r="J267" s="16" t="inlineStr">
+        <is>
+          <t>3 demand scenarios (base, upside, downside) per O&amp;D market for 3-year horizon</t>
+        </is>
+      </c>
+      <c r="K267" s="16" t="inlineStr">
+        <is>
+          <t>Scenario variance within ±15% of base-case for primary markets</t>
+        </is>
+      </c>
+      <c r="L267" s="16" t="inlineStr">
+        <is>
+          <t>SkySYM scenario runtime scales poorly for networks &gt;500 O&amp;D pairs; overnight batch required for full network runs</t>
+        </is>
+      </c>
+      <c r="M267" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N267" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="30" customHeight="1">
+      <c r="A268" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B268" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C268" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D268" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E268" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F268" s="18" t="inlineStr">
+        <is>
+          <t>Score and rank route opportunities by strategic fit</t>
+        </is>
+      </c>
+      <c r="G268" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H268" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I268" s="18" t="inlineStr">
+        <is>
+          <t>3 demand scenarios, strategic priority filters (geography, alliance fit, connectivity)</t>
+        </is>
+      </c>
+      <c r="J268" s="18" t="inlineStr">
+        <is>
+          <t>Ranked route opportunity scorecard (revenue potential, strategic score, competitive intensity)</t>
+        </is>
+      </c>
+      <c r="K268" s="18" t="inlineStr">
+        <is>
+          <t>Top-20 route list updated within 2 weeks of scenario generation</t>
+        </is>
+      </c>
+      <c r="L268" s="18" t="inlineStr">
+        <is>
+          <t>Scoring weights for 'strategic fit' are subjective; senior stakeholders override quantitative ranking without documented rationale</t>
+        </is>
+      </c>
+      <c r="M268" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N268" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="30" customHeight="1">
+      <c r="A269" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B269" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C269" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D269" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E269" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F269" s="16" t="inlineStr">
+        <is>
+          <t>Review route shortlist against network strategy guardrails</t>
+        </is>
+      </c>
+      <c r="G269" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H269" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I269" s="16" t="inlineStr">
+        <is>
+          <t>Ranked route opportunity scorecard, board-approved network strategy KPIs</t>
+        </is>
+      </c>
+      <c r="J269" s="16" t="inlineStr">
+        <is>
+          <t>Approved route shortlist (10–30 routes) for feasibility analysis</t>
+        </is>
+      </c>
+      <c r="K269" s="16" t="inlineStr">
+        <is>
+          <t>Shortlist approved within 5 business days of scorecard publication</t>
+        </is>
+      </c>
+      <c r="L269" s="16" t="inlineStr">
+        <is>
+          <t>No system-enforced guardrail check; planner reliance on manual KPI dashboard review risks missing constraints</t>
+        </is>
+      </c>
+      <c r="M269" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N269" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="30" customHeight="1">
+      <c r="A270" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B270" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C270" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D270" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E270" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F270" s="18" t="inlineStr">
+        <is>
+          <t>Run fleet assignment optimisation for shortlisted routes</t>
+        </is>
+      </c>
+      <c r="G270" s="18" t="inlineStr">
+        <is>
+          <t>Fleet Planning Analyst</t>
+        </is>
+      </c>
+      <c r="H270" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyMAX</t>
+        </is>
+      </c>
+      <c r="I270" s="18" t="inlineStr">
+        <is>
+          <t>Approved route shortlist, current fleet plan, aircraft availability calendar</t>
+        </is>
+      </c>
+      <c r="J270" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan with gauge recommendations per route</t>
+        </is>
+      </c>
+      <c r="K270" s="18" t="inlineStr">
+        <is>
+          <t>Fleet utilisation uplift ≥2% vs current plan in optimised output</t>
+        </is>
+      </c>
+      <c r="L270" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX optimisation assumes unconstrained maintenance slots; MRO visit conflicts discovered post-optimisation require manual iteration</t>
+        </is>
+      </c>
+      <c r="M270" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N270" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="30" customHeight="1">
+      <c r="A271" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B271" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C271" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D271" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E271" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F271" s="16" t="inlineStr">
+        <is>
+          <t>Assess slot &amp; airport capacity constraints</t>
+        </is>
+      </c>
+      <c r="G271" s="16" t="inlineStr">
+        <is>
+          <t>Slot Coordinator</t>
+        </is>
+      </c>
+      <c r="H271" s="16" t="inlineStr">
+        <is>
+          <t>IATA CRS (Coordinated Reservation System)</t>
+        </is>
+      </c>
+      <c r="I271" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan, IATA WSG slot library for target airports</t>
+        </is>
+      </c>
+      <c r="J271" s="16" t="inlineStr">
+        <is>
+          <t>Slot feasibility report (available, historic grandfather, needs application)</t>
+        </is>
+      </c>
+      <c r="K271" s="16" t="inlineStr">
+        <is>
+          <t>Slot feasibility assessment completed ≥90 days before IATA scheduling conference</t>
+        </is>
+      </c>
+      <c r="L271" s="16" t="inlineStr">
+        <is>
+          <t>Slot availability at Level 3 airports (LHR, AMS, CDG) is opaque until conference; strategic plans regularly revised post-conference</t>
+        </is>
+      </c>
+      <c r="M271" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N271" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="30" customHeight="1">
+      <c r="A272" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B272" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C272" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D272" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E272" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F272" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate airport infrastructure &amp; ground handling readiness</t>
+        </is>
+      </c>
+      <c r="G272" s="18" t="inlineStr">
+        <is>
+          <t>Airport Development Manager</t>
+        </is>
+      </c>
+      <c r="H272" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I272" s="18" t="inlineStr">
+        <is>
+          <t>Slot feasibility report, proposed frequencies, aircraft gauge</t>
+        </is>
+      </c>
+      <c r="J272" s="18" t="inlineStr">
+        <is>
+          <t>Airport readiness assessment (gates, ground handlers, customs, fuelling)</t>
+        </is>
+      </c>
+      <c r="K272" s="18" t="inlineStr">
+        <is>
+          <t>Infrastructure gap identified ≥12 months before proposed launch date</t>
+        </is>
+      </c>
+      <c r="L272" s="18" t="inlineStr">
+        <is>
+          <t>Ground handler capacity data at outstations not centrally held; planner must contact handlers individually, adding 3–6 weeks to cycle</t>
+        </is>
+      </c>
+      <c r="M272" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N272" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="30" customHeight="1">
+      <c r="A273" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B273" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C273" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D273" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E273" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F273" s="16" t="inlineStr">
+        <is>
+          <t>Confirm operational feasibility of candidate routes</t>
+        </is>
+      </c>
+      <c r="G273" s="16" t="inlineStr">
+        <is>
+          <t>Senior Network Planner</t>
+        </is>
+      </c>
+      <c r="H273" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I273" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan, slot feasibility report, airport readiness assessment</t>
+        </is>
+      </c>
+      <c r="J273" s="16" t="inlineStr">
+        <is>
+          <t>Operationally feasible route set confirmed in SkyWORKS schedule editor</t>
+        </is>
+      </c>
+      <c r="K273" s="16" t="inlineStr">
+        <is>
+          <t>≥80% of shortlisted routes confirmed feasible without major constraint</t>
+        </is>
+      </c>
+      <c r="L273" s="16" t="inlineStr">
+        <is>
+          <t>Crew base restrictions and FAR Part 117 duty-time rules reduce feasible rotations, particularly for ultra-long-haul additions</t>
+        </is>
+      </c>
+      <c r="M273" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N273" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="30" customHeight="1">
+      <c r="A274" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B274" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C274" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D274" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E274" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F274" s="18" t="inlineStr">
+        <is>
+          <t>Build unit revenue &amp; yield forecast per candidate route</t>
+        </is>
+      </c>
+      <c r="G274" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H274" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I274" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed feasible route set, demand scenarios, competitive fare data from ATPCO</t>
+        </is>
+      </c>
+      <c r="J274" s="18" t="inlineStr">
+        <is>
+          <t>PRASM and RASM forecast per route across base/upside/downside scenarios</t>
+        </is>
+      </c>
+      <c r="K274" s="18" t="inlineStr">
+        <is>
+          <t>RASM forecast accuracy within ±8% of actuals on launched routes (tracked retrospectively)</t>
+        </is>
+      </c>
+      <c r="L274" s="18" t="inlineStr">
+        <is>
+          <t>NRM is calibrated on existing routes; forecast reliability for new O&amp;D markets with no booking history is low — often requires manual analyst override</t>
+        </is>
+      </c>
+      <c r="M274" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N274" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="30" customHeight="1">
+      <c r="A275" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B275" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C275" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D275" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E275" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F275" s="16" t="inlineStr">
+        <is>
+          <t>Model direct operating costs per route</t>
+        </is>
+      </c>
+      <c r="G275" s="16" t="inlineStr">
+        <is>
+          <t>Finance Business Partner — Network</t>
+        </is>
+      </c>
+      <c r="H275" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I275" s="16" t="inlineStr">
+        <is>
+          <t>Fleet assignment plan (aircraft type, block hours), fuel price assumptions, airport charges schedule</t>
+        </is>
+      </c>
+      <c r="J275" s="16" t="inlineStr">
+        <is>
+          <t>CASM breakdown per route (fuel, airport, crew, maintenance, overhead allocation)</t>
+        </is>
+      </c>
+      <c r="K275" s="16" t="inlineStr">
+        <is>
+          <t>CASM model completed within 10 business days of receiving fleet assignment input</t>
+        </is>
+      </c>
+      <c r="L275" s="16" t="inlineStr">
+        <is>
+          <t>Airport charge schedules for new markets are not always available in SAP master data; finance team must source bilaterally from airport authorities</t>
+        </is>
+      </c>
+      <c r="M275" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N275" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="276" ht="30" customHeight="1">
+      <c r="A276" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B276" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C276" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D276" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E276" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F276" s="18" t="inlineStr">
+        <is>
+          <t>Assess route contribution margin and breakeven load factor</t>
+        </is>
+      </c>
+      <c r="G276" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H276" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I276" s="18" t="inlineStr">
+        <is>
+          <t>RASM forecast, CASM breakdown, targeted load factor assumptions</t>
+        </is>
+      </c>
+      <c r="J276" s="18" t="inlineStr">
+        <is>
+          <t>Route P&amp;L summary with breakeven load factor and payback period</t>
+        </is>
+      </c>
+      <c r="K276" s="18" t="inlineStr">
+        <is>
+          <t>Target contribution margin ≥12% in Year 2; breakeven load factor ≤75%</t>
+        </is>
+      </c>
+      <c r="L276" s="18" t="inlineStr">
+        <is>
+          <t>Sensitivity of breakeven load factor to fuel price is high; +10% fuel swing shifts breakeven by 4–6 ppts, making many routes marginal</t>
+        </is>
+      </c>
+      <c r="M276" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N276" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="30" customHeight="1">
+      <c r="A277" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B277" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C277" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D277" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E277" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F277" s="16" t="inlineStr">
+        <is>
+          <t>Aggregate network business case for plan period</t>
+        </is>
+      </c>
+      <c r="G277" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H277" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I277" s="16" t="inlineStr">
+        <is>
+          <t>Individual route P&amp;L summaries, network-level synergy assumptions (feed, connectivity)</t>
+        </is>
+      </c>
+      <c r="J277" s="16" t="inlineStr">
+        <is>
+          <t>3-year network business case document (revenue, cost, EBIT impact)</t>
+        </is>
+      </c>
+      <c r="K277" s="16" t="inlineStr">
+        <is>
+          <t>Network EBIT uplift ≥$150M over plan period vs do-nothing baseline</t>
+        </is>
+      </c>
+      <c r="L277" s="16" t="inlineStr">
+        <is>
+          <t>Network synergy benefits (connecting traffic uplift) are difficult to isolate and often overstated in bottom-up aggregation</t>
+        </is>
+      </c>
+      <c r="M277" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N277" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="30" customHeight="1">
+      <c r="A278" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B278" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C278" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D278" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E278" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F278" s="18" t="inlineStr">
+        <is>
+          <t>Package strategic plan for governance review</t>
+        </is>
+      </c>
+      <c r="G278" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H278" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I278" s="18" t="inlineStr">
+        <is>
+          <t>Network business case, route scorecard, risk register</t>
+        </is>
+      </c>
+      <c r="J278" s="18" t="inlineStr">
+        <is>
+          <t>Executive briefing pack: network strategy summary, investment ask, risk matrix</t>
+        </is>
+      </c>
+      <c r="K278" s="18" t="inlineStr">
+        <is>
+          <t>Briefing pack issued ≥5 business days before Network Strategy Committee meeting</t>
+        </is>
+      </c>
+      <c r="L278" s="18" t="inlineStr">
+        <is>
+          <t>Version control of the briefing pack is manual; late assumption changes from Revenue Management or Finance require last-minute slides rebuild</t>
+        </is>
+      </c>
+      <c r="M278" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N278" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="30" customHeight="1">
+      <c r="A279" s="15" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B279" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C279" s="16" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D279" s="16" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E279" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F279" s="16" t="inlineStr">
+        <is>
+          <t>Present plan to Network Strategy Committee</t>
+        </is>
+      </c>
+      <c r="G279" s="16" t="inlineStr">
+        <is>
+          <t>VP Network Planning</t>
+        </is>
+      </c>
+      <c r="H279" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I279" s="16" t="inlineStr">
+        <is>
+          <t>Executive briefing pack, committee member pre-read questions</t>
+        </is>
+      </c>
+      <c r="J279" s="16" t="inlineStr">
+        <is>
+          <t>Committee decision: approved / approved with conditions / rejected with rationale</t>
+        </is>
+      </c>
+      <c r="K279" s="16" t="inlineStr">
+        <is>
+          <t>Committee decision reached in ≤2 review cycles (no more than 1 deferral per plan)</t>
+        </is>
+      </c>
+      <c r="L279" s="16" t="inlineStr">
+        <is>
+          <t>Committee quorum requires C-suite attendance; scheduling conflicts routinely delay decision by 2–4 weeks, compressing scheduling window</t>
+        </is>
+      </c>
+      <c r="M279" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N279" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="280" ht="30" customHeight="1">
+      <c r="A280" s="17" t="inlineStr">
+        <is>
+          <t>NP-SP-15</t>
+        </is>
+      </c>
+      <c r="B280" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C280" s="18" t="inlineStr">
+        <is>
+          <t>Schedule Planning</t>
+        </is>
+      </c>
+      <c r="D280" s="18" t="inlineStr">
+        <is>
+          <t>Strategic Network Planning</t>
+        </is>
+      </c>
+      <c r="E280" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F280" s="18" t="inlineStr">
+        <is>
+          <t>Publish approved strategic network plan &amp; handoff to scheduling</t>
+        </is>
+      </c>
+      <c r="G280" s="18" t="inlineStr">
+        <is>
+          <t>Network Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H280" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="I280" s="18" t="inlineStr">
+        <is>
+          <t>Approved committee decision, final route list with gauge and frequency targets</t>
+        </is>
+      </c>
+      <c r="J280" s="18" t="inlineStr">
+        <is>
+          <t>Published strategic network plan loaded into SkyWORKS as planning baseline for Schedule Planning team</t>
+        </is>
+      </c>
+      <c r="K280" s="18" t="inlineStr">
+        <is>
+          <t>Plan published in SkyWORKS ≤3 business days after committee approval</t>
+        </is>
+      </c>
+      <c r="L280" s="18" t="inlineStr">
+        <is>
+          <t>SkyWORKS baseline lock-in creates downstream rigidity; late executive changes after publication require formal change request and delay tactical planning</t>
+        </is>
+      </c>
+      <c r="M280" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N280" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NP-RM-01: Inventory & Yield Optimization — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -22,6 +22,7 @@
     <sheet name="NP-SP-13" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="NP-SP-14" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="NP-SP-15" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="NP-RM-01" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1218,13 +1219,21 @@
           <t>Inventory &amp; Yield Optimization</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr"/>
-      <c r="G18" s="8" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-01</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -13149,13 +13158,1429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-01 — Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Ingest booking &amp; flown data from PSS</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Daily booking transactions, flown coupon data, no-show records</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Cleansed booking data feed loaded into RM data warehouse</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness ≥ 99.5% of all PNRs reconciled within 2 hours of departure</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS coupon reconciliation latency can delay same-day close files by up to 4 hours, compressing the overnight optimisation window</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Enrich data with competitive fare &amp; schedule feeds</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Competitor published schedules, OAG fare feeds, MIDT booking data</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Competitive context dataset appended to demand input files</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Competitive fare parity check completed for 100% of O&amp;D pairs within planning horizon</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>MIDT data lags actuals by 3–5 days, reducing confidence in competitor load factor estimates for near-term departures</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Run O&amp;D demand forecast model</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Cleansed booking data, competitive context, seasonal index, special-event calendar</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast by booking class for 330-day horizon</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 15% at O&amp;D level for departures within 30 days</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST demand models trained on pre-2020 data underweight volatile post-COVID travel patterns; requires periodic manual seasonality overrides</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Validate forecast accuracy against holdout set</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast, 30-day actuals from previous cycle</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report; approved or rejected forecast</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 15%; rejection triggers reforecast within 4 hours</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Redshift query contention during peak batch windows can delay accuracy checks, pushing AU updates past the 02:00 optimisation deadline</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Define booking class hierarchy and nested buckets</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Configuration Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Approved fare class structure from Pricing team, ATPCO filed classes</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Booking class hierarchy configuration in NRM (Y, B, M, H, Q, K … buckets)</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>100% of ATPCO-filed fare classes mapped to NRM booking classes before schedule activation</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Misalignment between ATPCO fare basis codes and NRM class definitions causes availability mismatches in GDS displays, leading to revenue leakage</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Set authorization unit (AU) levels per fare class</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast, fare class hierarchy, historical sell-up curves</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Initial AU limits loaded per booking class per flight</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>AU initialisation completed for 100% of flights ≥ 90 days prior to departure</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Manual AU overrides by market analysts outside NRM create version conflicts; no audit trail for override rationale increases regulatory audit risk</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Validate fare class mappings against ATPCO filings</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Configuration Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>NRM booking class configuration, ATPCO fare tariff tables</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Validated or flagged class mapping; exceptions escalated to Pricing team</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Zero GDS availability mismatches attributable to class mapping errors post-activation</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO filing changes by competitors can trigger a same-day re-mapping requirement; NRM does not auto-ingest ATPCO tariff updates in real time</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Activate nested inventory controls in Altéa</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Validated AU levels from NRM</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Live nested availability published to Altéa and GDS channels</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Availability synchronisation latency Altéa → GDS ≤ 5 minutes</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Altéa availability propagation to Sabre and Travelport GDS can lag by up to 15 minutes during peak filing windows, creating booking class sell-out errors</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Run EMSRb / O&amp;D seat allocation optimisation</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>AU levels, demand forecast, fare values, seat capacity</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Optimised AU recommendations per booking class per flight leg</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue per available seat kilometre (RASK) improvement ≥ 2% vs baseline AU</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>NRM O&amp;D optimiser requires full network connectivity data; partial connectivity caused by codeshare partner IT gaps degrades optimisation quality</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Review and approve AU recommendations</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>NRM-generated AU recommendations, market performance dashboard</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Approved or manually overridden AU file</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Analyst review cycle ≤ 90 minutes per market cluster; override rate ≤ 20%</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>High override rates in thin O&amp;D markets indicate NRM model underfitting; manual overrides are not fed back into the model, perpetuating forecast error</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Apply approved AU updates to live inventory</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Approved AU file</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Updated live availability across all GDS and direct channels</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>AU update applied to 100% of affected flights within 30 minutes of approval</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Bulk AU update jobs during peak hours can queue behind other NRM batch processes, delaying availability changes for same-day and next-day departures</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Monitor booking pace against forecast curve</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Real-time booking data from Altéa, forecast pace curve</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Pace deviation alert for flights outside ±10% of forecast</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Analyst response to pace deviation alert ≤ 2 hours for departures within 14 days</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Tableau dashboards pull from AWS Redshift snapshots with 1-hour refresh lag; real-time anomalies for high-demand events (concerts, sports) are missed until the next refresh</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Apply sell-up action or open lower classes</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Pace deviation alert, current AU levels, fare class sell-up elasticity data</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Revised AUs triggering sell-up (close lower classes) or stimulation (open lower classes)</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Yield improvement ≥ 1.5% per sell-up intervention vs control flights</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Sell-up elasticity coefficients in NRM are recalibrated only quarterly; rapid fare environment changes (fuel surcharge adjustments) make coefficients stale within weeks</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Update bid prices for O&amp;D revenue integrity</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Real-time load factors, revised demand signals, network connection values</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Updated bid price vector published to Altéa for itinerary acceptance control</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Bid price refresh cycle ≤ 4 hours for flights within 7 days of departure</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Bid price vector updates are network-wide calculations; during irregular ops, displaced passengers and re-accommodation can invalidate bid prices across 30+ connected flights simultaneously</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Manage group booking displacement impact</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Groups &amp; Allotments Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request (≥10 pax), current individual seat availability</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Group AU block allocated or declined; displacement cost calculated</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Group displacement cost ≤ 8% of group revenue contribution on affected flights</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Altéa group allotment module does not integrate real-time NRM bid prices; group pricing decisions rely on analyst manual look-up, creating inconsistent displacement cost accounting</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Capture post-departure spill and spoilage actuals</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Flown manifest from Altéa, final booking class loads, denied boarding records</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Spill / spoilage report by flight and booking class</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Spill (denied boardings) ≤ 1.5% of passengers carried; spoilage (empty seats in high class) ≤ 3% of capacity</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Denied boarding data from airport check-in is not always tagged with the booking class of the displaced passenger, reducing spill attribution accuracy</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate forecast model performance and recalibrate</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Spill / spoilage report, forecast vs actual load factor comparison</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Updated SkyCAST model parameters; recalibration report</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Model recalibration completed within 5 business days of departure; MAPE improvement ≥ 1 pp per calibration cycle</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST model recalibration requires manual parameter uploads; there is no automated feedback loop from NRM actuals to SkyCAST, creating a 5–7 day lag in model learning</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Publish yield performance report to stakeholders</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>RASK actuals, load factor, yield, spill/spoilage KPIs from Redshift</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Weekly yield performance report distributed to VP Revenue Management and Network Planning</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Report published within 2 business days of week close; RASK vs budget variance explained for all markets &gt; ±3%</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Manual data assembly from Altéa, NRM, and Redshift for the weekly report takes 6–8 analyst hours; no single integrated reporting layer across PSS and RM systems</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N280"/>
+  <dimension ref="A1:N298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -33266,6 +34691,1302 @@
       <c r="N280" s="17" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="30" customHeight="1">
+      <c r="A281" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B281" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C281" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D281" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E281" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F281" s="16" t="inlineStr">
+        <is>
+          <t>Ingest booking &amp; flown data from PSS</t>
+        </is>
+      </c>
+      <c r="G281" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H281" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I281" s="16" t="inlineStr">
+        <is>
+          <t>Daily booking transactions, flown coupon data, no-show records</t>
+        </is>
+      </c>
+      <c r="J281" s="16" t="inlineStr">
+        <is>
+          <t>Cleansed booking data feed loaded into RM data warehouse</t>
+        </is>
+      </c>
+      <c r="K281" s="16" t="inlineStr">
+        <is>
+          <t>Data completeness ≥ 99.5% of all PNRs reconciled within 2 hours of departure</t>
+        </is>
+      </c>
+      <c r="L281" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS coupon reconciliation latency can delay same-day close files by up to 4 hours, compressing the overnight optimisation window</t>
+        </is>
+      </c>
+      <c r="M281" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N281" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="30" customHeight="1">
+      <c r="A282" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B282" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C282" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D282" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E282" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F282" s="18" t="inlineStr">
+        <is>
+          <t>Enrich data with competitive fare &amp; schedule feeds</t>
+        </is>
+      </c>
+      <c r="G282" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H282" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I282" s="18" t="inlineStr">
+        <is>
+          <t>Competitor published schedules, OAG fare feeds, MIDT booking data</t>
+        </is>
+      </c>
+      <c r="J282" s="18" t="inlineStr">
+        <is>
+          <t>Competitive context dataset appended to demand input files</t>
+        </is>
+      </c>
+      <c r="K282" s="18" t="inlineStr">
+        <is>
+          <t>Competitive fare parity check completed for 100% of O&amp;D pairs within planning horizon</t>
+        </is>
+      </c>
+      <c r="L282" s="18" t="inlineStr">
+        <is>
+          <t>MIDT data lags actuals by 3–5 days, reducing confidence in competitor load factor estimates for near-term departures</t>
+        </is>
+      </c>
+      <c r="M282" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N282" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="30" customHeight="1">
+      <c r="A283" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B283" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C283" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D283" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E283" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F283" s="16" t="inlineStr">
+        <is>
+          <t>Run O&amp;D demand forecast model</t>
+        </is>
+      </c>
+      <c r="G283" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H283" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I283" s="16" t="inlineStr">
+        <is>
+          <t>Cleansed booking data, competitive context, seasonal index, special-event calendar</t>
+        </is>
+      </c>
+      <c r="J283" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast by booking class for 330-day horizon</t>
+        </is>
+      </c>
+      <c r="K283" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 15% at O&amp;D level for departures within 30 days</t>
+        </is>
+      </c>
+      <c r="L283" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST demand models trained on pre-2020 data underweight volatile post-COVID travel patterns; requires periodic manual seasonality overrides</t>
+        </is>
+      </c>
+      <c r="M283" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N283" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="30" customHeight="1">
+      <c r="A284" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B284" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C284" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D284" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E284" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F284" s="18" t="inlineStr">
+        <is>
+          <t>Validate forecast accuracy against holdout set</t>
+        </is>
+      </c>
+      <c r="G284" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H284" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I284" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast, 30-day actuals from previous cycle</t>
+        </is>
+      </c>
+      <c r="J284" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report; approved or rejected forecast</t>
+        </is>
+      </c>
+      <c r="K284" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 15%; rejection triggers reforecast within 4 hours</t>
+        </is>
+      </c>
+      <c r="L284" s="18" t="inlineStr">
+        <is>
+          <t>Redshift query contention during peak batch windows can delay accuracy checks, pushing AU updates past the 02:00 optimisation deadline</t>
+        </is>
+      </c>
+      <c r="M284" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N284" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="30" customHeight="1">
+      <c r="A285" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B285" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C285" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D285" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E285" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F285" s="16" t="inlineStr">
+        <is>
+          <t>Define booking class hierarchy and nested buckets</t>
+        </is>
+      </c>
+      <c r="G285" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Configuration Analyst</t>
+        </is>
+      </c>
+      <c r="H285" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I285" s="16" t="inlineStr">
+        <is>
+          <t>Approved fare class structure from Pricing team, ATPCO filed classes</t>
+        </is>
+      </c>
+      <c r="J285" s="16" t="inlineStr">
+        <is>
+          <t>Booking class hierarchy configuration in NRM (Y, B, M, H, Q, K … buckets)</t>
+        </is>
+      </c>
+      <c r="K285" s="16" t="inlineStr">
+        <is>
+          <t>100% of ATPCO-filed fare classes mapped to NRM booking classes before schedule activation</t>
+        </is>
+      </c>
+      <c r="L285" s="16" t="inlineStr">
+        <is>
+          <t>Misalignment between ATPCO fare basis codes and NRM class definitions causes availability mismatches in GDS displays, leading to revenue leakage</t>
+        </is>
+      </c>
+      <c r="M285" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N285" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="30" customHeight="1">
+      <c r="A286" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B286" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C286" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D286" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E286" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F286" s="18" t="inlineStr">
+        <is>
+          <t>Set authorization unit (AU) levels per fare class</t>
+        </is>
+      </c>
+      <c r="G286" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H286" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I286" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecast, fare class hierarchy, historical sell-up curves</t>
+        </is>
+      </c>
+      <c r="J286" s="18" t="inlineStr">
+        <is>
+          <t>Initial AU limits loaded per booking class per flight</t>
+        </is>
+      </c>
+      <c r="K286" s="18" t="inlineStr">
+        <is>
+          <t>AU initialisation completed for 100% of flights ≥ 90 days prior to departure</t>
+        </is>
+      </c>
+      <c r="L286" s="18" t="inlineStr">
+        <is>
+          <t>Manual AU overrides by market analysts outside NRM create version conflicts; no audit trail for override rationale increases regulatory audit risk</t>
+        </is>
+      </c>
+      <c r="M286" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N286" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="30" customHeight="1">
+      <c r="A287" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B287" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C287" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D287" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E287" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F287" s="16" t="inlineStr">
+        <is>
+          <t>Validate fare class mappings against ATPCO filings</t>
+        </is>
+      </c>
+      <c r="G287" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Configuration Analyst</t>
+        </is>
+      </c>
+      <c r="H287" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I287" s="16" t="inlineStr">
+        <is>
+          <t>NRM booking class configuration, ATPCO fare tariff tables</t>
+        </is>
+      </c>
+      <c r="J287" s="16" t="inlineStr">
+        <is>
+          <t>Validated or flagged class mapping; exceptions escalated to Pricing team</t>
+        </is>
+      </c>
+      <c r="K287" s="16" t="inlineStr">
+        <is>
+          <t>Zero GDS availability mismatches attributable to class mapping errors post-activation</t>
+        </is>
+      </c>
+      <c r="L287" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO filing changes by competitors can trigger a same-day re-mapping requirement; NRM does not auto-ingest ATPCO tariff updates in real time</t>
+        </is>
+      </c>
+      <c r="M287" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N287" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="288" ht="30" customHeight="1">
+      <c r="A288" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B288" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C288" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D288" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E288" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F288" s="18" t="inlineStr">
+        <is>
+          <t>Activate nested inventory controls in Altéa</t>
+        </is>
+      </c>
+      <c r="G288" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H288" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I288" s="18" t="inlineStr">
+        <is>
+          <t>Validated AU levels from NRM</t>
+        </is>
+      </c>
+      <c r="J288" s="18" t="inlineStr">
+        <is>
+          <t>Live nested availability published to Altéa and GDS channels</t>
+        </is>
+      </c>
+      <c r="K288" s="18" t="inlineStr">
+        <is>
+          <t>Availability synchronisation latency Altéa → GDS ≤ 5 minutes</t>
+        </is>
+      </c>
+      <c r="L288" s="18" t="inlineStr">
+        <is>
+          <t>Altéa availability propagation to Sabre and Travelport GDS can lag by up to 15 minutes during peak filing windows, creating booking class sell-out errors</t>
+        </is>
+      </c>
+      <c r="M288" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N288" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="30" customHeight="1">
+      <c r="A289" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B289" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C289" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D289" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E289" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F289" s="16" t="inlineStr">
+        <is>
+          <t>Run EMSRb / O&amp;D seat allocation optimisation</t>
+        </is>
+      </c>
+      <c r="G289" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H289" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I289" s="16" t="inlineStr">
+        <is>
+          <t>AU levels, demand forecast, fare values, seat capacity</t>
+        </is>
+      </c>
+      <c r="J289" s="16" t="inlineStr">
+        <is>
+          <t>Optimised AU recommendations per booking class per flight leg</t>
+        </is>
+      </c>
+      <c r="K289" s="16" t="inlineStr">
+        <is>
+          <t>Revenue per available seat kilometre (RASK) improvement ≥ 2% vs baseline AU</t>
+        </is>
+      </c>
+      <c r="L289" s="16" t="inlineStr">
+        <is>
+          <t>NRM O&amp;D optimiser requires full network connectivity data; partial connectivity caused by codeshare partner IT gaps degrades optimisation quality</t>
+        </is>
+      </c>
+      <c r="M289" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N289" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="30" customHeight="1">
+      <c r="A290" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B290" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C290" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D290" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E290" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F290" s="18" t="inlineStr">
+        <is>
+          <t>Review and approve AU recommendations</t>
+        </is>
+      </c>
+      <c r="G290" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H290" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I290" s="18" t="inlineStr">
+        <is>
+          <t>NRM-generated AU recommendations, market performance dashboard</t>
+        </is>
+      </c>
+      <c r="J290" s="18" t="inlineStr">
+        <is>
+          <t>Approved or manually overridden AU file</t>
+        </is>
+      </c>
+      <c r="K290" s="18" t="inlineStr">
+        <is>
+          <t>Analyst review cycle ≤ 90 minutes per market cluster; override rate ≤ 20%</t>
+        </is>
+      </c>
+      <c r="L290" s="18" t="inlineStr">
+        <is>
+          <t>High override rates in thin O&amp;D markets indicate NRM model underfitting; manual overrides are not fed back into the model, perpetuating forecast error</t>
+        </is>
+      </c>
+      <c r="M290" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N290" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="30" customHeight="1">
+      <c r="A291" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B291" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C291" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D291" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E291" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F291" s="16" t="inlineStr">
+        <is>
+          <t>Apply approved AU updates to live inventory</t>
+        </is>
+      </c>
+      <c r="G291" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H291" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I291" s="16" t="inlineStr">
+        <is>
+          <t>Approved AU file</t>
+        </is>
+      </c>
+      <c r="J291" s="16" t="inlineStr">
+        <is>
+          <t>Updated live availability across all GDS and direct channels</t>
+        </is>
+      </c>
+      <c r="K291" s="16" t="inlineStr">
+        <is>
+          <t>AU update applied to 100% of affected flights within 30 minutes of approval</t>
+        </is>
+      </c>
+      <c r="L291" s="16" t="inlineStr">
+        <is>
+          <t>Bulk AU update jobs during peak hours can queue behind other NRM batch processes, delaying availability changes for same-day and next-day departures</t>
+        </is>
+      </c>
+      <c r="M291" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N291" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="30" customHeight="1">
+      <c r="A292" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B292" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C292" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D292" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E292" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F292" s="18" t="inlineStr">
+        <is>
+          <t>Monitor booking pace against forecast curve</t>
+        </is>
+      </c>
+      <c r="G292" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H292" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I292" s="18" t="inlineStr">
+        <is>
+          <t>Real-time booking data from Altéa, forecast pace curve</t>
+        </is>
+      </c>
+      <c r="J292" s="18" t="inlineStr">
+        <is>
+          <t>Pace deviation alert for flights outside ±10% of forecast</t>
+        </is>
+      </c>
+      <c r="K292" s="18" t="inlineStr">
+        <is>
+          <t>Analyst response to pace deviation alert ≤ 2 hours for departures within 14 days</t>
+        </is>
+      </c>
+      <c r="L292" s="18" t="inlineStr">
+        <is>
+          <t>Tableau dashboards pull from AWS Redshift snapshots with 1-hour refresh lag; real-time anomalies for high-demand events (concerts, sports) are missed until the next refresh</t>
+        </is>
+      </c>
+      <c r="M292" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N292" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="30" customHeight="1">
+      <c r="A293" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B293" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C293" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D293" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E293" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F293" s="16" t="inlineStr">
+        <is>
+          <t>Apply sell-up action or open lower classes</t>
+        </is>
+      </c>
+      <c r="G293" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H293" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I293" s="16" t="inlineStr">
+        <is>
+          <t>Pace deviation alert, current AU levels, fare class sell-up elasticity data</t>
+        </is>
+      </c>
+      <c r="J293" s="16" t="inlineStr">
+        <is>
+          <t>Revised AUs triggering sell-up (close lower classes) or stimulation (open lower classes)</t>
+        </is>
+      </c>
+      <c r="K293" s="16" t="inlineStr">
+        <is>
+          <t>Yield improvement ≥ 1.5% per sell-up intervention vs control flights</t>
+        </is>
+      </c>
+      <c r="L293" s="16" t="inlineStr">
+        <is>
+          <t>Sell-up elasticity coefficients in NRM are recalibrated only quarterly; rapid fare environment changes (fuel surcharge adjustments) make coefficients stale within weeks</t>
+        </is>
+      </c>
+      <c r="M293" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N293" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="30" customHeight="1">
+      <c r="A294" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B294" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C294" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D294" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E294" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F294" s="18" t="inlineStr">
+        <is>
+          <t>Update bid prices for O&amp;D revenue integrity</t>
+        </is>
+      </c>
+      <c r="G294" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H294" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I294" s="18" t="inlineStr">
+        <is>
+          <t>Real-time load factors, revised demand signals, network connection values</t>
+        </is>
+      </c>
+      <c r="J294" s="18" t="inlineStr">
+        <is>
+          <t>Updated bid price vector published to Altéa for itinerary acceptance control</t>
+        </is>
+      </c>
+      <c r="K294" s="18" t="inlineStr">
+        <is>
+          <t>Bid price refresh cycle ≤ 4 hours for flights within 7 days of departure</t>
+        </is>
+      </c>
+      <c r="L294" s="18" t="inlineStr">
+        <is>
+          <t>Bid price vector updates are network-wide calculations; during irregular ops, displaced passengers and re-accommodation can invalidate bid prices across 30+ connected flights simultaneously</t>
+        </is>
+      </c>
+      <c r="M294" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N294" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="30" customHeight="1">
+      <c r="A295" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B295" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C295" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D295" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E295" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F295" s="16" t="inlineStr">
+        <is>
+          <t>Manage group booking displacement impact</t>
+        </is>
+      </c>
+      <c r="G295" s="16" t="inlineStr">
+        <is>
+          <t>Groups &amp; Allotments Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H295" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I295" s="16" t="inlineStr">
+        <is>
+          <t>Group booking request (≥10 pax), current individual seat availability</t>
+        </is>
+      </c>
+      <c r="J295" s="16" t="inlineStr">
+        <is>
+          <t>Group AU block allocated or declined; displacement cost calculated</t>
+        </is>
+      </c>
+      <c r="K295" s="16" t="inlineStr">
+        <is>
+          <t>Group displacement cost ≤ 8% of group revenue contribution on affected flights</t>
+        </is>
+      </c>
+      <c r="L295" s="16" t="inlineStr">
+        <is>
+          <t>Altéa group allotment module does not integrate real-time NRM bid prices; group pricing decisions rely on analyst manual look-up, creating inconsistent displacement cost accounting</t>
+        </is>
+      </c>
+      <c r="M295" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N295" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="30" customHeight="1">
+      <c r="A296" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B296" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C296" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D296" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E296" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F296" s="18" t="inlineStr">
+        <is>
+          <t>Capture post-departure spill and spoilage actuals</t>
+        </is>
+      </c>
+      <c r="G296" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H296" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I296" s="18" t="inlineStr">
+        <is>
+          <t>Flown manifest from Altéa, final booking class loads, denied boarding records</t>
+        </is>
+      </c>
+      <c r="J296" s="18" t="inlineStr">
+        <is>
+          <t>Spill / spoilage report by flight and booking class</t>
+        </is>
+      </c>
+      <c r="K296" s="18" t="inlineStr">
+        <is>
+          <t>Spill (denied boardings) ≤ 1.5% of passengers carried; spoilage (empty seats in high class) ≤ 3% of capacity</t>
+        </is>
+      </c>
+      <c r="L296" s="18" t="inlineStr">
+        <is>
+          <t>Denied boarding data from airport check-in is not always tagged with the booking class of the displaced passenger, reducing spill attribution accuracy</t>
+        </is>
+      </c>
+      <c r="M296" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N296" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="30" customHeight="1">
+      <c r="A297" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B297" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C297" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D297" s="16" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E297" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F297" s="16" t="inlineStr">
+        <is>
+          <t>Evaluate forecast model performance and recalibrate</t>
+        </is>
+      </c>
+      <c r="G297" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H297" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I297" s="16" t="inlineStr">
+        <is>
+          <t>Spill / spoilage report, forecast vs actual load factor comparison</t>
+        </is>
+      </c>
+      <c r="J297" s="16" t="inlineStr">
+        <is>
+          <t>Updated SkyCAST model parameters; recalibration report</t>
+        </is>
+      </c>
+      <c r="K297" s="16" t="inlineStr">
+        <is>
+          <t>Model recalibration completed within 5 business days of departure; MAPE improvement ≥ 1 pp per calibration cycle</t>
+        </is>
+      </c>
+      <c r="L297" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST model recalibration requires manual parameter uploads; there is no automated feedback loop from NRM actuals to SkyCAST, creating a 5–7 day lag in model learning</t>
+        </is>
+      </c>
+      <c r="M297" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N297" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="30" customHeight="1">
+      <c r="A298" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-01</t>
+        </is>
+      </c>
+      <c r="B298" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C298" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D298" s="18" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Yield Optimization</t>
+        </is>
+      </c>
+      <c r="E298" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F298" s="18" t="inlineStr">
+        <is>
+          <t>Publish yield performance report to stakeholders</t>
+        </is>
+      </c>
+      <c r="G298" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H298" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I298" s="18" t="inlineStr">
+        <is>
+          <t>RASK actuals, load factor, yield, spill/spoilage KPIs from Redshift</t>
+        </is>
+      </c>
+      <c r="J298" s="18" t="inlineStr">
+        <is>
+          <t>Weekly yield performance report distributed to VP Revenue Management and Network Planning</t>
+        </is>
+      </c>
+      <c r="K298" s="18" t="inlineStr">
+        <is>
+          <t>Report published within 2 business days of week close; RASK vs budget variance explained for all markets &gt; ±3%</t>
+        </is>
+      </c>
+      <c r="L298" s="18" t="inlineStr">
+        <is>
+          <t>Manual data assembly from Altéa, NRM, and Redshift for the weekly report takes 6–8 analyst hours; no single integrated reporting layer across PSS and RM systems</t>
+        </is>
+      </c>
+      <c r="M298" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N298" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NP-RM-02: Fare Class & Bucket Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -23,6 +23,7 @@
     <sheet name="NP-SP-14" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="NP-SP-15" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="NP-RM-01" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="NP-RM-02" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1256,13 +1257,21 @@
           <t>Fare Class &amp; Bucket Management</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr"/>
-      <c r="G19" s="10" t="inlineStr"/>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-02</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -14574,13 +14583,1429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-02 — Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Define fare class hierarchy in PSS</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Fare product strategy brief, IATA booking class standards</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Booking class configuration (Y, B, M, H, K, Q, V, W, L, G) in PSS</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>100% of active fare products mapped to a booking class within 2 business days of product launch</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa booking class table has finite slots; adding new classes for ancillary bundles requires PSS configuration freeze that blocks concurrent distribution updates</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Map booking classes to RM fare buckets</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Booking class list from Altéa, revenue segmentation guidelines</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Fare bucket mapping table in NRM linking each booking class to O&amp;D revenue tier</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Zero mismatches between Altéa booking class codes and NRM bucket definitions at go-live</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>NRM fare bucket schema uses internal numeric IDs that do not auto-sync with Altéa booking class labels; manual reconciliation required after each PSS config change</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate fare class structure against ATPCO rules</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Tariff Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>NRM bucket mapping, published ATPCO fare records (Records 1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Validation report confirming booking class eligibility rules match ATPCO Cat 25 combinability and Cat 5 advance purchase restrictions</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>0 ATPCO rule violations flagged by GDS edits at filing; audit pass rate 100%</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO Cat 25 combinability rules interact with NRM bucket nesting in non-obvious ways; misalignment causes ghost inventory — classes show available in GDS but are blocked in NRM</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Publish fare class availability to GDS channels</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated booking class configuration, SSIM schedule file</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Live availability display in Sabre, Travelport, and Amadeus GDS for all market O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>GDS availability refresh latency ≤ 90 seconds from NRM availability change; GDS parity rate ≥ 99.5%</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS availability cache TTL (up to 90 s) creates window where high-demand bucket closures are not yet reflected, enabling over-sell of discount classes during flash sales</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Extract historical O&amp;D booking data by fare class</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Altéa booking history (24 months), departure date range for planning horizon</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D booking curve dataset segmented by fare class, day-of-week, and booking lead time</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction covering ≥ 95% of historical departures within planning window; query SLA ≤ 4 hours</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Post-COVID booking patterns (2021–2022) distort historical curves; including them without seasonality dampening causes demand models to under-forecast leisure peak</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Run demand forecast model per O&amp;D bucket</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Historical booking curves, competitive fare inputs from OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Forecast demand curve per fare bucket per O&amp;D, including unconstrained demand estimate</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MASE (Mean Absolute Scaled Error) ≤ 0.25 for 90-day horizon; unconstrained demand estimate within ±12% of actuals at departure</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>NRM's detruncation algorithm underestimates unconstrained demand on routes with chronic sell-outs; results in systematic under-forecasting for high-yield buckets</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Review forecast variance and approve bucket plan</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>NRM forecast output, analyst commentary on anomalous markets</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Approved demand forecast for bucket sizing; markets flagged for manual review escalated</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Forecast review cycle ≤ 48 hours before system-generated availability updates are applied; &lt; 5% of markets requiring manual correction</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>High analyst workload during peak schedule planning cycles forces rubber-stamping of model outputs; errors not caught until post-departure revenue review</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Set initial bucket inventory levels for departure</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Approved demand forecast, aircraft capacity from Amadeus SkyMAX fleet assignment</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Initial bucket protection levels and booking limits per fare class per flight</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Bucket initialisation completed ≥ 330 days before departure for all long-haul markets; ≥ 90 days for short-haul</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>SkyMAX fleet assignment changes propagate to NRM with up to 6-hour lag; bucket limits set against wrong aircraft type cause premature close-out of discount classes</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Configure EMSR-b bid price and nesting strategy</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Approved bucket protection levels, fare class revenue values, willingness-to-pay estimates</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Bid price thresholds and virtual bucket nesting hierarchy loaded into NRM for each O&amp;D</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Bid price calibration complete ≥ 180 days before departure for long-haul; revenue uplift from nesting vs. partitioned control ≥ 2% RASM on calibrated markets</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>NRM's EMSR-b calculation does not natively account for ancillary revenue (bag fees, seat upgrades) in WTP estimates; bid prices structurally undervalue leisure segments</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Monitor booking pace against expected S-curve</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Real-time bookings from Altéa, expected booking curve from NRM forecast</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace index (BPI) per flight per fare class; pace alerts for flights deviating &gt; 20%</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>BPI monitored at T−90, T−60, T−30, T−14, T−7, T−3 checkpoints; alert resolution SLA ≤ 4 hours</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>NRM booking pace alerts have a minimum 15-minute polling interval; during flash sales or news events, early-warning signals arrive too late to prevent discount class oversell</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Adjust bucket thresholds based on pace deviation</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace alert, current bucket availability, revised demand estimate</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Updated protection levels and booking limits; change log entry in NRM audit trail</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Bucket adjustment applied within 2 hours of pace alert; average revenue recovery per adjustment ≥ $8/seat on affected flights</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Frequent intraday bucket adjustments on the same flight trigger NRM re-optimisation queue delays; changes queue behind batch jobs and may not take effect for up to 30 minutes</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Open or close fare classes per booking curve triggers</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>NRM availability recommendation, time-to-departure trigger rules</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Updated fare class availability in Altéa and reflected across GDS/NDC channels</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Availability update propagated to all GDS endpoints within 90 seconds; close-out of discount classes ≥ T−3 on flights with load factor forecast ≥ 90%</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway availability sync with Altéa runs on a separate thread from GDS availability; NDC channel may display open discount inventory up to 3 minutes after GDS close-out</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Monitor real-time bookings and cancellations by class</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Live Altéa booking stream, cancellation and refund events</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Real-time seat availability dashboard; auto-triggered re-open events when cancellations create sell-up opportunity</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue recovery from cancellation-triggered re-opens ≥ $15/seat; dashboard refresh ≤ 5-minute lag vs. Altéa booking engine</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>High-volume cancellation events (weather, IROPS) flood NRM with availability change events; system enters degraded mode and availability updates queue, causing stale GDS displays</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Process group booking requests against bucket availability</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Group booking request (≥10 pax), current bucket availability, group fare contract</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Group PNR with blocked inventory or counter-offer at higher fare class</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Group booking response time ≤ 24 hours; group revenue contribution ≥ 8% of total flight revenue on managed markets</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Altéa group booking module holds seats as option status for up to 72 hours; large group holds on high-demand flights suppress availability for individual high-yield bookings, eroding RASM</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Review exception queue for manual intervention flights</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>NRM exception queue (special events, comp schedule changes, distressed inventory flags)</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised list of flights requiring analyst action; override justification form initiated</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Exception queue reviewed twice daily (09:00 and 14:00 local); &lt; 3% of managed flights in exception state at any time</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>NRM exception queue intermingles flights flagged by automated rules with analyst-generated annotations; high-priority items can be buried under system noise during IROPS events</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Apply manual bucket override with audit justification</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Approved override justification, competitor fare filing from OAG Schedule Analyser, event calendar</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Manual availability override applied; audit log entry with approver, rationale, and expected revenue impact</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>100% of manual overrides documented in NRM audit trail; post-event review shows manual overrides outperform model recommendation in ≥ 60% of cases</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>NRM audit trail does not capture the external data (event calendars, competitor filings) that justified the override; institutional knowledge lost when analysts turn over</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Generate post-departure revenue performance report</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Analytics Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Altéa final booking close-out file, NRM forecast at departure, actual revenue by fare class</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Post-departure report: RASM, load factor, yield, and spill/spoilage by bucket for each departed flight</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Report generated within 48 hours of departure; RASM variance between actual and pre-departure NRM estimate reported for 100% of flights</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Altéa close-out files arrive in S3 in variable formats depending on PSS version; ETL pipeline requires manual intervention approximately 3% of the time due to schema drift</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Recalibrate NRM forecast model parameters</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Post-departure performance reports (rolling 13 weeks), MASE trend, spill and spoilage analysis</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Updated NRM model parameters; recalibration change log; improvement targets set for next review cycle</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Quarterly recalibration reduces MASE by ≥ 0.02 vs. prior quarter; spill rate ≤ 3% and spoilage rate ≤ 5% on managed O&amp;Ds post-calibration</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>NRM model recalibration requires a 72-hour training window during which live availability recommendations revert to static rules; scheduling this window without impacting peak sale periods is operationally difficult</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N298"/>
+  <dimension ref="A1:N316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -35985,6 +37410,1302 @@
         </is>
       </c>
       <c r="N298" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="30" customHeight="1">
+      <c r="A299" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B299" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C299" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D299" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E299" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F299" s="16" t="inlineStr">
+        <is>
+          <t>Define fare class hierarchy in PSS</t>
+        </is>
+      </c>
+      <c r="G299" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H299" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I299" s="16" t="inlineStr">
+        <is>
+          <t>Fare product strategy brief, IATA booking class standards</t>
+        </is>
+      </c>
+      <c r="J299" s="16" t="inlineStr">
+        <is>
+          <t>Booking class configuration (Y, B, M, H, K, Q, V, W, L, G) in PSS</t>
+        </is>
+      </c>
+      <c r="K299" s="16" t="inlineStr">
+        <is>
+          <t>100% of active fare products mapped to a booking class within 2 business days of product launch</t>
+        </is>
+      </c>
+      <c r="L299" s="16" t="inlineStr">
+        <is>
+          <t>Altéa booking class table has finite slots; adding new classes for ancillary bundles requires PSS configuration freeze that blocks concurrent distribution updates</t>
+        </is>
+      </c>
+      <c r="M299" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N299" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="30" customHeight="1">
+      <c r="A300" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B300" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C300" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D300" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E300" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F300" s="18" t="inlineStr">
+        <is>
+          <t>Map booking classes to RM fare buckets</t>
+        </is>
+      </c>
+      <c r="G300" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H300" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I300" s="18" t="inlineStr">
+        <is>
+          <t>Booking class list from Altéa, revenue segmentation guidelines</t>
+        </is>
+      </c>
+      <c r="J300" s="18" t="inlineStr">
+        <is>
+          <t>Fare bucket mapping table in NRM linking each booking class to O&amp;D revenue tier</t>
+        </is>
+      </c>
+      <c r="K300" s="18" t="inlineStr">
+        <is>
+          <t>Zero mismatches between Altéa booking class codes and NRM bucket definitions at go-live</t>
+        </is>
+      </c>
+      <c r="L300" s="18" t="inlineStr">
+        <is>
+          <t>NRM fare bucket schema uses internal numeric IDs that do not auto-sync with Altéa booking class labels; manual reconciliation required after each PSS config change</t>
+        </is>
+      </c>
+      <c r="M300" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N300" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="30" customHeight="1">
+      <c r="A301" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B301" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C301" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D301" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E301" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F301" s="16" t="inlineStr">
+        <is>
+          <t>Validate fare class structure against ATPCO rules</t>
+        </is>
+      </c>
+      <c r="G301" s="16" t="inlineStr">
+        <is>
+          <t>Pricing &amp; Tariff Analyst</t>
+        </is>
+      </c>
+      <c r="H301" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I301" s="16" t="inlineStr">
+        <is>
+          <t>NRM bucket mapping, published ATPCO fare records (Records 1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="J301" s="16" t="inlineStr">
+        <is>
+          <t>Validation report confirming booking class eligibility rules match ATPCO Cat 25 combinability and Cat 5 advance purchase restrictions</t>
+        </is>
+      </c>
+      <c r="K301" s="16" t="inlineStr">
+        <is>
+          <t>0 ATPCO rule violations flagged by GDS edits at filing; audit pass rate 100%</t>
+        </is>
+      </c>
+      <c r="L301" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO Cat 25 combinability rules interact with NRM bucket nesting in non-obvious ways; misalignment causes ghost inventory — classes show available in GDS but are blocked in NRM</t>
+        </is>
+      </c>
+      <c r="M301" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N301" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="30" customHeight="1">
+      <c r="A302" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B302" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C302" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D302" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E302" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F302" s="18" t="inlineStr">
+        <is>
+          <t>Publish fare class availability to GDS channels</t>
+        </is>
+      </c>
+      <c r="G302" s="18" t="inlineStr">
+        <is>
+          <t>Distribution &amp; GDS Analyst</t>
+        </is>
+      </c>
+      <c r="H302" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I302" s="18" t="inlineStr">
+        <is>
+          <t>Validated booking class configuration, SSIM schedule file</t>
+        </is>
+      </c>
+      <c r="J302" s="18" t="inlineStr">
+        <is>
+          <t>Live availability display in Sabre, Travelport, and Amadeus GDS for all market O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="K302" s="18" t="inlineStr">
+        <is>
+          <t>GDS availability refresh latency ≤ 90 seconds from NRM availability change; GDS parity rate ≥ 99.5%</t>
+        </is>
+      </c>
+      <c r="L302" s="18" t="inlineStr">
+        <is>
+          <t>Sabre GDS availability cache TTL (up to 90 s) creates window where high-demand bucket closures are not yet reflected, enabling over-sell of discount classes during flash sales</t>
+        </is>
+      </c>
+      <c r="M302" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N302" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="30" customHeight="1">
+      <c r="A303" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B303" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C303" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D303" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E303" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F303" s="16" t="inlineStr">
+        <is>
+          <t>Extract historical O&amp;D booking data by fare class</t>
+        </is>
+      </c>
+      <c r="G303" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H303" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I303" s="16" t="inlineStr">
+        <is>
+          <t>Altéa booking history (24 months), departure date range for planning horizon</t>
+        </is>
+      </c>
+      <c r="J303" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D booking curve dataset segmented by fare class, day-of-week, and booking lead time</t>
+        </is>
+      </c>
+      <c r="K303" s="16" t="inlineStr">
+        <is>
+          <t>Data extraction covering ≥ 95% of historical departures within planning window; query SLA ≤ 4 hours</t>
+        </is>
+      </c>
+      <c r="L303" s="16" t="inlineStr">
+        <is>
+          <t>Post-COVID booking patterns (2021–2022) distort historical curves; including them without seasonality dampening causes demand models to under-forecast leisure peak</t>
+        </is>
+      </c>
+      <c r="M303" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N303" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="30" customHeight="1">
+      <c r="A304" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B304" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C304" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D304" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E304" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F304" s="18" t="inlineStr">
+        <is>
+          <t>Run demand forecast model per O&amp;D bucket</t>
+        </is>
+      </c>
+      <c r="G304" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H304" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I304" s="18" t="inlineStr">
+        <is>
+          <t>Historical booking curves, competitive fare inputs from OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="J304" s="18" t="inlineStr">
+        <is>
+          <t>Forecast demand curve per fare bucket per O&amp;D, including unconstrained demand estimate</t>
+        </is>
+      </c>
+      <c r="K304" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MASE (Mean Absolute Scaled Error) ≤ 0.25 for 90-day horizon; unconstrained demand estimate within ±12% of actuals at departure</t>
+        </is>
+      </c>
+      <c r="L304" s="18" t="inlineStr">
+        <is>
+          <t>NRM's detruncation algorithm underestimates unconstrained demand on routes with chronic sell-outs; results in systematic under-forecasting for high-yield buckets</t>
+        </is>
+      </c>
+      <c r="M304" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N304" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="30" customHeight="1">
+      <c r="A305" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B305" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C305" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D305" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E305" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F305" s="16" t="inlineStr">
+        <is>
+          <t>Review forecast variance and approve bucket plan</t>
+        </is>
+      </c>
+      <c r="G305" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H305" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I305" s="16" t="inlineStr">
+        <is>
+          <t>NRM forecast output, analyst commentary on anomalous markets</t>
+        </is>
+      </c>
+      <c r="J305" s="16" t="inlineStr">
+        <is>
+          <t>Approved demand forecast for bucket sizing; markets flagged for manual review escalated</t>
+        </is>
+      </c>
+      <c r="K305" s="16" t="inlineStr">
+        <is>
+          <t>Forecast review cycle ≤ 48 hours before system-generated availability updates are applied; &lt; 5% of markets requiring manual correction</t>
+        </is>
+      </c>
+      <c r="L305" s="16" t="inlineStr">
+        <is>
+          <t>High analyst workload during peak schedule planning cycles forces rubber-stamping of model outputs; errors not caught until post-departure revenue review</t>
+        </is>
+      </c>
+      <c r="M305" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N305" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="30" customHeight="1">
+      <c r="A306" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B306" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C306" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D306" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E306" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F306" s="18" t="inlineStr">
+        <is>
+          <t>Set initial bucket inventory levels for departure</t>
+        </is>
+      </c>
+      <c r="G306" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H306" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I306" s="18" t="inlineStr">
+        <is>
+          <t>Approved demand forecast, aircraft capacity from Amadeus SkyMAX fleet assignment</t>
+        </is>
+      </c>
+      <c r="J306" s="18" t="inlineStr">
+        <is>
+          <t>Initial bucket protection levels and booking limits per fare class per flight</t>
+        </is>
+      </c>
+      <c r="K306" s="18" t="inlineStr">
+        <is>
+          <t>Bucket initialisation completed ≥ 330 days before departure for all long-haul markets; ≥ 90 days for short-haul</t>
+        </is>
+      </c>
+      <c r="L306" s="18" t="inlineStr">
+        <is>
+          <t>SkyMAX fleet assignment changes propagate to NRM with up to 6-hour lag; bucket limits set against wrong aircraft type cause premature close-out of discount classes</t>
+        </is>
+      </c>
+      <c r="M306" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N306" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="30" customHeight="1">
+      <c r="A307" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B307" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C307" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D307" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E307" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F307" s="16" t="inlineStr">
+        <is>
+          <t>Configure EMSR-b bid price and nesting strategy</t>
+        </is>
+      </c>
+      <c r="G307" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H307" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I307" s="16" t="inlineStr">
+        <is>
+          <t>Approved bucket protection levels, fare class revenue values, willingness-to-pay estimates</t>
+        </is>
+      </c>
+      <c r="J307" s="16" t="inlineStr">
+        <is>
+          <t>Bid price thresholds and virtual bucket nesting hierarchy loaded into NRM for each O&amp;D</t>
+        </is>
+      </c>
+      <c r="K307" s="16" t="inlineStr">
+        <is>
+          <t>Bid price calibration complete ≥ 180 days before departure for long-haul; revenue uplift from nesting vs. partitioned control ≥ 2% RASM on calibrated markets</t>
+        </is>
+      </c>
+      <c r="L307" s="16" t="inlineStr">
+        <is>
+          <t>NRM's EMSR-b calculation does not natively account for ancillary revenue (bag fees, seat upgrades) in WTP estimates; bid prices structurally undervalue leisure segments</t>
+        </is>
+      </c>
+      <c r="M307" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N307" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="30" customHeight="1">
+      <c r="A308" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B308" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C308" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D308" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E308" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F308" s="18" t="inlineStr">
+        <is>
+          <t>Monitor booking pace against expected S-curve</t>
+        </is>
+      </c>
+      <c r="G308" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H308" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I308" s="18" t="inlineStr">
+        <is>
+          <t>Real-time bookings from Altéa, expected booking curve from NRM forecast</t>
+        </is>
+      </c>
+      <c r="J308" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace index (BPI) per flight per fare class; pace alerts for flights deviating &gt; 20%</t>
+        </is>
+      </c>
+      <c r="K308" s="18" t="inlineStr">
+        <is>
+          <t>BPI monitored at T−90, T−60, T−30, T−14, T−7, T−3 checkpoints; alert resolution SLA ≤ 4 hours</t>
+        </is>
+      </c>
+      <c r="L308" s="18" t="inlineStr">
+        <is>
+          <t>NRM booking pace alerts have a minimum 15-minute polling interval; during flash sales or news events, early-warning signals arrive too late to prevent discount class oversell</t>
+        </is>
+      </c>
+      <c r="M308" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N308" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="30" customHeight="1">
+      <c r="A309" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B309" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C309" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D309" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E309" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F309" s="16" t="inlineStr">
+        <is>
+          <t>Adjust bucket thresholds based on pace deviation</t>
+        </is>
+      </c>
+      <c r="G309" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H309" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I309" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace alert, current bucket availability, revised demand estimate</t>
+        </is>
+      </c>
+      <c r="J309" s="16" t="inlineStr">
+        <is>
+          <t>Updated protection levels and booking limits; change log entry in NRM audit trail</t>
+        </is>
+      </c>
+      <c r="K309" s="16" t="inlineStr">
+        <is>
+          <t>Bucket adjustment applied within 2 hours of pace alert; average revenue recovery per adjustment ≥ $8/seat on affected flights</t>
+        </is>
+      </c>
+      <c r="L309" s="16" t="inlineStr">
+        <is>
+          <t>Frequent intraday bucket adjustments on the same flight trigger NRM re-optimisation queue delays; changes queue behind batch jobs and may not take effect for up to 30 minutes</t>
+        </is>
+      </c>
+      <c r="M309" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N309" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="30" customHeight="1">
+      <c r="A310" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B310" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C310" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D310" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E310" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F310" s="18" t="inlineStr">
+        <is>
+          <t>Open or close fare classes per booking curve triggers</t>
+        </is>
+      </c>
+      <c r="G310" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H310" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I310" s="18" t="inlineStr">
+        <is>
+          <t>NRM availability recommendation, time-to-departure trigger rules</t>
+        </is>
+      </c>
+      <c r="J310" s="18" t="inlineStr">
+        <is>
+          <t>Updated fare class availability in Altéa and reflected across GDS/NDC channels</t>
+        </is>
+      </c>
+      <c r="K310" s="18" t="inlineStr">
+        <is>
+          <t>Availability update propagated to all GDS endpoints within 90 seconds; close-out of discount classes ≥ T−3 on flights with load factor forecast ≥ 90%</t>
+        </is>
+      </c>
+      <c r="L310" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway availability sync with Altéa runs on a separate thread from GDS availability; NDC channel may display open discount inventory up to 3 minutes after GDS close-out</t>
+        </is>
+      </c>
+      <c r="M310" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N310" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="30" customHeight="1">
+      <c r="A311" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B311" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C311" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D311" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E311" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F311" s="16" t="inlineStr">
+        <is>
+          <t>Monitor real-time bookings and cancellations by class</t>
+        </is>
+      </c>
+      <c r="G311" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H311" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I311" s="16" t="inlineStr">
+        <is>
+          <t>Live Altéa booking stream, cancellation and refund events</t>
+        </is>
+      </c>
+      <c r="J311" s="16" t="inlineStr">
+        <is>
+          <t>Real-time seat availability dashboard; auto-triggered re-open events when cancellations create sell-up opportunity</t>
+        </is>
+      </c>
+      <c r="K311" s="16" t="inlineStr">
+        <is>
+          <t>Revenue recovery from cancellation-triggered re-opens ≥ $15/seat; dashboard refresh ≤ 5-minute lag vs. Altéa booking engine</t>
+        </is>
+      </c>
+      <c r="L311" s="16" t="inlineStr">
+        <is>
+          <t>High-volume cancellation events (weather, IROPS) flood NRM with availability change events; system enters degraded mode and availability updates queue, causing stale GDS displays</t>
+        </is>
+      </c>
+      <c r="M311" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N311" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="30" customHeight="1">
+      <c r="A312" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B312" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C312" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D312" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E312" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F312" s="18" t="inlineStr">
+        <is>
+          <t>Process group booking requests against bucket availability</t>
+        </is>
+      </c>
+      <c r="G312" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H312" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I312" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request (≥10 pax), current bucket availability, group fare contract</t>
+        </is>
+      </c>
+      <c r="J312" s="18" t="inlineStr">
+        <is>
+          <t>Group PNR with blocked inventory or counter-offer at higher fare class</t>
+        </is>
+      </c>
+      <c r="K312" s="18" t="inlineStr">
+        <is>
+          <t>Group booking response time ≤ 24 hours; group revenue contribution ≥ 8% of total flight revenue on managed markets</t>
+        </is>
+      </c>
+      <c r="L312" s="18" t="inlineStr">
+        <is>
+          <t>Altéa group booking module holds seats as option status for up to 72 hours; large group holds on high-demand flights suppress availability for individual high-yield bookings, eroding RASM</t>
+        </is>
+      </c>
+      <c r="M312" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N312" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="30" customHeight="1">
+      <c r="A313" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B313" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C313" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D313" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E313" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F313" s="16" t="inlineStr">
+        <is>
+          <t>Review exception queue for manual intervention flights</t>
+        </is>
+      </c>
+      <c r="G313" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H313" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I313" s="16" t="inlineStr">
+        <is>
+          <t>NRM exception queue (special events, comp schedule changes, distressed inventory flags)</t>
+        </is>
+      </c>
+      <c r="J313" s="16" t="inlineStr">
+        <is>
+          <t>Prioritised list of flights requiring analyst action; override justification form initiated</t>
+        </is>
+      </c>
+      <c r="K313" s="16" t="inlineStr">
+        <is>
+          <t>Exception queue reviewed twice daily (09:00 and 14:00 local); &lt; 3% of managed flights in exception state at any time</t>
+        </is>
+      </c>
+      <c r="L313" s="16" t="inlineStr">
+        <is>
+          <t>NRM exception queue intermingles flights flagged by automated rules with analyst-generated annotations; high-priority items can be buried under system noise during IROPS events</t>
+        </is>
+      </c>
+      <c r="M313" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N313" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="30" customHeight="1">
+      <c r="A314" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B314" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C314" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D314" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E314" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F314" s="18" t="inlineStr">
+        <is>
+          <t>Apply manual bucket override with audit justification</t>
+        </is>
+      </c>
+      <c r="G314" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H314" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I314" s="18" t="inlineStr">
+        <is>
+          <t>Approved override justification, competitor fare filing from OAG Schedule Analyser, event calendar</t>
+        </is>
+      </c>
+      <c r="J314" s="18" t="inlineStr">
+        <is>
+          <t>Manual availability override applied; audit log entry with approver, rationale, and expected revenue impact</t>
+        </is>
+      </c>
+      <c r="K314" s="18" t="inlineStr">
+        <is>
+          <t>100% of manual overrides documented in NRM audit trail; post-event review shows manual overrides outperform model recommendation in ≥ 60% of cases</t>
+        </is>
+      </c>
+      <c r="L314" s="18" t="inlineStr">
+        <is>
+          <t>NRM audit trail does not capture the external data (event calendars, competitor filings) that justified the override; institutional knowledge lost when analysts turn over</t>
+        </is>
+      </c>
+      <c r="M314" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N314" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="30" customHeight="1">
+      <c r="A315" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B315" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C315" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D315" s="16" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E315" s="15" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F315" s="16" t="inlineStr">
+        <is>
+          <t>Generate post-departure revenue performance report</t>
+        </is>
+      </c>
+      <c r="G315" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Analytics Analyst</t>
+        </is>
+      </c>
+      <c r="H315" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I315" s="16" t="inlineStr">
+        <is>
+          <t>Altéa final booking close-out file, NRM forecast at departure, actual revenue by fare class</t>
+        </is>
+      </c>
+      <c r="J315" s="16" t="inlineStr">
+        <is>
+          <t>Post-departure report: RASM, load factor, yield, and spill/spoilage by bucket for each departed flight</t>
+        </is>
+      </c>
+      <c r="K315" s="16" t="inlineStr">
+        <is>
+          <t>Report generated within 48 hours of departure; RASM variance between actual and pre-departure NRM estimate reported for 100% of flights</t>
+        </is>
+      </c>
+      <c r="L315" s="16" t="inlineStr">
+        <is>
+          <t>Altéa close-out files arrive in S3 in variable formats depending on PSS version; ETL pipeline requires manual intervention approximately 3% of the time due to schema drift</t>
+        </is>
+      </c>
+      <c r="M315" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N315" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="30" customHeight="1">
+      <c r="A316" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-02</t>
+        </is>
+      </c>
+      <c r="B316" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C316" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D316" s="18" t="inlineStr">
+        <is>
+          <t>Fare Class &amp; Bucket Management</t>
+        </is>
+      </c>
+      <c r="E316" s="17" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F316" s="18" t="inlineStr">
+        <is>
+          <t>Recalibrate NRM forecast model parameters</t>
+        </is>
+      </c>
+      <c r="G316" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System Analyst</t>
+        </is>
+      </c>
+      <c r="H316" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I316" s="18" t="inlineStr">
+        <is>
+          <t>Post-departure performance reports (rolling 13 weeks), MASE trend, spill and spoilage analysis</t>
+        </is>
+      </c>
+      <c r="J316" s="18" t="inlineStr">
+        <is>
+          <t>Updated NRM model parameters; recalibration change log; improvement targets set for next review cycle</t>
+        </is>
+      </c>
+      <c r="K316" s="18" t="inlineStr">
+        <is>
+          <t>Quarterly recalibration reduces MASE by ≥ 0.02 vs. prior quarter; spill rate ≤ 3% and spoilage rate ≤ 5% on managed O&amp;Ds post-calibration</t>
+        </is>
+      </c>
+      <c r="L316" s="18" t="inlineStr">
+        <is>
+          <t>NRM model recalibration requires a 72-hour training window during which live availability recommendations revert to static rules; scheduling this window without impacting peak sale periods is operationally difficult</t>
+        </is>
+      </c>
+      <c r="M316" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N316" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-RM-03: Overbooking Policy Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -24,6 +24,7 @@
     <sheet name="NP-SP-15" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="NP-RM-01" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="NP-RM-02" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="NP-RM-03" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1294,13 +1295,21 @@
           <t>Overbooking Policy Management</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr"/>
-      <c r="G20" s="8" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-03</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -15999,13 +16008,1429 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-03 — Overbooking Policy Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Overbooking Policy Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract booking &amp; no-show history from PSS</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Departed flight records, booking logs, check-in data — rolling 24 months</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Raw no-show and cancellation dataset by flight, fare class, and booking channel</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Dataset completeness ≥99% of departed flights</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS history exports require manual scheduling; ad-hoc pulls risk data truncation beyond 13-month rolling window</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Segment data by route, DOW, fare class, season</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Raw no-show dataset from Altéa PSS export</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Segmented no-show rate matrix with confidence intervals per cluster</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Minimum 90 observed flights per segment for statistical significance</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Thin markets (&lt;5 flights/week) produce unreliable segment-level no-show rates; pooled estimates inflate overbooking risk</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Run no-show forecast model and validate accuracy</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>RM Data Scientist</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Segmented no-show matrix, demand forecasts from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>No-show show-up curve per flight cluster; model accuracy report</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Forecast vs. actual no-show rate MAPE ≤5%</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>NRM show-up model requires retraining after major schedule restructures; post-COVID demand patterns invalidated legacy curves for 18+ months</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Calibrate show-up curve by fare class and lead time</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>RM Data Scientist</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated no-show forecast model; approved show-up curves</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Calibrated show-up probability curves published to AltéaRM overbooking module</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Show-up curve refresh cycle ≤30 days for high-frequency routes; ≤90 days for seasonal routes</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Fare class proliferation (Basic Economy vs. flexible fares) requires separate show-up curves; legacy model treats all economy as one class</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Generate recommended OB factors by flight segment</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Calibrated show-up curves; target load factor ≥83%; denied boarding cost assumptions</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Recommended overbooking factor per flight segment with expected IDB rate</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Expected IDB rate ≤0.05 per 10,000 enplaned passengers (DOT Part 250 benchmark)</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>NRM OB optimiser does not natively model denied boarding compensation cost per DOT 14 CFR 250 tiers; analyst must manually adjust factors to avoid regulatory overshoot</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Apply DOT 14 CFR 250 regulatory cap and fare rule check</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Compliance Manager</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Recommended OB factors; ATPCO fare conditions (refundability, cancellation fees)</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Compliance-reviewed OB factor set; flag for non-refundable fare interactions</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>100% of OB factors within DOT involuntary bump compensation trigger thresholds</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Non-refundable Basic Economy fares have near-zero pre-departure cancellations, artificially inflating apparent show-up rates; ATPCO Rule 35 interactions must be hand-checked</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Approve and publish booking limits to PSS inventory</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Director of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Compliance-reviewed OB factor set; Director sign-off</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Authorised overbooking limits loaded into Altéa inventory control per flight</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Limit publication latency ≤4 hours ahead of booking horizon open; 100% of flights have an active OB limit</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Altéa inventory control updates via batch file load — real-time limit changes mid-booking horizon require manual override in Altéa Inventory module, increasing error risk</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Monitor booking pace vs. authorised OB limits</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Live booking feed from Altéa PSS; authorised OB limits</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace dashboard with oversale risk flags per flight</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Alert response time ≤15 minutes of threshold breach detection</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>NRM booking pace alerts are polled every 30 minutes; fast-filling charter diversions or flash sales can exceed limits before alerts trigger</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Detect and triage oversale threshold breach</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace alert; current bookings vs. authorised limit</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Oversale risk classification (low / medium / high) with recommended action</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>False positive rate ≤10% of alerts triaged as high-risk</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Group booking blocks held in Altéa GRP segment are excluded from NRM oversale count until confirmed, masking true capacity exposure up to T-72h</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Adjust OB level or close booking class dynamically</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Oversale risk classification; updated show-up probability at current booking depth</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Revised OB factor or booking class closure instruction applied to Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>OB adjustment applied within 30 minutes of triage decision; no flight departs with OB factor &gt;20% above baseline</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Closing discount booking classes to reduce oversale pressure destroys revenue on price-sensitive leisure itineraries; analyst must balance IDB risk vs. yield impact</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Escalate high-risk oversale flights to RM Supervisor</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>RM Supervisor</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>High-risk oversale flag; passenger manifest; connecting itinerary exposure</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Escalation note with recommended corrective action; decision to hold or reduce OB</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Escalation-to-decision cycle time ≤1 hour; 100% of high-risk flights reviewed by T-24h</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Connecting passengers on interline itineraries (not native Altéa bookings) are not surfaced in NRM oversale count; last-minute IDB on these passengers triggers DOT reporting obligation</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Identify oversold flights at check-in closure</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Final check-in count; boarded passenger list; aircraft capacity</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed oversale count and list of checked-in passengers eligible for VDB/IDB</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Oversold flight identification completed ≥30 minutes before departure</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>SITA AMS and Altéa DCS (Departure Control System) seat count reconciliation can diverge by 1-2 seats when upgrade or UMNR seat blocks are reassigned at gate</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Solicit and screen volunteers for VDB compensation</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Oversold count; gate board call; compensation parameters from RM Supervisor</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed volunteer list with accepted compensation; rebooked itineraries in Altéa</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>VDB rate ≥80% of oversale situations resolved without IDB; average VDB compensation cost ≤$350</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Compensation authority is set centrally by RM; gate agents cannot negotiate above the pre-approved cap without supervisor override, slowing volunteer acquisition on high-demand flights</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Process involuntary denied boarding per 14 CFR 250</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent / Supervisor</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed oversale after VDB exhaustion; passenger priority matrix (status, fare, check-in time)</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>IDB passenger list; denied boarding compensation (cash/voucher at DOT-mandated 400% of OW fare, max $1,550)</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>IDB processing completed ≥15 minutes before door close; 0 IDB passengers with connecting flights missed due to rebooking delay</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>DOT priority boarding rules (status, early check-in) conflict with RM desire to protect high-yield last-minute fares; applying the correct matrix under gate pressure is error-prone</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Issue compensation and confirm rebooking for IDB/VDB pax</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>IDB/VDB passenger list; approved compensation values; next available flight inventory</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Compensation vouchers/cash issued; confirmed rebooking on next available service; IDB event logged</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>100% of IDB passengers offered confirmed rebooking within 2 hours; compensation issued at gate before passenger departs</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Electronic voucher issuance via Altéa is not integrated with the passenger's Rapid Rewards account; compensation is issued as a separate code, creating friction and loyalty defection risk</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Compile post-flight IDB/VDB statistics and cost data</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Altéa IDB/VDB event logs; gate agent reports; compensation cost records</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>IDB/VDB summary report: count, cost, route, fare class, DOW breakdown</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Report generated within 48 hours of flight departure; 100% event capture rate</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Gate agent IDB logs in Altéa DCS are free-text fields; structured data extraction requires ETL cleanup before Redshift load, delaying post-flight analytics by up to 5 days</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Review denied boarding KPIs against policy thresholds</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Director of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>IDB/VDB summary report; rolling 12-month trend; DOT Part 250 benchmark (0.05 IDB per 10k pax)</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>KPI review decision: policy adequate or recalibration required</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>IDB rate ≤0.05 per 10,000 enplaned passengers; VDB cost ≤$350 average per event</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal spikes (holiday periods, irregular operations) mask underlying OB model drift; point-in-time KPI review may miss structural deterioration in show-up accuracy</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Submit DOT quarterly denied boarding compliance report</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Compliance Manager</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>DOT Air Travel Consumer Report Submission Portal</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Validated IDB/VDB statistics; carrier passenger enplanement totals</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Filed DOT Part 250 quarterly report; internal compliance archive record</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>100% on-time filing by DOT deadline (30 days after quarter end); zero restatements</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>DOT requires IDB figures disaggregated by aircraft size categories; Altéa fleet-type tagging must be manually reconciled against FAA registration data to ensure accurate segment classification</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N316"/>
+  <dimension ref="A1:N334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -38706,6 +40131,1302 @@
         </is>
       </c>
       <c r="N316" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="30" customHeight="1">
+      <c r="A317" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B317" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C317" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D317" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E317" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F317" s="16" t="inlineStr">
+        <is>
+          <t>Extract booking &amp; no-show history from PSS</t>
+        </is>
+      </c>
+      <c r="G317" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H317" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I317" s="16" t="inlineStr">
+        <is>
+          <t>Departed flight records, booking logs, check-in data — rolling 24 months</t>
+        </is>
+      </c>
+      <c r="J317" s="16" t="inlineStr">
+        <is>
+          <t>Raw no-show and cancellation dataset by flight, fare class, and booking channel</t>
+        </is>
+      </c>
+      <c r="K317" s="16" t="inlineStr">
+        <is>
+          <t>Dataset completeness ≥99% of departed flights</t>
+        </is>
+      </c>
+      <c r="L317" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS history exports require manual scheduling; ad-hoc pulls risk data truncation beyond 13-month rolling window</t>
+        </is>
+      </c>
+      <c r="M317" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N317" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="30" customHeight="1">
+      <c r="A318" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B318" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C318" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D318" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E318" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F318" s="18" t="inlineStr">
+        <is>
+          <t>Segment data by route, DOW, fare class, season</t>
+        </is>
+      </c>
+      <c r="G318" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H318" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I318" s="18" t="inlineStr">
+        <is>
+          <t>Raw no-show dataset from Altéa PSS export</t>
+        </is>
+      </c>
+      <c r="J318" s="18" t="inlineStr">
+        <is>
+          <t>Segmented no-show rate matrix with confidence intervals per cluster</t>
+        </is>
+      </c>
+      <c r="K318" s="18" t="inlineStr">
+        <is>
+          <t>Minimum 90 observed flights per segment for statistical significance</t>
+        </is>
+      </c>
+      <c r="L318" s="18" t="inlineStr">
+        <is>
+          <t>Thin markets (&lt;5 flights/week) produce unreliable segment-level no-show rates; pooled estimates inflate overbooking risk</t>
+        </is>
+      </c>
+      <c r="M318" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N318" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="30" customHeight="1">
+      <c r="A319" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B319" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C319" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D319" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E319" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F319" s="16" t="inlineStr">
+        <is>
+          <t>Run no-show forecast model and validate accuracy</t>
+        </is>
+      </c>
+      <c r="G319" s="16" t="inlineStr">
+        <is>
+          <t>RM Data Scientist</t>
+        </is>
+      </c>
+      <c r="H319" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I319" s="16" t="inlineStr">
+        <is>
+          <t>Segmented no-show matrix, demand forecasts from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J319" s="16" t="inlineStr">
+        <is>
+          <t>No-show show-up curve per flight cluster; model accuracy report</t>
+        </is>
+      </c>
+      <c r="K319" s="16" t="inlineStr">
+        <is>
+          <t>Forecast vs. actual no-show rate MAPE ≤5%</t>
+        </is>
+      </c>
+      <c r="L319" s="16" t="inlineStr">
+        <is>
+          <t>NRM show-up model requires retraining after major schedule restructures; post-COVID demand patterns invalidated legacy curves for 18+ months</t>
+        </is>
+      </c>
+      <c r="M319" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N319" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="30" customHeight="1">
+      <c r="A320" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B320" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C320" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D320" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E320" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F320" s="18" t="inlineStr">
+        <is>
+          <t>Calibrate show-up curve by fare class and lead time</t>
+        </is>
+      </c>
+      <c r="G320" s="18" t="inlineStr">
+        <is>
+          <t>RM Data Scientist</t>
+        </is>
+      </c>
+      <c r="H320" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I320" s="18" t="inlineStr">
+        <is>
+          <t>Validated no-show forecast model; approved show-up curves</t>
+        </is>
+      </c>
+      <c r="J320" s="18" t="inlineStr">
+        <is>
+          <t>Calibrated show-up probability curves published to AltéaRM overbooking module</t>
+        </is>
+      </c>
+      <c r="K320" s="18" t="inlineStr">
+        <is>
+          <t>Show-up curve refresh cycle ≤30 days for high-frequency routes; ≤90 days for seasonal routes</t>
+        </is>
+      </c>
+      <c r="L320" s="18" t="inlineStr">
+        <is>
+          <t>Fare class proliferation (Basic Economy vs. flexible fares) requires separate show-up curves; legacy model treats all economy as one class</t>
+        </is>
+      </c>
+      <c r="M320" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N320" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="30" customHeight="1">
+      <c r="A321" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B321" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C321" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D321" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E321" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F321" s="16" t="inlineStr">
+        <is>
+          <t>Generate recommended OB factors by flight segment</t>
+        </is>
+      </c>
+      <c r="G321" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H321" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I321" s="16" t="inlineStr">
+        <is>
+          <t>Calibrated show-up curves; target load factor ≥83%; denied boarding cost assumptions</t>
+        </is>
+      </c>
+      <c r="J321" s="16" t="inlineStr">
+        <is>
+          <t>Recommended overbooking factor per flight segment with expected IDB rate</t>
+        </is>
+      </c>
+      <c r="K321" s="16" t="inlineStr">
+        <is>
+          <t>Expected IDB rate ≤0.05 per 10,000 enplaned passengers (DOT Part 250 benchmark)</t>
+        </is>
+      </c>
+      <c r="L321" s="16" t="inlineStr">
+        <is>
+          <t>NRM OB optimiser does not natively model denied boarding compensation cost per DOT 14 CFR 250 tiers; analyst must manually adjust factors to avoid regulatory overshoot</t>
+        </is>
+      </c>
+      <c r="M321" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N321" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="30" customHeight="1">
+      <c r="A322" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B322" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C322" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D322" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E322" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F322" s="18" t="inlineStr">
+        <is>
+          <t>Apply DOT 14 CFR 250 regulatory cap and fare rule check</t>
+        </is>
+      </c>
+      <c r="G322" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Compliance Manager</t>
+        </is>
+      </c>
+      <c r="H322" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I322" s="18" t="inlineStr">
+        <is>
+          <t>Recommended OB factors; ATPCO fare conditions (refundability, cancellation fees)</t>
+        </is>
+      </c>
+      <c r="J322" s="18" t="inlineStr">
+        <is>
+          <t>Compliance-reviewed OB factor set; flag for non-refundable fare interactions</t>
+        </is>
+      </c>
+      <c r="K322" s="18" t="inlineStr">
+        <is>
+          <t>100% of OB factors within DOT involuntary bump compensation trigger thresholds</t>
+        </is>
+      </c>
+      <c r="L322" s="18" t="inlineStr">
+        <is>
+          <t>Non-refundable Basic Economy fares have near-zero pre-departure cancellations, artificially inflating apparent show-up rates; ATPCO Rule 35 interactions must be hand-checked</t>
+        </is>
+      </c>
+      <c r="M322" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N322" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="30" customHeight="1">
+      <c r="A323" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B323" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C323" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D323" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E323" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F323" s="16" t="inlineStr">
+        <is>
+          <t>Approve and publish booking limits to PSS inventory</t>
+        </is>
+      </c>
+      <c r="G323" s="16" t="inlineStr">
+        <is>
+          <t>Director of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H323" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I323" s="16" t="inlineStr">
+        <is>
+          <t>Compliance-reviewed OB factor set; Director sign-off</t>
+        </is>
+      </c>
+      <c r="J323" s="16" t="inlineStr">
+        <is>
+          <t>Authorised overbooking limits loaded into Altéa inventory control per flight</t>
+        </is>
+      </c>
+      <c r="K323" s="16" t="inlineStr">
+        <is>
+          <t>Limit publication latency ≤4 hours ahead of booking horizon open; 100% of flights have an active OB limit</t>
+        </is>
+      </c>
+      <c r="L323" s="16" t="inlineStr">
+        <is>
+          <t>Altéa inventory control updates via batch file load — real-time limit changes mid-booking horizon require manual override in Altéa Inventory module, increasing error risk</t>
+        </is>
+      </c>
+      <c r="M323" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N323" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="30" customHeight="1">
+      <c r="A324" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B324" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C324" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D324" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E324" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F324" s="18" t="inlineStr">
+        <is>
+          <t>Monitor booking pace vs. authorised OB limits</t>
+        </is>
+      </c>
+      <c r="G324" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H324" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I324" s="18" t="inlineStr">
+        <is>
+          <t>Live booking feed from Altéa PSS; authorised OB limits</t>
+        </is>
+      </c>
+      <c r="J324" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace dashboard with oversale risk flags per flight</t>
+        </is>
+      </c>
+      <c r="K324" s="18" t="inlineStr">
+        <is>
+          <t>Alert response time ≤15 minutes of threshold breach detection</t>
+        </is>
+      </c>
+      <c r="L324" s="18" t="inlineStr">
+        <is>
+          <t>NRM booking pace alerts are polled every 30 minutes; fast-filling charter diversions or flash sales can exceed limits before alerts trigger</t>
+        </is>
+      </c>
+      <c r="M324" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N324" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="30" customHeight="1">
+      <c r="A325" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B325" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C325" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D325" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E325" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F325" s="16" t="inlineStr">
+        <is>
+          <t>Detect and triage oversale threshold breach</t>
+        </is>
+      </c>
+      <c r="G325" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H325" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I325" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace alert; current bookings vs. authorised limit</t>
+        </is>
+      </c>
+      <c r="J325" s="16" t="inlineStr">
+        <is>
+          <t>Oversale risk classification (low / medium / high) with recommended action</t>
+        </is>
+      </c>
+      <c r="K325" s="16" t="inlineStr">
+        <is>
+          <t>False positive rate ≤10% of alerts triaged as high-risk</t>
+        </is>
+      </c>
+      <c r="L325" s="16" t="inlineStr">
+        <is>
+          <t>Group booking blocks held in Altéa GRP segment are excluded from NRM oversale count until confirmed, masking true capacity exposure up to T-72h</t>
+        </is>
+      </c>
+      <c r="M325" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N325" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="30" customHeight="1">
+      <c r="A326" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B326" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C326" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D326" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E326" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F326" s="18" t="inlineStr">
+        <is>
+          <t>Adjust OB level or close booking class dynamically</t>
+        </is>
+      </c>
+      <c r="G326" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H326" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I326" s="18" t="inlineStr">
+        <is>
+          <t>Oversale risk classification; updated show-up probability at current booking depth</t>
+        </is>
+      </c>
+      <c r="J326" s="18" t="inlineStr">
+        <is>
+          <t>Revised OB factor or booking class closure instruction applied to Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K326" s="18" t="inlineStr">
+        <is>
+          <t>OB adjustment applied within 30 minutes of triage decision; no flight departs with OB factor &gt;20% above baseline</t>
+        </is>
+      </c>
+      <c r="L326" s="18" t="inlineStr">
+        <is>
+          <t>Closing discount booking classes to reduce oversale pressure destroys revenue on price-sensitive leisure itineraries; analyst must balance IDB risk vs. yield impact</t>
+        </is>
+      </c>
+      <c r="M326" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N326" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="30" customHeight="1">
+      <c r="A327" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B327" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C327" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D327" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E327" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F327" s="16" t="inlineStr">
+        <is>
+          <t>Escalate high-risk oversale flights to RM Supervisor</t>
+        </is>
+      </c>
+      <c r="G327" s="16" t="inlineStr">
+        <is>
+          <t>RM Supervisor</t>
+        </is>
+      </c>
+      <c r="H327" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I327" s="16" t="inlineStr">
+        <is>
+          <t>High-risk oversale flag; passenger manifest; connecting itinerary exposure</t>
+        </is>
+      </c>
+      <c r="J327" s="16" t="inlineStr">
+        <is>
+          <t>Escalation note with recommended corrective action; decision to hold or reduce OB</t>
+        </is>
+      </c>
+      <c r="K327" s="16" t="inlineStr">
+        <is>
+          <t>Escalation-to-decision cycle time ≤1 hour; 100% of high-risk flights reviewed by T-24h</t>
+        </is>
+      </c>
+      <c r="L327" s="16" t="inlineStr">
+        <is>
+          <t>Connecting passengers on interline itineraries (not native Altéa bookings) are not surfaced in NRM oversale count; last-minute IDB on these passengers triggers DOT reporting obligation</t>
+        </is>
+      </c>
+      <c r="M327" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N327" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="30" customHeight="1">
+      <c r="A328" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B328" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C328" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D328" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E328" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F328" s="18" t="inlineStr">
+        <is>
+          <t>Identify oversold flights at check-in closure</t>
+        </is>
+      </c>
+      <c r="G328" s="18" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H328" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I328" s="18" t="inlineStr">
+        <is>
+          <t>Final check-in count; boarded passenger list; aircraft capacity</t>
+        </is>
+      </c>
+      <c r="J328" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed oversale count and list of checked-in passengers eligible for VDB/IDB</t>
+        </is>
+      </c>
+      <c r="K328" s="18" t="inlineStr">
+        <is>
+          <t>Oversold flight identification completed ≥30 minutes before departure</t>
+        </is>
+      </c>
+      <c r="L328" s="18" t="inlineStr">
+        <is>
+          <t>SITA AMS and Altéa DCS (Departure Control System) seat count reconciliation can diverge by 1-2 seats when upgrade or UMNR seat blocks are reassigned at gate</t>
+        </is>
+      </c>
+      <c r="M328" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N328" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="30" customHeight="1">
+      <c r="A329" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B329" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C329" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D329" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E329" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F329" s="16" t="inlineStr">
+        <is>
+          <t>Solicit and screen volunteers for VDB compensation</t>
+        </is>
+      </c>
+      <c r="G329" s="16" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H329" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I329" s="16" t="inlineStr">
+        <is>
+          <t>Oversold count; gate board call; compensation parameters from RM Supervisor</t>
+        </is>
+      </c>
+      <c r="J329" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed volunteer list with accepted compensation; rebooked itineraries in Altéa</t>
+        </is>
+      </c>
+      <c r="K329" s="16" t="inlineStr">
+        <is>
+          <t>VDB rate ≥80% of oversale situations resolved without IDB; average VDB compensation cost ≤$350</t>
+        </is>
+      </c>
+      <c r="L329" s="16" t="inlineStr">
+        <is>
+          <t>Compensation authority is set centrally by RM; gate agents cannot negotiate above the pre-approved cap without supervisor override, slowing volunteer acquisition on high-demand flights</t>
+        </is>
+      </c>
+      <c r="M329" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N329" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="30" customHeight="1">
+      <c r="A330" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B330" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C330" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D330" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E330" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F330" s="18" t="inlineStr">
+        <is>
+          <t>Process involuntary denied boarding per 14 CFR 250</t>
+        </is>
+      </c>
+      <c r="G330" s="18" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent / Supervisor</t>
+        </is>
+      </c>
+      <c r="H330" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I330" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed oversale after VDB exhaustion; passenger priority matrix (status, fare, check-in time)</t>
+        </is>
+      </c>
+      <c r="J330" s="18" t="inlineStr">
+        <is>
+          <t>IDB passenger list; denied boarding compensation (cash/voucher at DOT-mandated 400% of OW fare, max $1,550)</t>
+        </is>
+      </c>
+      <c r="K330" s="18" t="inlineStr">
+        <is>
+          <t>IDB processing completed ≥15 minutes before door close; 0 IDB passengers with connecting flights missed due to rebooking delay</t>
+        </is>
+      </c>
+      <c r="L330" s="18" t="inlineStr">
+        <is>
+          <t>DOT priority boarding rules (status, early check-in) conflict with RM desire to protect high-yield last-minute fares; applying the correct matrix under gate pressure is error-prone</t>
+        </is>
+      </c>
+      <c r="M330" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N330" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="30" customHeight="1">
+      <c r="A331" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B331" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C331" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D331" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E331" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F331" s="16" t="inlineStr">
+        <is>
+          <t>Issue compensation and confirm rebooking for IDB/VDB pax</t>
+        </is>
+      </c>
+      <c r="G331" s="16" t="inlineStr">
+        <is>
+          <t>Airport Gate Agent</t>
+        </is>
+      </c>
+      <c r="H331" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I331" s="16" t="inlineStr">
+        <is>
+          <t>IDB/VDB passenger list; approved compensation values; next available flight inventory</t>
+        </is>
+      </c>
+      <c r="J331" s="16" t="inlineStr">
+        <is>
+          <t>Compensation vouchers/cash issued; confirmed rebooking on next available service; IDB event logged</t>
+        </is>
+      </c>
+      <c r="K331" s="16" t="inlineStr">
+        <is>
+          <t>100% of IDB passengers offered confirmed rebooking within 2 hours; compensation issued at gate before passenger departs</t>
+        </is>
+      </c>
+      <c r="L331" s="16" t="inlineStr">
+        <is>
+          <t>Electronic voucher issuance via Altéa is not integrated with the passenger's Rapid Rewards account; compensation is issued as a separate code, creating friction and loyalty defection risk</t>
+        </is>
+      </c>
+      <c r="M331" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N331" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="30" customHeight="1">
+      <c r="A332" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B332" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C332" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D332" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E332" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F332" s="18" t="inlineStr">
+        <is>
+          <t>Compile post-flight IDB/VDB statistics and cost data</t>
+        </is>
+      </c>
+      <c r="G332" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H332" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I332" s="18" t="inlineStr">
+        <is>
+          <t>Altéa IDB/VDB event logs; gate agent reports; compensation cost records</t>
+        </is>
+      </c>
+      <c r="J332" s="18" t="inlineStr">
+        <is>
+          <t>IDB/VDB summary report: count, cost, route, fare class, DOW breakdown</t>
+        </is>
+      </c>
+      <c r="K332" s="18" t="inlineStr">
+        <is>
+          <t>Report generated within 48 hours of flight departure; 100% event capture rate</t>
+        </is>
+      </c>
+      <c r="L332" s="18" t="inlineStr">
+        <is>
+          <t>Gate agent IDB logs in Altéa DCS are free-text fields; structured data extraction requires ETL cleanup before Redshift load, delaying post-flight analytics by up to 5 days</t>
+        </is>
+      </c>
+      <c r="M332" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N332" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="30" customHeight="1">
+      <c r="A333" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B333" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C333" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D333" s="16" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E333" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F333" s="16" t="inlineStr">
+        <is>
+          <t>Review denied boarding KPIs against policy thresholds</t>
+        </is>
+      </c>
+      <c r="G333" s="16" t="inlineStr">
+        <is>
+          <t>Director of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H333" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I333" s="16" t="inlineStr">
+        <is>
+          <t>IDB/VDB summary report; rolling 12-month trend; DOT Part 250 benchmark (0.05 IDB per 10k pax)</t>
+        </is>
+      </c>
+      <c r="J333" s="16" t="inlineStr">
+        <is>
+          <t>KPI review decision: policy adequate or recalibration required</t>
+        </is>
+      </c>
+      <c r="K333" s="16" t="inlineStr">
+        <is>
+          <t>IDB rate ≤0.05 per 10,000 enplaned passengers; VDB cost ≤$350 average per event</t>
+        </is>
+      </c>
+      <c r="L333" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal spikes (holiday periods, irregular operations) mask underlying OB model drift; point-in-time KPI review may miss structural deterioration in show-up accuracy</t>
+        </is>
+      </c>
+      <c r="M333" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N333" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="30" customHeight="1">
+      <c r="A334" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-03</t>
+        </is>
+      </c>
+      <c r="B334" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C334" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D334" s="18" t="inlineStr">
+        <is>
+          <t>Overbooking Policy Management</t>
+        </is>
+      </c>
+      <c r="E334" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F334" s="18" t="inlineStr">
+        <is>
+          <t>Submit DOT quarterly denied boarding compliance report</t>
+        </is>
+      </c>
+      <c r="G334" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Compliance Manager</t>
+        </is>
+      </c>
+      <c r="H334" s="18" t="inlineStr">
+        <is>
+          <t>DOT Air Travel Consumer Report Submission Portal</t>
+        </is>
+      </c>
+      <c r="I334" s="18" t="inlineStr">
+        <is>
+          <t>Validated IDB/VDB statistics; carrier passenger enplanement totals</t>
+        </is>
+      </c>
+      <c r="J334" s="18" t="inlineStr">
+        <is>
+          <t>Filed DOT Part 250 quarterly report; internal compliance archive record</t>
+        </is>
+      </c>
+      <c r="K334" s="18" t="inlineStr">
+        <is>
+          <t>100% on-time filing by DOT deadline (30 days after quarter end); zero restatements</t>
+        </is>
+      </c>
+      <c r="L334" s="18" t="inlineStr">
+        <is>
+          <t>DOT requires IDB figures disaggregated by aircraft size categories; Altéa fleet-type tagging must be manually reconciled against FAA registration data to ensure accurate segment classification</t>
+        </is>
+      </c>
+      <c r="M334" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N334" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-RM-04: Demand Forecasting & Modelling — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -25,6 +25,7 @@
     <sheet name="NP-RM-01" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="NP-RM-02" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="NP-RM-03" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="NP-RM-04" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1332,13 +1333,21 @@
           <t>Demand Forecasting &amp; Modelling</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr"/>
-      <c r="G21" s="10" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-04</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -17424,13 +17433,1357 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-04 — Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract historical booking &amp; ticketing data</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Scheduled forecast cycle trigger (daily/weekly batch)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Raw booking history file by O&amp;D, cabin, fare class and departure date</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness ≥ 99% of expected PNR records</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS booking history exports can lag 4–6 hours in peak windows, misaligning the daily forecast cycle and causing stale AU recommendations to persist in NRM overnight</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Ingest external demand &amp; traffic signals</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>OAG forward schedule feed, MIDT booking data, tourism board indices</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Enriched demand signal dataset merged with internal booking history</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>External signal ingestion latency ≤ 2 hours from OAG publish</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>MIDT data covers only GDS-booked itineraries, creating blind spots for NDC and direct-channel bookings — up to 30% of volume on some LCCs — leading to systematic under-forecasting on digitally distributed routes</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate &amp; cleanse data for anomalies</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Data Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Raw booking history + external signals from steps 1.1–1.2</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Cleansed, deduplicated demand dataset with anomaly flags</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Data quality score ≥ 95%; outlier rows flagged &lt; 2% of total</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>COVID-era booking collapse and recovery create structural breaks in training data; models trained on pre-2020 history without explicit break-point adjustment produce load-factor forecasts biased 6–12 pts below actuals on leisure routes</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Segment data by O&amp;D, cabin and booking curve</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Cleansed demand dataset</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Demand time-series per O&amp;D × cabin × day-of-week × season band</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Segment granularity covers ≥ 95% of revenue-bearing O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Thin O&amp;D markets (&lt; 200 observations per departure) produce statistically unstable booking curves; SkyCAST defaults to network-level priors which can over-smooth volatile new-route ramp-ups</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Identify constrained booking observations</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Segmented demand series + historical AU and sell limit records</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Flagged constrained observations (departures where AU was binding at close)</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Constrained-observation detection rate ≥ 90% vs manual audit sample</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>NRM does not retain intra-day AU change history at sufficient granularity; when AUs were changed multiple times within a day, the system only logs end-of-day state, causing the unconstraining algorithm to miss intermediate constraints</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Apply EM unconstraining to constrained series</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Constrained observation flags + observed booking counts</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Unconstrained demand estimate per O&amp;D × fare class × departure date</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Unconstraining variance (CV) ≤ 5% on routes with ≥ 90% load factor</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Expectation-Maximisation unconstraining can diverge on very high-load routes (LF &gt; 95%) where almost every observation is constrained — NRM falls back to simple censored-mean imputation which understates true demand by 8–15%</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Validate unconstrained demand estimates</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Unconstrained demand series from step 2.2</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Validated unconstrained demand series approved for model input</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Unconstrained mean ≤ 1.5× constrained mean on non-peak markets</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Overly aggressive unconstraining inflates unconstrained demand estimates, causing the optimiser to open excess inventory and erode yield on near-full flights — requires manual override on seasonal peak routes</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Select forecasting model type per market</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Validated unconstrained demand series, market volatility scores</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Model configuration file: additive vs multiplicative per O&amp;D × cabin</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Model selection logic applied to 100% of active O&amp;D pairs within 1 hour of data readiness</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST model selection heuristics default to additive models for thin markets regardless of demand variability; high-leisure volatile routes on short-haul thin sectors are systematically misconfigured, requiring manual analyst overrides each cycle</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Apply special-event &amp; seasonality overlays</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Model config + airline event calendar (holidays, conventions, sports, disruptions)</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Seasonality-adjusted demand series with event uplift / suppression factors</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Special-event adjustment coverage: ≥ 85% of Top-100 events per quarter captured before forecast run</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Event calendar maintenance is manual and decentralised — network RM team and regional market managers each maintain separate lists, causing duplicate or conflicting adjustments when the same event spans multiple O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Run O&amp;D demand forecast in SkyCAST</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Seasonality-adjusted unconstrained demand series + model config</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Point and probabilistic demand forecasts per O&amp;D × cabin × booking horizon</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 12% across all O&amp;D pairs; P90 forecast coverage ≥ 80% of actuals</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST batch forecast runs for a large network (500+ daily departures) can exceed the available processing window on peak planning days, causing downstream NRM optimisation to run on partially stale forecasts</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Disaggregate O&amp;D forecast to fare-class level</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecasts from step 3.3 + fare class demand share curves</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Fare-class level demand forecast input for EMSRb optimisation</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Fare-class forecast disaggregation completed within 30 min of O&amp;D forecast publish</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Fare-class demand share curves are estimated from historical booking curves; when airlines reprice aggressively (e.g. adding or retiring fare classes mid-season), the share curves become stale and misdirect inventory allocation toward retired buckets</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Analyst review of system-generated forecasts</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Fare-class demand forecasts from step 3.4, booking pace actuals</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Reviewed forecast report with analyst annotations and override candidates</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Analyst review completed within 4 hours of forecast publication; &lt; 15% of O&amp;D pairs require manual override</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>NRM forecast review UI surfaces only summary metrics per market; analysts cannot drill to individual booking-curve segments without exporting to Excel, slowing root-cause investigation and increasing override latency</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Apply market-level manual forecast adjustments</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Override candidate list from step 4.1, competitive intelligence, sales intelligence</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Adjusted demand forecast with analyst override log</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Override accuracy (post-departure MAPE for overridden markets) ≤ 10%</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Manual overrides are not systematically back-tested; analysts who override frequently cannot tell whether their interventions improve or degrade forecast accuracy versus the unmodified system forecast, making governance of override behaviour impossible</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Publish approved demand forecast to NRM</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Approved fare-class demand forecast (system + analyst overrides)</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Active demand forecast loaded into NRM for EMSRb optimisation cycle</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Forecast publish latency ≤ 30 min from analyst sign-off; 100% of departures within 330-day booking window covered</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>NRM forecast publish is a full-replace operation — partial updates are not supported; if a publish job fails mid-run (e.g. network timeout), the system may hold a mix of new and prior-cycle forecasts, causing inconsistent AU recommendations until the next full cycle</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Track post-departure forecast accuracy</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Departed flight actuals (load factor, revenue, fare-class mix) vs forecast</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy scorecard: MAPE, bias, coverage by O&amp;D, cabin, horizon</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Rolling 30-day network MAPE ≤ 12%; bias (mean signed error) within ±2%</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Post-departure actuals are available only after PSS ticket coupon reconciliation (typically T+2 days), creating a 48-hour blind spot between departure and accuracy reporting that delays identification of systematic forecast failures on new routes</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Detect systematic bias or model drift</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Forecast accuracy scorecard from step 5.1</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Bias / drift diagnostic report with affected O&amp;D segments identified</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Bias alert triggered when mean signed error exceeds ±3% for ≥ 5 consecutive departures on same O&amp;D</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau dashboards for RM forecast tracking are maintained by a separate analytics team; model drift alerts depend on manual dashboard reviews rather than automated statistical process control, meaning bias can persist for 2–3 weeks before analyst intervention</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Trigger model recalibration &amp; parameter update</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Bias / drift diagnostic report + recalibration threshold breach flags</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Updated model coefficients and booking-curve parameters deployed to SkyCAST</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Recalibration cycle completed within 48 hours of bias-alert trigger; post-recalibration MAPE improvement ≥ 2 percentage points</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST model parameter updates require a full re-training run on the rolling 2-year history window; on large networks this can take 6–8 hours, blocking the daily forecast cycle if recalibration is triggered mid-day rather than during the overnight batch window</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N334"/>
+  <dimension ref="A1:N351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -41429,6 +42782,1230 @@
       <c r="N334" s="17" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="30" customHeight="1">
+      <c r="A335" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B335" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C335" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D335" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E335" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F335" s="16" t="inlineStr">
+        <is>
+          <t>Extract historical booking &amp; ticketing data</t>
+        </is>
+      </c>
+      <c r="G335" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H335" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I335" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled forecast cycle trigger (daily/weekly batch)</t>
+        </is>
+      </c>
+      <c r="J335" s="16" t="inlineStr">
+        <is>
+          <t>Raw booking history file by O&amp;D, cabin, fare class and departure date</t>
+        </is>
+      </c>
+      <c r="K335" s="16" t="inlineStr">
+        <is>
+          <t>Data completeness ≥ 99% of expected PNR records</t>
+        </is>
+      </c>
+      <c r="L335" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS booking history exports can lag 4–6 hours in peak windows, misaligning the daily forecast cycle and causing stale AU recommendations to persist in NRM overnight</t>
+        </is>
+      </c>
+      <c r="M335" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N335" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="30" customHeight="1">
+      <c r="A336" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B336" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C336" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D336" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E336" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F336" s="18" t="inlineStr">
+        <is>
+          <t>Ingest external demand &amp; traffic signals</t>
+        </is>
+      </c>
+      <c r="G336" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H336" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I336" s="18" t="inlineStr">
+        <is>
+          <t>OAG forward schedule feed, MIDT booking data, tourism board indices</t>
+        </is>
+      </c>
+      <c r="J336" s="18" t="inlineStr">
+        <is>
+          <t>Enriched demand signal dataset merged with internal booking history</t>
+        </is>
+      </c>
+      <c r="K336" s="18" t="inlineStr">
+        <is>
+          <t>External signal ingestion latency ≤ 2 hours from OAG publish</t>
+        </is>
+      </c>
+      <c r="L336" s="18" t="inlineStr">
+        <is>
+          <t>MIDT data covers only GDS-booked itineraries, creating blind spots for NDC and direct-channel bookings — up to 30% of volume on some LCCs — leading to systematic under-forecasting on digitally distributed routes</t>
+        </is>
+      </c>
+      <c r="M336" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N336" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="30" customHeight="1">
+      <c r="A337" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B337" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C337" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D337" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E337" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F337" s="16" t="inlineStr">
+        <is>
+          <t>Validate &amp; cleanse data for anomalies</t>
+        </is>
+      </c>
+      <c r="G337" s="16" t="inlineStr">
+        <is>
+          <t>Data Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H337" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I337" s="16" t="inlineStr">
+        <is>
+          <t>Raw booking history + external signals from steps 1.1–1.2</t>
+        </is>
+      </c>
+      <c r="J337" s="16" t="inlineStr">
+        <is>
+          <t>Cleansed, deduplicated demand dataset with anomaly flags</t>
+        </is>
+      </c>
+      <c r="K337" s="16" t="inlineStr">
+        <is>
+          <t>Data quality score ≥ 95%; outlier rows flagged &lt; 2% of total</t>
+        </is>
+      </c>
+      <c r="L337" s="16" t="inlineStr">
+        <is>
+          <t>COVID-era booking collapse and recovery create structural breaks in training data; models trained on pre-2020 history without explicit break-point adjustment produce load-factor forecasts biased 6–12 pts below actuals on leisure routes</t>
+        </is>
+      </c>
+      <c r="M337" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N337" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="30" customHeight="1">
+      <c r="A338" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B338" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C338" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D338" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E338" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F338" s="18" t="inlineStr">
+        <is>
+          <t>Segment data by O&amp;D, cabin and booking curve</t>
+        </is>
+      </c>
+      <c r="G338" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H338" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I338" s="18" t="inlineStr">
+        <is>
+          <t>Cleansed demand dataset</t>
+        </is>
+      </c>
+      <c r="J338" s="18" t="inlineStr">
+        <is>
+          <t>Demand time-series per O&amp;D × cabin × day-of-week × season band</t>
+        </is>
+      </c>
+      <c r="K338" s="18" t="inlineStr">
+        <is>
+          <t>Segment granularity covers ≥ 95% of revenue-bearing O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="L338" s="18" t="inlineStr">
+        <is>
+          <t>Thin O&amp;D markets (&lt; 200 observations per departure) produce statistically unstable booking curves; SkyCAST defaults to network-level priors which can over-smooth volatile new-route ramp-ups</t>
+        </is>
+      </c>
+      <c r="M338" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N338" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="30" customHeight="1">
+      <c r="A339" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B339" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C339" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D339" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E339" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F339" s="16" t="inlineStr">
+        <is>
+          <t>Identify constrained booking observations</t>
+        </is>
+      </c>
+      <c r="G339" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H339" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I339" s="16" t="inlineStr">
+        <is>
+          <t>Segmented demand series + historical AU and sell limit records</t>
+        </is>
+      </c>
+      <c r="J339" s="16" t="inlineStr">
+        <is>
+          <t>Flagged constrained observations (departures where AU was binding at close)</t>
+        </is>
+      </c>
+      <c r="K339" s="16" t="inlineStr">
+        <is>
+          <t>Constrained-observation detection rate ≥ 90% vs manual audit sample</t>
+        </is>
+      </c>
+      <c r="L339" s="16" t="inlineStr">
+        <is>
+          <t>NRM does not retain intra-day AU change history at sufficient granularity; when AUs were changed multiple times within a day, the system only logs end-of-day state, causing the unconstraining algorithm to miss intermediate constraints</t>
+        </is>
+      </c>
+      <c r="M339" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N339" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="30" customHeight="1">
+      <c r="A340" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B340" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C340" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D340" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E340" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F340" s="18" t="inlineStr">
+        <is>
+          <t>Apply EM unconstraining to constrained series</t>
+        </is>
+      </c>
+      <c r="G340" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H340" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I340" s="18" t="inlineStr">
+        <is>
+          <t>Constrained observation flags + observed booking counts</t>
+        </is>
+      </c>
+      <c r="J340" s="18" t="inlineStr">
+        <is>
+          <t>Unconstrained demand estimate per O&amp;D × fare class × departure date</t>
+        </is>
+      </c>
+      <c r="K340" s="18" t="inlineStr">
+        <is>
+          <t>Unconstraining variance (CV) ≤ 5% on routes with ≥ 90% load factor</t>
+        </is>
+      </c>
+      <c r="L340" s="18" t="inlineStr">
+        <is>
+          <t>Expectation-Maximisation unconstraining can diverge on very high-load routes (LF &gt; 95%) where almost every observation is constrained — NRM falls back to simple censored-mean imputation which understates true demand by 8–15%</t>
+        </is>
+      </c>
+      <c r="M340" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N340" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="30" customHeight="1">
+      <c r="A341" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B341" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C341" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D341" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E341" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F341" s="16" t="inlineStr">
+        <is>
+          <t>Validate unconstrained demand estimates</t>
+        </is>
+      </c>
+      <c r="G341" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H341" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I341" s="16" t="inlineStr">
+        <is>
+          <t>Unconstrained demand series from step 2.2</t>
+        </is>
+      </c>
+      <c r="J341" s="16" t="inlineStr">
+        <is>
+          <t>Validated unconstrained demand series approved for model input</t>
+        </is>
+      </c>
+      <c r="K341" s="16" t="inlineStr">
+        <is>
+          <t>Unconstrained mean ≤ 1.5× constrained mean on non-peak markets</t>
+        </is>
+      </c>
+      <c r="L341" s="16" t="inlineStr">
+        <is>
+          <t>Overly aggressive unconstraining inflates unconstrained demand estimates, causing the optimiser to open excess inventory and erode yield on near-full flights — requires manual override on seasonal peak routes</t>
+        </is>
+      </c>
+      <c r="M341" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N341" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="30" customHeight="1">
+      <c r="A342" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B342" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C342" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D342" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E342" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F342" s="18" t="inlineStr">
+        <is>
+          <t>Select forecasting model type per market</t>
+        </is>
+      </c>
+      <c r="G342" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H342" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I342" s="18" t="inlineStr">
+        <is>
+          <t>Validated unconstrained demand series, market volatility scores</t>
+        </is>
+      </c>
+      <c r="J342" s="18" t="inlineStr">
+        <is>
+          <t>Model configuration file: additive vs multiplicative per O&amp;D × cabin</t>
+        </is>
+      </c>
+      <c r="K342" s="18" t="inlineStr">
+        <is>
+          <t>Model selection logic applied to 100% of active O&amp;D pairs within 1 hour of data readiness</t>
+        </is>
+      </c>
+      <c r="L342" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST model selection heuristics default to additive models for thin markets regardless of demand variability; high-leisure volatile routes on short-haul thin sectors are systematically misconfigured, requiring manual analyst overrides each cycle</t>
+        </is>
+      </c>
+      <c r="M342" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N342" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="30" customHeight="1">
+      <c r="A343" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B343" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C343" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D343" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E343" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F343" s="16" t="inlineStr">
+        <is>
+          <t>Apply special-event &amp; seasonality overlays</t>
+        </is>
+      </c>
+      <c r="G343" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H343" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I343" s="16" t="inlineStr">
+        <is>
+          <t>Model config + airline event calendar (holidays, conventions, sports, disruptions)</t>
+        </is>
+      </c>
+      <c r="J343" s="16" t="inlineStr">
+        <is>
+          <t>Seasonality-adjusted demand series with event uplift / suppression factors</t>
+        </is>
+      </c>
+      <c r="K343" s="16" t="inlineStr">
+        <is>
+          <t>Special-event adjustment coverage: ≥ 85% of Top-100 events per quarter captured before forecast run</t>
+        </is>
+      </c>
+      <c r="L343" s="16" t="inlineStr">
+        <is>
+          <t>Event calendar maintenance is manual and decentralised — network RM team and regional market managers each maintain separate lists, causing duplicate or conflicting adjustments when the same event spans multiple O&amp;D pairs</t>
+        </is>
+      </c>
+      <c r="M343" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N343" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="30" customHeight="1">
+      <c r="A344" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B344" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C344" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D344" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E344" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F344" s="18" t="inlineStr">
+        <is>
+          <t>Run O&amp;D demand forecast in SkyCAST</t>
+        </is>
+      </c>
+      <c r="G344" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H344" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I344" s="18" t="inlineStr">
+        <is>
+          <t>Seasonality-adjusted unconstrained demand series + model config</t>
+        </is>
+      </c>
+      <c r="J344" s="18" t="inlineStr">
+        <is>
+          <t>Point and probabilistic demand forecasts per O&amp;D × cabin × booking horizon</t>
+        </is>
+      </c>
+      <c r="K344" s="18" t="inlineStr">
+        <is>
+          <t>Forecast MAPE ≤ 12% across all O&amp;D pairs; P90 forecast coverage ≥ 80% of actuals</t>
+        </is>
+      </c>
+      <c r="L344" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST batch forecast runs for a large network (500+ daily departures) can exceed the available processing window on peak planning days, causing downstream NRM optimisation to run on partially stale forecasts</t>
+        </is>
+      </c>
+      <c r="M344" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N344" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="30" customHeight="1">
+      <c r="A345" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B345" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C345" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D345" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E345" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F345" s="16" t="inlineStr">
+        <is>
+          <t>Disaggregate O&amp;D forecast to fare-class level</t>
+        </is>
+      </c>
+      <c r="G345" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H345" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I345" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D demand forecasts from step 3.3 + fare class demand share curves</t>
+        </is>
+      </c>
+      <c r="J345" s="16" t="inlineStr">
+        <is>
+          <t>Fare-class level demand forecast input for EMSRb optimisation</t>
+        </is>
+      </c>
+      <c r="K345" s="16" t="inlineStr">
+        <is>
+          <t>Fare-class forecast disaggregation completed within 30 min of O&amp;D forecast publish</t>
+        </is>
+      </c>
+      <c r="L345" s="16" t="inlineStr">
+        <is>
+          <t>Fare-class demand share curves are estimated from historical booking curves; when airlines reprice aggressively (e.g. adding or retiring fare classes mid-season), the share curves become stale and misdirect inventory allocation toward retired buckets</t>
+        </is>
+      </c>
+      <c r="M345" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N345" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="30" customHeight="1">
+      <c r="A346" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B346" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C346" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D346" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E346" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F346" s="18" t="inlineStr">
+        <is>
+          <t>Analyst review of system-generated forecasts</t>
+        </is>
+      </c>
+      <c r="G346" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H346" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I346" s="18" t="inlineStr">
+        <is>
+          <t>Fare-class demand forecasts from step 3.4, booking pace actuals</t>
+        </is>
+      </c>
+      <c r="J346" s="18" t="inlineStr">
+        <is>
+          <t>Reviewed forecast report with analyst annotations and override candidates</t>
+        </is>
+      </c>
+      <c r="K346" s="18" t="inlineStr">
+        <is>
+          <t>Analyst review completed within 4 hours of forecast publication; &lt; 15% of O&amp;D pairs require manual override</t>
+        </is>
+      </c>
+      <c r="L346" s="18" t="inlineStr">
+        <is>
+          <t>NRM forecast review UI surfaces only summary metrics per market; analysts cannot drill to individual booking-curve segments without exporting to Excel, slowing root-cause investigation and increasing override latency</t>
+        </is>
+      </c>
+      <c r="M346" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N346" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="30" customHeight="1">
+      <c r="A347" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B347" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C347" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D347" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E347" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F347" s="16" t="inlineStr">
+        <is>
+          <t>Apply market-level manual forecast adjustments</t>
+        </is>
+      </c>
+      <c r="G347" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H347" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I347" s="16" t="inlineStr">
+        <is>
+          <t>Override candidate list from step 4.1, competitive intelligence, sales intelligence</t>
+        </is>
+      </c>
+      <c r="J347" s="16" t="inlineStr">
+        <is>
+          <t>Adjusted demand forecast with analyst override log</t>
+        </is>
+      </c>
+      <c r="K347" s="16" t="inlineStr">
+        <is>
+          <t>Override accuracy (post-departure MAPE for overridden markets) ≤ 10%</t>
+        </is>
+      </c>
+      <c r="L347" s="16" t="inlineStr">
+        <is>
+          <t>Manual overrides are not systematically back-tested; analysts who override frequently cannot tell whether their interventions improve or degrade forecast accuracy versus the unmodified system forecast, making governance of override behaviour impossible</t>
+        </is>
+      </c>
+      <c r="M347" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N347" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="30" customHeight="1">
+      <c r="A348" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B348" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C348" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D348" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E348" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F348" s="18" t="inlineStr">
+        <is>
+          <t>Publish approved demand forecast to NRM</t>
+        </is>
+      </c>
+      <c r="G348" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H348" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I348" s="18" t="inlineStr">
+        <is>
+          <t>Approved fare-class demand forecast (system + analyst overrides)</t>
+        </is>
+      </c>
+      <c r="J348" s="18" t="inlineStr">
+        <is>
+          <t>Active demand forecast loaded into NRM for EMSRb optimisation cycle</t>
+        </is>
+      </c>
+      <c r="K348" s="18" t="inlineStr">
+        <is>
+          <t>Forecast publish latency ≤ 30 min from analyst sign-off; 100% of departures within 330-day booking window covered</t>
+        </is>
+      </c>
+      <c r="L348" s="18" t="inlineStr">
+        <is>
+          <t>NRM forecast publish is a full-replace operation — partial updates are not supported; if a publish job fails mid-run (e.g. network timeout), the system may hold a mix of new and prior-cycle forecasts, causing inconsistent AU recommendations until the next full cycle</t>
+        </is>
+      </c>
+      <c r="M348" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N348" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="30" customHeight="1">
+      <c r="A349" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B349" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C349" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D349" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E349" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F349" s="16" t="inlineStr">
+        <is>
+          <t>Track post-departure forecast accuracy</t>
+        </is>
+      </c>
+      <c r="G349" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H349" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I349" s="16" t="inlineStr">
+        <is>
+          <t>Departed flight actuals (load factor, revenue, fare-class mix) vs forecast</t>
+        </is>
+      </c>
+      <c r="J349" s="16" t="inlineStr">
+        <is>
+          <t>Forecast accuracy scorecard: MAPE, bias, coverage by O&amp;D, cabin, horizon</t>
+        </is>
+      </c>
+      <c r="K349" s="16" t="inlineStr">
+        <is>
+          <t>Rolling 30-day network MAPE ≤ 12%; bias (mean signed error) within ±2%</t>
+        </is>
+      </c>
+      <c r="L349" s="16" t="inlineStr">
+        <is>
+          <t>Post-departure actuals are available only after PSS ticket coupon reconciliation (typically T+2 days), creating a 48-hour blind spot between departure and accuracy reporting that delays identification of systematic forecast failures on new routes</t>
+        </is>
+      </c>
+      <c r="M349" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N349" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="30" customHeight="1">
+      <c r="A350" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B350" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C350" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D350" s="18" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E350" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F350" s="18" t="inlineStr">
+        <is>
+          <t>Detect systematic bias or model drift</t>
+        </is>
+      </c>
+      <c r="G350" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H350" s="18" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I350" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy scorecard from step 5.1</t>
+        </is>
+      </c>
+      <c r="J350" s="18" t="inlineStr">
+        <is>
+          <t>Bias / drift diagnostic report with affected O&amp;D segments identified</t>
+        </is>
+      </c>
+      <c r="K350" s="18" t="inlineStr">
+        <is>
+          <t>Bias alert triggered when mean signed error exceeds ±3% for ≥ 5 consecutive departures on same O&amp;D</t>
+        </is>
+      </c>
+      <c r="L350" s="18" t="inlineStr">
+        <is>
+          <t>Tableau dashboards for RM forecast tracking are maintained by a separate analytics team; model drift alerts depend on manual dashboard reviews rather than automated statistical process control, meaning bias can persist for 2–3 weeks before analyst intervention</t>
+        </is>
+      </c>
+      <c r="M350" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N350" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="30" customHeight="1">
+      <c r="A351" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-04</t>
+        </is>
+      </c>
+      <c r="B351" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C351" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D351" s="16" t="inlineStr">
+        <is>
+          <t>Demand Forecasting &amp; Modelling</t>
+        </is>
+      </c>
+      <c r="E351" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F351" s="16" t="inlineStr">
+        <is>
+          <t>Trigger model recalibration &amp; parameter update</t>
+        </is>
+      </c>
+      <c r="G351" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H351" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I351" s="16" t="inlineStr">
+        <is>
+          <t>Bias / drift diagnostic report + recalibration threshold breach flags</t>
+        </is>
+      </c>
+      <c r="J351" s="16" t="inlineStr">
+        <is>
+          <t>Updated model coefficients and booking-curve parameters deployed to SkyCAST</t>
+        </is>
+      </c>
+      <c r="K351" s="16" t="inlineStr">
+        <is>
+          <t>Recalibration cycle completed within 48 hours of bias-alert trigger; post-recalibration MAPE improvement ≥ 2 percentage points</t>
+        </is>
+      </c>
+      <c r="L351" s="16" t="inlineStr">
+        <is>
+          <t>SkyCAST model parameter updates require a full re-training run on the rolling 2-year history window; on large networks this can take 6–8 hours, blocking the daily forecast cycle if recalibration is triggered mid-day rather than during the overnight batch window</t>
+        </is>
+      </c>
+      <c r="M351" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N351" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NP-RM-05: Group Sales Revenue Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -26,6 +26,7 @@
     <sheet name="NP-RM-02" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="NP-RM-03" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="NP-RM-04" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="NP-RM-05" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1370,13 +1371,21 @@
           <t>Group Sales Revenue Management</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="8" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-05</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -18783,7 +18792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N351"/>
+  <dimension ref="A1:N370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -44009,8 +44018,2864 @@
         </is>
       </c>
     </row>
+    <row r="352" ht="30" customHeight="1">
+      <c r="A352" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B352" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C352" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D352" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E352" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F352" s="18" t="inlineStr">
+        <is>
+          <t>Receive Group Booking Request</t>
+        </is>
+      </c>
+      <c r="G352" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H352" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I352" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request via SWABIZ portal, GDS, travel agency, or direct sales channel</t>
+        </is>
+      </c>
+      <c r="J352" s="18" t="inlineStr">
+        <is>
+          <t>Logged group enquiry record with O&amp;D, travel dates, pax count, and contact details</t>
+        </is>
+      </c>
+      <c r="K352" s="18" t="inlineStr">
+        <is>
+          <t>Request acknowledgement within 4 business hours; ≥95% SLA compliance</t>
+        </is>
+      </c>
+      <c r="L352" s="18" t="inlineStr">
+        <is>
+          <t>Requests arriving via multiple channels (email, GDS PNR, SWABIZ) require manual consolidation into Altéa — no single intake API across all channels</t>
+        </is>
+      </c>
+      <c r="M352" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N352" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="30" customHeight="1">
+      <c r="A353" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B353" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C353" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D353" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E353" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F353" s="16" t="inlineStr">
+        <is>
+          <t>Validate Group Size Eligibility</t>
+        </is>
+      </c>
+      <c r="G353" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H353" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I353" s="16" t="inlineStr">
+        <is>
+          <t>Passenger count stated in group request</t>
+        </is>
+      </c>
+      <c r="J353" s="16" t="inlineStr">
+        <is>
+          <t>Eligibility determination: group (≥10 pax) or retail redirection</t>
+        </is>
+      </c>
+      <c r="K353" s="16" t="inlineStr">
+        <is>
+          <t>100% of sub-threshold requests correctly redirected to retail within 1 business hour</t>
+        </is>
+      </c>
+      <c r="L353" s="16" t="inlineStr">
+        <is>
+          <t>Groups splitting into sub-10 clusters to access retail fares while exploiting group seat release policies — requires cross-PNR duplicate-name detection</t>
+        </is>
+      </c>
+      <c r="M353" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N353" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="30" customHeight="1">
+      <c r="A354" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B354" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C354" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D354" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E354" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F354" s="18" t="inlineStr">
+        <is>
+          <t>Check Blackout &amp; Peak Period Restrictions</t>
+        </is>
+      </c>
+      <c r="G354" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H354" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I354" s="18" t="inlineStr">
+        <is>
+          <t>Travel date range from group request; current peak calendar in NRM</t>
+        </is>
+      </c>
+      <c r="J354" s="18" t="inlineStr">
+        <is>
+          <t>Date eligibility flag; alternate date suggestions if blocked</t>
+        </is>
+      </c>
+      <c r="K354" s="18" t="inlineStr">
+        <is>
+          <t>Blackout date check completed in &lt;10 minutes; alternate date acceptance rate ≥40%</t>
+        </is>
+      </c>
+      <c r="L354" s="18" t="inlineStr">
+        <is>
+          <t>Peak calendars maintained manually in NRM and not automatically synced with marketing/events calendar — agents may quote blocked dates before checking</t>
+        </is>
+      </c>
+      <c r="M354" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N354" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="355" ht="30" customHeight="1">
+      <c r="A355" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B355" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C355" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D355" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E355" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F355" s="16" t="inlineStr">
+        <is>
+          <t>Confirm O&amp;D, Routing &amp; Itinerary</t>
+        </is>
+      </c>
+      <c r="G355" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H355" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I355" s="16" t="inlineStr">
+        <is>
+          <t>Validated group request with confirmed dates and pax count</t>
+        </is>
+      </c>
+      <c r="J355" s="16" t="inlineStr">
+        <is>
+          <t>Structured group itinerary record with flight segments and class of service</t>
+        </is>
+      </c>
+      <c r="K355" s="16" t="inlineStr">
+        <is>
+          <t>Itinerary confirmed and filed in PSS within 2 hours of initial request</t>
+        </is>
+      </c>
+      <c r="L355" s="16" t="inlineStr">
+        <is>
+          <t>Multi-segment itineraries require manual linking of PNRs across codeshare or interline partners — slow process for international group bookings</t>
+        </is>
+      </c>
+      <c r="M355" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N355" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="356" ht="30" customHeight="1">
+      <c r="A356" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B356" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C356" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D356" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E356" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F356" s="18" t="inlineStr">
+        <is>
+          <t>Query Real-Time O&amp;D Inventory Availability</t>
+        </is>
+      </c>
+      <c r="G356" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H356" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I356" s="18" t="inlineStr">
+        <is>
+          <t>Group itinerary with specific flight segments, dates, and fare class requirement</t>
+        </is>
+      </c>
+      <c r="J356" s="18" t="inlineStr">
+        <is>
+          <t>Current availability by booking class for each segment; load factor snapshot</t>
+        </is>
+      </c>
+      <c r="K356" s="18" t="inlineStr">
+        <is>
+          <t>Inventory query response in &lt;30 seconds; data freshness lag ≤5 minutes</t>
+        </is>
+      </c>
+      <c r="L356" s="18" t="inlineStr">
+        <is>
+          <t>NRM availability data can lag real-time PSS inventory by up to 5 minutes during high-volume periods — group blocks booked on stale data risk overbooking</t>
+        </is>
+      </c>
+      <c r="M356" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N356" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="30" customHeight="1">
+      <c r="A357" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B357" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C357" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D357" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E357" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F357" s="16" t="inlineStr">
+        <is>
+          <t>Run Displacement Cost Analysis</t>
+        </is>
+      </c>
+      <c r="G357" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H357" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I357" s="16" t="inlineStr">
+        <is>
+          <t>Requested seat block size; current booking curve; O&amp;D demand forecast from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J357" s="16" t="inlineStr">
+        <is>
+          <t>Displacement cost per seat (value of individual bookings that would be displaced); net revenue impact estimate</t>
+        </is>
+      </c>
+      <c r="K357" s="16" t="inlineStr">
+        <is>
+          <t>Displacement model accuracy ≥88% vs. actual realised revenue; analysis completed in &lt;15 minutes</t>
+        </is>
+      </c>
+      <c r="L357" s="16" t="inlineStr">
+        <is>
+          <t>Displacement models rely on NRM booking curves that may not fully account for last-minute premium fare uplift potential — groups in high-demand markets routinely under-priced</t>
+        </is>
+      </c>
+      <c r="M357" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N357" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="358" ht="30" customHeight="1">
+      <c r="A358" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B358" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C358" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D358" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E358" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F358" s="18" t="inlineStr">
+        <is>
+          <t>Assess Net Revenue Impact of Group Block</t>
+        </is>
+      </c>
+      <c r="G358" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H358" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I358" s="18" t="inlineStr">
+        <is>
+          <t>Displacement cost analysis; proposed group fare; seat block size</t>
+        </is>
+      </c>
+      <c r="J358" s="18" t="inlineStr">
+        <is>
+          <t>Net revenue positive/negative determination; RM recommendation (accept / reject / counter-date)</t>
+        </is>
+      </c>
+      <c r="K358" s="18" t="inlineStr">
+        <is>
+          <t>Group acceptance rate ≥65% of qualified requests; average group yield ≥85% of displacement cost</t>
+        </is>
+      </c>
+      <c r="L358" s="18" t="inlineStr">
+        <is>
+          <t>Sales teams operate under volume targets that incentivise accepting revenue-negative groups — tension between group sales quota and RM yield discipline</t>
+        </is>
+      </c>
+      <c r="M358" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N358" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="359" ht="30" customHeight="1">
+      <c r="A359" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B359" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C359" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D359" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E359" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F359" s="16" t="inlineStr">
+        <is>
+          <t>Calculate Block Fare Using Group Pricing Model</t>
+        </is>
+      </c>
+      <c r="G359" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H359" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I359" s="16" t="inlineStr">
+        <is>
+          <t>Net revenue impact assessment; group discount policy matrix; fare class availability</t>
+        </is>
+      </c>
+      <c r="J359" s="16" t="inlineStr">
+        <is>
+          <t>Proposed group fare per pax; total block revenue estimate</t>
+        </is>
+      </c>
+      <c r="K359" s="16" t="inlineStr">
+        <is>
+          <t>Group fare ≥95% of minimum acceptable yield threshold; pricing turnaround ≤30 minutes</t>
+        </is>
+      </c>
+      <c r="L359" s="16" t="inlineStr">
+        <is>
+          <t>Group pricing model does not natively integrate with ATPCO filed fares — group quotes are manual overrides that must be cross-checked against published fare rules to avoid BSP/ARC audit exceptions</t>
+        </is>
+      </c>
+      <c r="M359" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N359" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="360" ht="30" customHeight="1">
+      <c r="A360" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B360" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C360" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D360" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E360" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F360" s="18" t="inlineStr">
+        <is>
+          <t>Validate Fare Against Discount Authority Matrix</t>
+        </is>
+      </c>
+      <c r="G360" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H360" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I360" s="18" t="inlineStr">
+        <is>
+          <t>Proposed group fare; discount authority thresholds by market tier and season</t>
+        </is>
+      </c>
+      <c r="J360" s="18" t="inlineStr">
+        <is>
+          <t>Authority level determination: standard approval, RM manager review, or director escalation</t>
+        </is>
+      </c>
+      <c r="K360" s="18" t="inlineStr">
+        <is>
+          <t>100% of quotes validated against authority matrix before issue; zero out-of-authority quotes issued</t>
+        </is>
+      </c>
+      <c r="L360" s="18" t="inlineStr">
+        <is>
+          <t>Discount authority matrices are updated quarterly in spreadsheets and manually imported into NRM — stale thresholds lead to incorrect authority-level routing</t>
+        </is>
+      </c>
+      <c r="M360" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N360" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="361" ht="30" customHeight="1">
+      <c r="A361" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B361" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C361" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D361" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E361" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F361" s="16" t="inlineStr">
+        <is>
+          <t>Generate Formal Group Quote Document</t>
+        </is>
+      </c>
+      <c r="G361" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H361" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I361" s="16" t="inlineStr">
+        <is>
+          <t>Approved group fare; name release schedule; deposit terms; ticketing deadline</t>
+        </is>
+      </c>
+      <c r="J361" s="16" t="inlineStr">
+        <is>
+          <t>Formal group quote with fare, seat block, deposit amount, name release dates, and ticketing deadline</t>
+        </is>
+      </c>
+      <c r="K361" s="16" t="inlineStr">
+        <is>
+          <t>Quote issued within 24 hours of request receipt; quote acceptance rate ≥55%</t>
+        </is>
+      </c>
+      <c r="L361" s="16" t="inlineStr">
+        <is>
+          <t>Quote templates are maintained outside PSS in Word/PDF — manual population risks errors in fare amounts, deadlines, and contract terms; no audit trail within the booking system</t>
+        </is>
+      </c>
+      <c r="M361" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N361" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="362" ht="30" customHeight="1">
+      <c r="A362" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B362" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C362" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D362" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E362" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F362" s="18" t="inlineStr">
+        <is>
+          <t>Conduct Sales Negotiation with Group Organiser</t>
+        </is>
+      </c>
+      <c r="G362" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Manager</t>
+        </is>
+      </c>
+      <c r="H362" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM</t>
+        </is>
+      </c>
+      <c r="I362" s="18" t="inlineStr">
+        <is>
+          <t>Formal group quote; organiser counter-proposal (if any); competitive market rates</t>
+        </is>
+      </c>
+      <c r="J362" s="18" t="inlineStr">
+        <is>
+          <t>Agreed terms or revised counter-offer; negotiation log entry</t>
+        </is>
+      </c>
+      <c r="K362" s="18" t="inlineStr">
+        <is>
+          <t>Negotiation cycle ≤3 rounds to final agreement; average concession depth ≤5% below initial quote</t>
+        </is>
+      </c>
+      <c r="L362" s="18" t="inlineStr">
+        <is>
+          <t>Sales managers lack real-time competitive fare visibility during negotiation — competitors' group rates not available in PRISM, forcing reliance on OAG or manual fare searches</t>
+        </is>
+      </c>
+      <c r="M362" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N362" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="363" ht="30" customHeight="1">
+      <c r="A363" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B363" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C363" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D363" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E363" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F363" s="16" t="inlineStr">
+        <is>
+          <t>Obtain Final RM Approval for Confirmed Terms</t>
+        </is>
+      </c>
+      <c r="G363" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H363" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I363" s="16" t="inlineStr">
+        <is>
+          <t>Final agreed group terms; revenue impact recalculation at agreed fare</t>
+        </is>
+      </c>
+      <c r="J363" s="16" t="inlineStr">
+        <is>
+          <t>RM approval stamp; booking authority granted to sales team</t>
+        </is>
+      </c>
+      <c r="K363" s="16" t="inlineStr">
+        <is>
+          <t>Approval response within 4 business hours; ≤10% of groups requiring director-level escalation</t>
+        </is>
+      </c>
+      <c r="L363" s="16" t="inlineStr">
+        <is>
+          <t>Approval workflow is email-based with no system-enforced audit trail — SOX compliance reviews frequently flag missing RM sign-offs on large group bookings</t>
+        </is>
+      </c>
+      <c r="M363" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N363" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="364" ht="30" customHeight="1">
+      <c r="A364" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B364" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C364" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D364" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E364" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F364" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Group Booking &amp; Collect Deposit</t>
+        </is>
+      </c>
+      <c r="G364" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H364" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I364" s="18" t="inlineStr">
+        <is>
+          <t>RM approval; signed group contract; deposit payment from organiser</t>
+        </is>
+      </c>
+      <c r="J364" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed group PNR with seat block held; deposit receipt; booking confirmation to organiser</t>
+        </is>
+      </c>
+      <c r="K364" s="18" t="inlineStr">
+        <is>
+          <t>Deposit collection rate ≥98% of confirmed bookings; booking confirmation issued within 2 hours of receipt of signed contract</t>
+        </is>
+      </c>
+      <c r="L364" s="18" t="inlineStr">
+        <is>
+          <t>Deposit processing via bank transfer requires manual reconciliation against PNR in SAP S/4HANA Finance — 2-3 day lag between payment receipt and booking confirmation causes organiser escalations</t>
+        </is>
+      </c>
+      <c r="M364" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N364" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="365" ht="30" customHeight="1">
+      <c r="A365" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B365" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C365" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D365" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E365" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F365" s="16" t="inlineStr">
+        <is>
+          <t>Create Seat Block in PSS Inventory</t>
+        </is>
+      </c>
+      <c r="G365" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H365" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I365" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed group PNR; approved seat block size; fare class assignment</t>
+        </is>
+      </c>
+      <c r="J365" s="16" t="inlineStr">
+        <is>
+          <t>Hard-blocked seat inventory removed from open sale; group booking class activated</t>
+        </is>
+      </c>
+      <c r="K365" s="16" t="inlineStr">
+        <is>
+          <t>Seat block created within 1 hour of booking confirmation; zero inventory discrepancy vs. PNR</t>
+        </is>
+      </c>
+      <c r="L365" s="16" t="inlineStr">
+        <is>
+          <t>Hard blocks in Altéa reduce sellable capacity visible to GDS channels immediately — premature blocking of large groups in advance of name submission increases unsold seat risk</t>
+        </is>
+      </c>
+      <c r="M365" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N365" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="366" ht="30" customHeight="1">
+      <c r="A366" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B366" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C366" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D366" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E366" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F366" s="18" t="inlineStr">
+        <is>
+          <t>Monitor Name Release &amp; Ticketing Deadlines</t>
+        </is>
+      </c>
+      <c r="G366" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H366" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I366" s="18" t="inlineStr">
+        <is>
+          <t>Name release schedule from group contract; automated deadline alerts from PSS</t>
+        </is>
+      </c>
+      <c r="J366" s="18" t="inlineStr">
+        <is>
+          <t>Name submission status updates; reminder communications to group organiser</t>
+        </is>
+      </c>
+      <c r="K366" s="18" t="inlineStr">
+        <is>
+          <t>≥90% of names submitted by first release deadline; ticketing deadline breach rate &lt;5%</t>
+        </is>
+      </c>
+      <c r="L366" s="18" t="inlineStr">
+        <is>
+          <t>PSS deadline alerts are not integrated with CRM or email workflows — coordinators manually track deadlines in spreadsheets, leading to missed release dates and last-minute seat block management failures</t>
+        </is>
+      </c>
+      <c r="M366" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N366" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="367" ht="30" customHeight="1">
+      <c r="A367" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B367" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C367" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D367" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E367" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F367" s="16" t="inlineStr">
+        <is>
+          <t>Release Unsold Seats to Open Inventory</t>
+        </is>
+      </c>
+      <c r="G367" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H367" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I367" s="16" t="inlineStr">
+        <is>
+          <t>Final name count at ticketing deadline; remaining unoccupied seats in block</t>
+        </is>
+      </c>
+      <c r="J367" s="16" t="inlineStr">
+        <is>
+          <t>Released seats returned to NRM availability; booking class reopened for retail sale</t>
+        </is>
+      </c>
+      <c r="K367" s="16" t="inlineStr">
+        <is>
+          <t>Unsold seats released ≥72 hours before departure; recaptured revenue from released seats ≥60% of displacement cost on released units</t>
+        </is>
+      </c>
+      <c r="L367" s="16" t="inlineStr">
+        <is>
+          <t>Late seat release (within 72 hours of departure) significantly reduces recapture probability — NRM booking curves flatten below T-3 days, leaving released group seats unsold and generating direct revenue loss</t>
+        </is>
+      </c>
+      <c r="M367" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N367" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="368" ht="30" customHeight="1">
+      <c r="A368" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B368" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C368" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D368" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E368" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F368" s="18" t="inlineStr">
+        <is>
+          <t>Process Final Passenger Manifest &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="G368" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H368" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I368" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmed passenger names; actual tickets issued; deposit and balance payment records</t>
+        </is>
+      </c>
+      <c r="J368" s="18" t="inlineStr">
+        <is>
+          <t>Closed group PNR; final invoice; payment settled in SAP S/4HANA Finance</t>
+        </is>
+      </c>
+      <c r="K368" s="18" t="inlineStr">
+        <is>
+          <t>Final settlement completed within 5 business days post-travel; payment reconciliation accuracy ≥99.5%</t>
+        </is>
+      </c>
+      <c r="L368" s="18" t="inlineStr">
+        <is>
+          <t>Name changes and no-shows on group bookings trigger penalty fee calculations that must be manually computed and re-invoiced — no automated penalty engine in Altéa for group contracts</t>
+        </is>
+      </c>
+      <c r="M368" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N368" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="30" customHeight="1">
+      <c r="A369" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B369" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C369" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D369" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E369" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F369" s="16" t="inlineStr">
+        <is>
+          <t>Calculate Revenue Variance vs. Forecast</t>
+        </is>
+      </c>
+      <c r="G369" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H369" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I369" s="16" t="inlineStr">
+        <is>
+          <t>Actual group revenue from SAP FI; forecast revenue from NRM displacement model; seat block utilisation data</t>
+        </is>
+      </c>
+      <c r="J369" s="16" t="inlineStr">
+        <is>
+          <t>Revenue variance report; yield performance vs. plan; group booking contribution analysis</t>
+        </is>
+      </c>
+      <c r="K369" s="16" t="inlineStr">
+        <is>
+          <t>Forecast vs. actual variance ≤8%; group contribution to total flight revenue ≥12% on applicable routes</t>
+        </is>
+      </c>
+      <c r="L369" s="16" t="inlineStr">
+        <is>
+          <t>Revenue data from SAP FI and NRM actuals must be joined manually in Redshift — no automated group P&amp;L dashboard; variance analysis delayed by 2-3 days post-travel</t>
+        </is>
+      </c>
+      <c r="M369" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N369" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="370" ht="30" customHeight="1">
+      <c r="A370" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B370" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C370" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D370" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E370" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F370" s="18" t="inlineStr">
+        <is>
+          <t>Update RM Demand Forecasting Model with Actuals</t>
+        </is>
+      </c>
+      <c r="G370" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H370" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I370" s="18" t="inlineStr">
+        <is>
+          <t>Revenue variance report; actual load factor contribution from group block; group yield data</t>
+        </is>
+      </c>
+      <c r="J370" s="18" t="inlineStr">
+        <is>
+          <t>Updated demand coefficients in NRM forecasting model; group segment historical database entry</t>
+        </is>
+      </c>
+      <c r="K370" s="18" t="inlineStr">
+        <is>
+          <t>Model update completed within 10 business days post-travel; forecast accuracy improvement of ≥0.5% per cycle</t>
+        </is>
+      </c>
+      <c r="L370" s="18" t="inlineStr">
+        <is>
+          <t>NRM group booking actuals are not automatically tagged separately from retail bookings — group demand is blended into overall O&amp;D forecasts, distorting unconstrained demand estimates and causing systematic over-forecasting on high-group-volume routes</t>
+        </is>
+      </c>
+      <c r="M370" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N370" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-05 — Group Sales Revenue Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Group Sales Revenue Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Receive Group Booking Request</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request via SWABIZ portal, GDS, travel agency, or direct sales channel</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Logged group enquiry record with O&amp;D, travel dates, pax count, and contact details</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Request acknowledgement within 4 business hours; ≥95% SLA compliance</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Requests arriving via multiple channels (email, GDS PNR, SWABIZ) require manual consolidation into Altéa — no single intake API across all channels</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Validate Group Size Eligibility</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Passenger count stated in group request</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Eligibility determination: group (≥10 pax) or retail redirection</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>100% of sub-threshold requests correctly redirected to retail within 1 business hour</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Groups splitting into sub-10 clusters to access retail fares while exploiting group seat release policies — requires cross-PNR duplicate-name detection</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Check Blackout &amp; Peak Period Restrictions</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Travel date range from group request; current peak calendar in NRM</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Date eligibility flag; alternate date suggestions if blocked</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Blackout date check completed in &lt;10 minutes; alternate date acceptance rate ≥40%</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Peak calendars maintained manually in NRM and not automatically synced with marketing/events calendar — agents may quote blocked dates before checking</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Confirm O&amp;D, Routing &amp; Itinerary</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Validated group request with confirmed dates and pax count</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Structured group itinerary record with flight segments and class of service</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Itinerary confirmed and filed in PSS within 2 hours of initial request</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Multi-segment itineraries require manual linking of PNRs across codeshare or interline partners — slow process for international group bookings</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Query Real-Time O&amp;D Inventory Availability</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Group itinerary with specific flight segments, dates, and fare class requirement</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Current availability by booking class for each segment; load factor snapshot</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Inventory query response in &lt;30 seconds; data freshness lag ≤5 minutes</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>NRM availability data can lag real-time PSS inventory by up to 5 minutes during high-volume periods — group blocks booked on stale data risk overbooking</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Run Displacement Cost Analysis</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Requested seat block size; current booking curve; O&amp;D demand forecast from SkyCAST</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Displacement cost per seat (value of individual bookings that would be displaced); net revenue impact estimate</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Displacement model accuracy ≥88% vs. actual realised revenue; analysis completed in &lt;15 minutes</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Displacement models rely on NRM booking curves that may not fully account for last-minute premium fare uplift potential — groups in high-demand markets routinely under-priced</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Assess Net Revenue Impact of Group Block</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Displacement cost analysis; proposed group fare; seat block size</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Net revenue positive/negative determination; RM recommendation (accept / reject / counter-date)</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Group acceptance rate ≥65% of qualified requests; average group yield ≥85% of displacement cost</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Sales teams operate under volume targets that incentivise accepting revenue-negative groups — tension between group sales quota and RM yield discipline</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Calculate Block Fare Using Group Pricing Model</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Net revenue impact assessment; group discount policy matrix; fare class availability</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Proposed group fare per pax; total block revenue estimate</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Group fare ≥95% of minimum acceptable yield threshold; pricing turnaround ≤30 minutes</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Group pricing model does not natively integrate with ATPCO filed fares — group quotes are manual overrides that must be cross-checked against published fare rules to avoid BSP/ARC audit exceptions</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Validate Fare Against Discount Authority Matrix</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Proposed group fare; discount authority thresholds by market tier and season</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Authority level determination: standard approval, RM manager review, or director escalation</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>100% of quotes validated against authority matrix before issue; zero out-of-authority quotes issued</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Discount authority matrices are updated quarterly in spreadsheets and manually imported into NRM — stale thresholds lead to incorrect authority-level routing</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Generate Formal Group Quote Document</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Approved group fare; name release schedule; deposit terms; ticketing deadline</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Formal group quote with fare, seat block, deposit amount, name release dates, and ticketing deadline</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Quote issued within 24 hours of request receipt; quote acceptance rate ≥55%</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Quote templates are maintained outside PSS in Word/PDF — manual population risks errors in fare amounts, deadlines, and contract terms; no audit trail within the booking system</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Conduct Sales Negotiation with Group Organiser</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Formal group quote; organiser counter-proposal (if any); competitive market rates</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Agreed terms or revised counter-offer; negotiation log entry</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Negotiation cycle ≤3 rounds to final agreement; average concession depth ≤5% below initial quote</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Sales managers lack real-time competitive fare visibility during negotiation — competitors' group rates not available in PRISM, forcing reliance on OAG or manual fare searches</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Obtain Final RM Approval for Confirmed Terms</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Final agreed group terms; revenue impact recalculation at agreed fare</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>RM approval stamp; booking authority granted to sales team</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Approval response within 4 business hours; ≤10% of groups requiring director-level escalation</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Approval workflow is email-based with no system-enforced audit trail — SOX compliance reviews frequently flag missing RM sign-offs on large group bookings</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Group Booking &amp; Collect Deposit</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>RM approval; signed group contract; deposit payment from organiser</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed group PNR with seat block held; deposit receipt; booking confirmation to organiser</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Deposit collection rate ≥98% of confirmed bookings; booking confirmation issued within 2 hours of receipt of signed contract</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Deposit processing via bank transfer requires manual reconciliation against PNR in SAP S/4HANA Finance — 2-3 day lag between payment receipt and booking confirmation causes organiser escalations</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Create Seat Block in PSS Inventory</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed group PNR; approved seat block size; fare class assignment</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Hard-blocked seat inventory removed from open sale; group booking class activated</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Seat block created within 1 hour of booking confirmation; zero inventory discrepancy vs. PNR</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Hard blocks in Altéa reduce sellable capacity visible to GDS channels immediately — premature blocking of large groups in advance of name submission increases unsold seat risk</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Monitor Name Release &amp; Ticketing Deadlines</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Name release schedule from group contract; automated deadline alerts from PSS</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Name submission status updates; reminder communications to group organiser</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>≥90% of names submitted by first release deadline; ticketing deadline breach rate &lt;5%</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>PSS deadline alerts are not integrated with CRM or email workflows — coordinators manually track deadlines in spreadsheets, leading to missed release dates and last-minute seat block management failures</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Release Unsold Seats to Open Inventory</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Final name count at ticketing deadline; remaining unoccupied seats in block</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Released seats returned to NRM availability; booking class reopened for retail sale</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Unsold seats released ≥72 hours before departure; recaptured revenue from released seats ≥60% of displacement cost on released units</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Late seat release (within 72 hours of departure) significantly reduces recapture probability — NRM booking curves flatten below T-3 days, leaving released group seats unsold and generating direct revenue loss</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Process Final Passenger Manifest &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmed passenger names; actual tickets issued; deposit and balance payment records</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Closed group PNR; final invoice; payment settled in SAP S/4HANA Finance</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Final settlement completed within 5 business days post-travel; payment reconciliation accuracy ≥99.5%</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Name changes and no-shows on group bookings trigger penalty fee calculations that must be manually computed and re-invoiced — no automated penalty engine in Altéa for group contracts</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Calculate Revenue Variance vs. Forecast</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Actual group revenue from SAP FI; forecast revenue from NRM displacement model; seat block utilisation data</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue variance report; yield performance vs. plan; group booking contribution analysis</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Forecast vs. actual variance ≤8%; group contribution to total flight revenue ≥12% on applicable routes</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue data from SAP FI and NRM actuals must be joined manually in Redshift — no automated group P&amp;L dashboard; variance analysis delayed by 2-3 days post-travel</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-05</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Revenue Management</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Update RM Demand Forecasting Model with Actuals</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Revenue variance report; actual load factor contribution from group block; group yield data</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Updated demand coefficients in NRM forecasting model; group segment historical database entry</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>Model update completed within 10 business days post-travel; forecast accuracy improvement of ≥0.5% per cycle</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>NRM group booking actuals are not automatically tagged separately from retail bookings — group demand is blended into overall O&amp;D forecasts, distorting unconstrained demand estimates and causing systematic over-forecasting on high-group-volume routes</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add NP-RM-06: Upgrade & Upsell Revenue Optimization — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -27,6 +27,7 @@
     <sheet name="NP-RM-03" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="NP-RM-04" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="NP-RM-05" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="NP-RM-06" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1408,13 +1409,21 @@
           <t>Upgrade &amp; Upsell Revenue Optimization</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr"/>
-      <c r="G23" s="10" t="inlineStr"/>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-06</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -18792,7 +18801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N370"/>
+  <dimension ref="A1:N387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -45381,6 +45390,1230 @@
         </is>
       </c>
       <c r="N370" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="371" ht="30" customHeight="1">
+      <c r="A371" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B371" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C371" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D371" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E371" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F371" s="16" t="inlineStr">
+        <is>
+          <t>Extract PNR data for upsell candidate pool</t>
+        </is>
+      </c>
+      <c r="G371" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H371" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I371" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed bookings within 72-hour pre-departure window</t>
+        </is>
+      </c>
+      <c r="J371" s="16" t="inlineStr">
+        <is>
+          <t>Upsell candidate PNR list with cabin class, fare basis, and loyalty tier</t>
+        </is>
+      </c>
+      <c r="K371" s="16" t="inlineStr">
+        <is>
+          <t>Candidate pool coverage ≥95% of eligible bookings extracted</t>
+        </is>
+      </c>
+      <c r="L371" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PNR data exports can lag up to 15 min during peak schedule periods, narrowing the actionable upsell window for close-in departures</t>
+        </is>
+      </c>
+      <c r="M371" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N371" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="372" ht="30" customHeight="1">
+      <c r="A372" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B372" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C372" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D372" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E372" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F372" s="18" t="inlineStr">
+        <is>
+          <t>Score passengers using willingness-to-pay model</t>
+        </is>
+      </c>
+      <c r="G372" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Data Scientist</t>
+        </is>
+      </c>
+      <c r="H372" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I372" s="18" t="inlineStr">
+        <is>
+          <t>PNR list, historical upsell acceptance data, loyalty tier, booking channel</t>
+        </is>
+      </c>
+      <c r="J372" s="18" t="inlineStr">
+        <is>
+          <t>WTP score (0–100) and predicted upgrade revenue per passenger</t>
+        </is>
+      </c>
+      <c r="K372" s="18" t="inlineStr">
+        <is>
+          <t>WTP model accuracy ≥82% (lift vs. random baseline on holdout set)</t>
+        </is>
+      </c>
+      <c r="L372" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM WTP models trained on pre-COVID data can overestimate premium-cabin demand for leisure-heavy route clusters; requires quarterly recalibration</t>
+        </is>
+      </c>
+      <c r="M372" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N372" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" ht="30" customHeight="1">
+      <c r="A373" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B373" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C373" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D373" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E373" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F373" s="16" t="inlineStr">
+        <is>
+          <t>Check premium cabin inventory for upgrade availability</t>
+        </is>
+      </c>
+      <c r="G373" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H373" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I373" s="16" t="inlineStr">
+        <is>
+          <t>Flight departure date, cabin class inventory snapshot, current load factor by cabin</t>
+        </is>
+      </c>
+      <c r="J373" s="16" t="inlineStr">
+        <is>
+          <t>Available upgrade seats per cabin class per flight</t>
+        </is>
+      </c>
+      <c r="K373" s="16" t="inlineStr">
+        <is>
+          <t>Premium cabin upgrade seat availability query response time &lt;2 sec</t>
+        </is>
+      </c>
+      <c r="L373" s="16" t="inlineStr">
+        <is>
+          <t>Real-time seat availability from AltéaRM can conflict with GDS inventory counts when passive segments are not cancelled promptly, creating ghost-availability errors</t>
+        </is>
+      </c>
+      <c r="M373" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N373" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="30" customHeight="1">
+      <c r="A374" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B374" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C374" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D374" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E374" s="17" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F374" s="18" t="inlineStr">
+        <is>
+          <t>Segment eligible passengers by WTP tier and route</t>
+        </is>
+      </c>
+      <c r="G374" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H374" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I374" s="18" t="inlineStr">
+        <is>
+          <t>WTP scores, available upgrade inventory, route premium demand index</t>
+        </is>
+      </c>
+      <c r="J374" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised upsell target list segmented into High / Medium / Low WTP tiers</t>
+        </is>
+      </c>
+      <c r="K374" s="18" t="inlineStr">
+        <is>
+          <t>High-WTP tier (score ≥70) constitutes ≥30% of total candidate pool</t>
+        </is>
+      </c>
+      <c r="L374" s="18" t="inlineStr">
+        <is>
+          <t>Loyalty programme members in lower fare classes are frequently misclassified as low-WTP due to sparse ancillary purchase history in PROS RM</t>
+        </is>
+      </c>
+      <c r="M374" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N374" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="30" customHeight="1">
+      <c r="A375" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B375" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C375" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D375" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E375" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F375" s="16" t="inlineStr">
+        <is>
+          <t>Generate dynamic upgrade offer price per passenger</t>
+        </is>
+      </c>
+      <c r="G375" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Analyst</t>
+        </is>
+      </c>
+      <c r="H375" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I375" s="16" t="inlineStr">
+        <is>
+          <t>WTP score, fare differential (booked fare vs. premium cabin fare), route load factor</t>
+        </is>
+      </c>
+      <c r="J375" s="16" t="inlineStr">
+        <is>
+          <t>Personalised upgrade offer price in local currency</t>
+        </is>
+      </c>
+      <c r="K375" s="16" t="inlineStr">
+        <is>
+          <t>Average upgrade offer price within 15% of O&amp;D revenue maximisation model output</t>
+        </is>
+      </c>
+      <c r="L375" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM dynamic pricing engine does not natively ingest competitor same-day premium fare data, requiring manual competitive adjustment for price-sensitive O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="M375" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N375" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="30" customHeight="1">
+      <c r="A376" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B376" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C376" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D376" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E376" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F376" s="18" t="inlineStr">
+        <is>
+          <t>Apply ATPCO fare floor and ceiling constraints</t>
+        </is>
+      </c>
+      <c r="G376" s="18" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H376" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I376" s="18" t="inlineStr">
+        <is>
+          <t>Generated offer price, filed fare rules (Rule 010 / 015), minimum fare differentials</t>
+        </is>
+      </c>
+      <c r="J376" s="18" t="inlineStr">
+        <is>
+          <t>Validated upgrade offer price compliant with ATPCO fare rules</t>
+        </is>
+      </c>
+      <c r="K376" s="18" t="inlineStr">
+        <is>
+          <t>100% of published upgrade offers compliant with ATPCO Cat 25 negotiated fare rules</t>
+        </is>
+      </c>
+      <c r="L376" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO Cat 25 rule interpretation varies across PSS implementations; non-compliant upgrade offers can trigger GDS mis-pricing alerts and require emergency fare recall</t>
+        </is>
+      </c>
+      <c r="M376" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N376" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="30" customHeight="1">
+      <c r="A377" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B377" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C377" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D377" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E377" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F377" s="16" t="inlineStr">
+        <is>
+          <t>Bundle ancillary services with upgrade offer</t>
+        </is>
+      </c>
+      <c r="G377" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H377" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I377" s="16" t="inlineStr">
+        <is>
+          <t>Validated upgrade price, ancillary catalogue (lounge, extra baggage, priority boarding)</t>
+        </is>
+      </c>
+      <c r="J377" s="16" t="inlineStr">
+        <is>
+          <t>Bundled upsell offer package with itemised ancillary pricing</t>
+        </is>
+      </c>
+      <c r="K377" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary attach rate per upgrade offer ≥40% on applicable routes</t>
+        </is>
+      </c>
+      <c r="L377" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway bundle assembly fails when ancillary inventory systems (lounge access, seat maps) return timeout errors, forcing fallback to offer-only pricing with no bundle</t>
+        </is>
+      </c>
+      <c r="M377" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N377" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="30" customHeight="1">
+      <c r="A378" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B378" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C378" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D378" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E378" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F378" s="18" t="inlineStr">
+        <is>
+          <t>Publish upgrade offers via web check-in and mobile app</t>
+        </is>
+      </c>
+      <c r="G378" s="18" t="inlineStr">
+        <is>
+          <t>Digital Channel Manager</t>
+        </is>
+      </c>
+      <c r="H378" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I378" s="18" t="inlineStr">
+        <is>
+          <t>Bundled upgrade offer packages, passenger contact details from Altéa PSS</t>
+        </is>
+      </c>
+      <c r="J378" s="18" t="inlineStr">
+        <is>
+          <t>Live upsell offer presented in web check-in and airline mobile app</t>
+        </is>
+      </c>
+      <c r="K378" s="18" t="inlineStr">
+        <is>
+          <t>Offer display latency &lt;3 sec for ≥98% of web check-in sessions</t>
+        </is>
+      </c>
+      <c r="L378" s="18" t="inlineStr">
+        <is>
+          <t>NDC API retries during high-volume check-in peaks (T-24h departure) cause duplicate offer display or blank offer panels, degrading conversion rate</t>
+        </is>
+      </c>
+      <c r="M378" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N378" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="30" customHeight="1">
+      <c r="A379" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B379" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C379" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D379" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E379" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F379" s="16" t="inlineStr">
+        <is>
+          <t>Send targeted upsell email and push notifications</t>
+        </is>
+      </c>
+      <c r="G379" s="16" t="inlineStr">
+        <is>
+          <t>CRM Campaign Manager</t>
+        </is>
+      </c>
+      <c r="H379" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I379" s="16" t="inlineStr">
+        <is>
+          <t>Segmented passenger list with personalised offer price, departure T-48h and T-24h triggers</t>
+        </is>
+      </c>
+      <c r="J379" s="16" t="inlineStr">
+        <is>
+          <t>Email and push notification delivered with personalised upgrade CTA</t>
+        </is>
+      </c>
+      <c r="K379" s="16" t="inlineStr">
+        <is>
+          <t>Email open rate ≥28%; push notification click-through rate ≥12%</t>
+        </is>
+      </c>
+      <c r="L379" s="16" t="inlineStr">
+        <is>
+          <t>Altéa CRM notification engine does not suppress duplicate messages when passengers have both web and mobile sessions active, leading to over-communication complaints</t>
+        </is>
+      </c>
+      <c r="M379" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N379" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="380" ht="30" customHeight="1">
+      <c r="A380" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B380" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C380" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D380" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E380" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F380" s="18" t="inlineStr">
+        <is>
+          <t>Display upgrade prompts at airport check-in and kiosk</t>
+        </is>
+      </c>
+      <c r="G380" s="18" t="inlineStr">
+        <is>
+          <t>Airport Check-in Agent</t>
+        </is>
+      </c>
+      <c r="H380" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I380" s="18" t="inlineStr">
+        <is>
+          <t>Passenger check-in event, remaining upgrade inventory from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J380" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade upsell prompt displayed to agent and self-service kiosk</t>
+        </is>
+      </c>
+      <c r="K380" s="18" t="inlineStr">
+        <is>
+          <t>Airport upgrade conversion rate ≥8% of prompted passengers</t>
+        </is>
+      </c>
+      <c r="L380" s="18" t="inlineStr">
+        <is>
+          <t>SITA AMS kiosk software version lag (often 2+ major releases behind) causes offer display failures on older kiosk hardware at smaller outstations</t>
+        </is>
+      </c>
+      <c r="M380" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N380" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" ht="30" customHeight="1">
+      <c r="A381" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B381" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C381" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D381" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E381" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F381" s="16" t="inlineStr">
+        <is>
+          <t>Process upgrade payment via preferred channel</t>
+        </is>
+      </c>
+      <c r="G381" s="16" t="inlineStr">
+        <is>
+          <t>Airport Check-in Agent / Passenger (self-service)</t>
+        </is>
+      </c>
+      <c r="H381" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I381" s="16" t="inlineStr">
+        <is>
+          <t>Passenger acceptance of upgrade offer, payment card or loyalty points balance</t>
+        </is>
+      </c>
+      <c r="J381" s="16" t="inlineStr">
+        <is>
+          <t>Payment transaction record; EMD (Electronic Miscellaneous Document) issued</t>
+        </is>
+      </c>
+      <c r="K381" s="16" t="inlineStr">
+        <is>
+          <t>Payment processing success rate ≥98.5%; transaction time &lt;10 sec</t>
+        </is>
+      </c>
+      <c r="L381" s="16" t="inlineStr">
+        <is>
+          <t>Altéa EMD issuance for upgrade payments using loyalty currency (miles + cash) requires manual fare recalculation when the loyalty system API returns stale balance data</t>
+        </is>
+      </c>
+      <c r="M381" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N381" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="382" ht="30" customHeight="1">
+      <c r="A382" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B382" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C382" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D382" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E382" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F382" s="18" t="inlineStr">
+        <is>
+          <t>Reassign seat and update PNR cabin class</t>
+        </is>
+      </c>
+      <c r="G382" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System (automated)</t>
+        </is>
+      </c>
+      <c r="H382" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I382" s="18" t="inlineStr">
+        <is>
+          <t>Authorised payment confirmation, available premium cabin seat map</t>
+        </is>
+      </c>
+      <c r="J382" s="18" t="inlineStr">
+        <is>
+          <t>PNR updated with new cabin class, seat assignment, and fare basis code</t>
+        </is>
+      </c>
+      <c r="K382" s="18" t="inlineStr">
+        <is>
+          <t>PNR update latency &lt;5 sec; zero duplicate seat assignment errors per 10,000 upgrades</t>
+        </is>
+      </c>
+      <c r="L382" s="18" t="inlineStr">
+        <is>
+          <t>Concurrent upgrade processing for the same flight can cause seat-map race conditions in Altéa when two agents process the last available premium seat simultaneously</t>
+        </is>
+      </c>
+      <c r="M382" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N382" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="383" ht="30" customHeight="1">
+      <c r="A383" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B383" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C383" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D383" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E383" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F383" s="16" t="inlineStr">
+        <is>
+          <t>Provision premium cabin services and lounge access</t>
+        </is>
+      </c>
+      <c r="G383" s="16" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H383" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I383" s="16" t="inlineStr">
+        <is>
+          <t>Updated PNR with premium cabin indicator, lounge contract entitlements</t>
+        </is>
+      </c>
+      <c r="J383" s="16" t="inlineStr">
+        <is>
+          <t>Lounge access pass issued; premium meal and amenity kit flagged for catering</t>
+        </is>
+      </c>
+      <c r="K383" s="16" t="inlineStr">
+        <is>
+          <t>Premium service provisioning lead time ≥45 min before departure for ≥95% of upgrades</t>
+        </is>
+      </c>
+      <c r="L383" s="16" t="inlineStr">
+        <is>
+          <t>Catering uplift amendments post-upgrade are frequently missed when the upgrade is processed inside the catering finality window (T-2h), resulting in insufficient premium meals</t>
+        </is>
+      </c>
+      <c r="M383" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N383" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" ht="30" customHeight="1">
+      <c r="A384" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B384" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C384" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D384" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E384" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F384" s="18" t="inlineStr">
+        <is>
+          <t>Send upgrade confirmation and boarding pass to passenger</t>
+        </is>
+      </c>
+      <c r="G384" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System (automated)</t>
+        </is>
+      </c>
+      <c r="H384" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I384" s="18" t="inlineStr">
+        <is>
+          <t>PNR update complete, new boarding pass data, passenger email / mobile</t>
+        </is>
+      </c>
+      <c r="J384" s="18" t="inlineStr">
+        <is>
+          <t>Updated boarding pass (mobile and printable) and upgrade confirmation email</t>
+        </is>
+      </c>
+      <c r="K384" s="18" t="inlineStr">
+        <is>
+          <t>Confirmation delivery within 60 sec of PNR update for ≥99% of upgrades</t>
+        </is>
+      </c>
+      <c r="L384" s="18" t="inlineStr">
+        <is>
+          <t>Mobile boarding pass push fails for passengers using third-party wallet apps (non-Apple/Google Wallet) when Altéa PKPass API returns certificate validation errors</t>
+        </is>
+      </c>
+      <c r="M384" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N384" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" ht="30" customHeight="1">
+      <c r="A385" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B385" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C385" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D385" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E385" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F385" s="16" t="inlineStr">
+        <is>
+          <t>Aggregate upsell revenue and conversion metrics</t>
+        </is>
+      </c>
+      <c r="G385" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Analytics Analyst</t>
+        </is>
+      </c>
+      <c r="H385" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I385" s="16" t="inlineStr">
+        <is>
+          <t>EMD transaction records, PNR cabin upgrade events, offer impression logs</t>
+        </is>
+      </c>
+      <c r="J385" s="16" t="inlineStr">
+        <is>
+          <t>Daily upsell revenue report: impressions, conversions, revenue per upgrade, channel mix</t>
+        </is>
+      </c>
+      <c r="K385" s="16" t="inlineStr">
+        <is>
+          <t>Upsell revenue per available seat ≥$12 on applicable routes; daily report SLA &lt;6h after day-end</t>
+        </is>
+      </c>
+      <c r="L385" s="16" t="inlineStr">
+        <is>
+          <t>EMD revenue attribution in AWS Redshift is delayed by up to 4h due to batch ingestion from Altéa, preventing same-day intra-day optimisation of pricing parameters</t>
+        </is>
+      </c>
+      <c r="M385" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N385" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="30" customHeight="1">
+      <c r="A386" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B386" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C386" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D386" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E386" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F386" s="18" t="inlineStr">
+        <is>
+          <t>Compare actuals vs. forecast upsell revenue targets</t>
+        </is>
+      </c>
+      <c r="G386" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H386" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I386" s="18" t="inlineStr">
+        <is>
+          <t>Daily upsell revenue report, budgeted upsell revenue targets by route cluster</t>
+        </is>
+      </c>
+      <c r="J386" s="18" t="inlineStr">
+        <is>
+          <t>Variance report: actual vs. forecast with root-cause flags (pricing, inventory, channel)</t>
+        </is>
+      </c>
+      <c r="K386" s="18" t="inlineStr">
+        <is>
+          <t>Upsell revenue forecast accuracy within ±10% of actuals on rolling 7-day basis</t>
+        </is>
+      </c>
+      <c r="L386" s="18" t="inlineStr">
+        <is>
+          <t>Tableau dashboards pulling from AWS Redshift frequently timeout on full-network route-cluster queries, forcing analysts to run ad-hoc SQL instead of using governed reports</t>
+        </is>
+      </c>
+      <c r="M386" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N386" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="30" customHeight="1">
+      <c r="A387" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B387" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C387" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D387" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E387" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F387" s="16" t="inlineStr">
+        <is>
+          <t>Recalibrate WTP model and pricing parameters</t>
+        </is>
+      </c>
+      <c r="G387" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Data Scientist</t>
+        </is>
+      </c>
+      <c r="H387" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I387" s="16" t="inlineStr">
+        <is>
+          <t>Variance report, offer acceptance/rejection data, competitor fare changes from OAG</t>
+        </is>
+      </c>
+      <c r="J387" s="16" t="inlineStr">
+        <is>
+          <t>Updated WTP model weights; revised pricing floor and ceiling parameters in PROS RM</t>
+        </is>
+      </c>
+      <c r="K387" s="16" t="inlineStr">
+        <is>
+          <t>WTP model recalibration cycle ≤7 days after conversion target miss; post-recalibration lift ≥5%</t>
+        </is>
+      </c>
+      <c r="L387" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM model retraining requires a minimum 90-day historical acceptance dataset; insufficient data on new routes or post-schedule-change periods degrades model quality for at least one quarter</t>
+        </is>
+      </c>
+      <c r="M387" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N387" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -46868,6 +48101,1350 @@
         </is>
       </c>
       <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-06 — Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract PNR data for upsell candidate pool</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed bookings within 72-hour pre-departure window</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Upsell candidate PNR list with cabin class, fare basis, and loyalty tier</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Candidate pool coverage ≥95% of eligible bookings extracted</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PNR data exports can lag up to 15 min during peak schedule periods, narrowing the actionable upsell window for close-in departures</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Score passengers using willingness-to-pay model</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Data Scientist</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>PNR list, historical upsell acceptance data, loyalty tier, booking channel</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>WTP score (0–100) and predicted upgrade revenue per passenger</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>WTP model accuracy ≥82% (lift vs. random baseline on holdout set)</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM WTP models trained on pre-COVID data can overestimate premium-cabin demand for leisure-heavy route clusters; requires quarterly recalibration</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Check premium cabin inventory for upgrade availability</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Flight departure date, cabin class inventory snapshot, current load factor by cabin</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Available upgrade seats per cabin class per flight</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Premium cabin upgrade seat availability query response time &lt;2 sec</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Real-time seat availability from AltéaRM can conflict with GDS inventory counts when passive segments are not cancelled promptly, creating ghost-availability errors</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Segment eligible passengers by WTP tier and route</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>WTP scores, available upgrade inventory, route premium demand index</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Prioritised upsell target list segmented into High / Medium / Low WTP tiers</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>High-WTP tier (score ≥70) constitutes ≥30% of total candidate pool</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Loyalty programme members in lower fare classes are frequently misclassified as low-WTP due to sparse ancillary purchase history in PROS RM</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Generate dynamic upgrade offer price per passenger</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>WTP score, fare differential (booked fare vs. premium cabin fare), route load factor</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Personalised upgrade offer price in local currency</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Average upgrade offer price within 15% of O&amp;D revenue maximisation model output</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM dynamic pricing engine does not natively ingest competitor same-day premium fare data, requiring manual competitive adjustment for price-sensitive O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Apply ATPCO fare floor and ceiling constraints</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Generated offer price, filed fare rules (Rule 010 / 015), minimum fare differentials</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Validated upgrade offer price compliant with ATPCO fare rules</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>100% of published upgrade offers compliant with ATPCO Cat 25 negotiated fare rules</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO Cat 25 rule interpretation varies across PSS implementations; non-compliant upgrade offers can trigger GDS mis-pricing alerts and require emergency fare recall</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Bundle ancillary services with upgrade offer</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Validated upgrade price, ancillary catalogue (lounge, extra baggage, priority boarding)</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Bundled upsell offer package with itemised ancillary pricing</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary attach rate per upgrade offer ≥40% on applicable routes</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway bundle assembly fails when ancillary inventory systems (lounge access, seat maps) return timeout errors, forcing fallback to offer-only pricing with no bundle</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Publish upgrade offers via web check-in and mobile app</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Digital Channel Manager</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Bundled upgrade offer packages, passenger contact details from Altéa PSS</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Live upsell offer presented in web check-in and airline mobile app</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Offer display latency &lt;3 sec for ≥98% of web check-in sessions</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>NDC API retries during high-volume check-in peaks (T-24h departure) cause duplicate offer display or blank offer panels, degrading conversion rate</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Send targeted upsell email and push notifications</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>CRM Campaign Manager</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Segmented passenger list with personalised offer price, departure T-48h and T-24h triggers</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Email and push notification delivered with personalised upgrade CTA</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Email open rate ≥28%; push notification click-through rate ≥12%</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Altéa CRM notification engine does not suppress duplicate messages when passengers have both web and mobile sessions active, leading to over-communication complaints</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Display upgrade prompts at airport check-in and kiosk</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Airport Check-in Agent</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Passenger check-in event, remaining upgrade inventory from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade upsell prompt displayed to agent and self-service kiosk</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Airport upgrade conversion rate ≥8% of prompted passengers</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>SITA AMS kiosk software version lag (often 2+ major releases behind) causes offer display failures on older kiosk hardware at smaller outstations</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Process upgrade payment via preferred channel</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Airport Check-in Agent / Passenger (self-service)</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Passenger acceptance of upgrade offer, payment card or loyalty points balance</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Payment transaction record; EMD (Electronic Miscellaneous Document) issued</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Payment processing success rate ≥98.5%; transaction time &lt;10 sec</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Altéa EMD issuance for upgrade payments using loyalty currency (miles + cash) requires manual fare recalculation when the loyalty system API returns stale balance data</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Reassign seat and update PNR cabin class</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System (automated)</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Authorised payment confirmation, available premium cabin seat map</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>PNR updated with new cabin class, seat assignment, and fare basis code</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>PNR update latency &lt;5 sec; zero duplicate seat assignment errors per 10,000 upgrades</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Concurrent upgrade processing for the same flight can cause seat-map race conditions in Altéa when two agents process the last available premium seat simultaneously</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Provision premium cabin services and lounge access</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Airport Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>SITA Airport Management System (AMS)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Updated PNR with premium cabin indicator, lounge contract entitlements</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Lounge access pass issued; premium meal and amenity kit flagged for catering</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Premium service provisioning lead time ≥45 min before departure for ≥95% of upgrades</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Catering uplift amendments post-upgrade are frequently missed when the upgrade is processed inside the catering finality window (T-2h), resulting in insufficient premium meals</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Send upgrade confirmation and boarding pass to passenger</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management System (automated)</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>PNR update complete, new boarding pass data, passenger email / mobile</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Updated boarding pass (mobile and printable) and upgrade confirmation email</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Confirmation delivery within 60 sec of PNR update for ≥99% of upgrades</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Mobile boarding pass push fails for passengers using third-party wallet apps (non-Apple/Google Wallet) when Altéa PKPass API returns certificate validation errors</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Aggregate upsell revenue and conversion metrics</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Analytics Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>EMD transaction records, PNR cabin upgrade events, offer impression logs</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Daily upsell revenue report: impressions, conversions, revenue per upgrade, channel mix</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Upsell revenue per available seat ≥$12 on applicable routes; daily report SLA &lt;6h after day-end</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>EMD revenue attribution in AWS Redshift is delayed by up to 4h due to batch ingestion from Altéa, preventing same-day intra-day optimisation of pricing parameters</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Compare actuals vs. forecast upsell revenue targets</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Daily upsell revenue report, budgeted upsell revenue targets by route cluster</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Variance report: actual vs. forecast with root-cause flags (pricing, inventory, channel)</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Upsell revenue forecast accuracy within ±10% of actuals on rolling 7-day basis</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau dashboards pulling from AWS Redshift frequently timeout on full-network route-cluster queries, forcing analysts to run ad-hoc SQL instead of using governed reports</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-06</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Upgrade &amp; Upsell Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Recalibrate WTP model and pricing parameters</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimisation Data Scientist</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Variance report, offer acceptance/rejection data, competitor fare changes from OAG</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Updated WTP model weights; revised pricing floor and ceiling parameters in PROS RM</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>WTP model recalibration cycle ≤7 days after conversion target miss; post-recalibration lift ≥5%</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM model retraining requires a minimum 90-day historical acceptance dataset; insufficient data on new routes or post-schedule-change periods degrades model quality for at least one quarter</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Add NP-RM-07: Ancillary Revenue Optimization — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -28,6 +28,7 @@
     <sheet name="NP-RM-04" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="NP-RM-05" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="NP-RM-06" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="NP-RM-07" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1446,13 +1447,21 @@
           <t>Ancillary Revenue Optimization</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr"/>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-07</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -18801,7 +18810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N387"/>
+  <dimension ref="A1:N402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -46614,6 +46623,1086 @@
         </is>
       </c>
       <c r="N387" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" ht="30" customHeight="1">
+      <c r="A388" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B388" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C388" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D388" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E388" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F388" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark ancillary revenue vs. peer carriers</t>
+        </is>
+      </c>
+      <c r="G388" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H388" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I388" s="18" t="inlineStr">
+        <is>
+          <t>IATA annual ancillary revenue survey, peer carrier 10-K filings</t>
+        </is>
+      </c>
+      <c r="J388" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary benchmark report with gap analysis by product category</t>
+        </is>
+      </c>
+      <c r="K388" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue per passenger ≥ $35 (IATA LCC benchmark); report produced annually</t>
+        </is>
+      </c>
+      <c r="L388" s="18" t="inlineStr">
+        <is>
+          <t>IATA benchmark data lags 12–18 months; ultra-LCC peers (Spirit, Frontier) distort averages, masking true FSC comparison group and overstating apparent gap</t>
+        </is>
+      </c>
+      <c r="M388" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N388" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="30" customHeight="1">
+      <c r="A389" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B389" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C389" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D389" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E389" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F389" s="16" t="inlineStr">
+        <is>
+          <t>Analyse ancillary product mix by revenue category</t>
+        </is>
+      </c>
+      <c r="G389" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H389" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I389" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS booking records, ancillary sales transaction log</t>
+        </is>
+      </c>
+      <c r="J389" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary revenue decomposition: baggage, seat selection, F&amp;B, insurance, partner referrals</t>
+        </is>
+      </c>
+      <c r="K389" s="16" t="inlineStr">
+        <is>
+          <t>Top-3 categories contribute ≥70% of total ancillary revenue; data refresh ≤24 hours</t>
+        </is>
+      </c>
+      <c r="L389" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS ancillary sales codes are inconsistently applied by airport agents, causing product misclassification in Redshift that distorts category-level P&amp;L</t>
+        </is>
+      </c>
+      <c r="M389" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N389" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="30" customHeight="1">
+      <c r="A390" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B390" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C390" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D390" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E390" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F390" s="18" t="inlineStr">
+        <is>
+          <t>Identify new ancillary product opportunities</t>
+        </is>
+      </c>
+      <c r="G390" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H390" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I390" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark gap analysis, passenger demand segmentation, route O&amp;D traffic data</t>
+        </is>
+      </c>
+      <c r="J390" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary product roadmap with prioritised opportunities and revenue potential estimates</t>
+        </is>
+      </c>
+      <c r="K390" s="18" t="inlineStr">
+        <is>
+          <t>Minimum 3 new ancillary product candidates identified per annual review cycle</t>
+        </is>
+      </c>
+      <c r="L390" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D segmentation is designed for seat demand forecasting, not ancillary willingness-to-pay; proxy metrics must substitute for direct demand estimation, reducing confidence</t>
+        </is>
+      </c>
+      <c r="M390" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N390" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="30" customHeight="1">
+      <c r="A391" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B391" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C391" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D391" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E391" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F391" s="16" t="inlineStr">
+        <is>
+          <t>Configure ancillary service catalog in PSS</t>
+        </is>
+      </c>
+      <c r="G391" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H391" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I391" s="16" t="inlineStr">
+        <is>
+          <t>Approved ancillary product roadmap, IATA EMD (Electronic Miscellaneous Document) standards</t>
+        </is>
+      </c>
+      <c r="J391" s="16" t="inlineStr">
+        <is>
+          <t>Active ancillary service catalog with SSR/OSI codes and EMD settlement rules configured</t>
+        </is>
+      </c>
+      <c r="K391" s="16" t="inlineStr">
+        <is>
+          <t>100% of approved ancillaries configured and testable in Altéa within 5 business days of sign-off</t>
+        </is>
+      </c>
+      <c r="L391" s="16" t="inlineStr">
+        <is>
+          <t>EMD issuance rules require coordination with Finance for BSP settlement alignment; misconfigured EMD types generate revenue accounting errors and trigger BSP dispute processes</t>
+        </is>
+      </c>
+      <c r="M391" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N391" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="30" customHeight="1">
+      <c r="A392" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B392" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C392" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D392" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E392" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F392" s="18" t="inlineStr">
+        <is>
+          <t>Set dynamic pricing rules for seats and baggage</t>
+        </is>
+      </c>
+      <c r="G392" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H392" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I392" s="18" t="inlineStr">
+        <is>
+          <t>Historical ancillary demand elasticity data, booking curve by flight, load factor thresholds</t>
+        </is>
+      </c>
+      <c r="J392" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic ancillary price ladders by product, route, and days-to-departure bucket</t>
+        </is>
+      </c>
+      <c r="K392" s="18" t="inlineStr">
+        <is>
+          <t>Elasticity model coverage ≥80% of O&amp;D pairs; yield uplift ≥8% vs. static pricing baseline</t>
+        </is>
+      </c>
+      <c r="L392" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM dynamic ancillary pricing requires separate model training from core RM; data sparsity on thin routes produces unreliable elasticity estimates, defaulting to static fallback pricing</t>
+        </is>
+      </c>
+      <c r="M392" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N392" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" ht="30" customHeight="1">
+      <c r="A393" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B393" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C393" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D393" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E393" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F393" s="16" t="inlineStr">
+        <is>
+          <t>Design fare family bundles with ancillary inclusions</t>
+        </is>
+      </c>
+      <c r="G393" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H393" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I393" s="16" t="inlineStr">
+        <is>
+          <t>Fare family structure, ancillary cost-to-serve data, competitive bundle benchmarks</t>
+        </is>
+      </c>
+      <c r="J393" s="16" t="inlineStr">
+        <is>
+          <t>Defined fare family tiers (e.g. Basic / Standard / Flex) with ancillary inclusion matrix filed in ATPCO</t>
+        </is>
+      </c>
+      <c r="K393" s="16" t="inlineStr">
+        <is>
+          <t>Bundle attach rate ≥40% of total bookings; bundle margin ≥ à la carte revenue equivalent</t>
+        </is>
+      </c>
+      <c r="L393" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO Category 15 (Sales Restrictions) and Category 31 (Voluntary Changes) rules must be manually aligned with each bundle tier — a mismatch causes GDS display failures and customer refund claims</t>
+        </is>
+      </c>
+      <c r="M393" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N393" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" ht="30" customHeight="1">
+      <c r="A394" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B394" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C394" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D394" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E394" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F394" s="18" t="inlineStr">
+        <is>
+          <t>Validate ancillary offers in NDC API test environment</t>
+        </is>
+      </c>
+      <c r="G394" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H394" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I394" s="18" t="inlineStr">
+        <is>
+          <t>Configured ancillary catalog, fare family bundle definitions from ATPCO</t>
+        </is>
+      </c>
+      <c r="J394" s="18" t="inlineStr">
+        <is>
+          <t>Validated NDC offer schema with ancillaries returned in AirShopping and OrderCreate responses</t>
+        </is>
+      </c>
+      <c r="K394" s="18" t="inlineStr">
+        <is>
+          <t>100% of ancillary products surfaced in NDC AirShopping response; NDC API error rate &lt; 0.5%</t>
+        </is>
+      </c>
+      <c r="L394" s="18" t="inlineStr">
+        <is>
+          <t>IATA NDC 21.3 schema requires ancillaries as ServiceDefinitionID objects; legacy Altéa ancillary codes must be manually mapped — mappings break on Altéa version upgrades requiring re-validation</t>
+        </is>
+      </c>
+      <c r="M394" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N394" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="395" ht="30" customHeight="1">
+      <c r="A395" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B395" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C395" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D395" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E395" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F395" s="16" t="inlineStr">
+        <is>
+          <t>Segment passengers for targeted ancillary offers</t>
+        </is>
+      </c>
+      <c r="G395" s="16" t="inlineStr">
+        <is>
+          <t>Customer Analytics Manager</t>
+        </is>
+      </c>
+      <c r="H395" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I395" s="16" t="inlineStr">
+        <is>
+          <t>Loyalty programme profiles, booking history, route type (leisure/business), fare class</t>
+        </is>
+      </c>
+      <c r="J395" s="16" t="inlineStr">
+        <is>
+          <t>Passenger micro-segments with propensity scores for each ancillary product category</t>
+        </is>
+      </c>
+      <c r="K395" s="16" t="inlineStr">
+        <is>
+          <t>Propensity model AUC ≥0.72 for top-3 ancillary categories; segments refreshed ≤24 hours before departure</t>
+        </is>
+      </c>
+      <c r="L395" s="16" t="inlineStr">
+        <is>
+          <t>Loyalty data is siloed from GDS bookings — indirect-channel passengers have sparse profiles, reducing propensity model accuracy for ~35% of bookings and defaulting to generic offers</t>
+        </is>
+      </c>
+      <c r="M395" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N395" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="396" ht="30" customHeight="1">
+      <c r="A396" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B396" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C396" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D396" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E396" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F396" s="18" t="inlineStr">
+        <is>
+          <t>Configure real-time ancillary offer engine</t>
+        </is>
+      </c>
+      <c r="G396" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H396" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I396" s="18" t="inlineStr">
+        <is>
+          <t>Passenger propensity scores, dynamic price ladders from PROS RM, inventory availability</t>
+        </is>
+      </c>
+      <c r="J396" s="18" t="inlineStr">
+        <is>
+          <t>Personalised ancillary offer sets ranked by revenue contribution per passenger segment</t>
+        </is>
+      </c>
+      <c r="K396" s="18" t="inlineStr">
+        <is>
+          <t>Offer generation latency &lt; 200ms per PNR; personalised offer conversion rate ≥15%</t>
+        </is>
+      </c>
+      <c r="L396" s="18" t="inlineStr">
+        <is>
+          <t>AltéaRM offer engine integration with PROS dynamic ancillary prices requires a custom middleware API; latency spikes during peak booking windows trigger offer timeouts and fallback to static pricing</t>
+        </is>
+      </c>
+      <c r="M396" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N396" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="397" ht="30" customHeight="1">
+      <c r="A397" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B397" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C397" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D397" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E397" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F397" s="16" t="inlineStr">
+        <is>
+          <t>Deploy personalised offers via direct and GDS channels</t>
+        </is>
+      </c>
+      <c r="G397" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Channel Manager</t>
+        </is>
+      </c>
+      <c r="H397" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I397" s="16" t="inlineStr">
+        <is>
+          <t>Ranked personalised offer sets, channel capability matrix (NDC Level 3, GDS, direct web)</t>
+        </is>
+      </c>
+      <c r="J397" s="16" t="inlineStr">
+        <is>
+          <t>Live ancillary offers served to all booking channels with channel-specific display logic</t>
+        </is>
+      </c>
+      <c r="K397" s="16" t="inlineStr">
+        <is>
+          <t>NDC channel ancillary attach rate ≥ direct channel within 6 months of launch; GDS ancillary display compliance ≥90% of enabled PCCs</t>
+        </is>
+      </c>
+      <c r="L397" s="16" t="inlineStr">
+        <is>
+          <t>Travelport and Sabre GDS ancillary merchandising varies by Point of Sale — not all TMC-configured PCC terminals display ancillary offers, suppressing B2B ancillary revenue from managed travel</t>
+        </is>
+      </c>
+      <c r="M397" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N397" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="398" ht="30" customHeight="1">
+      <c r="A398" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B398" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C398" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D398" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E398" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F398" s="18" t="inlineStr">
+        <is>
+          <t>Monitor ancillary attach rates by channel and product</t>
+        </is>
+      </c>
+      <c r="G398" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H398" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I398" s="18" t="inlineStr">
+        <is>
+          <t>Real-time ancillary sales feed from Altéa PSS, channel booking logs, budget targets</t>
+        </is>
+      </c>
+      <c r="J398" s="18" t="inlineStr">
+        <is>
+          <t>Live ancillary performance dashboard: attach rate, revenue per pax, channel mix, trend</t>
+        </is>
+      </c>
+      <c r="K398" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue as % of total revenue ≥15%; dashboard data latency &lt; 4 hours</t>
+        </is>
+      </c>
+      <c r="L398" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS real-time data feed to Tableau relies on an AWS Kinesis stream — stream failures during high-volume booking periods create data gaps that delay corrective pricing actions by 8–12 hours</t>
+        </is>
+      </c>
+      <c r="M398" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N398" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="399" ht="30" customHeight="1">
+      <c r="A399" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B399" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C399" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D399" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E399" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F399" s="16" t="inlineStr">
+        <is>
+          <t>Conduct ancillary price elasticity A/B testing</t>
+        </is>
+      </c>
+      <c r="G399" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H399" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I399" s="16" t="inlineStr">
+        <is>
+          <t>Current ancillary price points, candidate test prices, booking volume thresholds for statistical significance</t>
+        </is>
+      </c>
+      <c r="J399" s="16" t="inlineStr">
+        <is>
+          <t>A/B test results with elasticity coefficient and recommended price adjustment per product</t>
+        </is>
+      </c>
+      <c r="K399" s="16" t="inlineStr">
+        <is>
+          <t>A/B test significance ≥95% confidence interval; minimum 500 transactions per test cell</t>
+        </is>
+      </c>
+      <c r="L399" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM A/B testing for ancillaries is not natively integrated with Altéa PSS booking flows — test cell assignment is enforced via custom middleware, increasing build and maintenance overhead</t>
+        </is>
+      </c>
+      <c r="M399" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N399" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="400" ht="30" customHeight="1">
+      <c r="A400" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B400" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C400" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D400" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E400" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F400" s="18" t="inlineStr">
+        <is>
+          <t>Optimise ancillary offer placement and sequencing</t>
+        </is>
+      </c>
+      <c r="G400" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H400" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I400" s="18" t="inlineStr">
+        <is>
+          <t>A/B test results, channel conversion data, passenger journey stage (search / select / pre-check-in)</t>
+        </is>
+      </c>
+      <c r="J400" s="18" t="inlineStr">
+        <is>
+          <t>Updated offer sequencing rules: optimal placement by journey stage and channel</t>
+        </is>
+      </c>
+      <c r="K400" s="18" t="inlineStr">
+        <is>
+          <t>Incremental ancillary revenue uplift ≥5% per optimisation cycle; cycle cadence monthly</t>
+        </is>
+      </c>
+      <c r="L400" s="18" t="inlineStr">
+        <is>
+          <t>Post-booking ancillary upsell in the pre-check-in window is constrained by Altéa PSS notification infrastructure — push notification capability requires a third-party integration not yet fully deployed at most carriers</t>
+        </is>
+      </c>
+      <c r="M400" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N400" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="401" ht="30" customHeight="1">
+      <c r="A401" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B401" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C401" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D401" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E401" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F401" s="16" t="inlineStr">
+        <is>
+          <t>Generate ancillary revenue performance report</t>
+        </is>
+      </c>
+      <c r="G401" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H401" s="16" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="I401" s="16" t="inlineStr">
+        <is>
+          <t>Monthly ancillary sales data from Redshift, budget targets, prior-period actuals</t>
+        </is>
+      </c>
+      <c r="J401" s="16" t="inlineStr">
+        <is>
+          <t>Monthly ancillary revenue report: actuals vs. budget, trend analysis, category and channel breakdown</t>
+        </is>
+      </c>
+      <c r="K401" s="16" t="inlineStr">
+        <is>
+          <t>Report delivered within 3 business days of month-end; forecast accuracy ≤5% variance vs. actuals</t>
+        </is>
+      </c>
+      <c r="L401" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance GL ancillary revenue codes do not always align with Altéa PSS ancillary sales codes — reconciliation requires a manual mapping table maintained by Finance that lags product catalog changes</t>
+        </is>
+      </c>
+      <c r="M401" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N401" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="402" ht="30" customHeight="1">
+      <c r="A402" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B402" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C402" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D402" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E402" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F402" s="18" t="inlineStr">
+        <is>
+          <t>Review portfolio and retire underperforming products</t>
+        </is>
+      </c>
+      <c r="G402" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H402" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I402" s="18" t="inlineStr">
+        <is>
+          <t>Monthly performance report, ancillary product P&amp;L, customer NPS scores by ancillary category</t>
+        </is>
+      </c>
+      <c r="J402" s="18" t="inlineStr">
+        <is>
+          <t>Portfolio rationalisation decision per product: retain / reprice / discontinue with timeline</t>
+        </is>
+      </c>
+      <c r="K402" s="18" t="inlineStr">
+        <is>
+          <t>Products with &lt;0.5% attach rate and negative NPS reviewed quarterly; discontinuation decision within 30 days of review</t>
+        </is>
+      </c>
+      <c r="L402" s="18" t="inlineStr">
+        <is>
+          <t>Discontinuing an ancillary product in Altéa PSS requires reversal of EMD settlement rules, ATPCO filing withdrawal, and NDC schema update — cross-system coordination takes 4–6 weeks, extending underperformer lifecycles</t>
+        </is>
+      </c>
+      <c r="M402" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N402" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -49459,6 +50548,1206 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-07 — Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark ancillary revenue vs. peer carriers</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>IATA annual ancillary revenue survey, peer carrier 10-K filings</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary benchmark report with gap analysis by product category</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue per passenger ≥ $35 (IATA LCC benchmark); report produced annually</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>IATA benchmark data lags 12–18 months; ultra-LCC peers (Spirit, Frontier) distort averages, masking true FSC comparison group and overstating apparent gap</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Analyse ancillary product mix by revenue category</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS booking records, ancillary sales transaction log</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary revenue decomposition: baggage, seat selection, F&amp;B, insurance, partner referrals</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Top-3 categories contribute ≥70% of total ancillary revenue; data refresh ≤24 hours</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Altéa PSS ancillary sales codes are inconsistently applied by airport agents, causing product misclassification in Redshift that distorts category-level P&amp;L</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Identify new ancillary product opportunities</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus SkyCAST</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark gap analysis, passenger demand segmentation, route O&amp;D traffic data</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary product roadmap with prioritised opportunities and revenue potential estimates</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Minimum 3 new ancillary product candidates identified per annual review cycle</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>SkyCAST O&amp;D segmentation is designed for seat demand forecasting, not ancillary willingness-to-pay; proxy metrics must substitute for direct demand estimation, reducing confidence</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Configure ancillary service catalog in PSS</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Approved ancillary product roadmap, IATA EMD (Electronic Miscellaneous Document) standards</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Active ancillary service catalog with SSR/OSI codes and EMD settlement rules configured</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>100% of approved ancillaries configured and testable in Altéa within 5 business days of sign-off</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>EMD issuance rules require coordination with Finance for BSP settlement alignment; misconfigured EMD types generate revenue accounting errors and trigger BSP dispute processes</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Set dynamic pricing rules for seats and baggage</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Historical ancillary demand elasticity data, booking curve by flight, load factor thresholds</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic ancillary price ladders by product, route, and days-to-departure bucket</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Elasticity model coverage ≥80% of O&amp;D pairs; yield uplift ≥8% vs. static pricing baseline</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM dynamic ancillary pricing requires separate model training from core RM; data sparsity on thin routes produces unreliable elasticity estimates, defaulting to static fallback pricing</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Design fare family bundles with ancillary inclusions</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Strategy Manager</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Fare family structure, ancillary cost-to-serve data, competitive bundle benchmarks</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Defined fare family tiers (e.g. Basic / Standard / Flex) with ancillary inclusion matrix filed in ATPCO</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Bundle attach rate ≥40% of total bookings; bundle margin ≥ à la carte revenue equivalent</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO Category 15 (Sales Restrictions) and Category 31 (Voluntary Changes) rules must be manually aligned with each bundle tier — a mismatch causes GDS display failures and customer refund claims</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Validate ancillary offers in NDC API test environment</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Configured ancillary catalog, fare family bundle definitions from ATPCO</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Validated NDC offer schema with ancillaries returned in AirShopping and OrderCreate responses</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>100% of ancillary products surfaced in NDC AirShopping response; NDC API error rate &lt; 0.5%</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>IATA NDC 21.3 schema requires ancillaries as ServiceDefinitionID objects; legacy Altéa ancillary codes must be manually mapped — mappings break on Altéa version upgrades requiring re-validation</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Segment passengers for targeted ancillary offers</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Customer Analytics Manager</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Loyalty programme profiles, booking history, route type (leisure/business), fare class</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Passenger micro-segments with propensity scores for each ancillary product category</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Propensity model AUC ≥0.72 for top-3 ancillary categories; segments refreshed ≤24 hours before departure</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Loyalty data is siloed from GDS bookings — indirect-channel passengers have sparse profiles, reducing propensity model accuracy for ~35% of bookings and defaulting to generic offers</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Configure real-time ancillary offer engine</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Passenger propensity scores, dynamic price ladders from PROS RM, inventory availability</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Personalised ancillary offer sets ranked by revenue contribution per passenger segment</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Offer generation latency &lt; 200ms per PNR; personalised offer conversion rate ≥15%</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>AltéaRM offer engine integration with PROS dynamic ancillary prices requires a custom middleware API; latency spikes during peak booking windows trigger offer timeouts and fallback to static pricing</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Deploy personalised offers via direct and GDS channels</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Channel Manager</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Ranked personalised offer sets, channel capability matrix (NDC Level 3, GDS, direct web)</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Live ancillary offers served to all booking channels with channel-specific display logic</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>NDC channel ancillary attach rate ≥ direct channel within 6 months of launch; GDS ancillary display compliance ≥90% of enabled PCCs</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Travelport and Sabre GDS ancillary merchandising varies by Point of Sale — not all TMC-configured PCC terminals display ancillary offers, suppressing B2B ancillary revenue from managed travel</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Monitor ancillary attach rates by channel and product</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Real-time ancillary sales feed from Altéa PSS, channel booking logs, budget targets</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Live ancillary performance dashboard: attach rate, revenue per pax, channel mix, trend</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue as % of total revenue ≥15%; dashboard data latency &lt; 4 hours</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS real-time data feed to Tableau relies on an AWS Kinesis stream — stream failures during high-volume booking periods create data gaps that delay corrective pricing actions by 8–12 hours</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Conduct ancillary price elasticity A/B testing</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Current ancillary price points, candidate test prices, booking volume thresholds for statistical significance</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>A/B test results with elasticity coefficient and recommended price adjustment per product</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>A/B test significance ≥95% confidence interval; minimum 500 transactions per test cell</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM A/B testing for ancillaries is not natively integrated with Altéa PSS booking flows — test cell assignment is enforced via custom middleware, increasing build and maintenance overhead</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Optimise ancillary offer placement and sequencing</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>A/B test results, channel conversion data, passenger journey stage (search / select / pre-check-in)</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Updated offer sequencing rules: optimal placement by journey stage and channel</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Incremental ancillary revenue uplift ≥5% per optimisation cycle; cycle cadence monthly</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Post-booking ancillary upsell in the pre-check-in window is constrained by Altéa PSS notification infrastructure — push notification capability requires a third-party integration not yet fully deployed at most carriers</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Generate ancillary revenue performance report</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Monthly ancillary sales data from Redshift, budget targets, prior-period actuals</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Monthly ancillary revenue report: actuals vs. budget, trend analysis, category and channel breakdown</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Report delivered within 3 business days of month-end; forecast accuracy ≤5% variance vs. actuals</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance GL ancillary revenue codes do not always align with Altéa PSS ancillary sales codes — reconciliation requires a manual mapping table maintained by Finance that lags product catalog changes</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-07</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Optimization</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Review portfolio and retire underperforming products</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Monthly performance report, ancillary product P&amp;L, customer NPS scores by ancillary category</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Portfolio rationalisation decision per product: retain / reprice / discontinue with timeline</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Products with &lt;0.5% attach rate and negative NPS reviewed quarterly; discontinuation decision within 30 days of review</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Discontinuing an ancillary product in Altéa PSS requires reversal of EMD settlement rules, ATPCO filing withdrawal, and NDC schema update — cross-system coordination takes 4–6 weeks, extending underperformer lifecycles</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add NP-RM-08: RM System Calibration & Tuning — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -29,6 +29,7 @@
     <sheet name="NP-RM-05" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="NP-RM-06" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="NP-RM-07" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="NP-RM-08" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1484,13 +1485,21 @@
           <t>RM System Calibration &amp; Tuning</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="10" t="inlineStr"/>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-08</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -18810,7 +18819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N402"/>
+  <dimension ref="A1:N418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -47705,6 +47714,1158 @@
       <c r="N402" s="17" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="403" ht="30" customHeight="1">
+      <c r="A403" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B403" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C403" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D403" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E403" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F403" s="16" t="inlineStr">
+        <is>
+          <t>Extract RM forecast accuracy metrics</t>
+        </is>
+      </c>
+      <c r="G403" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H403" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I403" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled monthly calibration cycle or ad-hoc trigger from revenue variance alert</t>
+        </is>
+      </c>
+      <c r="J403" s="16" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report: MAPE by market, booking class, and horizon</t>
+        </is>
+      </c>
+      <c r="K403" s="16" t="inlineStr">
+        <is>
+          <t>Mean Absolute Percentage Error (MAPE) ≤15% across all O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="L403" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM MAPE reporting requires custom extract scripts; no native scheduled accuracy dashboard, increasing analyst effort and risk of metric inconsistency</t>
+        </is>
+      </c>
+      <c r="M403" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N403" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="30" customHeight="1">
+      <c r="A404" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B404" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C404" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D404" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E404" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F404" s="18" t="inlineStr">
+        <is>
+          <t>Identify underperforming O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="G404" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H404" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I404" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report from step 1.1; actuals from AWS Redshift booking data warehouse</t>
+        </is>
+      </c>
+      <c r="J404" s="18" t="inlineStr">
+        <is>
+          <t>Ranked list of O&amp;D markets with MAPE &gt;15% or revenue variance &gt;3% vs. plan</t>
+        </is>
+      </c>
+      <c r="K404" s="18" t="inlineStr">
+        <is>
+          <t>≥90% of O&amp;D markets within MAPE threshold within 30 days of calibration cycle</t>
+        </is>
+      </c>
+      <c r="L404" s="18" t="inlineStr">
+        <is>
+          <t>Cross-market comparison requires manual joins between Amadeus NRM outputs and AWS Redshift actuals; data latency of up to 24 hrs can mask intra-day booking pattern shifts</t>
+        </is>
+      </c>
+      <c r="M404" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N404" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="405" ht="30" customHeight="1">
+      <c r="A405" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B405" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C405" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D405" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E405" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F405" s="16" t="inlineStr">
+        <is>
+          <t>Assess booking curve deviations from expected pickup</t>
+        </is>
+      </c>
+      <c r="G405" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Analyst</t>
+        </is>
+      </c>
+      <c r="H405" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I405" s="16" t="inlineStr">
+        <is>
+          <t>Ranked O&amp;D market list; historical booking curve profiles from NRM</t>
+        </is>
+      </c>
+      <c r="J405" s="16" t="inlineStr">
+        <is>
+          <t>Deviation analysis report flagging systematic early/late booking shifts and class-mix anomalies</t>
+        </is>
+      </c>
+      <c r="K405" s="16" t="inlineStr">
+        <is>
+          <t>Booking curve R² ≥0.92 across flagged markets; decision to proceed with recalibration if ≥3 markets fail threshold</t>
+        </is>
+      </c>
+      <c r="L405" s="16" t="inlineStr">
+        <is>
+          <t>Structural demand shifts post-COVID (early leisure surge, late corporate recovery) have permanently altered booking curves; NRM baseline curves calibrated pre-2023 may no longer reflect current market behaviour</t>
+        </is>
+      </c>
+      <c r="M405" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N405" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="406" ht="30" customHeight="1">
+      <c r="A406" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B406" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C406" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D406" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E406" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F406" s="18" t="inlineStr">
+        <is>
+          <t>Extract historical booking and ticketing data</t>
+        </is>
+      </c>
+      <c r="G406" s="18" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="H406" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I406" s="18" t="inlineStr">
+        <is>
+          <t>Calibration scope (markets, date range, booking classes) from deviation analysis report</t>
+        </is>
+      </c>
+      <c r="J406" s="18" t="inlineStr">
+        <is>
+          <t>Structured training dataset: O&amp;D bookings, fares paid, cancellation rates, no-show rates — 24-month rolling window</t>
+        </is>
+      </c>
+      <c r="K406" s="18" t="inlineStr">
+        <is>
+          <t>Dataset completeness ≥98% of scheduled departures in scope; extract runtime &lt;2 hours</t>
+        </is>
+      </c>
+      <c r="L406" s="18" t="inlineStr">
+        <is>
+          <t>AWS Redshift query performance degrades on unpartitioned historical tables; full 24-month O&amp;D extracts for 100+ markets can exceed 4-hour SLA without query optimisation</t>
+        </is>
+      </c>
+      <c r="M406" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N406" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="407" ht="30" customHeight="1">
+      <c r="A407" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B407" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C407" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D407" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E407" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F407" s="16" t="inlineStr">
+        <is>
+          <t>Validate input data quality and completeness</t>
+        </is>
+      </c>
+      <c r="G407" s="16" t="inlineStr">
+        <is>
+          <t>Data Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H407" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I407" s="16" t="inlineStr">
+        <is>
+          <t>Raw extract from AWS Redshift; data quality ruleset stored in S3</t>
+        </is>
+      </c>
+      <c r="J407" s="16" t="inlineStr">
+        <is>
+          <t>Data quality scorecard with pass/fail per validation rule; cleansed dataset or rejection notice</t>
+        </is>
+      </c>
+      <c r="K407" s="16" t="inlineStr">
+        <is>
+          <t>Data quality score ≥95% (null rate &lt;2%, duplicate bookings &lt;0.5%, fare outliers &lt;1%)</t>
+        </is>
+      </c>
+      <c r="L407" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS ticket voids and exchanges frequently generate duplicate or partial booking records that inflate cancellation rate inputs to the NRM demand model, distorting recalibration outputs</t>
+        </is>
+      </c>
+      <c r="M407" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N407" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="408" ht="30" customHeight="1">
+      <c r="A408" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B408" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C408" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D408" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E408" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F408" s="18" t="inlineStr">
+        <is>
+          <t>Load competitive fare and capacity benchmarks</t>
+        </is>
+      </c>
+      <c r="G408" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H408" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I408" s="18" t="inlineStr">
+        <is>
+          <t>Competitor fare filing data from ATPCO; OAG Schedule Analyser capacity data for target O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="J408" s="18" t="inlineStr">
+        <is>
+          <t>Competitive context dataset: competitor fare ladder, capacity by carrier, schedule frequency</t>
+        </is>
+      </c>
+      <c r="K408" s="18" t="inlineStr">
+        <is>
+          <t>Competitive data coverage ≥85% of target O&amp;D markets; data freshness within 48 hours of filing date</t>
+        </is>
+      </c>
+      <c r="L408" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO fare data covers only filed public fares; negotiated corporate and NDC-only fares are not visible, creating a systematic blind spot in price elasticity model inputs for corporate-heavy routes</t>
+        </is>
+      </c>
+      <c r="M408" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N408" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="409" ht="30" customHeight="1">
+      <c r="A409" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B409" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C409" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D409" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E409" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F409" s="16" t="inlineStr">
+        <is>
+          <t>Recalibrate demand forecast model coefficients</t>
+        </is>
+      </c>
+      <c r="G409" s="16" t="inlineStr">
+        <is>
+          <t>RM Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H409" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I409" s="16" t="inlineStr">
+        <is>
+          <t>Cleansed 24-month historical dataset; competitive context dataset; current NRM model parameter set</t>
+        </is>
+      </c>
+      <c r="J409" s="16" t="inlineStr">
+        <is>
+          <t>Updated demand model coefficients (seasonality indices, trend factors, day-of-week multipliers) staged in NRM test partition</t>
+        </is>
+      </c>
+      <c r="K409" s="16" t="inlineStr">
+        <is>
+          <t>Post-recalibration MAPE improvement ≥10% vs. baseline on hold-out validation set</t>
+        </is>
+      </c>
+      <c r="L409" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM parameter update interface requires batch file upload in proprietary format; no API-driven calibration workflow, increasing manual error risk and extending cycle time to 3–5 business days</t>
+        </is>
+      </c>
+      <c r="M409" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N409" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="410" ht="30" customHeight="1">
+      <c r="A410" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B410" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C410" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D410" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E410" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F410" s="18" t="inlineStr">
+        <is>
+          <t>Update price elasticity and WTP model curves</t>
+        </is>
+      </c>
+      <c r="G410" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Analyst</t>
+        </is>
+      </c>
+      <c r="H410" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I410" s="18" t="inlineStr">
+        <is>
+          <t>Updated demand model coefficients; ATPCO competitive fare ladder; passenger segment willingness-to-pay data</t>
+        </is>
+      </c>
+      <c r="J410" s="18" t="inlineStr">
+        <is>
+          <t>Revised price elasticity curves and class-specific bid price adjustments per O&amp;D market cluster</t>
+        </is>
+      </c>
+      <c r="K410" s="18" t="inlineStr">
+        <is>
+          <t>Bid price accuracy: simulated revenue within ±2% of optimal on hold-out markets; elasticity curve R² ≥0.88</t>
+        </is>
+      </c>
+      <c r="L410" s="18" t="inlineStr">
+        <is>
+          <t>WTP segmentation in Amadeus NRM is limited to cabin-level; lack of sub-segment granularity (e.g. loyalty tier, corporate account) reduces model precision for high-value O&amp;D pairs with mixed traffic composition</t>
+        </is>
+      </c>
+      <c r="M410" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N410" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="411" ht="30" customHeight="1">
+      <c r="A411" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B411" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C411" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D411" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E411" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F411" s="16" t="inlineStr">
+        <is>
+          <t>Tune overbooking safety factors by route type</t>
+        </is>
+      </c>
+      <c r="G411" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H411" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I411" s="16" t="inlineStr">
+        <is>
+          <t>Updated elasticity curves; historical no-show and cancellation rates by route category (short-haul leisure, long-haul corporate, thin route)</t>
+        </is>
+      </c>
+      <c r="J411" s="16" t="inlineStr">
+        <is>
+          <t>Revised overbooking multipliers per route cluster; updated denied boarding risk scores</t>
+        </is>
+      </c>
+      <c r="K411" s="16" t="inlineStr">
+        <is>
+          <t>Denied boarding rate ≤0.05 per 1,000 passengers; seat spoilage rate ≤2% of available seats</t>
+        </is>
+      </c>
+      <c r="L411" s="16" t="inlineStr">
+        <is>
+          <t>Denied boarding compensation exposure under EU261/2004 and DOT rules creates asymmetric financial risk; NRM overbooking model does not natively incorporate regulatory compensation cost as an optimisation constraint</t>
+        </is>
+      </c>
+      <c r="M411" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N411" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="412" ht="30" customHeight="1">
+      <c r="A412" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B412" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C412" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D412" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E412" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F412" s="18" t="inlineStr">
+        <is>
+          <t>Execute shadow-mode simulation on hold-out period</t>
+        </is>
+      </c>
+      <c r="G412" s="18" t="inlineStr">
+        <is>
+          <t>RM Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H412" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I412" s="18" t="inlineStr">
+        <is>
+          <t>Updated NRM parameter set (demand model + elasticity curves + overbooking factors); hold-out historical period (most recent 90 days not used in training)</t>
+        </is>
+      </c>
+      <c r="J412" s="18" t="inlineStr">
+        <is>
+          <t>Shadow revenue report: simulated revenue and load factor for each O&amp;D flight in hold-out period</t>
+        </is>
+      </c>
+      <c r="K412" s="18" t="inlineStr">
+        <is>
+          <t>Shadow simulation runtime ≤8 hours; simulated revenue variance vs. actuals ≤2%</t>
+        </is>
+      </c>
+      <c r="L412" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM shadow mode does not replicate real-time competitor price reactions; static competitor assumptions in simulation overstate revenue uplift potential by an estimated 0.5–1.0% on competitive routes</t>
+        </is>
+      </c>
+      <c r="M412" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N412" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="413" ht="30" customHeight="1">
+      <c r="A413" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B413" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C413" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D413" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E413" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F413" s="16" t="inlineStr">
+        <is>
+          <t>Evaluate shadow revenue vs. actual revenue</t>
+        </is>
+      </c>
+      <c r="G413" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Manager</t>
+        </is>
+      </c>
+      <c r="H413" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I413" s="16" t="inlineStr">
+        <is>
+          <t>Shadow revenue report; actual revenue actuals from AWS Redshift for the same hold-out period</t>
+        </is>
+      </c>
+      <c r="J413" s="16" t="inlineStr">
+        <is>
+          <t>Calibration validation dashboard: revenue lift by market cluster, load factor delta, booking class mix comparison</t>
+        </is>
+      </c>
+      <c r="K413" s="16" t="inlineStr">
+        <is>
+          <t>Simulated revenue uplift ≥1.0% vs. actuals across all market clusters; no individual cluster showing revenue degradation &gt;0.5%</t>
+        </is>
+      </c>
+      <c r="L413" s="16" t="inlineStr">
+        <is>
+          <t>Revenue attribution between calibration changes and external demand factors (events, competitor capacity changes) is not automated; manual attribution analysis adds 1–2 days to the validation cycle</t>
+        </is>
+      </c>
+      <c r="M413" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N413" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="414" ht="30" customHeight="1">
+      <c r="A414" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B414" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C414" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D414" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E414" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F414" s="18" t="inlineStr">
+        <is>
+          <t>Run live A/B test on selected pilot markets</t>
+        </is>
+      </c>
+      <c r="G414" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H414" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I414" s="18" t="inlineStr">
+        <is>
+          <t>Validated calibration parameter set; pilot market selection (10–15 O&amp;D pairs representative of route clusters)</t>
+        </is>
+      </c>
+      <c r="J414" s="18" t="inlineStr">
+        <is>
+          <t>A/B test results: revenue per available seat kilometre (RASK) and load factor for treatment vs. control group over 4-week period</t>
+        </is>
+      </c>
+      <c r="K414" s="18" t="inlineStr">
+        <is>
+          <t>A/B revenue uplift ≥1.5% in pilot markets over 4-week test window at 95% statistical confidence</t>
+        </is>
+      </c>
+      <c r="L414" s="18" t="inlineStr">
+        <is>
+          <t>Selecting statistically valid control markets is difficult on thin-route network where few true analogues exist; contamination risk between test and control markets sharing connections distorts A/B results</t>
+        </is>
+      </c>
+      <c r="M414" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N414" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="415" ht="30" customHeight="1">
+      <c r="A415" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B415" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C415" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D415" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E415" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F415" s="16" t="inlineStr">
+        <is>
+          <t>Stage calibrated parameters in UAT environment</t>
+        </is>
+      </c>
+      <c r="G415" s="16" t="inlineStr">
+        <is>
+          <t>RM Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H415" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I415" s="16" t="inlineStr">
+        <is>
+          <t>Approved calibration parameter set from A/B test; UAT deployment checklist</t>
+        </is>
+      </c>
+      <c r="J415" s="16" t="inlineStr">
+        <is>
+          <t>UAT environment loaded with new parameters; regression test results confirming no unintended impacts to adjacent processes (pricing, inventory, interline)</t>
+        </is>
+      </c>
+      <c r="K415" s="16" t="inlineStr">
+        <is>
+          <t>UAT regression test pass rate 100% on critical path; deployment staging completed within 1 business day</t>
+        </is>
+      </c>
+      <c r="L415" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM UAT environment is shared with pricing and ancillary revenue teams; uncoordinated deployments from parallel projects create parameter conflicts that require vendor support engagement to resolve</t>
+        </is>
+      </c>
+      <c r="M415" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N415" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="416" ht="30" customHeight="1">
+      <c r="A416" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B416" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C416" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D416" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E416" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F416" s="18" t="inlineStr">
+        <is>
+          <t>Present calibration results for RM leadership sign-off</t>
+        </is>
+      </c>
+      <c r="G416" s="18" t="inlineStr">
+        <is>
+          <t>Head of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H416" s="18" t="inlineStr">
+        <is>
+          <t>Microsoft Azure Synapse</t>
+        </is>
+      </c>
+      <c r="I416" s="18" t="inlineStr">
+        <is>
+          <t>Calibration validation dashboard; A/B test results; UAT regression summary; estimated annual revenue impact</t>
+        </is>
+      </c>
+      <c r="J416" s="18" t="inlineStr">
+        <is>
+          <t>Signed approval record or change request with required amendments; go/no-go decision for production deployment</t>
+        </is>
+      </c>
+      <c r="K416" s="18" t="inlineStr">
+        <is>
+          <t>Sign-off decision turnaround ≤2 business days; zero production deployments without documented approval</t>
+        </is>
+      </c>
+      <c r="L416" s="18" t="inlineStr">
+        <is>
+          <t>Calibration approval process is undocumented in most carriers; absence of a formal change control board for RM model changes means deployments can proceed without revenue risk assessment, creating audit exposure</t>
+        </is>
+      </c>
+      <c r="M416" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N416" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="417" ht="30" customHeight="1">
+      <c r="A417" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B417" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C417" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D417" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E417" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F417" s="16" t="inlineStr">
+        <is>
+          <t>Deploy calibrated parameters to production NRM</t>
+        </is>
+      </c>
+      <c r="G417" s="16" t="inlineStr">
+        <is>
+          <t>RM Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H417" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I417" s="16" t="inlineStr">
+        <is>
+          <t>Signed approval record; staged parameter set from UAT; deployment runbook</t>
+        </is>
+      </c>
+      <c r="J417" s="16" t="inlineStr">
+        <is>
+          <t>Production NRM updated with new demand model coefficients, elasticity curves, and overbooking factors; deployment confirmation log</t>
+        </is>
+      </c>
+      <c r="K417" s="16" t="inlineStr">
+        <is>
+          <t>Production deployment completed within 4-hour maintenance window; zero unplanned system downtime during deployment</t>
+        </is>
+      </c>
+      <c r="L417" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM production parameter updates require a maintenance window coordinated with Amadeus support; last-minute scheduling conflicts with Altéa PSS maintenance windows have caused deployment delays of up to 72 hours</t>
+        </is>
+      </c>
+      <c r="M417" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N417" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="418" ht="30" customHeight="1">
+      <c r="A418" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B418" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C418" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D418" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E418" s="17" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F418" s="18" t="inlineStr">
+        <is>
+          <t>Monitor live KPIs post-deployment</t>
+        </is>
+      </c>
+      <c r="G418" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H418" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I418" s="18" t="inlineStr">
+        <is>
+          <t>Live booking data from Amadeus NRM; post-deployment KPI dashboard; baseline metrics from pre-calibration period</t>
+        </is>
+      </c>
+      <c r="J418" s="18" t="inlineStr">
+        <is>
+          <t>30-day post-deployment performance report; rollback recommendation if KPIs deteriorate beyond threshold</t>
+        </is>
+      </c>
+      <c r="K418" s="18" t="inlineStr">
+        <is>
+          <t>RASK improvement ≥1.0% vs. pre-calibration baseline within 30 days; no market showing load factor decline &gt;2 percentage points</t>
+        </is>
+      </c>
+      <c r="L418" s="18" t="inlineStr">
+        <is>
+          <t>Post-deployment monitoring relies on manual Tableau dashboard review; absence of automated anomaly detection means revenue degradation from a miscalibrated market cluster may go undetected for 3–5 days, compounding financial impact</t>
+        </is>
+      </c>
+      <c r="M418" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N418" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -51748,6 +52909,1278 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-08 — RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Extract RM forecast accuracy metrics</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Scheduled monthly calibration cycle or ad-hoc trigger from revenue variance alert</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report: MAPE by market, booking class, and horizon</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Mean Absolute Percentage Error (MAPE) ≤15% across all O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM MAPE reporting requires custom extract scripts; no native scheduled accuracy dashboard, increasing analyst effort and risk of metric inconsistency</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Identify underperforming O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Forecast accuracy report from step 1.1; actuals from AWS Redshift booking data warehouse</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Ranked list of O&amp;D markets with MAPE &gt;15% or revenue variance &gt;3% vs. plan</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>≥90% of O&amp;D markets within MAPE threshold within 30 days of calibration cycle</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Cross-market comparison requires manual joins between Amadeus NRM outputs and AWS Redshift actuals; data latency of up to 24 hrs can mask intra-day booking pattern shifts</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Assess booking curve deviations from expected pickup</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Ranked O&amp;D market list; historical booking curve profiles from NRM</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Deviation analysis report flagging systematic early/late booking shifts and class-mix anomalies</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Booking curve R² ≥0.92 across flagged markets; decision to proceed with recalibration if ≥3 markets fail threshold</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Structural demand shifts post-COVID (early leisure surge, late corporate recovery) have permanently altered booking curves; NRM baseline curves calibrated pre-2023 may no longer reflect current market behaviour</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Extract historical booking and ticketing data</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Calibration scope (markets, date range, booking classes) from deviation analysis report</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Structured training dataset: O&amp;D bookings, fares paid, cancellation rates, no-show rates — 24-month rolling window</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Dataset completeness ≥98% of scheduled departures in scope; extract runtime &lt;2 hours</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift query performance degrades on unpartitioned historical tables; full 24-month O&amp;D extracts for 100+ markets can exceed 4-hour SLA without query optimisation</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Validate input data quality and completeness</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Data Quality Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Raw extract from AWS Redshift; data quality ruleset stored in S3</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Data quality scorecard with pass/fail per validation rule; cleansed dataset or rejection notice</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Data quality score ≥95% (null rate &lt;2%, duplicate bookings &lt;0.5%, fare outliers &lt;1%)</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS ticket voids and exchanges frequently generate duplicate or partial booking records that inflate cancellation rate inputs to the NRM demand model, distorting recalibration outputs</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Load competitive fare and capacity benchmarks</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Competitor fare filing data from ATPCO; OAG Schedule Analyser capacity data for target O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Competitive context dataset: competitor fare ladder, capacity by carrier, schedule frequency</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Competitive data coverage ≥85% of target O&amp;D markets; data freshness within 48 hours of filing date</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare data covers only filed public fares; negotiated corporate and NDC-only fares are not visible, creating a systematic blind spot in price elasticity model inputs for corporate-heavy routes</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Recalibrate demand forecast model coefficients</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>RM Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Cleansed 24-month historical dataset; competitive context dataset; current NRM model parameter set</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Updated demand model coefficients (seasonality indices, trend factors, day-of-week multipliers) staged in NRM test partition</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Post-recalibration MAPE improvement ≥10% vs. baseline on hold-out validation set</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM parameter update interface requires batch file upload in proprietary format; no API-driven calibration workflow, increasing manual error risk and extending cycle time to 3–5 business days</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Update price elasticity and WTP model curves</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Updated demand model coefficients; ATPCO competitive fare ladder; passenger segment willingness-to-pay data</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Revised price elasticity curves and class-specific bid price adjustments per O&amp;D market cluster</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Bid price accuracy: simulated revenue within ±2% of optimal on hold-out markets; elasticity curve R² ≥0.88</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>WTP segmentation in Amadeus NRM is limited to cabin-level; lack of sub-segment granularity (e.g. loyalty tier, corporate account) reduces model precision for high-value O&amp;D pairs with mixed traffic composition</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Tune overbooking safety factors by route type</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Updated elasticity curves; historical no-show and cancellation rates by route category (short-haul leisure, long-haul corporate, thin route)</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Revised overbooking multipliers per route cluster; updated denied boarding risk scores</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Denied boarding rate ≤0.05 per 1,000 passengers; seat spoilage rate ≤2% of available seats</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Denied boarding compensation exposure under EU261/2004 and DOT rules creates asymmetric financial risk; NRM overbooking model does not natively incorporate regulatory compensation cost as an optimisation constraint</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Execute shadow-mode simulation on hold-out period</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>RM Systems Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Updated NRM parameter set (demand model + elasticity curves + overbooking factors); hold-out historical period (most recent 90 days not used in training)</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Shadow revenue report: simulated revenue and load factor for each O&amp;D flight in hold-out period</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Shadow simulation runtime ≤8 hours; simulated revenue variance vs. actuals ≤2%</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM shadow mode does not replicate real-time competitor price reactions; static competitor assumptions in simulation overstate revenue uplift potential by an estimated 0.5–1.0% on competitive routes</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate shadow revenue vs. actual revenue</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Optimization Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Shadow revenue report; actual revenue actuals from AWS Redshift for the same hold-out period</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Calibration validation dashboard: revenue lift by market cluster, load factor delta, booking class mix comparison</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Simulated revenue uplift ≥1.0% vs. actuals across all market clusters; no individual cluster showing revenue degradation &gt;0.5%</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue attribution between calibration changes and external demand factors (events, competitor capacity changes) is not automated; manual attribution analysis adds 1–2 days to the validation cycle</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Run live A/B test on selected pilot markets</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Validated calibration parameter set; pilot market selection (10–15 O&amp;D pairs representative of route clusters)</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>A/B test results: revenue per available seat kilometre (RASK) and load factor for treatment vs. control group over 4-week period</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>A/B revenue uplift ≥1.5% in pilot markets over 4-week test window at 95% statistical confidence</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Selecting statistically valid control markets is difficult on thin-route network where few true analogues exist; contamination risk between test and control markets sharing connections distorts A/B results</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Stage calibrated parameters in UAT environment</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>RM Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Approved calibration parameter set from A/B test; UAT deployment checklist</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>UAT environment loaded with new parameters; regression test results confirming no unintended impacts to adjacent processes (pricing, inventory, interline)</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>UAT regression test pass rate 100% on critical path; deployment staging completed within 1 business day</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM UAT environment is shared with pricing and ancillary revenue teams; uncoordinated deployments from parallel projects create parameter conflicts that require vendor support engagement to resolve</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Present calibration results for RM leadership sign-off</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Head of Revenue Management</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Microsoft Azure Synapse</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Calibration validation dashboard; A/B test results; UAT regression summary; estimated annual revenue impact</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Signed approval record or change request with required amendments; go/no-go decision for production deployment</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Sign-off decision turnaround ≤2 business days; zero production deployments without documented approval</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Calibration approval process is undocumented in most carriers; absence of a formal change control board for RM model changes means deployments can proceed without revenue risk assessment, creating audit exposure</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Deploy calibrated parameters to production NRM</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>RM Systems Engineer</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Signed approval record; staged parameter set from UAT; deployment runbook</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Production NRM updated with new demand model coefficients, elasticity curves, and overbooking factors; deployment confirmation log</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Production deployment completed within 4-hour maintenance window; zero unplanned system downtime during deployment</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM production parameter updates require a maintenance window coordinated with Amadeus support; last-minute scheduling conflicts with Altéa PSS maintenance windows have caused deployment delays of up to 72 hours</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-08</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>RM System Calibration &amp; Tuning</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Monitor live KPIs post-deployment</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Live booking data from Amadeus NRM; post-deployment KPI dashboard; baseline metrics from pre-calibration period</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>30-day post-deployment performance report; rollback recommendation if KPIs deteriorate beyond threshold</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>RASK improvement ≥1.0% vs. pre-calibration baseline within 30 days; no market showing load factor decline &gt;2 percentage points</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Post-deployment monitoring relies on manual Tableau dashboard review; absence of automated anomaly detection means revenue degradation from a miscalibrated market cluster may go undetected for 3–5 days, compounding financial impact</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add NP-RM-09: Post-Departure Revenue Reporting — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -30,6 +30,7 @@
     <sheet name="NP-RM-06" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="NP-RM-07" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="NP-RM-08" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="NP-RM-09" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1522,13 +1523,21 @@
           <t>Post-Departure Revenue Reporting</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="8" t="inlineStr"/>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-09</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -18819,7 +18828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N418"/>
+  <dimension ref="A1:N435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -48866,6 +48875,1230 @@
       <c r="N418" s="17" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="419" ht="30" customHeight="1">
+      <c r="A419" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B419" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C419" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D419" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E419" s="15" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F419" s="16" t="inlineStr">
+        <is>
+          <t>Trigger post-departure PSS revenue extract</t>
+        </is>
+      </c>
+      <c r="G419" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H419" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I419" s="16" t="inlineStr">
+        <is>
+          <t>Flight departure confirmation signal from Altéa DCS</t>
+        </is>
+      </c>
+      <c r="J419" s="16" t="inlineStr">
+        <is>
+          <t>Raw booking &amp; ticketing record extract per flight</t>
+        </is>
+      </c>
+      <c r="K419" s="16" t="inlineStr">
+        <is>
+          <t>Extract available within 30 min of block-in; ≥99.5% flight coverage</t>
+        </is>
+      </c>
+      <c r="L419" s="16" t="inlineStr">
+        <is>
+          <t>Altéa extract latency spikes during high-frequency bank departures, delaying same-day reporting windows</t>
+        </is>
+      </c>
+      <c r="M419" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N419" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="420" ht="30" customHeight="1">
+      <c r="A420" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B420" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C420" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D420" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E420" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F420" s="18" t="inlineStr">
+        <is>
+          <t>Pull ancillary revenue feeds from ancillary platform</t>
+        </is>
+      </c>
+      <c r="G420" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H420" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa Ancillary (Ancillary Services Manager)</t>
+        </is>
+      </c>
+      <c r="I420" s="18" t="inlineStr">
+        <is>
+          <t>Completed flight leg; ancillary transaction logs</t>
+        </is>
+      </c>
+      <c r="J420" s="18" t="inlineStr">
+        <is>
+          <t>Per-flight ancillary revenue breakdown (bags, seat upgrades, extras)</t>
+        </is>
+      </c>
+      <c r="K420" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary revenue captured per passenger ≥ airline target (e.g. USD 28/pax industry benchmark)</t>
+        </is>
+      </c>
+      <c r="L420" s="18" t="inlineStr">
+        <is>
+          <t>Ancillary items sold via NDC API Gateway may not post to Altéa in real time, creating gaps in same-day reporting</t>
+        </is>
+      </c>
+      <c r="M420" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N420" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="421" ht="30" customHeight="1">
+      <c r="A421" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B421" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C421" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D421" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E421" s="15" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F421" s="16" t="inlineStr">
+        <is>
+          <t>Validate booking-to-flown passenger completeness</t>
+        </is>
+      </c>
+      <c r="G421" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H421" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I421" s="16" t="inlineStr">
+        <is>
+          <t>DCS final manifest; booking record extract</t>
+        </is>
+      </c>
+      <c r="J421" s="16" t="inlineStr">
+        <is>
+          <t>Reconciled flown passenger count with no-show &amp; offload flags</t>
+        </is>
+      </c>
+      <c r="K421" s="16" t="inlineStr">
+        <is>
+          <t>Booking-to-manifest match rate ≥99.8% before proceeding</t>
+        </is>
+      </c>
+      <c r="L421" s="16" t="inlineStr">
+        <is>
+          <t>Last-minute irregular operations (IROPs) create orphan booking records that misstate flown revenue</t>
+        </is>
+      </c>
+      <c r="M421" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N421" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="422" ht="30" customHeight="1">
+      <c r="A422" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B422" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C422" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D422" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E422" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F422" s="18" t="inlineStr">
+        <is>
+          <t>Reconcile ticketed revenue vs. flown revenue</t>
+        </is>
+      </c>
+      <c r="G422" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H422" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I422" s="18" t="inlineStr">
+        <is>
+          <t>Altéa ticketing extract; flown passenger manifest</t>
+        </is>
+      </c>
+      <c r="J422" s="18" t="inlineStr">
+        <is>
+          <t>Flight-level ticketed vs. flown revenue variance report</t>
+        </is>
+      </c>
+      <c r="K422" s="18" t="inlineStr">
+        <is>
+          <t>Revenue variance tolerance ≤1% of flight revenue before exception flag</t>
+        </is>
+      </c>
+      <c r="L422" s="18" t="inlineStr">
+        <is>
+          <t>Multi-coupon interline tickets generate partial-revenue allocations that SAP FI cannot auto-match without manual MITA settlement codes</t>
+        </is>
+      </c>
+      <c r="M422" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N422" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="423" ht="30" customHeight="1">
+      <c r="A423" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B423" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C423" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D423" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E423" s="15" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F423" s="16" t="inlineStr">
+        <is>
+          <t>Match BSP &amp; interline settlement amounts</t>
+        </is>
+      </c>
+      <c r="G423" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H423" s="16" t="inlineStr">
+        <is>
+          <t>IATA BSPlink</t>
+        </is>
+      </c>
+      <c r="I423" s="16" t="inlineStr">
+        <is>
+          <t>BSP billing files; interline prorate agreements</t>
+        </is>
+      </c>
+      <c r="J423" s="16" t="inlineStr">
+        <is>
+          <t>Settled interline revenue allocation per flight segment</t>
+        </is>
+      </c>
+      <c r="K423" s="16" t="inlineStr">
+        <is>
+          <t>BSP settlement matched within 48 hours of departure; dispute rate &lt;0.5%</t>
+        </is>
+      </c>
+      <c r="L423" s="16" t="inlineStr">
+        <is>
+          <t>Prorate disputes with interline partners under MITA/BIMA can take 30–90 days to resolve, overstating interim revenue</t>
+        </is>
+      </c>
+      <c r="M423" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N423" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="424" ht="30" customHeight="1">
+      <c r="A424" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B424" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C424" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D424" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E424" s="17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F424" s="18" t="inlineStr">
+        <is>
+          <t>Validate upgrade &amp; no-show revenue capture</t>
+        </is>
+      </c>
+      <c r="G424" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H424" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I424" s="18" t="inlineStr">
+        <is>
+          <t>No-show records; upgrade transaction log from DCS</t>
+        </is>
+      </c>
+      <c r="J424" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed no-show penalty revenue and upgrade delta postings</t>
+        </is>
+      </c>
+      <c r="K424" s="18" t="inlineStr">
+        <is>
+          <t>No-show revenue leakage &lt;0.2% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L424" s="18" t="inlineStr">
+        <is>
+          <t>Oversold flights with denied boarding (IDB/VDB) generate compensation cost offsets that are frequently mis-posted against revenue rather than cost accounts</t>
+        </is>
+      </c>
+      <c r="M424" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N424" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="425" ht="30" customHeight="1">
+      <c r="A425" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B425" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C425" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D425" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E425" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F425" s="16" t="inlineStr">
+        <is>
+          <t>Aggregate O&amp;D revenue by fare class &amp; cabin</t>
+        </is>
+      </c>
+      <c r="G425" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H425" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I425" s="16" t="inlineStr">
+        <is>
+          <t>Reconciled flight revenue records; booking class mapping</t>
+        </is>
+      </c>
+      <c r="J425" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix by fare class, cabin, and market pair</t>
+        </is>
+      </c>
+      <c r="K425" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D attribution completeness ≥98% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L425" s="16" t="inlineStr">
+        <is>
+          <t>Point-to-point carriers with connecting itineraries lack native O&amp;D proration logic in Altéa; NRM must apply estimated prorate splits</t>
+        </is>
+      </c>
+      <c r="M425" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N425" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="426" ht="30" customHeight="1">
+      <c r="A426" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B426" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C426" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D426" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E426" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F426" s="18" t="inlineStr">
+        <is>
+          <t>Calculate RASM, PRASM, and load factor vs. forecast</t>
+        </is>
+      </c>
+      <c r="G426" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H426" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I426" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix; capacity data from Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J426" s="18" t="inlineStr">
+        <is>
+          <t>Flight-level RASM, PRASM, load factor actuals vs. forecast delta</t>
+        </is>
+      </c>
+      <c r="K426" s="18" t="inlineStr">
+        <is>
+          <t>RASM actuals within ±3% of pre-departure NRM forecast; load factor ≥83%</t>
+        </is>
+      </c>
+      <c r="L426" s="18" t="inlineStr">
+        <is>
+          <t>NRM forecast baseline uses O&amp;D demand curves that require 12+ months of history — new routes show high forecast error in first two seasons</t>
+        </is>
+      </c>
+      <c r="M426" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N426" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="427" ht="30" customHeight="1">
+      <c r="A427" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B427" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C427" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D427" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E427" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F427" s="16" t="inlineStr">
+        <is>
+          <t>Identify revenue spoilage and dilution events</t>
+        </is>
+      </c>
+      <c r="G427" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H427" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I427" s="16" t="inlineStr">
+        <is>
+          <t>RASM/PRASM variance report; fare class booking curve</t>
+        </is>
+      </c>
+      <c r="J427" s="16" t="inlineStr">
+        <is>
+          <t>Spoilage flag (unsold high-yield seats) or dilution flag (over-discounted load)</t>
+        </is>
+      </c>
+      <c r="K427" s="16" t="inlineStr">
+        <is>
+          <t>Spoilage rate ≤4% of available seats on constrained routes; dilution rate ≤2%</t>
+        </is>
+      </c>
+      <c r="L427" s="16" t="inlineStr">
+        <is>
+          <t>Automated RM bid-price controls in NRM cannot retroactively explain spoilage caused by schedule irregularities or competitor fare wars without manual analyst annotation</t>
+        </is>
+      </c>
+      <c r="M427" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N427" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="428" ht="30" customHeight="1">
+      <c r="A428" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B428" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C428" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D428" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E428" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F428" s="18" t="inlineStr">
+        <is>
+          <t>Generate flight-level post-departure P&amp;L report</t>
+        </is>
+      </c>
+      <c r="G428" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H428" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I428" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled revenue; ancillary revenue; prorate settlements</t>
+        </is>
+      </c>
+      <c r="J428" s="18" t="inlineStr">
+        <is>
+          <t>Flight-level revenue P&amp;L report with actuals vs. plan variance</t>
+        </is>
+      </c>
+      <c r="K428" s="18" t="inlineStr">
+        <is>
+          <t>Report generation within 4 hours of block-in for priority routes</t>
+        </is>
+      </c>
+      <c r="L428" s="18" t="inlineStr">
+        <is>
+          <t>SAP FI cost allocations for fuel and crew are posted at cost-centre level, not flight level — flight P&amp;L requires manual allocation keys that reduce accuracy</t>
+        </is>
+      </c>
+      <c r="M428" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N428" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="429" ht="30" customHeight="1">
+      <c r="A429" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B429" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C429" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D429" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E429" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F429" s="16" t="inlineStr">
+        <is>
+          <t>Publish variance dashboard for RM and Finance</t>
+        </is>
+      </c>
+      <c r="G429" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H429" s="16" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I429" s="16" t="inlineStr">
+        <is>
+          <t>Flight P&amp;L report; RASM/PRASM variance data</t>
+        </is>
+      </c>
+      <c r="J429" s="16" t="inlineStr">
+        <is>
+          <t>Interactive revenue variance dashboard published to BI portal</t>
+        </is>
+      </c>
+      <c r="K429" s="16" t="inlineStr">
+        <is>
+          <t>Dashboard refresh latency ≤1 hour from report generation; stakeholder access rate ≥90%</t>
+        </is>
+      </c>
+      <c r="L429" s="16" t="inlineStr">
+        <is>
+          <t>Tableau data extracts from SAP and NRM use separate ETL schedules, causing dashboard columns to reflect mixed reporting periods during refresh windows</t>
+        </is>
+      </c>
+      <c r="M429" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N429" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="430" ht="30" customHeight="1">
+      <c r="A430" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B430" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C430" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D430" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E430" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F430" s="18" t="inlineStr">
+        <is>
+          <t>Route significant variances to Revenue Director</t>
+        </is>
+      </c>
+      <c r="G430" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H430" s="18" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I430" s="18" t="inlineStr">
+        <is>
+          <t>Variance dashboard; threshold breach flags</t>
+        </is>
+      </c>
+      <c r="J430" s="18" t="inlineStr">
+        <is>
+          <t>Escalation notification with variance summary and root-cause annotation</t>
+        </is>
+      </c>
+      <c r="K430" s="18" t="inlineStr">
+        <is>
+          <t>Escalation triggered within 2 hours for variances ≥5% of planned flight revenue</t>
+        </is>
+      </c>
+      <c r="L430" s="18" t="inlineStr">
+        <is>
+          <t>No automated escalation workflow in SAP FI — analysts rely on manual email alerts, creating inconsistent escalation timing across regions</t>
+        </is>
+      </c>
+      <c r="M430" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N430" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="431" ht="30" customHeight="1">
+      <c r="A431" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B431" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C431" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D431" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E431" s="15" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F431" s="16" t="inlineStr">
+        <is>
+          <t>Distribute approved reports to RM and Finance teams</t>
+        </is>
+      </c>
+      <c r="G431" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Director</t>
+        </is>
+      </c>
+      <c r="H431" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I431" s="16" t="inlineStr">
+        <is>
+          <t>Approved flight-level revenue reports</t>
+        </is>
+      </c>
+      <c r="J431" s="16" t="inlineStr">
+        <is>
+          <t>Published report package to S3 data lake for downstream consumption</t>
+        </is>
+      </c>
+      <c r="K431" s="16" t="inlineStr">
+        <is>
+          <t>Distribution to all stakeholders within 6 hours of block-in for same-day flights</t>
+        </is>
+      </c>
+      <c r="L431" s="16" t="inlineStr">
+        <is>
+          <t>S3 IAM access policies differ between Revenue Management and Finance teams, requiring duplicate report versions with different data masking levels</t>
+        </is>
+      </c>
+      <c r="M431" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N431" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="432" ht="30" customHeight="1">
+      <c r="A432" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B432" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C432" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D432" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E432" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F432" s="18" t="inlineStr">
+        <is>
+          <t>Feed actuals into NRM for forecast comparison</t>
+        </is>
+      </c>
+      <c r="G432" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H432" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I432" s="18" t="inlineStr">
+        <is>
+          <t>Finalised flight revenue actuals from S3 data lake</t>
+        </is>
+      </c>
+      <c r="J432" s="18" t="inlineStr">
+        <is>
+          <t>Actuals posted to NRM historical performance database</t>
+        </is>
+      </c>
+      <c r="K432" s="18" t="inlineStr">
+        <is>
+          <t>Actuals feed completed within 24 hours of departure; data completeness ≥99%</t>
+        </is>
+      </c>
+      <c r="L432" s="18" t="inlineStr">
+        <is>
+          <t>NRM actuals ingestion pipeline requires structured SSIM-aligned flight keys — IROPs-affected flights with revised flight numbers create orphan actuals that must be manually re-keyed</t>
+        </is>
+      </c>
+      <c r="M432" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N432" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="433" ht="30" customHeight="1">
+      <c r="A433" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B433" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C433" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D433" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E433" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F433" s="16" t="inlineStr">
+        <is>
+          <t>Assess forecast model error vs. recalibration threshold</t>
+        </is>
+      </c>
+      <c r="G433" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H433" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I433" s="16" t="inlineStr">
+        <is>
+          <t>Actuals vs. NRM forecast delta; rolling MAPE statistics</t>
+        </is>
+      </c>
+      <c r="J433" s="16" t="inlineStr">
+        <is>
+          <t>Recalibration decision flag: proceed or trigger model update</t>
+        </is>
+      </c>
+      <c r="K433" s="16" t="inlineStr">
+        <is>
+          <t>MAPE ≤8% on 30-day rolling basis; trigger recalibration if MAPE &gt;10% for 5 consecutive days</t>
+        </is>
+      </c>
+      <c r="L433" s="16" t="inlineStr">
+        <is>
+          <t>NRM model recalibration jobs require 4–6 hour processing windows that temporarily freeze bid-price updates, creating yield management blind spots during peak booking periods</t>
+        </is>
+      </c>
+      <c r="M433" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N433" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="434" ht="30" customHeight="1">
+      <c r="A434" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B434" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C434" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D434" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E434" s="17" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F434" s="18" t="inlineStr">
+        <is>
+          <t>Trigger NRM demand model recalibration job</t>
+        </is>
+      </c>
+      <c r="G434" s="18" t="inlineStr">
+        <is>
+          <t>RM Systems Administrator</t>
+        </is>
+      </c>
+      <c r="H434" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I434" s="18" t="inlineStr">
+        <is>
+          <t>Recalibration trigger flag; accumulated actuals dataset</t>
+        </is>
+      </c>
+      <c r="J434" s="18" t="inlineStr">
+        <is>
+          <t>Updated NRM demand model parameters; recalibration completion log</t>
+        </is>
+      </c>
+      <c r="K434" s="18" t="inlineStr">
+        <is>
+          <t>Recalibration job completes within 6-hour maintenance window; model improvement verified by ≥1% MAPE reduction</t>
+        </is>
+      </c>
+      <c r="L434" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus NRM recalibration requires coordination with Amadeus managed services SLA (8-hour response window), delaying urgent corrections during high-yield periods such as holiday blocks</t>
+        </is>
+      </c>
+      <c r="M434" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N434" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="435" ht="30" customHeight="1">
+      <c r="A435" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B435" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C435" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D435" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E435" s="15" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F435" s="16" t="inlineStr">
+        <is>
+          <t>Archive finalised flight revenue record to data lake</t>
+        </is>
+      </c>
+      <c r="G435" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H435" s="16" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I435" s="16" t="inlineStr">
+        <is>
+          <t>Validated &amp; reconciled flight revenue package</t>
+        </is>
+      </c>
+      <c r="J435" s="16" t="inlineStr">
+        <is>
+          <t>Immutable flight revenue archive record in S3 with audit trail</t>
+        </is>
+      </c>
+      <c r="K435" s="16" t="inlineStr">
+        <is>
+          <t>100% of departed flights archived within 24 hours; retention compliance per IATA Resolution 787 (7-year minimum)</t>
+        </is>
+      </c>
+      <c r="L435" s="16" t="inlineStr">
+        <is>
+          <t>S3 lifecycle policies must balance cost (Glacier transition) against ad-hoc audit retrieval SLAs — retrieval from Glacier takes 3–5 hours, conflicting with same-day audit requests</t>
+        </is>
+      </c>
+      <c r="M435" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N435" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -54181,6 +55414,1350 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-09 — Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Trigger post-departure PSS revenue extract</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Flight departure confirmation signal from Altéa DCS</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Raw booking &amp; ticketing record extract per flight</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Extract available within 30 min of block-in; ≥99.5% flight coverage</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Altéa extract latency spikes during high-frequency bank departures, delaying same-day reporting windows</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Pull ancillary revenue feeds from ancillary platform</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa Ancillary (Ancillary Services Manager)</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Completed flight leg; ancillary transaction logs</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Per-flight ancillary revenue breakdown (bags, seat upgrades, extras)</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary revenue captured per passenger ≥ airline target (e.g. USD 28/pax industry benchmark)</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Ancillary items sold via NDC API Gateway may not post to Altéa in real time, creating gaps in same-day reporting</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Validate booking-to-flown passenger completeness</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>DCS final manifest; booking record extract</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled flown passenger count with no-show &amp; offload flags</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Booking-to-manifest match rate ≥99.8% before proceeding</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Last-minute irregular operations (IROPs) create orphan booking records that misstate flown revenue</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Reconcile ticketed revenue vs. flown revenue</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Altéa ticketing extract; flown passenger manifest</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Flight-level ticketed vs. flown revenue variance report</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue variance tolerance ≤1% of flight revenue before exception flag</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Multi-coupon interline tickets generate partial-revenue allocations that SAP FI cannot auto-match without manual MITA settlement codes</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Match BSP &amp; interline settlement amounts</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>IATA BSPlink</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>BSP billing files; interline prorate agreements</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Settled interline revenue allocation per flight segment</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>BSP settlement matched within 48 hours of departure; dispute rate &lt;0.5%</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Prorate disputes with interline partners under MITA/BIMA can take 30–90 days to resolve, overstating interim revenue</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Validate upgrade &amp; no-show revenue capture</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Accounting Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>No-show records; upgrade transaction log from DCS</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed no-show penalty revenue and upgrade delta postings</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>No-show revenue leakage &lt;0.2% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Oversold flights with denied boarding (IDB/VDB) generate compensation cost offsets that are frequently mis-posted against revenue rather than cost accounts</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Aggregate O&amp;D revenue by fare class &amp; cabin</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled flight revenue records; booking class mapping</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix by fare class, cabin, and market pair</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>O&amp;D attribution completeness ≥98% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Point-to-point carriers with connecting itineraries lack native O&amp;D proration logic in Altéa; NRM must apply estimated prorate splits</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Calculate RASM, PRASM, and load factor vs. forecast</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>O&amp;D revenue matrix; capacity data from Amadeus SkyWORKS</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Flight-level RASM, PRASM, load factor actuals vs. forecast delta</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>RASM actuals within ±3% of pre-departure NRM forecast; load factor ≥83%</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>NRM forecast baseline uses O&amp;D demand curves that require 12+ months of history — new routes show high forecast error in first two seasons</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Identify revenue spoilage and dilution events</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>RASM/PRASM variance report; fare class booking curve</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Spoilage flag (unsold high-yield seats) or dilution flag (over-discounted load)</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Spoilage rate ≤4% of available seats on constrained routes; dilution rate ≤2%</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Automated RM bid-price controls in NRM cannot retroactively explain spoilage caused by schedule irregularities or competitor fare wars without manual analyst annotation</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Generate flight-level post-departure P&amp;L report</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Reconciled revenue; ancillary revenue; prorate settlements</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Flight-level revenue P&amp;L report with actuals vs. plan variance</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Report generation within 4 hours of block-in for priority routes</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>SAP FI cost allocations for fuel and crew are posted at cost-centre level, not flight level — flight P&amp;L requires manual allocation keys that reduce accuracy</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Publish variance dashboard for RM and Finance</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Flight P&amp;L report; RASM/PRASM variance data</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Interactive revenue variance dashboard published to BI portal</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Dashboard refresh latency ≤1 hour from report generation; stakeholder access rate ≥90%</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Tableau data extracts from SAP and NRM use separate ETL schedules, causing dashboard columns to reflect mixed reporting periods during refresh windows</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Route significant variances to Revenue Director</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Manager</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA Finance (FI/CO)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Variance dashboard; threshold breach flags</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Escalation notification with variance summary and root-cause annotation</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Escalation triggered within 2 hours for variances ≥5% of planned flight revenue</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>No automated escalation workflow in SAP FI — analysts rely on manual email alerts, creating inconsistent escalation timing across regions</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Distribute approved reports to RM and Finance teams</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Director</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Approved flight-level revenue reports</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Published report package to S3 data lake for downstream consumption</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Distribution to all stakeholders within 6 hours of block-in for same-day flights</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>S3 IAM access policies differ between Revenue Management and Finance teams, requiring duplicate report versions with different data masking levels</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Feed actuals into NRM for forecast comparison</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Finalised flight revenue actuals from S3 data lake</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Actuals posted to NRM historical performance database</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Actuals feed completed within 24 hours of departure; data completeness ≥99%</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>NRM actuals ingestion pipeline requires structured SSIM-aligned flight keys — IROPs-affected flights with revised flight numbers create orphan actuals that must be manually re-keyed</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Assess forecast model error vs. recalibration threshold</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Actuals vs. NRM forecast delta; rolling MAPE statistics</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Recalibration decision flag: proceed or trigger model update</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>MAPE ≤8% on 30-day rolling basis; trigger recalibration if MAPE &gt;10% for 5 consecutive days</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>NRM model recalibration jobs require 4–6 hour processing windows that temporarily freeze bid-price updates, creating yield management blind spots during peak booking periods</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Trigger NRM demand model recalibration job</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>RM Systems Administrator</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Recalibration trigger flag; accumulated actuals dataset</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Updated NRM demand model parameters; recalibration completion log</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Recalibration job completes within 6-hour maintenance window; model improvement verified by ≥1% MAPE reduction</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus NRM recalibration requires coordination with Amadeus managed services SLA (8-hour response window), delaying urgent corrections during high-yield periods such as holiday blocks</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-09</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Post-Departure Revenue Reporting</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Archive finalised flight revenue record to data lake</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Validated &amp; reconciled flight revenue package</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Immutable flight revenue archive record in S3 with audit trail</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>100% of departed flights archived within 24 hours; retention compliance per IATA Resolution 787 (7-year minimum)</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>S3 lifecycle policies must balance cost (Glacier transition) against ad-hoc audit retrieval SLAs — retrieval from Glacier takes 3–5 hours, conflicting with same-day audit requests</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add NP-RM-10: Competitive Fare Monitoring & Response — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -31,6 +31,7 @@
     <sheet name="NP-RM-07" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="NP-RM-08" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="NP-RM-09" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="NP-RM-10" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1560,13 +1561,21 @@
           <t>Competitive Fare Monitoring &amp; Response</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr"/>
-      <c r="G27" s="10" t="inlineStr"/>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-10</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -18828,7 +18837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N435"/>
+  <dimension ref="A1:N451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -50097,6 +50106,1158 @@
         </is>
       </c>
       <c r="N435" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="436" ht="30" customHeight="1">
+      <c r="A436" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B436" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C436" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D436" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E436" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F436" s="18" t="inlineStr">
+        <is>
+          <t>Ingest ATPCO competitor fare feed</t>
+        </is>
+      </c>
+      <c r="G436" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H436" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I436" s="18" t="inlineStr">
+        <is>
+          <t>Scheduled ATPCO Fare Update (FU) and Fare Distribution (FD) transmissions</t>
+        </is>
+      </c>
+      <c r="J436" s="18" t="inlineStr">
+        <is>
+          <t>Structured fare change dataset by O&amp;D, booking class, and carrier</t>
+        </is>
+      </c>
+      <c r="K436" s="18" t="inlineStr">
+        <is>
+          <t>Feed latency ≤30 min from ATPCO publication; 100% O&amp;D coverage on monitored routes</t>
+        </is>
+      </c>
+      <c r="L436" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO batch update cycles (typically 3× daily) create lag vs. real-time OTA price changes; competitor fares visible on GDS before ATPCO reflects them</t>
+        </is>
+      </c>
+      <c r="M436" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N436" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="437" ht="30" customHeight="1">
+      <c r="A437" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B437" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C437" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D437" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E437" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F437" s="16" t="inlineStr">
+        <is>
+          <t>Scrape OTA &amp; metasearch displayed fares</t>
+        </is>
+      </c>
+      <c r="G437" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H437" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I437" s="16" t="inlineStr">
+        <is>
+          <t>Automated scrape schedule for key O&amp;D markets; ATPCO baseline fare dataset</t>
+        </is>
+      </c>
+      <c r="J437" s="16" t="inlineStr">
+        <is>
+          <t>Displayed-price dataset including taxes, carrier surcharges, and ancillary bundling</t>
+        </is>
+      </c>
+      <c r="K437" s="16" t="inlineStr">
+        <is>
+          <t>Scrape coverage ≥95% of tier-1 competitive routes; data freshness ≤60 min</t>
+        </is>
+      </c>
+      <c r="L437" s="16" t="inlineStr">
+        <is>
+          <t>NDC-sourced fares from competitors bypass ATPCO and are invisible to traditional monitoring tools; requires separate NDC channel scraping capability not standard in OAG</t>
+        </is>
+      </c>
+      <c r="M437" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N437" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="438" ht="30" customHeight="1">
+      <c r="A438" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B438" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C438" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D438" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E438" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F438" s="18" t="inlineStr">
+        <is>
+          <t>Detect and flag material fare changes</t>
+        </is>
+      </c>
+      <c r="G438" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H438" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I438" s="18" t="inlineStr">
+        <is>
+          <t>Combined ATPCO and OTA fare datasets; pre-configured alert thresholds by market tier</t>
+        </is>
+      </c>
+      <c r="J438" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised alert queue: fare changes ≥10% on tier-1 routes, ≥15% on tier-2</t>
+        </is>
+      </c>
+      <c r="K438" s="18" t="inlineStr">
+        <is>
+          <t>False-positive alert rate ≤5%; mean time to analyst notification ≤15 min from ingestion</t>
+        </is>
+      </c>
+      <c r="L438" s="18" t="inlineStr">
+        <is>
+          <t>Threshold calibration is static; promotional fare launches by LCCs in thin markets trigger high false-positive volumes that overwhelm analyst queues</t>
+        </is>
+      </c>
+      <c r="M438" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N438" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="439" ht="30" customHeight="1">
+      <c r="A439" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B439" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C439" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D439" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E439" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F439" s="16" t="inlineStr">
+        <is>
+          <t>Analyse competitor O&amp;D fare positioning</t>
+        </is>
+      </c>
+      <c r="G439" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H439" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I439" s="16" t="inlineStr">
+        <is>
+          <t>Flagged fare alert; historical competitor fare trend data from data lake</t>
+        </is>
+      </c>
+      <c r="J439" s="16" t="inlineStr">
+        <is>
+          <t>Competitive positioning report: own fare vs. competitor by cabin, booking class, and departure window</t>
+        </is>
+      </c>
+      <c r="K439" s="16" t="inlineStr">
+        <is>
+          <t>Analysis turnaround ≤2 hr for tier-1 alerts; ≤8 hr for tier-2</t>
+        </is>
+      </c>
+      <c r="L439" s="16" t="inlineStr">
+        <is>
+          <t>NRM lacks a native competitor fare visualisation layer; analysts context-switch between NRM and Tableau dashboards, increasing error risk and analysis time</t>
+        </is>
+      </c>
+      <c r="M439" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N439" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="440" ht="30" customHeight="1">
+      <c r="A440" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B440" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C440" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D440" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E440" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F440" s="18" t="inlineStr">
+        <is>
+          <t>Assess impact on O&amp;D demand forecast</t>
+        </is>
+      </c>
+      <c r="G440" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H440" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I440" s="18" t="inlineStr">
+        <is>
+          <t>Competitive positioning report; current NRM demand forecast and booking curve</t>
+        </is>
+      </c>
+      <c r="J440" s="18" t="inlineStr">
+        <is>
+          <t>Demand sensitivity estimate: projected booking-curve shift under current and revised fare scenarios</t>
+        </is>
+      </c>
+      <c r="K440" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy within ±5% MAPE post-response on monitored O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L440" s="18" t="inlineStr">
+        <is>
+          <t>NRM demand models have limited sensitivity to intraday competitor fare moves on ultra-short booking windows (&lt;72 hr); last-minute price wars require manual forecast override</t>
+        </is>
+      </c>
+      <c r="M440" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N440" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="441" ht="30" customHeight="1">
+      <c r="A441" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B441" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C441" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D441" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E441" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F441" s="16" t="inlineStr">
+        <is>
+          <t>Classify response urgency and route tier</t>
+        </is>
+      </c>
+      <c r="G441" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H441" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I441" s="16" t="inlineStr">
+        <is>
+          <t>Demand impact estimate; route revenue contribution ranking; days-to-departure</t>
+        </is>
+      </c>
+      <c r="J441" s="16" t="inlineStr">
+        <is>
+          <t>Urgency classification: Immediate (≤4 hr), Same-day, Scheduled review</t>
+        </is>
+      </c>
+      <c r="K441" s="16" t="inlineStr">
+        <is>
+          <t>Immediate-class alerts actioned within 4 hr in ≥90% of cases</t>
+        </is>
+      </c>
+      <c r="L441" s="16" t="inlineStr">
+        <is>
+          <t>Revenue contribution rankings in Tableau are refreshed nightly; intraday revenue shifts on high-value routes are not reflected in urgency scoring during the same business day</t>
+        </is>
+      </c>
+      <c r="M441" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N441" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="442" ht="30" customHeight="1">
+      <c r="A442" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B442" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C442" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D442" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E442" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F442" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate inventory availability and load factor</t>
+        </is>
+      </c>
+      <c r="G442" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H442" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I442" s="18" t="inlineStr">
+        <is>
+          <t>Urgency classification; current fare bucket availability by flight and departure date</t>
+        </is>
+      </c>
+      <c r="J442" s="18" t="inlineStr">
+        <is>
+          <t>Inventory health snapshot: available seats by fare bucket, current load factor, revenue-per-available-seat-mile (RASM)</t>
+        </is>
+      </c>
+      <c r="K442" s="18" t="inlineStr">
+        <is>
+          <t>Load factor target ≥83% on relevant departure; RASM ≥ route budget</t>
+        </is>
+      </c>
+      <c r="L442" s="18" t="inlineStr">
+        <is>
+          <t>Opening low fare buckets to match competitor on near-full flights cannibalises higher-yield bookings already in the pipe; NRM bid-price guardrails may not prevent this on short notice</t>
+        </is>
+      </c>
+      <c r="M442" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N442" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="443" ht="30" customHeight="1">
+      <c r="A443" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B443" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C443" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D443" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E443" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F443" s="16" t="inlineStr">
+        <is>
+          <t>Model fare response scenarios in NRM</t>
+        </is>
+      </c>
+      <c r="G443" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H443" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I443" s="16" t="inlineStr">
+        <is>
+          <t>Inventory health snapshot; competitor fare structure; elasticity parameters from historical data</t>
+        </is>
+      </c>
+      <c r="J443" s="16" t="inlineStr">
+        <is>
+          <t>3–5 response scenario outputs: match, undercut, hold, selective open/close by booking window</t>
+        </is>
+      </c>
+      <c r="K443" s="16" t="inlineStr">
+        <is>
+          <t>Scenario modelling completed within 1 hr of escalation; ≥3 scenarios produced per alert</t>
+        </is>
+      </c>
+      <c r="L443" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM scenario engine requires clean elasticity inputs; thin-route O&amp;Ds with &lt;12 months of data produce unreliable price-sensitivity curves, forcing analyst judgment over model output</t>
+        </is>
+      </c>
+      <c r="M443" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N443" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="444" ht="30" customHeight="1">
+      <c r="A444" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B444" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C444" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D444" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E444" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F444" s="18" t="inlineStr">
+        <is>
+          <t>Review and approve response strategy</t>
+        </is>
+      </c>
+      <c r="G444" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H444" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I444" s="18" t="inlineStr">
+        <is>
+          <t>Modelled response scenarios; route revenue budget; commercial policy guardrails</t>
+        </is>
+      </c>
+      <c r="J444" s="18" t="inlineStr">
+        <is>
+          <t>Approved response strategy with rationale, fare targets, booking-class assignments, and validity period</t>
+        </is>
+      </c>
+      <c r="K444" s="18" t="inlineStr">
+        <is>
+          <t>Approval cycle ≤2 hr for immediate-class alerts; sign-off documented in NRM audit trail</t>
+        </is>
+      </c>
+      <c r="L444" s="18" t="inlineStr">
+        <is>
+          <t>Commercial policy guardrails (minimum fare floors, allotment restrictions for corporate accounts) are maintained separately in ATPCO and not surfaced within NRM approval workflow, risking policy violations</t>
+        </is>
+      </c>
+      <c r="M444" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N444" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="445" ht="30" customHeight="1">
+      <c r="A445" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B445" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C445" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D445" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E445" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F445" s="16" t="inlineStr">
+        <is>
+          <t>File revised fares via ATPCO submissions</t>
+        </is>
+      </c>
+      <c r="G445" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H445" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I445" s="16" t="inlineStr">
+        <is>
+          <t>Approved response strategy; current fare tariff record for affected O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="J445" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare submission batch: new or amended fare basis codes, amounts, and effective dates</t>
+        </is>
+      </c>
+      <c r="K445" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO filing completeness 100% for approved O&amp;Ds; filing-to-effective lag ≤3 hr (next ATPCO update cycle)</t>
+        </is>
+      </c>
+      <c r="L445" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO update cycles constrain real-time parity; competitors using direct NDC filing can respond 2–3 hr faster, creating a temporary price-visibility disadvantage in GDS</t>
+        </is>
+      </c>
+      <c r="M445" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N445" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="446" ht="30" customHeight="1">
+      <c r="A446" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B446" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C446" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D446" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E446" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F446" s="18" t="inlineStr">
+        <is>
+          <t>Configure fare rules, restrictions, and RBDs</t>
+        </is>
+      </c>
+      <c r="G446" s="18" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H446" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I446" s="18" t="inlineStr">
+        <is>
+          <t>Approved response strategy; existing rule categories (Cat 2, 3, 5, 14, 15, 35)</t>
+        </is>
+      </c>
+      <c r="J446" s="18" t="inlineStr">
+        <is>
+          <t>Updated fare rules: advance purchase, minimum stay, combinability, blackout dates, refund conditions</t>
+        </is>
+      </c>
+      <c r="K446" s="18" t="inlineStr">
+        <is>
+          <t>Zero ATPCO rule validation errors on submission; rules audit-compliant with IATA Resolution 024</t>
+        </is>
+      </c>
+      <c r="L446" s="18" t="inlineStr">
+        <is>
+          <t>Complex combinability rules (Cat 10) for interline itineraries require manual review against partner agreements; errors result in GDS pricing rejections and customer-visible mispricing</t>
+        </is>
+      </c>
+      <c r="M446" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N446" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="447" ht="30" customHeight="1">
+      <c r="A447" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B447" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C447" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D447" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E447" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F447" s="16" t="inlineStr">
+        <is>
+          <t>Verify fare distribution across GDS channels</t>
+        </is>
+      </c>
+      <c r="G447" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H447" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I447" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO effective fare update notification; test O&amp;D city pairs</t>
+        </is>
+      </c>
+      <c r="J447" s="16" t="inlineStr">
+        <is>
+          <t>GDS distribution verification report: fare visible and correctly priced in Sabre, Travelport, and Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="K447" s="16" t="inlineStr">
+        <is>
+          <t>Fare parity confirmed across ≥3 GDS within 60 min of ATPCO effective time; zero pricing discrepancies on spot-check O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L447" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS cache refresh lags Sabre by up to 45 min post-ATPCO update; customers on Travelport-connected TMCs see stale competitor fares, causing booking leakage during the gap</t>
+        </is>
+      </c>
+      <c r="M447" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N447" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="448" ht="30" customHeight="1">
+      <c r="A448" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B448" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C448" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D448" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E448" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F448" s="18" t="inlineStr">
+        <is>
+          <t>Activate fares in PSS inventory and NDC</t>
+        </is>
+      </c>
+      <c r="G448" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H448" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I448" s="18" t="inlineStr">
+        <is>
+          <t>GDS verification sign-off; NDC API Gateway configuration</t>
+        </is>
+      </c>
+      <c r="J448" s="18" t="inlineStr">
+        <is>
+          <t>Live fare availability confirmed in Altéa inventory and NDC API offer response</t>
+        </is>
+      </c>
+      <c r="K448" s="18" t="inlineStr">
+        <is>
+          <t>NDC offer response includes new fare within 30 min of Altéa activation; booking class availability aligned with approved strategy</t>
+        </is>
+      </c>
+      <c r="L448" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS inventory bucket mapping to ATPCO booking class codes requires manual reconciliation when new fare basis codes are introduced; mapping errors cause sell-up failures</t>
+        </is>
+      </c>
+      <c r="M448" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N448" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="449" ht="30" customHeight="1">
+      <c r="A449" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B449" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C449" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D449" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E449" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F449" s="16" t="inlineStr">
+        <is>
+          <t>Monitor booking velocity post-response</t>
+        </is>
+      </c>
+      <c r="G449" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H449" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I449" s="16" t="inlineStr">
+        <is>
+          <t>Live booking stream from Altéa PSS; pre-response booking curve baseline</t>
+        </is>
+      </c>
+      <c r="J449" s="16" t="inlineStr">
+        <is>
+          <t>Booking velocity dashboard: actual vs. forecast bookings by fare bucket, hourly cadence for 24 hr post-activation</t>
+        </is>
+      </c>
+      <c r="K449" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace recovery to baseline curve within 24 hr on ≥80% of actioned O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L449" s="16" t="inlineStr">
+        <is>
+          <t>NRM booking-curve comparison uses historical same-departure-day data that may not account for week-of-year seasonality shifts; recovery signals can be misread on holidays or event periods</t>
+        </is>
+      </c>
+      <c r="M449" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N449" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="450" ht="30" customHeight="1">
+      <c r="A450" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B450" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C450" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D450" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E450" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F450" s="18" t="inlineStr">
+        <is>
+          <t>Assess revenue impact against route budget</t>
+        </is>
+      </c>
+      <c r="G450" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H450" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I450" s="18" t="inlineStr">
+        <is>
+          <t>48-hr post-response booking and revenue data from Redshift data lake; route budget targets</t>
+        </is>
+      </c>
+      <c r="J450" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact report: incremental revenue vs. estimated dilution cost; net yield delta</t>
+        </is>
+      </c>
+      <c r="K450" s="18" t="inlineStr">
+        <is>
+          <t>Net yield delta ≥0% vs. pre-response baseline within 48 hr; RASM maintained ≥ route budget</t>
+        </is>
+      </c>
+      <c r="L450" s="18" t="inlineStr">
+        <is>
+          <t>Dilution cost from opening low fare buckets is not automatically calculated in NRM; analysts must manually query Redshift to isolate response-attributable revenue changes from organic demand shifts</t>
+        </is>
+      </c>
+      <c r="M450" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N450" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="451" ht="30" customHeight="1">
+      <c r="A451" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B451" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C451" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D451" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E451" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F451" s="16" t="inlineStr">
+        <is>
+          <t>Conduct post-action review and update playbook</t>
+        </is>
+      </c>
+      <c r="G451" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H451" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I451" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact report; response timeline audit trail from ATPCO and NRM</t>
+        </is>
+      </c>
+      <c r="J451" s="16" t="inlineStr">
+        <is>
+          <t>Post-action review record: strategy effectiveness score, lessons learned, and updated competitive response playbook entry</t>
+        </is>
+      </c>
+      <c r="K451" s="16" t="inlineStr">
+        <is>
+          <t>Post-action review completed within 5 business days for tier-1 alerts; playbook updated within 10 business days</t>
+        </is>
+      </c>
+      <c r="L451" s="16" t="inlineStr">
+        <is>
+          <t>Competitive response playbooks are maintained as unstructured documents outside RM systems; institutional knowledge of effective response patterns is lost when analysts rotate, and playbook entries are rarely linked to outcome data</t>
+        </is>
+      </c>
+      <c r="M451" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N451" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -56758,6 +57919,1278 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-10 — Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Ingest ATPCO competitor fare feed</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Scheduled ATPCO Fare Update (FU) and Fare Distribution (FD) transmissions</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Structured fare change dataset by O&amp;D, booking class, and carrier</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Feed latency ≤30 min from ATPCO publication; 100% O&amp;D coverage on monitored routes</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO batch update cycles (typically 3× daily) create lag vs. real-time OTA price changes; competitor fares visible on GDS before ATPCO reflects them</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Scrape OTA &amp; metasearch displayed fares</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Intelligence Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>OAG Schedule Analyser</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Automated scrape schedule for key O&amp;D markets; ATPCO baseline fare dataset</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Displayed-price dataset including taxes, carrier surcharges, and ancillary bundling</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Scrape coverage ≥95% of tier-1 competitive routes; data freshness ≤60 min</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>NDC-sourced fares from competitors bypass ATPCO and are invisible to traditional monitoring tools; requires separate NDC channel scraping capability not standard in OAG</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Detect and flag material fare changes</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management System</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Combined ATPCO and OTA fare datasets; pre-configured alert thresholds by market tier</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Prioritised alert queue: fare changes ≥10% on tier-1 routes, ≥15% on tier-2</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>False-positive alert rate ≤5%; mean time to analyst notification ≤15 min from ingestion</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Threshold calibration is static; promotional fare launches by LCCs in thin markets trigger high false-positive volumes that overwhelm analyst queues</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Analyse competitor O&amp;D fare positioning</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Flagged fare alert; historical competitor fare trend data from data lake</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Competitive positioning report: own fare vs. competitor by cabin, booking class, and departure window</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Analysis turnaround ≤2 hr for tier-1 alerts; ≤8 hr for tier-2</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>NRM lacks a native competitor fare visualisation layer; analysts context-switch between NRM and Tableau dashboards, increasing error risk and analysis time</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Assess impact on O&amp;D demand forecast</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Competitive positioning report; current NRM demand forecast and booking curve</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Demand sensitivity estimate: projected booking-curve shift under current and revised fare scenarios</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Forecast accuracy within ±5% MAPE post-response on monitored O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>NRM demand models have limited sensitivity to intraday competitor fare moves on ultra-short booking windows (&lt;72 hr); last-minute price wars require manual forecast override</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Classify response urgency and route tier</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Demand impact estimate; route revenue contribution ranking; days-to-departure</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Urgency classification: Immediate (≤4 hr), Same-day, Scheduled review</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Immediate-class alerts actioned within 4 hr in ≥90% of cases</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue contribution rankings in Tableau are refreshed nightly; intraday revenue shifts on high-value routes are not reflected in urgency scoring during the same business day</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate inventory availability and load factor</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Urgency classification; current fare bucket availability by flight and departure date</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Inventory health snapshot: available seats by fare bucket, current load factor, revenue-per-available-seat-mile (RASM)</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Load factor target ≥83% on relevant departure; RASM ≥ route budget</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Opening low fare buckets to match competitor on near-full flights cannibalises higher-yield bookings already in the pipe; NRM bid-price guardrails may not prevent this on short notice</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Model fare response scenarios in NRM</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Inventory health snapshot; competitor fare structure; elasticity parameters from historical data</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>3–5 response scenario outputs: match, undercut, hold, selective open/close by booking window</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Scenario modelling completed within 1 hr of escalation; ≥3 scenarios produced per alert</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>PROS RM scenario engine requires clean elasticity inputs; thin-route O&amp;Ds with &lt;12 months of data produce unreliable price-sensitivity curves, forcing analyst judgment over model output</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Review and approve response strategy</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Modelled response scenarios; route revenue budget; commercial policy guardrails</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Approved response strategy with rationale, fare targets, booking-class assignments, and validity period</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Approval cycle ≤2 hr for immediate-class alerts; sign-off documented in NRM audit trail</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Commercial policy guardrails (minimum fare floors, allotment restrictions for corporate accounts) are maintained separately in ATPCO and not surfaced within NRM approval workflow, risking policy violations</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>File revised fares via ATPCO submissions</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Approved response strategy; current fare tariff record for affected O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare submission batch: new or amended fare basis codes, amounts, and effective dates</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO filing completeness 100% for approved O&amp;Ds; filing-to-effective lag ≤3 hr (next ATPCO update cycle)</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO update cycles constrain real-time parity; competitors using direct NDC filing can respond 2–3 hr faster, creating a temporary price-visibility disadvantage in GDS</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Configure fare rules, restrictions, and RBDs</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Approved response strategy; existing rule categories (Cat 2, 3, 5, 14, 15, 35)</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Updated fare rules: advance purchase, minimum stay, combinability, blackout dates, refund conditions</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Zero ATPCO rule validation errors on submission; rules audit-compliant with IATA Resolution 024</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Complex combinability rules (Cat 10) for interline itineraries require manual review against partner agreements; errors result in GDS pricing rejections and customer-visible mispricing</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Verify fare distribution across GDS channels</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Sabre GDS</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO effective fare update notification; test O&amp;D city pairs</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>GDS distribution verification report: fare visible and correctly priced in Sabre, Travelport, and Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Fare parity confirmed across ≥3 GDS within 60 min of ATPCO effective time; zero pricing discrepancies on spot-check O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Travelport GDS cache refresh lags Sabre by up to 45 min post-ATPCO update; customers on Travelport-connected TMCs see stale competitor fares, causing booking leakage during the gap</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Activate fares in PSS inventory and NDC</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>GDS verification sign-off; NDC API Gateway configuration</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Live fare availability confirmed in Altéa inventory and NDC API offer response</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>NDC offer response includes new fare within 30 min of Altéa activation; booking class availability aligned with approved strategy</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Altéa PSS inventory bucket mapping to ATPCO booking class codes requires manual reconciliation when new fare basis codes are introduced; mapping errors cause sell-up failures</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Monitor booking velocity post-response</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM / AltéaRM)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Live booking stream from Altéa PSS; pre-response booking curve baseline</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Booking velocity dashboard: actual vs. forecast bookings by fare bucket, hourly cadence for 24 hr post-activation</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace recovery to baseline curve within 24 hr on ≥80% of actioned O&amp;Ds</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>NRM booking-curve comparison uses historical same-departure-day data that may not account for week-of-year seasonality shifts; recovery signals can be misread on holidays or event periods</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Assess revenue impact against route budget</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Manager</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>AWS S3 / Redshift</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>48-hr post-response booking and revenue data from Redshift data lake; route budget targets</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue impact report: incremental revenue vs. estimated dilution cost; net yield delta</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Net yield delta ≥0% vs. pre-response baseline within 48 hr; RASM maintained ≥ route budget</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Dilution cost from opening low fare buckets is not automatically calculated in NRM; analysts must manually query Redshift to isolate response-attributable revenue changes from organic demand shifts</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-10</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Competitive Fare Monitoring &amp; Response</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Conduct post-action review and update playbook</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Tableau / Power BI</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact report; response timeline audit trail from ATPCO and NRM</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Post-action review record: strategy effectiveness score, lessons learned, and updated competitive response playbook entry</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Post-action review completed within 5 business days for tier-1 alerts; playbook updated within 10 business days</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Competitive response playbooks are maintained as unstructured documents outside RM systems; institutional knowledge of effective response patterns is lost when analysts rotate, and playbook entries are rarely linked to outcome data</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add NP-RM-11: Corporate & Negotiated Rate Management — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -32,6 +32,7 @@
     <sheet name="NP-RM-08" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="NP-RM-09" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="NP-RM-10" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="NP-RM-11" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1598,13 +1599,21 @@
           <t>Corporate &amp; Negotiated Rate Management</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr"/>
-      <c r="G28" s="8" t="inlineStr"/>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-11</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -18837,7 +18846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N451"/>
+  <dimension ref="A1:N469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -51260,6 +51269,1302 @@
       <c r="N451" s="15" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="452" ht="30" customHeight="1">
+      <c r="A452" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B452" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C452" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D452" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E452" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F452" s="18" t="inlineStr">
+        <is>
+          <t>Receive &amp; log corporate RFP in CRM</t>
+        </is>
+      </c>
+      <c r="G452" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H452" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I452" s="18" t="inlineStr">
+        <is>
+          <t>RFP submission from corporate buyer or TMC (email / GBTA RFP tool)</t>
+        </is>
+      </c>
+      <c r="J452" s="18" t="inlineStr">
+        <is>
+          <t>Qualified lead record with travel volume, routes, and preferred travel dates</t>
+        </is>
+      </c>
+      <c r="K452" s="18" t="inlineStr">
+        <is>
+          <t>RFP response time ≤3 business days; 100% RFPs logged in Salesforce within 24 hrs</t>
+        </is>
+      </c>
+      <c r="L452" s="18" t="inlineStr">
+        <is>
+          <t>RFPs arrive via multiple untracked channels (email, broker portals, GBTA RFP Hub); manual logging causes duplicates and missed responses</t>
+        </is>
+      </c>
+      <c r="M452" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N452" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="453" ht="30" customHeight="1">
+      <c r="A453" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B453" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C453" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D453" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E453" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F453" s="16" t="inlineStr">
+        <is>
+          <t>Assess historical travel volume &amp; route overlap</t>
+        </is>
+      </c>
+      <c r="G453" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H453" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I453" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM opportunity record; prior booking history if existing account</t>
+        </is>
+      </c>
+      <c r="J453" s="16" t="inlineStr">
+        <is>
+          <t>Volume assessment report: annual passenger yield, top 10 routes, seasonality profile</t>
+        </is>
+      </c>
+      <c r="K453" s="16" t="inlineStr">
+        <is>
+          <t>Volume data pull completed within 4 hours of RFP receipt</t>
+        </is>
+      </c>
+      <c r="L453" s="16" t="inlineStr">
+        <is>
+          <t>New corporate accounts have no booking history; reliance on self-reported volume figures that may be overstated by 20–40% to secure deeper discounts</t>
+        </is>
+      </c>
+      <c r="M453" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N453" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="454" ht="30" customHeight="1">
+      <c r="A454" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B454" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C454" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D454" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E454" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F454" s="18" t="inlineStr">
+        <is>
+          <t>Qualify account against minimum volume threshold</t>
+        </is>
+      </c>
+      <c r="G454" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H454" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I454" s="18" t="inlineStr">
+        <is>
+          <t>Volume assessment report from step 1.2</t>
+        </is>
+      </c>
+      <c r="J454" s="18" t="inlineStr">
+        <is>
+          <t>Qualification decision: proceed to negotiation or decline/redirect to SME program</t>
+        </is>
+      </c>
+      <c r="K454" s="18" t="inlineStr">
+        <is>
+          <t>Minimum qualifying threshold: 200 segments/year or $150K annual spend</t>
+        </is>
+      </c>
+      <c r="L454" s="18" t="inlineStr">
+        <is>
+          <t>Sub-threshold accounts consuming senior sales capacity; no automated triage in Salesforce to enforce volume floors consistently across regions</t>
+        </is>
+      </c>
+      <c r="M454" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N454" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="455" ht="30" customHeight="1">
+      <c r="A455" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B455" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C455" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D455" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E455" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F455" s="16" t="inlineStr">
+        <is>
+          <t>Model discount tiers against NRM inventory</t>
+        </is>
+      </c>
+      <c r="G455" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H455" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I455" s="16" t="inlineStr">
+        <is>
+          <t>Qualified account route/volume profile; current O&amp;D bid-price curves from Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="J455" s="16" t="inlineStr">
+        <is>
+          <t>Discount tier matrix (3–5 tiers) with revenue impact per tier at projected volume</t>
+        </is>
+      </c>
+      <c r="K455" s="16" t="inlineStr">
+        <is>
+          <t>Modelled revenue dilution &lt;3% vs. unconstrained mix; analysis completed within 2 business days</t>
+        </is>
+      </c>
+      <c r="L455" s="16" t="inlineStr">
+        <is>
+          <t>NRM bid-price data is point-in-time; discount tiers fixed at contract signing may become revenue-dilutive during high-demand periods without dynamic override capability</t>
+        </is>
+      </c>
+      <c r="M455" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N455" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="456" ht="30" customHeight="1">
+      <c r="A456" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B456" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C456" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D456" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E456" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F456" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark proposed rates vs. ATPCO published fares</t>
+        </is>
+      </c>
+      <c r="G456" s="18" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H456" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I456" s="18" t="inlineStr">
+        <is>
+          <t>Discount tier matrix from step 2.1; ATPCO fare tariff for relevant O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="J456" s="18" t="inlineStr">
+        <is>
+          <t>Competitive rate benchmark showing proposed negotiated fare vs. lowest published fare and competitor filing</t>
+        </is>
+      </c>
+      <c r="K456" s="18" t="inlineStr">
+        <is>
+          <t>Negotiated rate within 5–15% below lowest unrestricted published fare for target markets</t>
+        </is>
+      </c>
+      <c r="L456" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO tariff data has a 48-hour publication lag; competitor last-minute fare reductions not captured, causing negotiated rates to inadvertently undercut market</t>
+        </is>
+      </c>
+      <c r="M456" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N456" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="457" ht="30" customHeight="1">
+      <c r="A457" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B457" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C457" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D457" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E457" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F457" s="16" t="inlineStr">
+        <is>
+          <t>Validate revenue impact against load factor targets</t>
+        </is>
+      </c>
+      <c r="G457" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H457" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I457" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark report from step 2.2; route load factor targets from network plan</t>
+        </is>
+      </c>
+      <c r="J457" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact sign-off: approved discount tier set with floor rates per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K457" s="16" t="inlineStr">
+        <is>
+          <t>Approved rates must preserve projected route load factor ≥83% and RASK within 2% of unconstrained forecast</t>
+        </is>
+      </c>
+      <c r="L457" s="16" t="inlineStr">
+        <is>
+          <t>NRM does not natively model corporate volume displacement of leisure inventory; manual override required to test scenarios on constrained peak departures</t>
+        </is>
+      </c>
+      <c r="M457" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N457" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="458" ht="30" customHeight="1">
+      <c r="A458" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B458" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C458" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D458" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E458" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F458" s="18" t="inlineStr">
+        <is>
+          <t>Draft contract terms and route coverage schedule</t>
+        </is>
+      </c>
+      <c r="G458" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H458" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I458" s="18" t="inlineStr">
+        <is>
+          <t>Approved discount tier set; legal contract template; blackout date calendar</t>
+        </is>
+      </c>
+      <c r="J458" s="18" t="inlineStr">
+        <is>
+          <t>Draft corporate travel agreement: discount schedule, route coverage, blackout dates, minimum commitment, audit rights</t>
+        </is>
+      </c>
+      <c r="K458" s="18" t="inlineStr">
+        <is>
+          <t>Contract draft delivered to corporate buyer within 5 business days of rate approval</t>
+        </is>
+      </c>
+      <c r="L458" s="18" t="inlineStr">
+        <is>
+          <t>Contract templates not version-controlled in Salesforce; legal redlines handled via email, creating misalignment between signed terms and fare filing parameters in ATPCO</t>
+        </is>
+      </c>
+      <c r="M458" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N458" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="459" ht="30" customHeight="1">
+      <c r="A459" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B459" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C459" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D459" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E459" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F459" s="16" t="inlineStr">
+        <is>
+          <t>File private negotiated fares in ATPCO</t>
+        </is>
+      </c>
+      <c r="G459" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H459" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I459" s="16" t="inlineStr">
+        <is>
+          <t>Signed corporate travel agreement; approved discount tier set</t>
+        </is>
+      </c>
+      <c r="J459" s="16" t="inlineStr">
+        <is>
+          <t>Private fare codes filed in ATPCO with account-specific fare basis codes, routing rules, and booking class restrictions</t>
+        </is>
+      </c>
+      <c r="K459" s="16" t="inlineStr">
+        <is>
+          <t>Fare filing completed within 24 hours of contract execution; zero filing errors on first submission</t>
+        </is>
+      </c>
+      <c r="L459" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO private fare filing requires precise fare basis code structuring; errors in Rule 15 (Sales Restrictions) or Rule 35 (Negotiated Fares) cause incorrect TMC access or public leakage of private rates</t>
+        </is>
+      </c>
+      <c r="M459" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N459" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="460" ht="30" customHeight="1">
+      <c r="A460" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B460" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C460" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D460" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E460" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F460" s="18" t="inlineStr">
+        <is>
+          <t>Configure Sabre PRISM access for TMC booking</t>
+        </is>
+      </c>
+      <c r="G460" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H460" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM</t>
+        </is>
+      </c>
+      <c r="I460" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO private fare codes; TMC agency IATA codes from contract</t>
+        </is>
+      </c>
+      <c r="J460" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM corporate account record with pseudo-city codes, negotiated fare credentials, and booking class availability</t>
+        </is>
+      </c>
+      <c r="K460" s="18" t="inlineStr">
+        <is>
+          <t>PRISM configuration active and tested within 48 hours of ATPCO filing; TMC confirmation of successful test booking</t>
+        </is>
+      </c>
+      <c r="L460" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM configuration requires manual pseudo-city mapping for each TMC location; large corporates with 50+ TMC offices create significant setup overhead with no bulk-load API</t>
+        </is>
+      </c>
+      <c r="M460" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N460" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="461" ht="30" customHeight="1">
+      <c r="A461" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B461" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C461" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D461" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E461" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F461" s="16" t="inlineStr">
+        <is>
+          <t>Set up NDC private offer for NDC-enabled corporates</t>
+        </is>
+      </c>
+      <c r="G461" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H461" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I461" s="16" t="inlineStr">
+        <is>
+          <t>Corporate account ID; approved discount tier set; NDC-capable TMC flag from contract</t>
+        </is>
+      </c>
+      <c r="J461" s="16" t="inlineStr">
+        <is>
+          <t>NDC private offer configured with corporate token, ancillary bundle inclusions, and fare eligibility rules</t>
+        </is>
+      </c>
+      <c r="K461" s="16" t="inlineStr">
+        <is>
+          <t>NDC offer live within 72 hours for NDC-enabled accounts; ancillary attach rate target ≥35% on NDC-booked itineraries</t>
+        </is>
+      </c>
+      <c r="L461" s="16" t="inlineStr">
+        <is>
+          <t>NDC adoption among corporate TMCs remains below 30%; ATPCO and NDC offer parameters must be maintained in parallel, creating dual-maintenance risk and version drift between channels</t>
+        </is>
+      </c>
+      <c r="M461" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N461" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="462" ht="30" customHeight="1">
+      <c r="A462" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B462" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C462" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D462" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E462" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F462" s="18" t="inlineStr">
+        <is>
+          <t>Validate fare accessibility across all booked channels</t>
+        </is>
+      </c>
+      <c r="G462" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H462" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I462" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO private fares; Sabre PRISM config; NDC offer (if applicable)</t>
+        </is>
+      </c>
+      <c r="J462" s="18" t="inlineStr">
+        <is>
+          <t>Channel validation report confirming fare availability in Amadeus GDS, Sabre GDS, Travelport GDS, and NDC</t>
+        </is>
+      </c>
+      <c r="K462" s="18" t="inlineStr">
+        <is>
+          <t>100% fare accessibility in contracted channels before contract activation date; zero public display of private fares</t>
+        </is>
+      </c>
+      <c r="L462" s="18" t="inlineStr">
+        <is>
+          <t>GDS fare display inconsistencies across Amadeus, Sabre, and Travelport due to differing cache refresh cycles (up to 4-hour lag); corporate bookers may see incorrect rates during the window</t>
+        </is>
+      </c>
+      <c r="M462" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N462" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="30" customHeight="1">
+      <c r="A463" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B463" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C463" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D463" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E463" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F463" s="16" t="inlineStr">
+        <is>
+          <t>Track monthly booking volume vs. contracted commitment</t>
+        </is>
+      </c>
+      <c r="G463" s="16" t="inlineStr">
+        <is>
+          <t>Corporate Account Analyst</t>
+        </is>
+      </c>
+      <c r="H463" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I463" s="16" t="inlineStr">
+        <is>
+          <t>GDS booking data feed; Amadeus Altéa PSS ticketing records; contract commitment thresholds</t>
+        </is>
+      </c>
+      <c r="J463" s="16" t="inlineStr">
+        <is>
+          <t>Monthly corporate account scorecard: booked segments, revenue, yield vs. target, commitment attainment %</t>
+        </is>
+      </c>
+      <c r="K463" s="16" t="inlineStr">
+        <is>
+          <t>Volume commitment attainment reported by 5th business day of following month; data completeness ≥99% across all channels</t>
+        </is>
+      </c>
+      <c r="L463" s="16" t="inlineStr">
+        <is>
+          <t>Booking data from NDC channel not consistently flowing into Redshift reconciliation pipeline; NDC-booked corporate trips may be excluded from volume commitment tracking, understating attainment</t>
+        </is>
+      </c>
+      <c r="M463" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N463" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="464" ht="30" customHeight="1">
+      <c r="A464" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B464" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C464" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D464" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E464" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F464" s="18" t="inlineStr">
+        <is>
+          <t>Generate quarterly corporate performance report</t>
+        </is>
+      </c>
+      <c r="G464" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H464" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I464" s="18" t="inlineStr">
+        <is>
+          <t>Monthly scorecard data from AWS Redshift; account-level revenue and yield benchmarks</t>
+        </is>
+      </c>
+      <c r="J464" s="18" t="inlineStr">
+        <is>
+          <t>Quarterly business review (QBR) deck: volume trend, route penetration, yield analysis, missed booking analysis</t>
+        </is>
+      </c>
+      <c r="K464" s="18" t="inlineStr">
+        <is>
+          <t>QBR delivered to corporate buyer within 15 business days of quarter close; 100% of tier-1 accounts receive QBR</t>
+        </is>
+      </c>
+      <c r="L464" s="18" t="inlineStr">
+        <is>
+          <t>Manual extraction from Redshift to Tableau for QBR preparation takes 2–3 days per account; no automated QBR generation for the long tail of mid-market accounts (typically 200+ accounts per analyst)</t>
+        </is>
+      </c>
+      <c r="M464" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N464" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="465" ht="30" customHeight="1">
+      <c r="A465" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B465" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C465" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D465" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E465" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F465" s="16" t="inlineStr">
+        <is>
+          <t>Assess volume commitment attainment threshold</t>
+        </is>
+      </c>
+      <c r="G465" s="16" t="inlineStr">
+        <is>
+          <t>Senior Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H465" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I465" s="16" t="inlineStr">
+        <is>
+          <t>Quarterly performance report; contract minimum commitment clause</t>
+        </is>
+      </c>
+      <c r="J465" s="16" t="inlineStr">
+        <is>
+          <t>Attainment decision: compliant (≥85%), at-risk (70–84%), or non-compliant (&lt;70%) classification</t>
+        </is>
+      </c>
+      <c r="K465" s="16" t="inlineStr">
+        <is>
+          <t>≥85% of tier-1 accounts maintaining contracted commitment; non-compliant accounts actioned within 10 business days</t>
+        </is>
+      </c>
+      <c r="L465" s="16" t="inlineStr">
+        <is>
+          <t>Contracts with volume commitment clauses rarely include enforceable penalties; non-compliant accounts may retain full discount tier without commercial consequence, eroding revenue quality</t>
+        </is>
+      </c>
+      <c r="M465" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N465" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="466" ht="30" customHeight="1">
+      <c r="A466" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B466" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C466" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D466" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E466" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F466" s="18" t="inlineStr">
+        <is>
+          <t>Trigger rate adjustment or incentive review</t>
+        </is>
+      </c>
+      <c r="G466" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H466" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I466" s="18" t="inlineStr">
+        <is>
+          <t>Non-compliant or at-risk account classification; current route load factor data from NRM</t>
+        </is>
+      </c>
+      <c r="J466" s="18" t="inlineStr">
+        <is>
+          <t>Rate adjustment proposal: discount tier reduction, incentive bonus offer, or remediation plan submitted to corporate buyer</t>
+        </is>
+      </c>
+      <c r="K466" s="18" t="inlineStr">
+        <is>
+          <t>Rate adjustment applied within 30 days of non-compliance trigger; targeted return to ≥85% commitment attainment within 1 quarter</t>
+        </is>
+      </c>
+      <c r="L466" s="18" t="inlineStr">
+        <is>
+          <t>NRM does not have a corporate account module; rate adjustment modelling must be done manually outside the system, with no automated link between attainment tracking in Salesforce and NRM inventory controls</t>
+        </is>
+      </c>
+      <c r="M466" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N466" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="467" ht="30" customHeight="1">
+      <c r="A467" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B467" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C467" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D467" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E467" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F467" s="16" t="inlineStr">
+        <is>
+          <t>Initiate contract renewal 90 days before expiry</t>
+        </is>
+      </c>
+      <c r="G467" s="16" t="inlineStr">
+        <is>
+          <t>Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H467" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I467" s="16" t="inlineStr">
+        <is>
+          <t>Contract expiry date alert from Salesforce; account performance history</t>
+        </is>
+      </c>
+      <c r="J467" s="16" t="inlineStr">
+        <is>
+          <t>Renewal opportunity record opened in Salesforce; renewal kick-off meeting scheduled with corporate buyer</t>
+        </is>
+      </c>
+      <c r="K467" s="16" t="inlineStr">
+        <is>
+          <t>100% of active contracts have renewal opportunity opened ≥90 days before expiry; zero lapsed contracts due to missed renewal trigger</t>
+        </is>
+      </c>
+      <c r="L467" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce contract expiry alerts not configured for all accounts due to inconsistent contract record hygiene; lapsed contracts default to published fares, triggering reactive re-negotiation with weakened leverage</t>
+        </is>
+      </c>
+      <c r="M467" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N467" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="468" ht="30" customHeight="1">
+      <c r="A468" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B468" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C468" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D468" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E468" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F468" s="18" t="inlineStr">
+        <is>
+          <t>Re-model renewal rates using updated RM forecast</t>
+        </is>
+      </c>
+      <c r="G468" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H468" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I468" s="18" t="inlineStr">
+        <is>
+          <t>Updated O&amp;D demand forecast from NRM; account performance history; competitor rate intelligence from ATPCO</t>
+        </is>
+      </c>
+      <c r="J468" s="18" t="inlineStr">
+        <is>
+          <t>Renewal rate proposal with updated discount tiers, revised route coverage, and projected revenue impact</t>
+        </is>
+      </c>
+      <c r="K468" s="18" t="inlineStr">
+        <is>
+          <t>Renewal rates modelled to deliver ≥2% RASK improvement vs. expiring contract; analysis completed 60 days before expiry</t>
+        </is>
+      </c>
+      <c r="L468" s="18" t="inlineStr">
+        <is>
+          <t>12-month forward NRM forecasts used for renewal modelling have ±8% accuracy on thin routes; locking renewal rates to inaccurate forecasts on marginal routes risks over-discounting into peak periods</t>
+        </is>
+      </c>
+      <c r="M468" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N468" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="469" ht="30" customHeight="1">
+      <c r="A469" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B469" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C469" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D469" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E469" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F469" s="16" t="inlineStr">
+        <is>
+          <t>Approve renewal, renegotiate, or exit account</t>
+        </is>
+      </c>
+      <c r="G469" s="16" t="inlineStr">
+        <is>
+          <t>Director of Corporate Sales</t>
+        </is>
+      </c>
+      <c r="H469" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I469" s="16" t="inlineStr">
+        <is>
+          <t>Renewal rate proposal; account strategic value score; competitive RFP comparison</t>
+        </is>
+      </c>
+      <c r="J469" s="16" t="inlineStr">
+        <is>
+          <t>Renewal decision: signed contract renewal, counter-proposal issued, or account exit with fare code deactivation notice</t>
+        </is>
+      </c>
+      <c r="K469" s="16" t="inlineStr">
+        <is>
+          <t>Tier-1 account renewal rate ≥90%; tier-2 renewal rate ≥75%; exit decision documented in Salesforce within 5 business days of final negotiation</t>
+        </is>
+      </c>
+      <c r="L469" s="16" t="inlineStr">
+        <is>
+          <t>No systematic strategic value scoring model in Salesforce; renewal decisions on borderline accounts rely on relationship judgment rather than data, leading to inconsistent discount policy across the portfolio</t>
+        </is>
+      </c>
+      <c r="M469" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N469" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -59191,6 +60496,1422 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-11 — Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Receive &amp; log corporate RFP in CRM</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>RFP submission from corporate buyer or TMC (email / GBTA RFP tool)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Qualified lead record with travel volume, routes, and preferred travel dates</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>RFP response time ≤3 business days; 100% RFPs logged in Salesforce within 24 hrs</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>RFPs arrive via multiple untracked channels (email, broker portals, GBTA RFP Hub); manual logging causes duplicates and missed responses</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Assess historical travel volume &amp; route overlap</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM opportunity record; prior booking history if existing account</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Volume assessment report: annual passenger yield, top 10 routes, seasonality profile</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>Volume data pull completed within 4 hours of RFP receipt</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>New corporate accounts have no booking history; reliance on self-reported volume figures that may be overstated by 20–40% to secure deeper discounts</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Qualify account against minimum volume threshold</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Volume assessment report from step 1.2</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Qualification decision: proceed to negotiation or decline/redirect to SME program</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Minimum qualifying threshold: 200 segments/year or $150K annual spend</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Sub-threshold accounts consuming senior sales capacity; no automated triage in Salesforce to enforce volume floors consistently across regions</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Model discount tiers against NRM inventory</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Qualified account route/volume profile; current O&amp;D bid-price curves from Amadeus NRM</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Discount tier matrix (3–5 tiers) with revenue impact per tier at projected volume</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Modelled revenue dilution &lt;3% vs. unconstrained mix; analysis completed within 2 business days</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>NRM bid-price data is point-in-time; discount tiers fixed at contract signing may become revenue-dilutive during high-demand periods without dynamic override capability</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Benchmark proposed rates vs. ATPCO published fares</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Discount tier matrix from step 2.1; ATPCO fare tariff for relevant O&amp;D markets</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Competitive rate benchmark showing proposed negotiated fare vs. lowest published fare and competitor filing</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>Negotiated rate within 5–15% below lowest unrestricted published fare for target markets</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO tariff data has a 48-hour publication lag; competitor last-minute fare reductions not captured, causing negotiated rates to inadvertently undercut market</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Validate revenue impact against load factor targets</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Benchmark report from step 2.2; route load factor targets from network plan</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue impact sign-off: approved discount tier set with floor rates per O&amp;D</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Approved rates must preserve projected route load factor ≥83% and RASK within 2% of unconstrained forecast</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>NRM does not natively model corporate volume displacement of leisure inventory; manual override required to test scenarios on constrained peak departures</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Draft contract terms and route coverage schedule</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Sales Manager</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Approved discount tier set; legal contract template; blackout date calendar</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Draft corporate travel agreement: discount schedule, route coverage, blackout dates, minimum commitment, audit rights</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Contract draft delivered to corporate buyer within 5 business days of rate approval</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>Contract templates not version-controlled in Salesforce; legal redlines handled via email, creating misalignment between signed terms and fare filing parameters in ATPCO</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>File private negotiated fares in ATPCO</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Pricing Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Signed corporate travel agreement; approved discount tier set</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Private fare codes filed in ATPCO with account-specific fare basis codes, routing rules, and booking class restrictions</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Fare filing completed within 24 hours of contract execution; zero filing errors on first submission</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO private fare filing requires precise fare basis code structuring; errors in Rule 15 (Sales Restrictions) or Rule 35 (Negotiated Fares) cause incorrect TMC access or public leakage of private rates</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Configure Sabre PRISM access for TMC booking</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO private fare codes; TMC agency IATA codes from contract</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM corporate account record with pseudo-city codes, negotiated fare credentials, and booking class availability</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>PRISM configuration active and tested within 48 hours of ATPCO filing; TMC confirmation of successful test booking</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Sabre PRISM configuration requires manual pseudo-city mapping for each TMC location; large corporates with 50+ TMC offices create significant setup overhead with no bulk-load API</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Set up NDC private offer for NDC-enabled corporates</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Corporate account ID; approved discount tier set; NDC-capable TMC flag from contract</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>NDC private offer configured with corporate token, ancillary bundle inclusions, and fare eligibility rules</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>NDC offer live within 72 hours for NDC-enabled accounts; ancillary attach rate target ≥35% on NDC-booked itineraries</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>NDC adoption among corporate TMCs remains below 30%; ATPCO and NDC offer parameters must be maintained in parallel, creating dual-maintenance risk and version drift between channels</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Validate fare accessibility across all booked channels</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Distribution Analyst</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus GDS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>ATPCO private fares; Sabre PRISM config; NDC offer (if applicable)</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Channel validation report confirming fare availability in Amadeus GDS, Sabre GDS, Travelport GDS, and NDC</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>100% fare accessibility in contracted channels before contract activation date; zero public display of private fares</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>GDS fare display inconsistencies across Amadeus, Sabre, and Travelport due to differing cache refresh cycles (up to 4-hour lag); corporate bookers may see incorrect rates during the window</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Track monthly booking volume vs. contracted commitment</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Corporate Account Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>AWS Redshift</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>GDS booking data feed; Amadeus Altéa PSS ticketing records; contract commitment thresholds</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Monthly corporate account scorecard: booked segments, revenue, yield vs. target, commitment attainment %</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Volume commitment attainment reported by 5th business day of following month; data completeness ≥99% across all channels</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Booking data from NDC channel not consistently flowing into Redshift reconciliation pipeline; NDC-booked corporate trips may be excluded from volume commitment tracking, understating attainment</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Generate quarterly corporate performance report</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Monthly scorecard data from AWS Redshift; account-level revenue and yield benchmarks</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Quarterly business review (QBR) deck: volume trend, route penetration, yield analysis, missed booking analysis</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>QBR delivered to corporate buyer within 15 business days of quarter close; 100% of tier-1 accounts receive QBR</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Manual extraction from Redshift to Tableau for QBR preparation takes 2–3 days per account; no automated QBR generation for the long tail of mid-market accounts (typically 200+ accounts per analyst)</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Assess volume commitment attainment threshold</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Senior Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Quarterly performance report; contract minimum commitment clause</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Attainment decision: compliant (≥85%), at-risk (70–84%), or non-compliant (&lt;70%) classification</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>≥85% of tier-1 accounts maintaining contracted commitment; non-compliant accounts actioned within 10 business days</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Contracts with volume commitment clauses rarely include enforceable penalties; non-compliant accounts may retain full discount tier without commercial consequence, eroding revenue quality</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Trigger rate adjustment or incentive review</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Non-compliant or at-risk account classification; current route load factor data from NRM</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Rate adjustment proposal: discount tier reduction, incentive bonus offer, or remediation plan submitted to corporate buyer</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Rate adjustment applied within 30 days of non-compliance trigger; targeted return to ≥85% commitment attainment within 1 quarter</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>NRM does not have a corporate account module; rate adjustment modelling must be done manually outside the system, with no automated link between attainment tracking in Salesforce and NRM inventory controls</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Initiate contract renewal 90 days before expiry</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Corporate Account Manager</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Contract expiry date alert from Salesforce; account performance history</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Renewal opportunity record opened in Salesforce; renewal kick-off meeting scheduled with corporate buyer</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>100% of active contracts have renewal opportunity opened ≥90 days before expiry; zero lapsed contracts due to missed renewal trigger</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce contract expiry alerts not configured for all accounts due to inconsistent contract record hygiene; lapsed contracts default to published fares, triggering reactive re-negotiation with weakened leverage</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Re-model renewal rates using updated RM forecast</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Revenue Management (NRM)</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Updated O&amp;D demand forecast from NRM; account performance history; competitor rate intelligence from ATPCO</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Renewal rate proposal with updated discount tiers, revised route coverage, and projected revenue impact</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Renewal rates modelled to deliver ≥2% RASK improvement vs. expiring contract; analysis completed 60 days before expiry</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>12-month forward NRM forecasts used for renewal modelling have ±8% accuracy on thin routes; locking renewal rates to inaccurate forecasts on marginal routes risks over-discounting into peak periods</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-11</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Corporate &amp; Negotiated Rate Management</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Approve renewal, renegotiate, or exit account</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Director of Corporate Sales</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce CRM</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Renewal rate proposal; account strategic value score; competitive RFP comparison</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Renewal decision: signed contract renewal, counter-proposal issued, or account exit with fare code deactivation notice</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Tier-1 account renewal rate ≥90%; tier-2 renewal rate ≥75%; exit decision documented in Salesforce within 5 business days of final negotiation</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>No systematic strategic value scoring model in Salesforce; renewal decisions on borderline accounts rely on relationship judgment rather than data, leading to inconsistent discount policy across the portfolio</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add NP-RM-12: Real-Time Availability & Seat Inventory Control — L4 steps, BPMN, slides, wiki page
</commit_message>
<xml_diff>
--- a/data/Airlines_Process_Catalog.xlsx
+++ b/data/Airlines_Process_Catalog.xlsx
@@ -33,6 +33,7 @@
     <sheet name="NP-RM-09" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="NP-RM-10" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="NP-RM-11" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="NP-RM-12" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1636,13 +1637,21 @@
           <t>Real-Time Availability &amp; Seat Inventory Control</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>⏳ Queued</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="10" t="inlineStr"/>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>network-and-pricing/revenue-management/np-rm-12</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -18846,7 +18855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N469"/>
+  <dimension ref="A1:N486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -52563,6 +52572,1230 @@
         </is>
       </c>
       <c r="N469" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="30" customHeight="1">
+      <c r="A470" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B470" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C470" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D470" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E470" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F470" s="18" t="inlineStr">
+        <is>
+          <t>Load authorized capacity &amp; fleet config</t>
+        </is>
+      </c>
+      <c r="G470" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H470" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I470" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment output, aircraft subtype capacity tables</t>
+        </is>
+      </c>
+      <c r="J470" s="18" t="inlineStr">
+        <is>
+          <t>Authorized capacity record per flight-date with cabin split</t>
+        </is>
+      </c>
+      <c r="K470" s="18" t="inlineStr">
+        <is>
+          <t>Capacity load accuracy 100% before sales open</t>
+        </is>
+      </c>
+      <c r="L470" s="18" t="inlineStr">
+        <is>
+          <t>Late fleet swaps from network planning trigger manual capacity corrections in AltéaRM; no automated re-sync with SkyMAX fleet assignment module</t>
+        </is>
+      </c>
+      <c r="M470" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N470" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="471" ht="30" customHeight="1">
+      <c r="A471" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B471" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C471" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D471" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E471" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F471" s="16" t="inlineStr">
+        <is>
+          <t>Initialize fare class booking buckets</t>
+        </is>
+      </c>
+      <c r="G471" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H471" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I471" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare class definitions, historical booking curve by O&amp;D</t>
+        </is>
+      </c>
+      <c r="J471" s="16" t="inlineStr">
+        <is>
+          <t>Booking class hierarchy (Y, B, M, H, Q, K, L, U, T, X) with initial seat counts</t>
+        </is>
+      </c>
+      <c r="K471" s="16" t="inlineStr">
+        <is>
+          <t>All booking classes live ≥14 days before departure; 0 missing bucket errors at booking open</t>
+        </is>
+      </c>
+      <c r="L471" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare class proliferation (20+ classes on competitive routes) increases bucket management complexity; AltéaRM UI does not support bulk bucket edits</t>
+        </is>
+      </c>
+      <c r="M471" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N471" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="472" ht="30" customHeight="1">
+      <c r="A472" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B472" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C472" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D472" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E472" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F472" s="18" t="inlineStr">
+        <is>
+          <t>Apply overbooking factors by flight segment</t>
+        </is>
+      </c>
+      <c r="G472" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H472" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I472" s="18" t="inlineStr">
+        <is>
+          <t>Historical no-show rates, cancellation curves, load factor targets</t>
+        </is>
+      </c>
+      <c r="J472" s="18" t="inlineStr">
+        <is>
+          <t>Authorized booking limit (ABL) per flight exceeding physical capacity</t>
+        </is>
+      </c>
+      <c r="K472" s="18" t="inlineStr">
+        <is>
+          <t>Target involuntary denied boarding rate ≤0.05 per 10,000 passengers</t>
+        </is>
+      </c>
+      <c r="L472" s="18" t="inlineStr">
+        <is>
+          <t>No-show model degrades on routes with recent schedule changes or post-event demand spikes; manual recalibration required in AltéaRM — no auto-retraining trigger</t>
+        </is>
+      </c>
+      <c r="M472" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N472" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="473" ht="30" customHeight="1">
+      <c r="A473" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B473" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C473" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D473" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E473" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F473" s="16" t="inlineStr">
+        <is>
+          <t>Monitor real-time booking pace vs forecast</t>
+        </is>
+      </c>
+      <c r="G473" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H473" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I473" s="16" t="inlineStr">
+        <is>
+          <t>Live booking transactions from Amadeus Altéa PSS, SkyCAST demand forecast</t>
+        </is>
+      </c>
+      <c r="J473" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace index (actual/forecast ratio) per flight per class</t>
+        </is>
+      </c>
+      <c r="K473" s="16" t="inlineStr">
+        <is>
+          <t>Pace variance alert triggered within 15 minutes of threshold breach</t>
+        </is>
+      </c>
+      <c r="L473" s="16" t="inlineStr">
+        <is>
+          <t>AltéaRM polling interval from Altéa PSS is near-real-time but not event-driven; sudden group bookings or flash sales can spike pace index before alert fires</t>
+        </is>
+      </c>
+      <c r="M473" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N473" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="474" ht="30" customHeight="1">
+      <c r="A474" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B474" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C474" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D474" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E474" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F474" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate booking pace deviation threshold</t>
+        </is>
+      </c>
+      <c r="G474" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H474" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I474" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace index, departure date proximity, current load factor</t>
+        </is>
+      </c>
+      <c r="J474" s="18" t="inlineStr">
+        <is>
+          <t>Availability action flag: accelerated close, hold, or open lower class</t>
+        </is>
+      </c>
+      <c r="K474" s="18" t="inlineStr">
+        <is>
+          <t>System recommendation generated within 5 minutes of threshold breach; analyst review SLA ≤30 min</t>
+        </is>
+      </c>
+      <c r="L474" s="18" t="inlineStr">
+        <is>
+          <t>Threshold calibration is static per route cluster — unusual demand patterns (e.g. redirected traffic, airline irregular operations) generate false positive alerts requiring analyst intervention</t>
+        </is>
+      </c>
+      <c r="M474" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N474" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="475" ht="30" customHeight="1">
+      <c r="A475" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B475" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C475" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D475" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E475" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F475" s="16" t="inlineStr">
+        <is>
+          <t>Flag flight for priority availability review</t>
+        </is>
+      </c>
+      <c r="G475" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H475" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I475" s="16" t="inlineStr">
+        <is>
+          <t>Availability action flag from automated pace evaluation</t>
+        </is>
+      </c>
+      <c r="J475" s="16" t="inlineStr">
+        <is>
+          <t>Flight placed in analyst work queue with recommended action and revenue impact estimate</t>
+        </is>
+      </c>
+      <c r="K475" s="16" t="inlineStr">
+        <is>
+          <t>≥90% of flagged flights actioned within analyst SLA; &lt;5% false-positive escalation rate</t>
+        </is>
+      </c>
+      <c r="L475" s="16" t="inlineStr">
+        <is>
+          <t>High-frequency flagging on congested departure banks (e.g. Monday AM banks) overwhelms analyst queues; PROS RM AI prioritisation not yet integrated at this carrier</t>
+        </is>
+      </c>
+      <c r="M475" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N475" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="476" ht="30" customHeight="1">
+      <c r="A476" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B476" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C476" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D476" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E476" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F476" s="18" t="inlineStr">
+        <is>
+          <t>Generate availability adjustment recommendation</t>
+        </is>
+      </c>
+      <c r="G476" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H476" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I476" s="18" t="inlineStr">
+        <is>
+          <t>Current bucket availability, forecast demand, competitive fare filings from ATPCO</t>
+        </is>
+      </c>
+      <c r="J476" s="18" t="inlineStr">
+        <is>
+          <t>Recommended bucket open/close action with projected revenue impact delta</t>
+        </is>
+      </c>
+      <c r="K476" s="18" t="inlineStr">
+        <is>
+          <t>Revenue uplift from accepted recommendations ≥1.5% per adjusted flight vs control group</t>
+        </is>
+      </c>
+      <c r="L476" s="18" t="inlineStr">
+        <is>
+          <t>AltéaRM recommendations do not factor competitor real-time availability in Sabre/Travelport GDS; ATPCO fare data lags competitor filing by up to 2 hours</t>
+        </is>
+      </c>
+      <c r="M476" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N476" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="477" ht="30" customHeight="1">
+      <c r="A477" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B477" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C477" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D477" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E477" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F477" s="16" t="inlineStr">
+        <is>
+          <t>Validate recommendation against RM policy bounds</t>
+        </is>
+      </c>
+      <c r="G477" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H477" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I477" s="16" t="inlineStr">
+        <is>
+          <t>System recommendation, RM policy rules (minimum bucket sizes, blackout dates, alliance blocks)</t>
+        </is>
+      </c>
+      <c r="J477" s="16" t="inlineStr">
+        <is>
+          <t>Approved or overridden availability action</t>
+        </is>
+      </c>
+      <c r="K477" s="16" t="inlineStr">
+        <is>
+          <t>Policy override rate ≤8% of system recommendations; override reason coded for feedback loop</t>
+        </is>
+      </c>
+      <c r="L477" s="16" t="inlineStr">
+        <is>
+          <t>RM policy rules are maintained in AltéaRM configuration tables — change request lead time is 5 business days, creating misalignment during rapid competitive responses</t>
+        </is>
+      </c>
+      <c r="M477" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N477" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="478" ht="30" customHeight="1">
+      <c r="A478" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B478" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C478" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D478" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E478" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F478" s="18" t="inlineStr">
+        <is>
+          <t>Apply manual override with documented reason</t>
+        </is>
+      </c>
+      <c r="G478" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H478" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I478" s="18" t="inlineStr">
+        <is>
+          <t>Out-of-bounds recommendation, analyst market intelligence, competitive intelligence feed</t>
+        </is>
+      </c>
+      <c r="J478" s="18" t="inlineStr">
+        <is>
+          <t>Manually adjusted bucket availability with override reason code logged</t>
+        </is>
+      </c>
+      <c r="K478" s="18" t="inlineStr">
+        <is>
+          <t>Manual override revenue outcome tracked: ≥60% of overrides must outperform system recommendation at T+7 days post-departure</t>
+        </is>
+      </c>
+      <c r="L478" s="18" t="inlineStr">
+        <is>
+          <t>Override audit trail in AltéaRM is flight-level only — no automatic post-departure outcome attribution; manual tracking in spreadsheets introduces error</t>
+        </is>
+      </c>
+      <c r="M478" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N478" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="30" customHeight="1">
+      <c r="A479" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B479" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C479" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D479" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E479" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F479" s="16" t="inlineStr">
+        <is>
+          <t>Broadcast availability updates to all channels</t>
+        </is>
+      </c>
+      <c r="G479" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS (automated)</t>
+        </is>
+      </c>
+      <c r="H479" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I479" s="16" t="inlineStr">
+        <is>
+          <t>Approved bucket availability changes from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J479" s="16" t="inlineStr">
+        <is>
+          <t>Updated availability published to Sabre GDS, Travelport GDS, Amadeus GDS, and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="K479" s="16" t="inlineStr">
+        <is>
+          <t>Availability propagation to all GDS channels within 60 seconds of AltéaRM commit; NDC API latency ≤5 seconds</t>
+        </is>
+      </c>
+      <c r="L479" s="16" t="inlineStr">
+        <is>
+          <t>Sabre and Travelport GDS availability caching can delay display of closed classes by up to 90 seconds — undercuts intended revenue protection window on high-demand flights</t>
+        </is>
+      </c>
+      <c r="M479" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N479" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="480" ht="30" customHeight="1">
+      <c r="A480" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B480" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C480" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D480" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E480" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F480" s="18" t="inlineStr">
+        <is>
+          <t>Receive and assess group booking request</t>
+        </is>
+      </c>
+      <c r="G480" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H480" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I480" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request (pax count, travel date, origin/destination, fare requirements)</t>
+        </is>
+      </c>
+      <c r="J480" s="18" t="inlineStr">
+        <is>
+          <t>Group inventory assessment report: available seats, impact on individual yield</t>
+        </is>
+      </c>
+      <c r="K480" s="18" t="inlineStr">
+        <is>
+          <t>Group quote turnaround ≤4 hours for ≤50 pax; ≤24 hours for &gt;50 pax</t>
+        </is>
+      </c>
+      <c r="L480" s="18" t="inlineStr">
+        <is>
+          <t>Group bookings bypass normal availability controls in Altéa PSS — large groups (&gt;30 pax) can displace higher-yield individual bookings if allotment limits not enforced in real time</t>
+        </is>
+      </c>
+      <c r="M480" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N480" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="481" ht="30" customHeight="1">
+      <c r="A481" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B481" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C481" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D481" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E481" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F481" s="16" t="inlineStr">
+        <is>
+          <t>Validate group request against allotment policy</t>
+        </is>
+      </c>
+      <c r="G481" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H481" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I481" s="16" t="inlineStr">
+        <is>
+          <t>Group assessment report, flight allotment policy (max % of capacity per group), current availability</t>
+        </is>
+      </c>
+      <c r="J481" s="16" t="inlineStr">
+        <is>
+          <t>Approved or rejected group allotment decision with conditional availability hold</t>
+        </is>
+      </c>
+      <c r="K481" s="16" t="inlineStr">
+        <is>
+          <t>Group allotment approval rate within policy: ≥95% handled without senior escalation; group revenue mix target ≤20% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L481" s="16" t="inlineStr">
+        <is>
+          <t>AltéaRM group allotment module requires manual entry of allotment limits per flight — no automated inheritance from network-level group policy, causing inconsistency across the system</t>
+        </is>
+      </c>
+      <c r="M481" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N481" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="482" ht="30" customHeight="1">
+      <c r="A482" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B482" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C482" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D482" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E482" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F482" s="18" t="inlineStr">
+        <is>
+          <t>Confirm group block and adjust net inventory</t>
+        </is>
+      </c>
+      <c r="G482" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H482" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I482" s="18" t="inlineStr">
+        <is>
+          <t>Approved group allotment decision, group fare agreement</t>
+        </is>
+      </c>
+      <c r="J482" s="18" t="inlineStr">
+        <is>
+          <t>Group PNR block confirmed; individual booking class availability reduced by block size</t>
+        </is>
+      </c>
+      <c r="K482" s="18" t="inlineStr">
+        <is>
+          <t>Group block confirmation rate ≥85% within quoted hold period; no-show rate on confirmed groups ≤12%</t>
+        </is>
+      </c>
+      <c r="L482" s="18" t="inlineStr">
+        <is>
+          <t>Group blocks held without deposit reduce effective inventory for individual revenue-maximising bookings — Altéa PSS release rules must be manually configured per group record</t>
+        </is>
+      </c>
+      <c r="M482" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N482" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="483" ht="30" customHeight="1">
+      <c r="A483" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B483" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C483" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D483" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E483" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F483" s="16" t="inlineStr">
+        <is>
+          <t>Conduct T-72h pre-departure inventory review</t>
+        </is>
+      </c>
+      <c r="G483" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H483" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I483" s="16" t="inlineStr">
+        <is>
+          <t>Current booking count, remaining availability, forecast final load factor, waitlist count</t>
+        </is>
+      </c>
+      <c r="J483" s="16" t="inlineStr">
+        <is>
+          <t>Pre-departure availability strategy: sell-up, open low classes, or hold current position</t>
+        </is>
+      </c>
+      <c r="K483" s="16" t="inlineStr">
+        <is>
+          <t>Final load factor target ≥83%; revenue per available seat kilometre (RASK) vs budget reviewed at T-72h</t>
+        </is>
+      </c>
+      <c r="L483" s="16" t="inlineStr">
+        <is>
+          <t>T-72h review is manual and sequential per flight — on banks of 80+ departures, analyst capacity limits force triage; lower-revenue routes reviewed last or skipped entirely</t>
+        </is>
+      </c>
+      <c r="M483" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N483" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="484" ht="30" customHeight="1">
+      <c r="A484" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B484" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C484" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D484" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E484" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F484" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate unsold inventory against threshold</t>
+        </is>
+      </c>
+      <c r="G484" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H484" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I484" s="18" t="inlineStr">
+        <is>
+          <t>Current load factor, departure proximity, unsold seat count, waitlist queue depth</t>
+        </is>
+      </c>
+      <c r="J484" s="18" t="inlineStr">
+        <is>
+          <t>Decision flag: open lower fare classes or maintain current availability strategy</t>
+        </is>
+      </c>
+      <c r="K484" s="18" t="inlineStr">
+        <is>
+          <t>Unsold seat recovery via last-minute availability opening: target ≥65% of exposed seats sold at ≥breakeven yield</t>
+        </is>
+      </c>
+      <c r="L484" s="18" t="inlineStr">
+        <is>
+          <t>Static threshold rules for opening lower classes do not account for connecting passenger itinerary value — opening cheap last-minute classes may dilute O&amp;D revenue on competitive routes</t>
+        </is>
+      </c>
+      <c r="M484" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N484" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="485" ht="30" customHeight="1">
+      <c r="A485" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B485" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C485" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D485" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E485" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F485" s="16" t="inlineStr">
+        <is>
+          <t>Open lower fare classes and clear waitlist</t>
+        </is>
+      </c>
+      <c r="G485" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H485" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I485" s="16" t="inlineStr">
+        <is>
+          <t>Availability action flag, waitlist passenger queue from Altéa PSS</t>
+        </is>
+      </c>
+      <c r="J485" s="16" t="inlineStr">
+        <is>
+          <t>Lower classes opened in AltéaRM; waitlist passengers auto-confirmed via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K485" s="16" t="inlineStr">
+        <is>
+          <t>Waitlist clearance rate ≥90% within 2 hours of class opening; confirmed waitlist pax CSAT ≥4.2/5</t>
+        </is>
+      </c>
+      <c r="L485" s="16" t="inlineStr">
+        <is>
+          <t>Waitlist auto-confirmation in Altéa PSS sends immediate ticketing deadline — passengers who do not respond within 2 hours forfeit the seat, requiring manual re-processing by reservations agents</t>
+        </is>
+      </c>
+      <c r="M485" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N485" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="486" ht="30" customHeight="1">
+      <c r="A486" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B486" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C486" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D486" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E486" s="17" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F486" s="18" t="inlineStr">
+        <is>
+          <t>Freeze availability at check-in cutoff</t>
+        </is>
+      </c>
+      <c r="G486" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS (automated)</t>
+        </is>
+      </c>
+      <c r="H486" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I486" s="18" t="inlineStr">
+        <is>
+          <t>Departure time, check-in cutoff rule (route-specific: 45–90 min before departure)</t>
+        </is>
+      </c>
+      <c r="J486" s="18" t="inlineStr">
+        <is>
+          <t>Availability closed to all booking channels; final booked load factor locked for departure</t>
+        </is>
+      </c>
+      <c r="K486" s="18" t="inlineStr">
+        <is>
+          <t>Check-in cutoff applied accurately on 100% of departures; overbooking resolution (VDB/IDB) initiated within 30 minutes of cutoff if overbooked</t>
+        </is>
+      </c>
+      <c r="L486" s="18" t="inlineStr">
+        <is>
+          <t>Irregular operations (IROPS) delay departures after availability freeze — stranded passengers rebooked on alternate flights consume inventory already frozen for those flights, requiring emergency availability unlocks in Altéa PSS</t>
+        </is>
+      </c>
+      <c r="M486" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N486" s="17" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -61912,6 +63145,1350 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>NP-RM-12 — Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>L1: Network Planning &amp; Scheduling  |  L2: Revenue Management  |  L3: Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Process ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 Domain</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>L2 Process</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>L3 Name</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step #</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L4 Step Name</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Role / Swim Lane</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pain Point / Risk</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Decision Point</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Load authorized capacity &amp; fleet config</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Fleet assignment output, aircraft subtype capacity tables</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Authorized capacity record per flight-date with cabin split</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Capacity load accuracy 100% before sales open</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Late fleet swaps from network planning trigger manual capacity corrections in AltéaRM; no automated re-sync with SkyMAX fleet assignment module</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Initialize fare class booking buckets</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare class definitions, historical booking curve by O&amp;D</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Booking class hierarchy (Y, B, M, H, Q, K, L, U, T, X) with initial seat counts</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>All booking classes live ≥14 days before departure; 0 missing bucket errors at booking open</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>ATPCO fare class proliferation (20+ classes on competitive routes) increases bucket management complexity; AltéaRM UI does not support bulk bucket edits</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Apply overbooking factors by flight segment</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Historical no-show rates, cancellation curves, load factor targets</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Authorized booking limit (ABL) per flight exceeding physical capacity</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Target involuntary denied boarding rate ≤0.05 per 10,000 passengers</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>No-show model degrades on routes with recent schedule changes or post-event demand spikes; manual recalibration required in AltéaRM — no auto-retraining trigger</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Monitor real-time booking pace vs forecast</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Live booking transactions from Amadeus Altéa PSS, SkyCAST demand forecast</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Booking pace index (actual/forecast ratio) per flight per class</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Pace variance alert triggered within 15 minutes of threshold breach</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>AltéaRM polling interval from Altéa PSS is near-real-time but not event-driven; sudden group bookings or flash sales can spike pace index before alert fires</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate booking pace deviation threshold</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Booking pace index, departure date proximity, current load factor</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Availability action flag: accelerated close, hold, or open lower class</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>System recommendation generated within 5 minutes of threshold breach; analyst review SLA ≤30 min</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Threshold calibration is static per route cluster — unusual demand patterns (e.g. redirected traffic, airline irregular operations) generate false positive alerts requiring analyst intervention</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Flag flight for priority availability review</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Availability action flag from automated pace evaluation</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Flight placed in analyst work queue with recommended action and revenue impact estimate</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>≥90% of flagged flights actioned within analyst SLA; &lt;5% false-positive escalation rate</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>High-frequency flagging on congested departure banks (e.g. Monday AM banks) overwhelms analyst queues; PROS RM AI prioritisation not yet integrated at this carrier</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Generate availability adjustment recommendation</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Current bucket availability, forecast demand, competitive fare filings from ATPCO</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>Recommended bucket open/close action with projected revenue impact delta</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>Revenue uplift from accepted recommendations ≥1.5% per adjusted flight vs control group</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>AltéaRM recommendations do not factor competitor real-time availability in Sabre/Travelport GDS; ATPCO fare data lags competitor filing by up to 2 hours</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Validate recommendation against RM policy bounds</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>System recommendation, RM policy rules (minimum bucket sizes, blackout dates, alliance blocks)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Approved or overridden availability action</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Policy override rate ≤8% of system recommendations; override reason coded for feedback loop</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>RM policy rules are maintained in AltéaRM configuration tables — change request lead time is 5 business days, creating misalignment during rapid competitive responses</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Apply manual override with documented reason</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Senior Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Out-of-bounds recommendation, analyst market intelligence, competitive intelligence feed</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>Manually adjusted bucket availability with override reason code logged</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>Manual override revenue outcome tracked: ≥60% of overrides must outperform system recommendation at T+7 days post-departure</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>Override audit trail in AltéaRM is flight-level only — no automatic post-departure outcome attribution; manual tracking in spreadsheets introduces error</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Broadcast availability updates to all channels</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS (automated)</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Approved bucket availability changes from AltéaRM</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Updated availability published to Sabre GDS, Travelport GDS, Amadeus GDS, and NDC API Gateway</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Availability propagation to all GDS channels within 60 seconds of AltéaRM commit; NDC API latency ≤5 seconds</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Sabre and Travelport GDS availability caching can delay display of closed classes by up to 90 seconds — undercuts intended revenue protection window on high-demand flights</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Receive and assess group booking request</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Group booking request (pax count, travel date, origin/destination, fare requirements)</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Group inventory assessment report: available seats, impact on individual yield</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Group quote turnaround ≤4 hours for ≤50 pax; ≤24 hours for &gt;50 pax</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Group bookings bypass normal availability controls in Altéa PSS — large groups (&gt;30 pax) can displace higher-yield individual bookings if allotment limits not enforced in real time</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Validate group request against allotment policy</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Group assessment report, flight allotment policy (max % of capacity per group), current availability</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Approved or rejected group allotment decision with conditional availability hold</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Group allotment approval rate within policy: ≥95% handled without senior escalation; group revenue mix target ≤20% of total flight revenue</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>AltéaRM group allotment module requires manual entry of allotment limits per flight — no automated inheritance from network-level group policy, causing inconsistency across the system</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Confirm group block and adjust net inventory</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales Coordinator</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Approved group allotment decision, group fare agreement</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Group PNR block confirmed; individual booking class availability reduced by block size</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Group block confirmation rate ≥85% within quoted hold period; no-show rate on confirmed groups ≤12%</t>
+        </is>
+      </c>
+      <c r="L16" s="18" t="inlineStr">
+        <is>
+          <t>Group blocks held without deposit reduce effective inventory for individual revenue-maximising bookings — Altéa PSS release rules must be manually configured per group record</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Conduct T-72h pre-departure inventory review</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Current booking count, remaining availability, forecast final load factor, waitlist count</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Pre-departure availability strategy: sell-up, open low classes, or hold current position</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Final load factor target ≥83%; revenue per available seat kilometre (RASK) vs budget reviewed at T-72h</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>T-72h review is manual and sequential per flight — on banks of 80+ departures, analyst capacity limits force triage; lower-revenue routes reviewed last or skipped entirely</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate unsold inventory against threshold</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Current load factor, departure proximity, unsold seat count, waitlist queue depth</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Decision flag: open lower fare classes or maintain current availability strategy</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>Unsold seat recovery via last-minute availability opening: target ≥65% of exposed seats sold at ≥breakeven yield</t>
+        </is>
+      </c>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t>Static threshold rules for opening lower classes do not account for connecting passenger itinerary value — opening cheap last-minute classes may dilute O&amp;D revenue on competitive routes</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Open lower fare classes and clear waitlist</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Revenue Management Analyst</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Amadeus AltéaRM (NRM)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Availability action flag, waitlist passenger queue from Altéa PSS</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>Lower classes opened in AltéaRM; waitlist passengers auto-confirmed via Altéa PSS</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Waitlist clearance rate ≥90% within 2 hours of class opening; confirmed waitlist pax CSAT ≥4.2/5</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Waitlist auto-confirmation in Altéa PSS sends immediate ticketing deadline — passengers who do not respond within 2 hours forfeit the seat, requiring manual re-processing by reservations agents</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>NP-RM-12</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Network Planning &amp; Scheduling</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Management</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Real-Time Availability &amp; Seat Inventory Control</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Freeze availability at check-in cutoff</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS (automated)</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Amadeus Altéa PSS</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Departure time, check-in cutoff rule (route-specific: 45–90 min before departure)</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>Availability closed to all booking channels; final booked load factor locked for departure</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>Check-in cutoff applied accurately on 100% of departures; overbooking resolution (VDB/IDB) initiated within 30 minutes of cutoff if overbooked</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>Irregular operations (IROPS) delay departures after availability freeze — stranded passengers rebooked on alternate flights consume inventory already frozen for those flights, requiring emergency availability unlocks in Altéa PSS</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>